<commit_message>
Kundregler i konteringen, 3108/3308 för EU-försäljning
- Konteringens modeller väljer vilka kundregler som gäller transaktionen
  (src/lib/transaktioner/kundregler.ts) och följer dem. Valet sparas i
  konteringar.regler och visas under förslagen i flödesschemat.
- Första regeln: periodisk sammanställning. EU-försäljning till företag
  bokförs på 3108 (varor) eller 3308 (tjänster), aldrig på 3100.
- 3108 och 3308 inlagda i K1-arbetsboken, k1.json ombyggd (164 konton).
- Tillräckligt?: med köparens utländska VAT-nummer och inget utskrivet
  momsbelopp antas omvänd betalningsskyldighet eller momsfri unionsintern
  varuförsäljning.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/K1_kontobeskrivningar_v1_5.xlsx
+++ b/K1_kontobeskrivningar_v1_5.xlsx
@@ -570,7 +570,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="KontobeskrivningarTable" displayName="KontobeskrivningarTable" ref="A1:Q163" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="KontobeskrivningarTable" displayName="KontobeskrivningarTable" ref="A1:Q165" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="account_number"/>
     <x:tableColumn id="2" name="account_name"/>
@@ -5680,7 +5680,7 @@
         <x:v>Försäljningen hör till företagets normala verksamhet|En dokumenterad momsregel visar att ingen svensk utgående moms ska debiteras|Intäkten ska redovisas på R2 och kan styrkas med försäljningsunderlag</x:v>
       </x:c>
       <x:c r="E99" s="14" t="str">
-        <x:v>Försäljningen är momspliktig; använd 3000|Beloppet är ett offentligt stöd eller bidrag; pröva 3980|Beloppet är vinst vid avyttring av anläggningstillgång; använd 3970|Beloppet är ränta eller annan finansiell intäkt|Momsbehandlingen är bara oklar eller kunden finns utomlands utan att beskattningslandet har utretts|Beloppet är kundförskott över 5 000 kronor för en prestation som inte påbörjats</x:v>
+        <x:v>Försäljningen är momspliktig; använd 3000|Beloppet är ett offentligt stöd eller bidrag; pröva 3980|Beloppet är vinst vid avyttring av anläggningstillgång; använd 3970|Beloppet är ränta eller annan finansiell intäkt|Momsbehandlingen är bara oklar eller kunden finns utomlands utan att beskattningslandet har utretts|Beloppet är kundförskott över 5 000 kronor för en prestation som inte påbörjats|Försäljning av varor till ett företag i ett annat EU-land; använd 3108|Försäljning av tjänster till ett företag i ett annat EU-land; använd 3308</x:v>
       </x:c>
       <x:c r="F99" s="14" t="str">
         <x:v>Identifiera den exakta grunden för att ingen svensk utgående moms ska redovisas|Skilj momsfri svensk omsättning från export, unionsintern försäljning, omsättning utanför landet och transaktion utanför momsens tillämpningsområde|Redovisa intäkten till ersättningen exklusive eventuell utländsk skatt som inte är företagets intäkt|Tillämpa samma K1-justeringar för kundfordringar, ofakturerad försäljning och kundförskott som för momspliktig försäljning|Koppla varje bokning till momskod, deklarationsfält eller dokumenterad orsak till att inget svenskt momsbelopp finns|Stäm av R2 mot försäljningsunderlag, 1500, 2900 och momsdeklaration|Håll R2-intäkter som ingår i nettoomsättningen åtskilda från bidrag och reavinster som inte ingår|Märk varje försäljning som svensk momsfri, export, unionsintern varuförsäljning, tjänst omsatt utomlands eller utanför momsens område|Vid granskningsflagga begär in faktura eller försäljningsunderlag, avtal, kundland och dokumenterad rättslig grund för att svensk utgående moms inte tas ut|Sätt ärendet till väntar på underlag tills momsfri svensk omsättning kan skiljas från export, EU-handel, omsättning utomlands, bidrag och annan intäkt|Godkänn 3100 för dokumenterad momsfri huvudintäkt som ska ingå i nettoomsättningen|Föreslå 3000, 3970, 3980, 8310, rätt utlandskategori eller scope-eskalering när intäktens natur eller momsbehandling är en annan</x:v>
@@ -5719,290 +5719,292 @@
     </x:row>
     <x:row r="100" ht="430" customHeight="1">
       <x:c r="A100" s="14" t="str">
-        <x:v>3200</x:v>
+        <x:v>3108</x:v>
       </x:c>
       <x:c r="B100" s="14" t="str">
-        <x:v>Bil- och bostadsförmån m.m.</x:v>
+        <x:v>Försäljning varor till annat EU-land, momsfri</x:v>
       </x:c>
       <x:c r="C100" s="14" t="str">
-        <x:v>Intäktskonto på R3 för värdet av bil-, bostads- och andra förmåner eller privata nyttjanden som ska tas upp i den enskilda näringsverksamheten. Kontot är motpart till ägarens uttag och avser inte en anställds löneförmån.</x:v>
+        <x:v>Intäktskonto för försäljning av varor till en momsregistrerad köpare i ett annat EU-land, där varan transporteras dit och köparen redovisar momsen. Ingen svensk utgående moms. Redovisas i momsdeklarationens ruta 35 och i den periodiska sammanställningen.</x:v>
       </x:c>
       <x:c r="D100" s="14" t="str">
-        <x:v>Företagaren använder en bil, bostad, lokal eller annan tillgång som är bokförd i företaget privat|Ett uttag av tjänst eller nyttjande av mer än ringa värde ska redovisas|Ett aktuellt och dokumenterat förmånsvärde, marknadsvärde eller föreskrivet schablonvärde har fastställts</x:v>
+        <x:v>Företaget säljer varor till ett företag i ett annat EU-land|Köparen har ett giltigt VAT-nummer från ett annat EU-land|Varan transporteras från Sverige till ett annat EU-land|Ingen svensk utgående moms har debiterats</x:v>
       </x:c>
       <x:c r="E100" s="14" t="str">
-        <x:v>Tillgången är privat och inte bokförd i företaget|Händelsen är uttag av pengar; använd 2013 utan intäktskonto|En vara lämnar företaget permanent; pröva varuuttag på 2011 och relevant uttagsintäkt|Förmånen avser en anställd och ska hanteras i lönesystemet|Privat användning är inte styrkt eller värdet är inte fastställt</x:v>
+        <x:v>Köparen är en privatperson|Köparen är ett svenskt företag; använd 3000|Försäljningen avser tjänster; använd 3308|Varan säljs till ett land utanför EU|Köparens VAT-nummer saknas</x:v>
       </x:c>
       <x:c r="F100" s="14" t="str">
-        <x:v>Verifiera att tillgången eller tjänsten hör till företaget|Identifiera användare, period, omfattning och typ av privat nyttjande|Fastställ värdet enligt aktuell inkomstskatteregel: marknadsvärde exklusive moms eller föreskrivet schablonvärde när sådant finns|Bokför förmånsintäkten på 3200 och ägaruttaget på 2014 enligt dokumenterad konteringsrutin|Bedöm utgående moms separat; momsens beskattningsunderlag behöver inte vara samma som förmånsvärdet|Koppla till körjournal, bostadsberäkning, nyttjandeunderlag eller annan dokumentation|Stäm av årets belopp mot R3 och deklarationsunderlaget|Versionsstyr bilförmåns-, bostadsförmåns- och andra schablonvärden|Använd endast efter manuell bedömning av förmån eller privat nyttjande|Versionsstyr värde per förmånstyp och beskattningsår|Skilj resultatvärde, eget uttag och momsunderlag|Vid granskningsflagga begär in körjournal, nyttjandeunderlag, tillgångsuppgifter och beräkning av förmånsvärde och moms|Sätt ärendet till väntar på underlag tills privat användning, värdering, beskattningsår och motpost på 2014 är verifierade|Godkänn 3200 endast för verifierad förmånsintäkt som hör till företagaren i den enskilda firman|Föreslå 2011, 2013, privat kostnad eller scope-eskalering när posten avser varuuttag, betalning, anställd, bostad eller annat komplicerat upplägg</x:v>
+        <x:v>Kontrollera att köparens VAT-nummer från ett annat EU-land finns på fakturan|Kontrollera att fakturan anger omvänd skattskyldighet eller unionsintern leverans|Bokför hela beloppet utan svensk utgående moms|Försäljningen ska redovisas i ruta 35 och i den periodiska sammanställningen med köparens VAT-nummer|Skilj varor från tjänster; tjänster bokförs på 3308|Godkänn 3108 för dokumenterad varuförsäljning till momsregistrerad köpare i annat EU-land</x:v>
       </x:c>
       <x:c r="G100" s="14" t="str">
-        <x:v>2014|2612|2622|2632|1240|5000</x:v>
+        <x:v>1930|2013|1500</x:v>
       </x:c>
       <x:c r="H100" s="14" t="str">
-        <x:v>Privat användning av en företagsbokförd bil redovisas som förmånsintäkt på 3200 och som eget uttag på 2014 efter fastställd värdering|Eventuell uttagsmoms bokförs separat på rätt momskonto</x:v>
+        <x:v>En webbshop säljer produkter till ett företag i Tyskland med tyskt VAT-nummer; fakturan anger reverse charge och beloppet bokförs på 3108 utan moms</x:v>
       </x:c>
       <x:c r="I100" s="14" t="str">
-        <x:v>Enskild näringsidkare är inte anställd i den egna firman|Förmånsvärdet i inkomstbeskattningen och momsens beskattningsunderlag kan skilja sig|Aktuella schablonvärden får inte hårdkodas utan årsversion|Bil, bostad och fastighet har särskilda regler och kräver normalt manuell granskning|Förmånsvärden får inte hårdkodas eller återanvändas mellan år</x:v>
+        <x:v>Försäljning till privatpersoner i andra EU-länder är inte momsfri på det här sättet|Utan köparens VAT-nummer gäller inte undantaget|Försäljningen ska med i den periodiska sammanställningen</x:v>
       </x:c>
       <x:c r="J100" s="14" t="str">
-        <x:v>bilförmån|bostadsförmån|privat nyttjande|uttag av tjänst|R3|förmånsvärde</x:v>
+        <x:v>EU-försäljning varor|unionsintern försäljning|reverse charge|omvänd skattskyldighet|periodisk sammanställning|ruta 35|VAT-nummer</x:v>
       </x:c>
       <x:c r="K100" s="14" t="str">
-        <x:v>2014|1240|2612|2622|2632|3000</x:v>
+        <x:v>3000|3100|3308</x:v>
       </x:c>
       <x:c r="L100" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 4, konto 3200, rad R3|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.3, 3.1 och 3.17 samt exempel 3-1|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, exempel 5-1, steg 9</x:v>
+        <x:v>BAS-kontoplanen, konto 3108|Skatteverket, momsdeklarationen ruta 35 och periodisk sammanställning</x:v>
       </x:c>
       <x:c r="M100" s="14" t="str">
-        <x:v>Tillgången används både privat och i företaget|Bil, bostad, lokal eller fastighet berörs|Förmånsvärde eller schablonregel saknas|Momsens uttagsregel är oklar|Händelsen kan avse anställd i stället för företagaren|Bil-, bostads- eller annan förmån förekommer</x:v>
+        <x:v>Köparens VAT-nummer saknas eller är svenskt|Det är oklart om köparen är ett företag|Det är oklart om det är varor eller tjänster|Varan har inte lämnat Sverige</x:v>
       </x:c>
       <x:c r="N100" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="O100" s="14" t="n">
-        <x:v>3</x:v>
+      <x:c r="O100" s="14" t="str">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P100" s="14"/>
-      <x:c r="Q100" s="12" t="str"/>
+      <x:c r="Q100" s="14" t="str">
+        <x:v>Tillagt 2026-10-23: EU-försäljning ska inte bokföras på 3100</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="430" customHeight="1">
       <x:c r="A101" s="14" t="str">
-        <x:v>3211</x:v>
+        <x:v>3308</x:v>
       </x:c>
       <x:c r="B101" s="14" t="str">
-        <x:v>Försäljning, positiv VMB</x:v>
+        <x:v>Försäljning tjänster till annat EU-land</x:v>
       </x:c>
       <x:c r="C101" s="14" t="str">
-        <x:v>Försäljningskonto för VMB-transaktioner eller VMB-perioder där försäljningspriset överstiger inköpspriset och marginalen är positiv.</x:v>
+        <x:v>Intäktskonto för försäljning av tjänster till en momsregistrerad köpare i ett annat EU-land enligt huvudregeln, där köparen redovisar momsen. Ingen svensk utgående moms. Redovisas i momsdeklarationens ruta 39 och i den periodiska sammanställningen.</x:v>
       </x:c>
       <x:c r="D101" s="14" t="str">
-        <x:v>Varan omfattas av VMB|Normal VMB ger positiv marginal för varan eller förenklad VMB ger positiv periodmarginal</x:v>
+        <x:v>Företaget säljer tjänster till ett företag i ett annat EU-land|Köparen har ett giltigt VAT-nummer från ett annat EU-land|Fakturan anger omvänd skattskyldighet eller reverse charge|Ingen svensk utgående moms har debiterats</x:v>
       </x:c>
       <x:c r="E101" s="14" t="str">
-        <x:v>Marginalen är negativ; använd 3212|Vanlig moms gäller för hela försäljningspriset|Försäljningen avser omvänd skattskyldighet utan VMB</x:v>
+        <x:v>Köparen är en privatperson|Köparen är ett svenskt företag; använd 3000|Försäljningen avser varor; använd 3108|Köparen finns utanför EU|Tjänsten är knuten till fastighet i Sverige, persontransport, tillträde till evenemang eller restaurang, där andra regler gäller|Köparens VAT-nummer saknas</x:v>
       </x:c>
       <x:c r="F101" s="14" t="str">
-        <x:v>Matcha försäljningen mot rätt VMB-varukostnad|Beräkna utgående moms på den positiva marginalen på 2616, 2626 eller 2636|Håll normal och förenklad VMB spårbara i underlaget|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Kontrollera att köparens VAT-nummer från ett annat EU-land finns på fakturan|Kontrollera att fakturan anger omvänd skattskyldighet eller reverse charge|Bokför hela beloppet utan svensk utgående moms|Försäljningen ska redovisas i ruta 39 och i den periodiska sammanställningen med köparens VAT-nummer|Skilj tjänster från varor; varor bokförs på 3108|Godkänn 3308 för dokumenterad tjänsteförsäljning till momsregistrerad köpare i annat EU-land</x:v>
       </x:c>
       <x:c r="G101" s="14" t="str">
-        <x:v>1930|1500|2616|2626|2636|4211</x:v>
+        <x:v>1930|2013|1500</x:v>
       </x:c>
       <x:c r="H101" s="14" t="str">
-        <x:v>En begagnad vara säljs för mer än inköpspriset och försäljningen bokförs som positiv VMB</x:v>
+        <x:v>En konsult fakturerar ett företag i Danmark med danskt VAT-nummer för ett uppdrag; fakturan anger reverse charge och beloppet bokförs på 3308 utan moms</x:v>
       </x:c>
       <x:c r="I101" s="14" t="str">
-        <x:v>Kontonamnet anger positiv marginal men ersätter inte den underliggande marginalberäkningen|Hela ersättningen ska kunna stämmas av mot kundbetalningen</x:v>
+        <x:v>Försäljning till privatpersoner i andra EU-länder beskattas normalt i Sverige|Vissa tjänster har särskilda regler för omsättningsland|Försäljningen ska med i den periodiska sammanställningen</x:v>
       </x:c>
       <x:c r="J101" s="14" t="str">
-        <x:v>positiv VMB|försäljning begagnade varor|vinstmarginal|VMB-intäkt</x:v>
+        <x:v>EU-försäljning tjänster|reverse charge|omvänd skattskyldighet|periodisk sammanställning|ruta 39|VAT-nummer|konsulttjänst EU</x:v>
       </x:c>
       <x:c r="K101" s="14" t="str">
-        <x:v>3212|2616|2626|2636|4211|1465|1467</x:v>
+        <x:v>3000|3100|3108</x:v>
       </x:c>
       <x:c r="L101" s="14" t="str">
-        <x:v>BAS_FULL_2022, konto 3211|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
+        <x:v>BAS-kontoplanen, konto 3308|Skatteverket, momsdeklarationen ruta 39 och periodisk sammanställning</x:v>
       </x:c>
       <x:c r="M101" s="14" t="str">
-        <x:v>Marginalen eller inköpspriset saknas|Flera momssatser blandas|Det är oklart om normal eller förenklad VMB används</x:v>
+        <x:v>Köparens VAT-nummer saknas eller är svenskt|Det är oklart om köparen är ett företag|Det är oklart om det är varor eller tjänster|Tjänsten kan omfattas av ett undantag från huvudregeln</x:v>
       </x:c>
       <x:c r="N101" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="O101" s="14" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="P101" s="14" t="str"/>
-      <x:c r="Q101" s="12" t="str"/>
+      <x:c r="O101" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P101" s="14"/>
+      <x:c r="Q101" s="14" t="str">
+        <x:v>Tillagt 2026-10-23: EU-försäljning ska inte bokföras på 3100</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" ht="430" customHeight="1">
       <x:c r="A102" s="14" t="str">
-        <x:v>3212</x:v>
+        <x:v>3200</x:v>
       </x:c>
       <x:c r="B102" s="14" t="str">
-        <x:v>Försäljning, negativ VMB</x:v>
+        <x:v>Bil- och bostadsförmån m.m.</x:v>
       </x:c>
       <x:c r="C102" s="14" t="str">
-        <x:v>Försäljningskonto för VMB-transaktioner eller VMB-perioder där försäljningspriset understiger inköpspriset och marginalen är negativ.</x:v>
+        <x:v>Intäktskonto på R3 för värdet av bil-, bostads- och andra förmåner eller privata nyttjanden som ska tas upp i den enskilda näringsverksamheten. Kontot är motpart till ägarens uttag och avser inte en anställds löneförmån.</x:v>
       </x:c>
       <x:c r="D102" s="14" t="str">
-        <x:v>Varan omfattas av VMB|Normal VMB ger negativ marginal för varan eller förenklad VMB ger negativ periodmarginal</x:v>
+        <x:v>Företagaren använder en bil, bostad, lokal eller annan tillgång som är bokförd i företaget privat|Ett uttag av tjänst eller nyttjande av mer än ringa värde ska redovisas|Ett aktuellt och dokumenterat förmånsvärde, marknadsvärde eller föreskrivet schablonvärde har fastställts</x:v>
       </x:c>
       <x:c r="E102" s="14" t="str">
-        <x:v>Marginalen är positiv; använd 3211|Vanlig moms gäller|En lagernedskrivning bokförs utan försäljning</x:v>
+        <x:v>Tillgången är privat och inte bokförd i företaget|Händelsen är uttag av pengar; använd 2013 utan intäktskonto|En vara lämnar företaget permanent; pröva varuuttag på 2011 och relevant uttagsintäkt|Förmånen avser en anställd och ska hanteras i lönesystemet|Privat användning är inte styrkt eller värdet är inte fastställt</x:v>
       </x:c>
       <x:c r="F102" s="14" t="str">
-        <x:v>Matcha försäljningen mot rätt VMB-varukostnad på 4212|Bokför ingen negativ utgående moms|Vid förenklad VMB ska eventuell framåtförd negativ marginal följas separat enligt momsreglerna|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Verifiera att tillgången eller tjänsten hör till företaget|Identifiera användare, period, omfattning och typ av privat nyttjande|Fastställ värdet enligt aktuell inkomstskatteregel: marknadsvärde exklusive moms eller föreskrivet schablonvärde när sådant finns|Bokför förmånsintäkten på 3200 och ägaruttaget på 2014 enligt dokumenterad konteringsrutin|Bedöm utgående moms separat; momsens beskattningsunderlag behöver inte vara samma som förmånsvärdet|Koppla till körjournal, bostadsberäkning, nyttjandeunderlag eller annan dokumentation|Stäm av årets belopp mot R3 och deklarationsunderlaget|Versionsstyr bilförmåns-, bostadsförmåns- och andra schablonvärden|Använd endast efter manuell bedömning av förmån eller privat nyttjande|Versionsstyr värde per förmånstyp och beskattningsår|Skilj resultatvärde, eget uttag och momsunderlag|Vid granskningsflagga begär in körjournal, nyttjandeunderlag, tillgångsuppgifter och beräkning av förmånsvärde och moms|Sätt ärendet till väntar på underlag tills privat användning, värdering, beskattningsår och motpost på 2014 är verifierade|Godkänn 3200 endast för verifierad förmånsintäkt som hör till företagaren i den enskilda firman|Föreslå 2011, 2013, privat kostnad eller scope-eskalering när posten avser varuuttag, betalning, anställd, bostad eller annat komplicerat upplägg</x:v>
       </x:c>
       <x:c r="G102" s="14" t="str">
-        <x:v>1930|1500|4212</x:v>
+        <x:v>2014|2612|2622|2632|1240|5000</x:v>
       </x:c>
       <x:c r="H102" s="14" t="str">
-        <x:v>En VMB-vara säljs för mindre än inköpspriset och försäljningen klassificeras som negativ VMB</x:v>
+        <x:v>Privat användning av en företagsbokförd bil redovisas som förmånsintäkt på 3200 och som eget uttag på 2014 efter fastställd värdering|Eventuell uttagsmoms bokförs separat på rätt momskonto</x:v>
       </x:c>
       <x:c r="I102" s="14" t="str">
-        <x:v>Negativ marginal får inte användas för att minska moms på positiva marginaler när reglerna inte medger det|Ingen utgående VMB-moms bokförs på en negativ marginal</x:v>
+        <x:v>Enskild näringsidkare är inte anställd i den egna firman|Förmånsvärdet i inkomstbeskattningen och momsens beskattningsunderlag kan skilja sig|Aktuella schablonvärden får inte hårdkodas utan årsversion|Bil, bostad och fastighet har särskilda regler och kräver normalt manuell granskning|Förmånsvärden får inte hårdkodas eller återanvändas mellan år</x:v>
       </x:c>
       <x:c r="J102" s="14" t="str">
-        <x:v>negativ VMB|förlustmarginal|försäljning begagnade varor|VMB-intäkt</x:v>
+        <x:v>bilförmån|bostadsförmån|privat nyttjande|uttag av tjänst|R3|förmånsvärde</x:v>
       </x:c>
       <x:c r="K102" s="14" t="str">
-        <x:v>3211|4212|1465|1467|2616|2626|2636</x:v>
+        <x:v>2014|1240|2612|2622|2632|3000</x:v>
       </x:c>
       <x:c r="L102" s="14" t="str">
-        <x:v>BAS_FULL_2022, konto 3212|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 4, konto 3200, rad R3|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.3, 3.1 och 3.17 samt exempel 3-1|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, exempel 5-1, steg 9</x:v>
       </x:c>
       <x:c r="M102" s="14" t="str">
-        <x:v>All negativ marginal vid förenklad VMB|Marginalen eller inköpspriset saknas|Kvittning mot positiva marginaler övervägs</x:v>
+        <x:v>Tillgången används både privat och i företaget|Bil, bostad, lokal eller fastighet berörs|Förmånsvärde eller schablonregel saknas|Momsens uttagsregel är oklar|Händelsen kan avse anställd i stället för företagaren|Bil-, bostads- eller annan förmån förekommer</x:v>
       </x:c>
       <x:c r="N102" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O102" s="14" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="P102" s="14" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P102" s="14"/>
       <x:c r="Q102" s="12" t="str"/>
     </x:row>
     <x:row r="103" ht="430" customHeight="1">
       <x:c r="A103" s="14" t="str">
-        <x:v>3500</x:v>
+        <x:v>3211</x:v>
       </x:c>
       <x:c r="B103" s="14" t="str">
-        <x:v>Fakturerade kostnader</x:v>
+        <x:v>Försäljning, positiv VMB</x:v>
       </x:c>
       <x:c r="C103" s="14" t="str">
-        <x:v>Intäkter när företaget först har haft en kostnad i eget namn och sedan tar betalt av kunden för den, till exempel frakt, emballage, faktureringsavgift eller resa. Den ursprungliga kostnaden ligger kvar som kostnad och ersättningen bokförs som försäljning.</x:v>
+        <x:v>Försäljningskonto för VMB-transaktioner eller VMB-perioder där försäljningspriset överstiger inköpspriset och marginalen är positiv.</x:v>
       </x:c>
       <x:c r="D103" s="14" t="str">
-        <x:v>Företaget har köpt varan eller tjänsten i eget namn och ansvarat för betalningen|Kunden debiteras för exempelvis frakt, emballage, faktureringsavgift eller resekostnad som en del av företagets egen försäljning|Underlaget visar vad som har fakturerats och vilken moms som gäller för försäljningen</x:v>
+        <x:v>Varan omfattas av VMB|Normal VMB ger positiv marginal för varan eller förenklad VMB ger positiv periodmarginal</x:v>
       </x:c>
       <x:c r="E103" s="14" t="str">
-        <x:v>Företaget har bara gjort ett verkligt utlägg för kundens räkning där kunden själv är betalningsskyldig; bokför då inte ersättningen som egen intäkt|Beloppet är den egentliga försäljningen av en vara eller tjänst; använd relevant försäljningskonto|Posten avser EU-land eller export och momshanteringen inte är säker|Tull- eller speditionskostnaden kan vara ett utlägg eller hör till varuinköpet|Underlaget är ospecificerat eller kontot används som restkonto</x:v>
+        <x:v>Marginalen är negativ; använd 3212|Vanlig moms gäller för hela försäljningspriset|Försäljningen avser omvänd skattskyldighet utan VMB</x:v>
       </x:c>
       <x:c r="F103" s="14" t="str">
-        <x:v>Kontrollera först i vems namn kostnaden uppkom: företagets eget namn talar för vidarefakturering, kundens namn för verkligt utlägg|Vid vidarefakturering ligger den ursprungliga kostnaden kvar och kundens ersättning bokförs som företagets intäkt|Vid verkligt utlägg ska beloppet normalt inte påverka företagets resultat|BAS 3510, 3511, 3518, 3520, 3540 och 3550 får sammanföras automatiskt till 3500 när kontots innebörd stämmer|BAS 3518 behåller sitt tecken så att returnerat emballage minskar intäkten|BAS 3500 och 3590 kräver specificering eftersom de är generella konton|BAS 3521, 3522, 3541 och 3542 kräver kontroll av kundland och moms|BAS 3530 kräver kontroll av om posten är egen vidarefakturering, verkligt utlägg eller del av ett varuinköp|Använd samma momsbedömning som för den försäljning som den fakturerade kostnaden hör till|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Matcha försäljningen mot rätt VMB-varukostnad|Beräkna utgående moms på den positiva marginalen på 2616, 2626 eller 2636|Håll normal och förenklad VMB spårbara i underlaget|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G103" s="14" t="str">
-        <x:v>1510|1930|3000|4000|5700|5800</x:v>
+        <x:v>1930|1500|2616|2626|2636|4211</x:v>
       </x:c>
       <x:c r="H103" s="14" t="str">
-        <x:v>Företaget betalar frakten i eget namn och tar sedan betalt av kunden; fraktkostnaden ligger kvar och ersättningen bokförs på 3500|Företaget tar ut en faktureringsavgift av kunden och bokför avgiften som intäkt på 3500|Kunden står själv på kvittot och företaget får exakt samma belopp tillbaka; kontrollera om det är ett verkligt utlägg och inte egen försäljning|Returnerat emballage bokförs med bevarat tecken så att intäkten minskar</x:v>
+        <x:v>En begagnad vara säljs för mer än inköpspriset och försäljningen bokförs som positiv VMB</x:v>
       </x:c>
       <x:c r="I103" s="14" t="str">
-        <x:v>Blanda inte ihop vidarefakturering med verkligt utlägg|Att kunden ersätter kostnaden gör inte automatiskt posten till ett utlägg|EU-, export-, tull- och speditionsposter kräver kontroll innan bokföringen godkänns|3500 får inte användas som ospecificerat restkonto|Spara kostnadsunderlaget och kopplingen till kundfakturan</x:v>
+        <x:v>Kontonamnet anger positiv marginal men ersätter inte den underliggande marginalberäkningen|Hela ersättningen ska kunna stämmas av mot kundbetalningen</x:v>
       </x:c>
       <x:c r="J103" s="14" t="str">
-        <x:v>fakturerade kostnader|vidarefakturering|utlägg|kundersättning|R1|påslag</x:v>
+        <x:v>positiv VMB|försäljning begagnade varor|vinstmarginal|VMB-intäkt</x:v>
       </x:c>
       <x:c r="K103" s="14" t="str">
-        <x:v>3000|1510|4000|5700|5800</x:v>
+        <x:v>3212|2616|2626|2636|4211|1465|1467</x:v>
       </x:c>
       <x:c r="L103" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 4, konto 3500, rad R1|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 7.1|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sambandet mellan affärshändelser</x:v>
+        <x:v>BAS_FULL_2022, konto 3211|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
       </x:c>
       <x:c r="M103" s="14" t="str">
-        <x:v>Det är oklart om kostnaden uppkom i företagets eller kundens namn|Posten kan vara ett verkligt utlägg|Kunden finns i ett annat land eller momshanteringen är oklar|Posten avser tull eller spedition|BAS-kontot är 3500 eller 3590 och underlaget är inte tillräckligt specificerat</x:v>
+        <x:v>Marginalen eller inköpspriset saknas|Flera momssatser blandas|Det är oklart om normal eller förenklad VMB används</x:v>
       </x:c>
       <x:c r="N103" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O103" s="14" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P103" s="14" t="str">
-        <x:v>customer_advance_over_5000</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P103" s="14" t="str"/>
       <x:c r="Q103" s="12" t="str"/>
     </x:row>
     <x:row r="104" ht="430" customHeight="1">
       <x:c r="A104" s="14" t="str">
-        <x:v>3700</x:v>
+        <x:v>3212</x:v>
       </x:c>
       <x:c r="B104" s="14" t="str">
-        <x:v>Lämnade rabatter, bonus etc.</x:v>
+        <x:v>Försäljning, negativ VMB</x:v>
       </x:c>
       <x:c r="C104" s="14" t="str">
-        <x:v>K1-konto på R1 eller R2 för rabatter, bonusar och andra verkliga prisnedsättningar som företaget lämnar till sina kunder. Beloppet minskar den ursprungliga försäljningen.</x:v>
+        <x:v>Försäljningskonto för VMB-transaktioner eller VMB-perioder där försäljningspriset understiger inköpspriset och marginalen är negativ.</x:v>
       </x:c>
       <x:c r="D104" s="14" t="str">
-        <x:v>Företaget lämnar rabatt, bonus eller återbäring som sänker priset på en försäljning|Prisnedsättningen kan kopplas till en kund, försäljning och momssats|Det finns kreditnota, bonusavtal eller annat underlag som visar nedsättningen|Beloppet avser normal öres- eller kronutjämning i samband med försäljning</x:v>
+        <x:v>Varan omfattas av VMB|Normal VMB ger negativ marginal för varan eller förenklad VMB ger negativ periodmarginal</x:v>
       </x:c>
       <x:c r="E104" s="14" t="str">
-        <x:v>Beloppet är reklam, gåva, representation eller annan marknadsföringskostnad|Beloppet är kundförlust, ackord eller skadestånd och inte en verklig prisnedsättning|Beloppet är en rabatt som företaget själv har fått vid inköp; använd 4700|Posten avser punktskatt; detta ligger utanför tjänstens standardomfattning|Posten saknar koppling till en försäljning eller underlag för momshanteringen</x:v>
+        <x:v>Marginalen är positiv; använd 3211|Vanlig moms gäller|En lagernedskrivning bokförs utan försäljning</x:v>
       </x:c>
       <x:c r="F104" s="14" t="str">
-        <x:v>Kontrollera att händelsen är en verklig prisnedsättning och inte en kostnad eller kundförlust|Koppla rabatten till ursprungsförsäljningen och använd samma momssats|Kräv kreditnota eller annat dokumenterat underlag när priset sätts ned i efterhand|BAS 3730, 3731, 3732 och 3740 får sammanföras automatiskt till 3700|BAS 3700, 3710 och 3790 kräver kontroll eftersom kontona är generella eller ofördelade|BAS 3750, 3751 och 3752 avser punktskatter och ligger utanför standardflödet|Fördela beloppet mellan R1 och R2 om rabatten avser både momspliktig och momsfri försäljning|Stäm av kreditnota eller bonus mot kundfordran, betalning och redovisad försäljning|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Matcha försäljningen mot rätt VMB-varukostnad på 4212|Bokför ingen negativ utgående moms|Vid förenklad VMB ska eventuell framåtförd negativ marginal följas separat enligt momsreglerna|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G104" s="14" t="str">
-        <x:v>1500|1910|1930|2610|2620|2630|3000|3100</x:v>
+        <x:v>1930|1500|4212</x:v>
       </x:c>
       <x:c r="H104" s="14" t="str">
-        <x:v>En kreditnota för en tidigare försäljning bokförs som minskad försäljning på 3700 och minskad utgående moms med samma momssats som originalfakturan|En dokumenterad årsbonus till en kund bokförs på 3700 och fördelas efter de försäljningar och momssatser som bonusen avser|Normal öresutjämning från en kundbetalning sammanförs till 3700</x:v>
+        <x:v>En VMB-vara säljs för mindre än inköpspriset och försäljningen klassificeras som negativ VMB</x:v>
       </x:c>
       <x:c r="I104" s="14" t="str">
-        <x:v>Rabatten ska minska försäljningen och inte bokföras som en vanlig kostnad|Momsjusteringen måste följa ursprungsförsäljningen|Generella intäktskorrigeringar utan underlag eller momssats ska granskas|Kundförlust, skadestånd och rabatt är olika händelser|Punktskatter får inte behandlas som kundrabatter</x:v>
+        <x:v>Negativ marginal får inte användas för att minska moms på positiva marginaler när reglerna inte medger det|Ingen utgående VMB-moms bokförs på en negativ marginal</x:v>
       </x:c>
       <x:c r="J104" s="14" t="str">
-        <x:v>lämnad rabatt|bonus|återbäring|kreditnota|prisnedsättning|öresutjämning|R1|R2</x:v>
+        <x:v>negativ VMB|förlustmarginal|försäljning begagnade varor|VMB-intäkt</x:v>
       </x:c>
       <x:c r="K104" s="14" t="str">
-        <x:v>3000|3100|3500|4700|1500|2610|2620|2630</x:v>
+        <x:v>3211|4212|1465|1467|2616|2626|2636</x:v>
       </x:c>
       <x:c r="L104" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – konto 3700, rad R1/R2|BFNAR 2006:1 senast ändrat genom BFNAR 2025:1, definitionen av nettoomsättning och punkt 7.1|Skatteverkets rättsliga vägledning om kreditnota och prisnedsättning i efterhand, 2026</x:v>
+        <x:v>BAS_FULL_2022, konto 3212|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
       </x:c>
       <x:c r="M104" s="14" t="str">
-        <x:v>Posten kommer från BAS 3700, 3710 eller 3790|Ursprungsförsäljning, kund eller momssats saknas|Händelsen kan vara kundförlust, kostnad, reklamation eller skadestånd i stället för rabatt|Kreditnota eller bonusunderlag saknas|Rabatten avser flera momssatser eller både momspliktig och momsfri försäljning</x:v>
+        <x:v>All negativ marginal vid förenklad VMB|Marginalen eller inköpspriset saknas|Kvittning mot positiva marginaler övervägs</x:v>
       </x:c>
       <x:c r="N104" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O104" s="14" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P104" s="14"/>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P104" s="14" t="str"/>
       <x:c r="Q104" s="12" t="str"/>
     </x:row>
     <x:row r="105" ht="430" customHeight="1">
       <x:c r="A105" s="14" t="str">
-        <x:v>3900</x:v>
+        <x:v>3500</x:v>
       </x:c>
       <x:c r="B105" s="14" t="str">
-        <x:v>Övriga rörelseintäkter</x:v>
+        <x:v>Fakturerade kostnader</x:v>
       </x:c>
       <x:c r="C105" s="14" t="str">
-        <x:v>Samlingskonto på R1 eller R2 för rörelseintäkter som hör till företaget men inte är huvudförsäljning, fakturerade kostnader, förmåner, vinst vid anläggningstillgångsförsäljning eller erhållna bidrag.</x:v>
+        <x:v>Intäkter när företaget först har haft en kostnad i eget namn och sedan tar betalt av kunden för den, till exempel frakt, emballage, faktureringsavgift eller resa. Den ursprungliga kostnaden ligger kvar som kostnad och ersättningen bokförs som försäljning.</x:v>
       </x:c>
       <x:c r="D105" s="14" t="str">
-        <x:v>Inkomsten är sekundär i förhållande till företagets normala huvudverksamhet|Inkomsten hör till rörelsen och ska redovisas på R1 eller R2|Inkomstens art, momsbehandling och redovisningstidpunkt är dokumenterade|En tidigare direkt kostnadsförd inventarie säljs</x:v>
+        <x:v>Företaget har köpt varan eller tjänsten i eget namn och ansvarat för betalningen|Kunden debiteras för exempelvis frakt, emballage, faktureringsavgift eller resekostnad som en del av företagets egen försäljning|Underlaget visar vad som har fakturerats och vilken moms som gäller för försäljningen</x:v>
       </x:c>
       <x:c r="E105" s="14" t="str">
-        <x:v>Inkomsten är normal huvudförsäljning; använd 3000 eller 3100|Beloppet är fakturerad kostnad, bil- eller bostadsförmån, anläggningstillgångsvinst eller bidrag|Beloppet är ränteintäkt eller annan finansiell intäkt|Beloppet hör till privatpersonen|Inkomstens art är okänd och 3900 används som restkonto|Intäkten avser säkringsinstrument eller annan avancerad finansiell transaktion|Intäkten förutsätter anställda, exempelvis sjuklöneersättning</x:v>
+        <x:v>Företaget har bara gjort ett verkligt utlägg för kundens räkning där kunden själv är betalningsskyldig; bokför då inte ersättningen som egen intäkt|Beloppet är den egentliga försäljningen av en vara eller tjänst; använd relevant försäljningskonto|Posten avser EU-land eller export och momshanteringen inte är säker|Tull- eller speditionskostnaden kan vara ett utlägg eller hör till varuinköpet|Underlaget är ospecificerat eller kontot används som restkonto</x:v>
       </x:c>
       <x:c r="F105" s="14" t="str">
-        <x:v>Identifiera inkomsttypen och dokumentera varför den är en sekundär rörelseintäkt|Fastställ om intäkten ska redovisas på R1 eller R2, om den ingår i nettoomsättningen och om utgående moms ska redovisas|Hyres- och arrendeintäkter kräver manuell granskning; frivillig beskattning för lokaluthyrning får aldrig hanteras automatiskt|Konfliktersättning, skadestånd, gåvor, försäkringsersättning och skuldackord kräver manuell granskning av grund, skatteplikt, moms och koppling till kostnad, tillgång eller skuld|Säkringsinstrument och orealiserade värdeförändringar ligger utanför tjänstens standardomfattning|Sjuklöneersättning och andra intäkter som förutsätter anställda ligger utanför tjänstens målgrupp|För försäljning av en tidigare direkt kostnadsförd inventarie: bokför ersättningen på 3900 och redovisa eventuell utgående moms separat|Fördela inkomsten över flera år endast när det är uppenbart att den avser flera år enligt K1|Kontrollera om ersättningen i stället ska påverka en tillgångs anskaffningsvärde, en vinst vid avyttring, ett bidrag eller en kostnad|Koppla intäkten till dokumenterad kategori och motpart och stäm av fordran, bankbetalning och efterföljande reglering|Blockera ospecificerade bokningar och använd aldrig 3900 som restkonto för okända insättningar</x:v>
+        <x:v>Kontrollera först i vems namn kostnaden uppkom: företagets eget namn talar för vidarefakturering, kundens namn för verkligt utlägg|Vid vidarefakturering ligger den ursprungliga kostnaden kvar och kundens ersättning bokförs som företagets intäkt|Vid verkligt utlägg ska beloppet normalt inte påverka företagets resultat|BAS 3510, 3511, 3518, 3520, 3540 och 3550 får sammanföras automatiskt till 3500 när kontots innebörd stämmer|BAS 3518 behåller sitt tecken så att returnerat emballage minskar intäkten|BAS 3500 och 3590 kräver specificering eftersom de är generella konton|BAS 3521, 3522, 3541 och 3542 kräver kontroll av kundland och moms|BAS 3530 kräver kontroll av om posten är egen vidarefakturering, verkligt utlägg eller del av ett varuinköp|Använd samma momsbedömning som för den försäljning som den fakturerade kostnaden hör till|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G105" s="14" t="str">
-        <x:v>1600|1500|1910|1930|2610|2620|2630</x:v>
+        <x:v>1510|1930|3000|4000|5700|5800</x:v>
       </x:c>
       <x:c r="H105" s="14" t="str">
-        <x:v>En dokumenterad sekundär provisions- eller licensintäkt kan bokföras på 3900 med rätt momsbehandling|Hyresintäkt eller försäkringsersättning skickas till manuell granskning innan konto och moms fastställs|En tidigare kostnadsförd dator säljs och ersättningen bokförs på 3900 med eventuell moms separat</x:v>
+        <x:v>Företaget betalar frakten i eget namn och tar sedan betalt av kunden; fraktkostnaden ligger kvar och ersättningen bokförs på 3500|Företaget tar ut en faktureringsavgift av kunden och bokför avgiften som intäkt på 3500|Kunden står själv på kvittot och företaget får exakt samma belopp tillbaka; kontrollera om det är ett verkligt utlägg och inte egen försäljning|Returnerat emballage bokförs med bevarat tecken så att intäkten minskar</x:v>
       </x:c>
       <x:c r="I105" s="14" t="str">
-        <x:v>3900 får inte bli ett restkonto för okända insättningar|R1 eller R2, nettoomsättning och momsbehandling måste fastställas per intäkt|Hyresintäkter, försäkringsersättning, skadestånd, gåvor och skuldackord kräver manuell granskning|Sekundär intäkt kan ändå ingå i nettoomsättningen beroende på verksamheten|Använd inte 1222 när tillgången aldrig har ingått i inventariegruppen|Säkringsinstrument och personalrelaterade ersättningar ligger utanför standardtjänsten</x:v>
+        <x:v>Blanda inte ihop vidarefakturering med verkligt utlägg|Att kunden ersätter kostnaden gör inte automatiskt posten till ett utlägg|EU-, export-, tull- och speditionsposter kräver kontroll innan bokföringen godkänns|3500 får inte användas som ospecificerat restkonto|Spara kostnadsunderlaget och kopplingen till kundfakturan</x:v>
       </x:c>
       <x:c r="J105" s="14" t="str">
-        <x:v>övrig rörelseintäkt|sekundär intäkt|försäkringsersättning|skadestånd|R1|R2</x:v>
+        <x:v>fakturerade kostnader|vidarefakturering|utlägg|kundersättning|R1|påslag</x:v>
       </x:c>
       <x:c r="K105" s="14" t="str">
-        <x:v>3000|3100|3500|3970|3980|1600|8310</x:v>
+        <x:v>3000|1510|4000|5700|5800</x:v>
       </x:c>
       <x:c r="L105" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 3900, rad R1/R2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.17 och 7.2|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sidoordnad specifikation|Skatteverket – Uthyrning av fastighet och frivillig beskattning, kontrollerat 2026-09-20</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 4, konto 3500, rad R1|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 7.1|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sambandet mellan affärshändelser</x:v>
       </x:c>
       <x:c r="M105" s="14" t="str">
-        <x:v>Intäktstyp, redovisningsrad eller momsbehandling är oklar|Hyres- eller arrendeintäkt förekommer|Försäkringsersättning, konfliktersättning, skadestånd, gåva eller skuldackord förekommer|Intäkten kan vara huvudförsäljning, bidrag, vinst vid avyttring eller finansiell intäkt|Beslut, avtal eller annan dokumentation saknas|Intäkten kan påverka en tillgång, kostnad eller skuld på annat sätt än som vanlig rörelseintäkt</x:v>
+        <x:v>Det är oklart om kostnaden uppkom i företagets eller kundens namn|Posten kan vara ett verkligt utlägg|Kunden finns i ett annat land eller momshanteringen är oklar|Posten avser tull eller spedition|BAS-kontot är 3500 eller 3590 och underlaget är inte tillräckligt specificerat</x:v>
       </x:c>
       <x:c r="N105" s="14" t="str">
         <x:v>active</x:v>
@@ -6010,146 +6012,148 @@
       <x:c r="O105" s="14" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="P105" s="14"/>
+      <x:c r="P105" s="14" t="str">
+        <x:v>customer_advance_over_5000</x:v>
+      </x:c>
       <x:c r="Q105" s="12" t="str"/>
     </x:row>
     <x:row r="106" ht="430" customHeight="1">
       <x:c r="A106" s="14" t="str">
-        <x:v>3970</x:v>
+        <x:v>3700</x:v>
       </x:c>
       <x:c r="B106" s="14" t="str">
-        <x:v>Vinst vid avyttring av immateriella och materiella anläggningstillgångar</x:v>
+        <x:v>Lämnade rabatter, bonus etc.</x:v>
       </x:c>
       <x:c r="C106" s="14" t="str">
-        <x:v>Intäktskonto på R2 för en positiv skillnad mellan försäljningsinkomst och bokfört värde när en individuellt värderad immateriell eller materiell anläggningstillgång avyttras.</x:v>
+        <x:v>K1-konto på R1 eller R2 för rabatter, bonusar och andra verkliga prisnedsättningar som företaget lämnar till sina kunder. Beloppet minskar den ursprungliga försäljningen.</x:v>
       </x:c>
       <x:c r="D106" s="14" t="str">
-        <x:v>En byggnad, mark, markanläggning, förvärvad immateriell tillgång eller annan individuellt hanterad anläggningstillgång har avyttrats|Försäljningsinkomst, bokfört värde och bortbokning av tillgången är verifierade|Skillnaden är positiv och ska redovisas som vinst</x:v>
+        <x:v>Företaget lämnar rabatt, bonus eller återbäring som sänker priset på en försäljning|Prisnedsättningen kan kopplas till en kund, försäljning och momssats|Det finns kreditnota, bonusavtal eller annat underlag som visar nedsättningen|Beloppet avser normal öres- eller kronutjämning i samband med försäljning</x:v>
       </x:c>
       <x:c r="E106" s="14" t="str">
-        <x:v>Avyttringen gäller maskiner, inventarier, byggnads- och markinventarier eller fordon som hanteras kollektivt via 1222, 1232 eller 1242|Skillnaden är negativ; använd 7970|Beloppet är hela försäljningsersättningen och inte endast vinsten|Tillgångens bokförda värde eller ackumulerade avskrivning är inte fastställd|Försäljningen gäller lager eller privat tillgång</x:v>
+        <x:v>Beloppet är reklam, gåva, representation eller annan marknadsföringskostnad|Beloppet är kundförlust, ackord eller skadestånd och inte en verklig prisnedsättning|Beloppet är en rabatt som företaget själv har fått vid inköp; använd 4700|Posten avser punktskatt; detta ligger utanför tjänstens standardomfattning|Posten saknar koppling till en försäljning eller underlag för momshanteringen</x:v>
       </x:c>
       <x:c r="F106" s="14" t="str">
-        <x:v>Identifiera tillgången i förteckningen över anläggningstillgångar|Fastställ försäljningsinkomst exklusive eventuell utgående moms|Beräkna bokfört värde efter årets avskrivning och nedskrivning enligt tillämplig K1-regel|Boka bort anskaffningsvärde och ackumulerade avskrivningar|Redovisa endast positiv nettoskillnad på 3970|Bokför eventuell utgående moms separat; momsen ingår inte i vinsten|Kontrollera att kollektivt värderade inventariegrupper i stället hanteras genom försäljningsersättning på balansunderkonto|Koppla till avtal, betalning, tillgångspost och skatteberäkning|Använd endast när individuell vinstberäkning ska göras|Kräv försäljningspris, bokfört värde, årets avskrivning, kostnader och tillgångsslag|Vid granskningsflagga begär in försäljningsavtal, faktura, betalning och uppdaterad tillgångsförteckning|Sätt ärendet till väntar på underlag tills försäljningspris, bokfört värde, årets avskrivning och moms är avstämda|Godkänn 3970 endast när en individuell avyttring ger en verifierad positiv skillnad|Föreslå kollektiv inventariemodell, 7970 eller eskalering när tillgångsslag, redovisningsmodell eller beräkning är oklar</x:v>
+        <x:v>Kontrollera att händelsen är en verklig prisnedsättning och inte en kostnad eller kundförlust|Koppla rabatten till ursprungsförsäljningen och använd samma momssats|Kräv kreditnota eller annat dokumenterat underlag när priset sätts ned i efterhand|BAS 3730, 3731, 3732 och 3740 får sammanföras automatiskt till 3700|BAS 3700, 3710 och 3790 kräver kontroll eftersom kontona är generella eller ofördelade|BAS 3750, 3751 och 3752 avser punktskatter och ligger utanför standardflödet|Fördela beloppet mellan R1 och R2 om rabatten avser både momspliktig och momsfri försäljning|Stäm av kreditnota eller bonus mot kundfordran, betalning och redovisad försäljning|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G106" s="14" t="str">
-        <x:v>1000|1009|1110|1119|1130|1150|1159|1500|1930|2610</x:v>
+        <x:v>1500|1910|1930|2610|2620|2630|3000|3100</x:v>
       </x:c>
       <x:c r="H106" s="14" t="str">
-        <x:v>En byggnad säljs och tillgångens bokförda värde tas bort; positiv skillnad mot försäljningsinkomsten redovisas på 3970|Försäljning av en maskin i den kollektivt värderade inventariegruppen bokförs inte som individuell vinst på 3970</x:v>
+        <x:v>En kreditnota för en tidigare försäljning bokförs som minskad försäljning på 3700 och minskad utgående moms med samma momssats som originalfakturan|En dokumenterad årsbonus till en kund bokförs på 3700 och fördelas efter de försäljningar och momssatser som bonusen avser|Normal öresutjämning från en kundbetalning sammanförs till 3700</x:v>
       </x:c>
       <x:c r="I106" s="14" t="str">
-        <x:v>3970 innehåller vinsten, inte bruttoersättningen|K1:s kollektiva värdering av inventarier innebär att individuell vinst normalt inte beräknas för 1220-, 1230- och 1240-grupperna|Moms och transaktionskostnader måste behandlas separat|Försäljning till företagaren eller närstående kräver marknadsvärdeskontroll|Kollektivt hanterade inventarier ska normalt inte ge individuell vinst här</x:v>
+        <x:v>Rabatten ska minska försäljningen och inte bokföras som en vanlig kostnad|Momsjusteringen måste följa ursprungsförsäljningen|Generella intäktskorrigeringar utan underlag eller momssats ska granskas|Kundförlust, skadestånd och rabatt är olika händelser|Punktskatter får inte behandlas som kundrabatter</x:v>
       </x:c>
       <x:c r="J106" s="14" t="str">
-        <x:v>vinst avyttring|anläggningstillgång|reavinst|byggnad|mark|immateriell tillgång|R2</x:v>
+        <x:v>lämnad rabatt|bonus|återbäring|kreditnota|prisnedsättning|öresutjämning|R1|R2</x:v>
       </x:c>
       <x:c r="K106" s="14" t="str">
-        <x:v>7970|1000|1110|1130|1150|1222|1232|1242|2610</x:v>
+        <x:v>3000|3100|3500|4700|1500|2610|2620|2630</x:v>
       </x:c>
       <x:c r="L106" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 3970, rad R2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.16, 6.27, 6.37–6.38 och kapitel 7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, exemplen 6-7 och 6-8</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – konto 3700, rad R1/R2|BFNAR 2006:1 senast ändrat genom BFNAR 2025:1, definitionen av nettoomsättning och punkt 7.1|Skatteverkets rättsliga vägledning om kreditnota och prisnedsättning i efterhand, 2026</x:v>
       </x:c>
       <x:c r="M106" s="14" t="str">
-        <x:v>Tillgångstyp eller bokfört värde är oklart|Avyttringen gäller kollektivt värderad inventariegrupp|Moms, transaktionskostnader eller närståendeförsäljning förekommer|Tillgången är endast delvis avyttrad|Skillnaden kan vara förlust|Tillgångsslag eller redovisningsmodell är oklar</x:v>
+        <x:v>Posten kommer från BAS 3700, 3710 eller 3790|Ursprungsförsäljning, kund eller momssats saknas|Händelsen kan vara kundförlust, kostnad, reklamation eller skadestånd i stället för rabatt|Kreditnota eller bonusunderlag saknas|Rabatten avser flera momssatser eller både momspliktig och momsfri försäljning</x:v>
       </x:c>
       <x:c r="N106" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O106" s="14" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P106" s="14"/>
       <x:c r="Q106" s="12" t="str"/>
     </x:row>
     <x:row r="107" ht="430" customHeight="1">
       <x:c r="A107" s="14" t="str">
-        <x:v>3980</x:v>
+        <x:v>3900</x:v>
       </x:c>
       <x:c r="B107" s="14" t="str">
-        <x:v>Erhållna bidrag</x:v>
+        <x:v>Övriga rörelseintäkter</x:v>
       </x:c>
       <x:c r="C107" s="14" t="str">
-        <x:v>Intäktskonto på R2 för offentliga stöd och andra bidrag som hör till verksamheten och ska intäktsredovisas. Stöd som direkt hänför sig till förvärv av en tillgång ska i stället minska tillgångens anskaffningsvärde.</x:v>
+        <x:v>Samlingskonto på R1 eller R2 för rörelseintäkter som hör till företaget men inte är huvudförsäljning, fakturerade kostnader, förmåner, vinst vid anläggningstillgångsförsäljning eller erhållna bidrag.</x:v>
       </x:c>
       <x:c r="D107" s="14" t="str">
-        <x:v>Ett offentligt stöd eller bidrag har beviljats verksamheten|Beslut, överenskommelse eller dispositionsrätt visar att inkomsten ska redovisas|Stödet är inte ett privat stöd och ska inte minska en tillgångs anskaffningsvärde</x:v>
+        <x:v>Inkomsten är sekundär i förhållande till företagets normala huvudverksamhet|Inkomsten hör till rörelsen och ska redovisas på R1 eller R2|Inkomstens art, momsbehandling och redovisningstidpunkt är dokumenterade|En tidigare direkt kostnadsförd inventarie säljs</x:v>
       </x:c>
       <x:c r="E107" s="14" t="str">
-        <x:v>Stödet har beviljats företagaren privat|Stödet hänför sig direkt till förvärv av byggnad, markanläggning, inventarie eller annan tillgång; minska anskaffningsvärdet enligt tillämplig regel|Ansökan är inskickad men beslut eller dispositionsrätt saknas|Beloppet är lån, kundbetalning eller ersättning för en levererad prestation|Stödets villkor eller period är oklar</x:v>
+        <x:v>Inkomsten är normal huvudförsäljning; använd 3000 eller 3100|Beloppet är fakturerad kostnad, bil- eller bostadsförmån, anläggningstillgångsvinst eller bidrag|Beloppet är ränteintäkt eller annan finansiell intäkt|Beloppet hör till privatpersonen|Inkomstens art är okänd och 3900 används som restkonto|Intäkten avser säkringsinstrument eller annan avancerad finansiell transaktion|Intäkten förutsätter anställda, exempelvis sjuklöneersättning</x:v>
       </x:c>
       <x:c r="F107" s="14" t="str">
-        <x:v>Verifiera stödmottagare, stödtyp, beslut, villkor, belopp och beslutsdatum|Redovisa stödet när beslut eller överenskommelse finns med dokumenterat belopp, eller när företaget annars kan förfoga över inkomsten|Om stödet uppenbart avser flera år ska intäkten fördelas på de år den avser|Årliga stöd som betalas under löpande år ska inte periodiseras enbart därför att de avser tolv månader|Kontrollera om stödet hänför sig till ett tillgångsförvärv och därför ska minska anskaffningsvärdet|Bokför beslutad men ännu inte utbetald intäkt mot 1600|Stäm av 3980 mot beslut, bank, fordran och deklarationsunderlag|Dokumentera eventuella återbetalningsvillkor och återkrav|Använd för verksamhetsstöd när beslut och rätt till stödet finns|Spara stödgivare, villkor, ändamål, belopp, beslutsdatum, utbetalningsplan och återbetalningsrisk|Vid granskningsflagga begär in bidragsbeslut, villkor, ändamål, beslutsdatum och utbetalningsplan|Sätt ärendet till väntar på underlag tills rätten till stödet, period, återbetalningsrisk och tillgångskoppling är verifierade|Godkänn 3980 när bidraget hör till verksamheten och ska intäktsredovisas|Föreslå minskat anskaffningsvärde, periodisering, fordran eller eskalering när villkoren kräver annan behandling</x:v>
+        <x:v>Identifiera inkomsttypen och dokumentera varför den är en sekundär rörelseintäkt|Fastställ om intäkten ska redovisas på R1 eller R2, om den ingår i nettoomsättningen och om utgående moms ska redovisas|Hyres- och arrendeintäkter kräver manuell granskning; frivillig beskattning för lokaluthyrning får aldrig hanteras automatiskt|Konfliktersättning, skadestånd, gåvor, försäkringsersättning och skuldackord kräver manuell granskning av grund, skatteplikt, moms och koppling till kostnad, tillgång eller skuld|Säkringsinstrument och orealiserade värdeförändringar ligger utanför tjänstens standardomfattning|Sjuklöneersättning och andra intäkter som förutsätter anställda ligger utanför tjänstens målgrupp|För försäljning av en tidigare direkt kostnadsförd inventarie: bokför ersättningen på 3900 och redovisa eventuell utgående moms separat|Fördela inkomsten över flera år endast när det är uppenbart att den avser flera år enligt K1|Kontrollera om ersättningen i stället ska påverka en tillgångs anskaffningsvärde, en vinst vid avyttring, ett bidrag eller en kostnad|Koppla intäkten till dokumenterad kategori och motpart och stäm av fordran, bankbetalning och efterföljande reglering|Blockera ospecificerade bokningar och använd aldrig 3900 som restkonto för okända insättningar</x:v>
       </x:c>
       <x:c r="G107" s="14" t="str">
-        <x:v>1600|1930|1110|1150|1220|1230|1240</x:v>
+        <x:v>1600|1500|1910|1930|2610|2620|2630</x:v>
       </x:c>
       <x:c r="H107" s="14" t="str">
-        <x:v>Ett beslutat verksamhetsbidrag som avser innevarande år bokförs på 3980 mot bank eller fordran|Ett investeringsbidrag som hänför sig till en maskin minskar maskinens anskaffningsvärde och bokförs inte som vanlig intäkt på 3980</x:v>
+        <x:v>En dokumenterad sekundär provisions- eller licensintäkt kan bokföras på 3900 med rätt momsbehandling|Hyresintäkt eller försäkringsersättning skickas till manuell granskning innan konto och moms fastställs|En tidigare kostnadsförd dator säljs och ersättningen bokförs på 3900 med eventuell moms separat</x:v>
       </x:c>
       <x:c r="I107" s="14" t="str">
-        <x:v>Bidrag och stöd ingår inte alltid i nettoomsättningen även om de redovisas på R2|Beslutstidpunkt och dispositionsrätt styr intäktsredovisningen|Tillgångsanknutna stöd behandlas annorlunda än verksamhetsstöd|Privata stöd får inte bokföras i företaget|Tillgångsanknutet stöd kan minska anskaffningsvärdet och kräver manuell bedömning</x:v>
+        <x:v>3900 får inte bli ett restkonto för okända insättningar|R1 eller R2, nettoomsättning och momsbehandling måste fastställas per intäkt|Hyresintäkter, försäkringsersättning, skadestånd, gåvor och skuldackord kräver manuell granskning|Sekundär intäkt kan ändå ingå i nettoomsättningen beroende på verksamheten|Använd inte 1222 när tillgången aldrig har ingått i inventariegruppen|Säkringsinstrument och personalrelaterade ersättningar ligger utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="J107" s="14" t="str">
-        <x:v>erhållet bidrag|offentligt stöd|verksamhetsstöd|investeringsbidrag|R2|beslut</x:v>
+        <x:v>övrig rörelseintäkt|sekundär intäkt|försäkringsersättning|skadestånd|R1|R2</x:v>
       </x:c>
       <x:c r="K107" s="14" t="str">
-        <x:v>1600|3900|3970|1110|1150|1220|1230|1240</x:v>
+        <x:v>3000|3100|3500|3970|3980|1600|8310</x:v>
       </x:c>
       <x:c r="L107" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 3980, rad R2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 3.17, punkt 6.61 och punkt 7.2 samt exempel 7-2</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 3900, rad R1/R2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.17 och 7.2|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sidoordnad specifikation|Skatteverket – Uthyrning av fastighet och frivillig beskattning, kontrollerat 2026-09-20</x:v>
       </x:c>
       <x:c r="M107" s="14" t="str">
-        <x:v>Beslut, villkor eller stödmottagare är oklar|Stödet kan vara privat eller tillgångsanknutet|Stödet avser flera år eller kan återkrävas|Moms- eller skattebehandlingen är oklar|Fordran eller utbetalning stämmer inte med beslutet|Stödvillkor, periodisering eller koppling till tillgång är oklar</x:v>
+        <x:v>Intäktstyp, redovisningsrad eller momsbehandling är oklar|Hyres- eller arrendeintäkt förekommer|Försäkringsersättning, konfliktersättning, skadestånd, gåva eller skuldackord förekommer|Intäkten kan vara huvudförsäljning, bidrag, vinst vid avyttring eller finansiell intäkt|Beslut, avtal eller annan dokumentation saknas|Intäkten kan påverka en tillgång, kostnad eller skuld på annat sätt än som vanlig rörelseintäkt</x:v>
       </x:c>
       <x:c r="N107" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O107" s="14" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P107" s="14"/>
       <x:c r="Q107" s="12" t="str"/>
     </x:row>
     <x:row r="108" ht="430" customHeight="1">
       <x:c r="A108" s="14" t="str">
-        <x:v>4000</x:v>
+        <x:v>3970</x:v>
       </x:c>
       <x:c r="B108" s="14" t="str">
-        <x:v>Varor</x:v>
+        <x:v>Vinst vid avyttring av immateriella och materiella anläggningstillgångar</x:v>
       </x:c>
       <x:c r="C108" s="14" t="str">
-        <x:v>Kostnadskonto på R5 för inköp av varor och material som ska säljas vidare, förbrukas i produktion eller direkt ingå i företagets leverans till kund.</x:v>
+        <x:v>Intäktskonto på R2 för en positiv skillnad mellan försäljningsinkomst och bokfört värde när en individuellt värderad immateriell eller materiell anläggningstillgång avyttras.</x:v>
       </x:c>
       <x:c r="D108" s="14" t="str">
-        <x:v>Företaget köper handelsvaror, råvaror eller material för försäljning eller produktion|Utgiften hör till verksamheten och är inte en anläggningstillgång|Varuinköpet ska ingå i beräkningen av årets kostnad på R5</x:v>
+        <x:v>En byggnad, mark, markanläggning, förvärvad immateriell tillgång eller annan individuellt hanterad anläggningstillgång har avyttrats|Försäljningsinkomst, bokfört värde och bortbokning av tillgången är verifierade|Skillnaden är positiv och ska redovisas som vinst</x:v>
       </x:c>
       <x:c r="E108" s="14" t="str">
-        <x:v>Inköpet är maskin, inventarie, bil, byggnad eller annan anläggningstillgång|Inköpet är allmän förbrukningsinventarie eller förbrukningsmaterial som hör till 5400|Utgiften avser underentreprenör eller köpt arbete; använd 4600|Beloppet är lokal-, rese-, reklam- eller annan extern kostnad|Betalningen är förskott över 5 000 kronor och leverans inte har påbörjats|Inköpet är privat</x:v>
+        <x:v>Avyttringen gäller maskiner, inventarier, byggnads- och markinventarier eller fordon som hanteras kollektivt via 1222, 1232 eller 1242|Skillnaden är negativ; använd 7970|Beloppet är hela försäljningsersättningen och inte endast vinsten|Tillgångens bokförda värde eller ackumulerade avskrivning är inte fastställd|Försäljningen gäller lager eller privat tillgång</x:v>
       </x:c>
       <x:c r="F108" s="14" t="str">
-        <x:v>Identifiera varutyp, användning och koppling till företagets försäljning eller produktion|Bokför inköpet exklusive avdragsgill ingående moms|Vid kontantmetoden justeras årets utbetalningar för leverantörsskulder och leverantörsförskott i bokslutet|Vid faktureringsmetoden utgår kostnaden från fakturerade inköp och justeras för förskott samt inköp som borde ha fakturerats|Ta inte med varor som ska aktiveras som anläggningstillgång|Inventera och värdera varor som finns kvar på balansdagen på 1400|Bokför lagerförändringen separat på 4900 så att R5 avser årets varukostnad|Bokför erhållna rabatter och bonusar på 4700 enligt kontoplanen|Stäm av 4000 mot leverantörsreskontra, bank, 1700, 2440, 1400 och 4900|Använd för varor och material som säljs vidare eller direkt ingår i kundens leverans|Klassificera efter inköpets användning|Stäm av mot lager och leverantörsskulder vid bokslut|Bokför varu- och materialinköp som ska säljas vidare eller direkt ingå i leveransen på 4000 exklusive avdragsgill moms|Begär faktura och uppgift om användning när inköpet kan vara inventarie, privat kostnad, förskott eller något som finns kvar i lager|Vid bokslut stäms årets inköp av mot leverantörsskulder, leverantörsförskott och inventeringslistan|Godkänn slutlig R5-kostnad först efter att utgående lager på 1400 och lagerförändringen på 4900 har bokförts</x:v>
+        <x:v>Identifiera tillgången i förteckningen över anläggningstillgångar|Fastställ försäljningsinkomst exklusive eventuell utgående moms|Beräkna bokfört värde efter årets avskrivning och nedskrivning enligt tillämplig K1-regel|Boka bort anskaffningsvärde och ackumulerade avskrivningar|Redovisa endast positiv nettoskillnad på 3970|Bokför eventuell utgående moms separat; momsen ingår inte i vinsten|Kontrollera att kollektivt värderade inventariegrupper i stället hanteras genom försäljningsersättning på balansunderkonto|Koppla till avtal, betalning, tillgångspost och skatteberäkning|Använd endast när individuell vinstberäkning ska göras|Kräv försäljningspris, bokfört värde, årets avskrivning, kostnader och tillgångsslag|Vid granskningsflagga begär in försäljningsavtal, faktura, betalning och uppdaterad tillgångsförteckning|Sätt ärendet till väntar på underlag tills försäljningspris, bokfört värde, årets avskrivning och moms är avstämda|Godkänn 3970 endast när en individuell avyttring ger en verifierad positiv skillnad|Föreslå kollektiv inventariemodell, 7970 eller eskalering när tillgångsslag, redovisningsmodell eller beräkning är oklar</x:v>
       </x:c>
       <x:c r="G108" s="14" t="str">
-        <x:v>2440|1930|2641|1700|1400|4700|4900</x:v>
+        <x:v>1000|1009|1110|1119|1130|1150|1159|1500|1930|2610</x:v>
       </x:c>
       <x:c r="H108" s="14" t="str">
-        <x:v>Inköpta handelsvaror bokförs på 4000 exklusive avdragsgill moms|Varor som finns kvar vid årets slut tas upp som lager på 1400 och lagerförändringen bokförs på 4900</x:v>
+        <x:v>En byggnad säljs och tillgångens bokförda värde tas bort; positiv skillnad mot försäljningsinkomsten redovisas på 3970|Försäljning av en maskin i den kollektivt värderade inventariegruppen bokförs inte som individuell vinst på 3970</x:v>
       </x:c>
       <x:c r="I108" s="14" t="str">
-        <x:v>Varuinköp och varukostnad är inte alltid samma belopp på grund av lagerförändring|Förskott och obetalda leverantörsfakturor måste justeras vid bokslutet|Ej avdragsgill moms ingår i kostnaden eller lagervärdet|Köp av anläggningstillgång får inte kostnadsföras som varor|Använd inte för externa tjänster, förbrukningsinventarier, anläggningstillgångar eller privata inköp</x:v>
+        <x:v>3970 innehåller vinsten, inte bruttoersättningen|K1:s kollektiva värdering av inventarier innebär att individuell vinst normalt inte beräknas för 1220-, 1230- och 1240-grupperna|Moms och transaktionskostnader måste behandlas separat|Försäljning till företagaren eller närstående kräver marknadsvärdeskontroll|Kollektivt hanterade inventarier ska normalt inte ge individuell vinst här</x:v>
       </x:c>
       <x:c r="J108" s="14" t="str">
-        <x:v>varuinköp|handelsvaror|material|råvara|R5|lager|leverantörsskuld</x:v>
+        <x:v>vinst avyttring|anläggningstillgång|reavinst|byggnad|mark|immateriell tillgång|R2</x:v>
       </x:c>
       <x:c r="K108" s="14" t="str">
-        <x:v>1400|1700|2440|4600|4700|4900|5400|2641</x:v>
+        <x:v>7970|1000|1110|1130|1150|1222|1232|1242|2610</x:v>
       </x:c>
       <x:c r="L108" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 4000, rad R5|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 7.5–7.7 och exemplen 7-3a och 7-3b|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.45–6.55</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 3970, rad R2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.16, 6.27, 6.37–6.38 och kapitel 7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, exemplen 6-7 och 6-8</x:v>
       </x:c>
       <x:c r="M108" s="14" t="str">
-        <x:v>Varans användning eller klassificering är oklar|Leverantörsförskott eller obetald faktura finns|Lagerinventering saknas|Inköpet kan vara anläggningstillgång eller privat|Momsavdraget är begränsat|Användningen är oklar eller bokslutssekvensen mot lager är inte verifierad</x:v>
+        <x:v>Tillgångstyp eller bokfört värde är oklart|Avyttringen gäller kollektivt värderad inventariegrupp|Moms, transaktionskostnader eller närståendeförsäljning förekommer|Tillgången är endast delvis avyttrad|Skillnaden kan vara förlust|Tillgångsslag eller redovisningsmodell är oklar</x:v>
       </x:c>
       <x:c r="N108" s="14" t="str">
         <x:v>active</x:v>
@@ -6157,148 +6161,148 @@
       <x:c r="O108" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P108" s="14" t="str">
-        <x:v>supplier_advance_over_5000</x:v>
-      </x:c>
+      <x:c r="P108" s="14"/>
       <x:c r="Q108" s="12" t="str"/>
     </x:row>
     <x:row r="109" ht="430" customHeight="1">
       <x:c r="A109" s="14" t="str">
-        <x:v>4200</x:v>
+        <x:v>3980</x:v>
       </x:c>
       <x:c r="B109" s="14" t="str">
-        <x:v>Sålda varor VMB</x:v>
+        <x:v>Erhållna bidrag</x:v>
       </x:c>
       <x:c r="C109" s="14" t="str">
-        <x:v>Samlat kostnadskonto för anskaffningsvärdet på sålda VMB-varor när materialet inte redan är uppdelat mellan positiv och negativ marginal.</x:v>
+        <x:v>Intäktskonto på R2 för offentliga stöd och andra bidrag som hör till verksamheten och ska intäktsredovisas. Stöd som direkt hänför sig till förvärv av en tillgång ska i stället minska tillgångens anskaffningsvärde.</x:v>
       </x:c>
       <x:c r="D109" s="14" t="str">
-        <x:v>Importerad bokföring använder BAS 4200 för VMB-varukostnad|VMB-varukostnaden är korrekt men saknar uppdelning på 4211 och 4212</x:v>
+        <x:v>Ett offentligt stöd eller bidrag har beviljats verksamheten|Beslut, överenskommelse eller dispositionsrätt visar att inkomsten ska redovisas|Stödet är inte ett privat stöd och ska inte minska en tillgångs anskaffningsvärde</x:v>
       </x:c>
       <x:c r="E109" s="14" t="str">
-        <x:v>Positiv eller negativ marginal kan identifieras; använd 4211 respektive 4212|Varorna omfattas av vanlig moms|Posten avser inköp som fortfarande finns i lager</x:v>
+        <x:v>Stödet har beviljats företagaren privat|Stödet hänför sig direkt till förvärv av byggnad, markanläggning, inventarie eller annan tillgång; minska anskaffningsvärdet enligt tillämplig regel|Ansökan är inskickad men beslut eller dispositionsrätt saknas|Beloppet är lån, kundbetalning eller ersättning för en levererad prestation|Stödets villkor eller period är oklar</x:v>
       </x:c>
       <x:c r="F109" s="14" t="str">
-        <x:v>Stäm av kostnaden mot sålda VMB-varors inköpspris|Försök vid granskning dela upp 4200 mellan 4211 och 4212|Håll VMB-varukostnad skild från vanliga varuinköp|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Verifiera stödmottagare, stödtyp, beslut, villkor, belopp och beslutsdatum|Redovisa stödet när beslut eller överenskommelse finns med dokumenterat belopp, eller när företaget annars kan förfoga över inkomsten|Om stödet uppenbart avser flera år ska intäkten fördelas på de år den avser|Årliga stöd som betalas under löpande år ska inte periodiseras enbart därför att de avser tolv månader|Kontrollera om stödet hänför sig till ett tillgångsförvärv och därför ska minska anskaffningsvärdet|Bokför beslutad men ännu inte utbetald intäkt mot 1600|Stäm av 3980 mot beslut, bank, fordran och deklarationsunderlag|Dokumentera eventuella återbetalningsvillkor och återkrav|Använd för verksamhetsstöd när beslut och rätt till stödet finns|Spara stödgivare, villkor, ändamål, belopp, beslutsdatum, utbetalningsplan och återbetalningsrisk|Vid granskningsflagga begär in bidragsbeslut, villkor, ändamål, beslutsdatum och utbetalningsplan|Sätt ärendet till väntar på underlag tills rätten till stödet, period, återbetalningsrisk och tillgångskoppling är verifierade|Godkänn 3980 när bidraget hör till verksamheten och ska intäktsredovisas|Föreslå minskat anskaffningsvärde, periodisering, fordran eller eskalering när villkoren kräver annan behandling</x:v>
       </x:c>
       <x:c r="G109" s="14" t="str">
-        <x:v>1465|1467|3211|3212</x:v>
+        <x:v>1600|1930|1110|1150|1220|1230|1240</x:v>
       </x:c>
       <x:c r="H109" s="14" t="str">
-        <x:v>En importerad SIE-fil har anskaffningsvärdet för sålda VMB-varor bokfört på BAS 4200 och förs över utan att blandas med 4000</x:v>
+        <x:v>Ett beslutat verksamhetsbidrag som avser innevarande år bokförs på 3980 mot bank eller fordran|Ett investeringsbidrag som hänför sig till en maskin minskar maskinens anskaffningsvärde och bokförs inte som vanlig intäkt på 3980</x:v>
       </x:c>
       <x:c r="I109" s="14" t="str">
-        <x:v>4200 är ett samlingskonto och ger inte ensam tillräckligt underlag för momsberäkningen|Ny löpande bokföring bör använda 4211 eller 4212 när marginalens tecken är känt</x:v>
+        <x:v>Bidrag och stöd ingår inte alltid i nettoomsättningen även om de redovisas på R2|Beslutstidpunkt och dispositionsrätt styr intäktsredovisningen|Tillgångsanknutna stöd behandlas annorlunda än verksamhetsstöd|Privata stöd får inte bokföras i företaget|Tillgångsanknutet stöd kan minska anskaffningsvärdet och kräver manuell bedömning</x:v>
       </x:c>
       <x:c r="J109" s="14" t="str">
-        <x:v>sålda VMB-varor|varukostnad|inköpspris|begagnade varor|BAS 4200</x:v>
+        <x:v>erhållet bidrag|offentligt stöd|verksamhetsstöd|investeringsbidrag|R2|beslut</x:v>
       </x:c>
       <x:c r="K109" s="14" t="str">
-        <x:v>4211|4212|1465|1467|3211|3212</x:v>
+        <x:v>1600|3900|3970|1110|1150|1220|1230|1240</x:v>
       </x:c>
       <x:c r="L109" s="14" t="str">
-        <x:v>BAS_FULL_2022, konto 4200|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 3980, rad R2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 3.17, punkt 6.61 och punkt 7.2 samt exempel 7-2</x:v>
       </x:c>
       <x:c r="M109" s="14" t="str">
-        <x:v>4200 används i ny löpande bokföring|Varukostnaden kan inte stämmas av mot lager eller försäljning|Momsberäkningen saknar uppdelning</x:v>
+        <x:v>Beslut, villkor eller stödmottagare är oklar|Stödet kan vara privat eller tillgångsanknutet|Stödet avser flera år eller kan återkrävas|Moms- eller skattebehandlingen är oklar|Fordran eller utbetalning stämmer inte med beslutet|Stödvillkor, periodisering eller koppling till tillgång är oklar</x:v>
       </x:c>
       <x:c r="N109" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O109" s="14" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="P109" s="14" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P109" s="14"/>
       <x:c r="Q109" s="12" t="str"/>
     </x:row>
     <x:row r="110" ht="430" customHeight="1">
       <x:c r="A110" s="14" t="str">
-        <x:v>4211</x:v>
+        <x:v>4000</x:v>
       </x:c>
       <x:c r="B110" s="14" t="str">
-        <x:v>Sålda varor, positiv VMB</x:v>
+        <x:v>Varor</x:v>
       </x:c>
       <x:c r="C110" s="14" t="str">
-        <x:v>Kostnadskonto för inköpspriset på sålda VMB-varor som har positiv vinstmarginal.</x:v>
+        <x:v>Kostnadskonto på R5 för inköp av varor och material som ska säljas vidare, förbrukas i produktion eller direkt ingå i företagets leverans till kund.</x:v>
       </x:c>
       <x:c r="D110" s="14" t="str">
-        <x:v>En VMB-vara eller tillåten VMB-period har positiv marginal|Inköpspriset ska matchas mot försäljningen på 3211</x:v>
+        <x:v>Företaget köper handelsvaror, råvaror eller material för försäljning eller produktion|Utgiften hör till verksamheten och är inte en anläggningstillgång|Varuinköpet ska ingå i beräkningen av årets kostnad på R5</x:v>
       </x:c>
       <x:c r="E110" s="14" t="str">
-        <x:v>Marginalen är negativ; använd 4212|Varan finns kvar i lager|Inköpet omfattas av vanlig moms</x:v>
+        <x:v>Inköpet är maskin, inventarie, bil, byggnad eller annan anläggningstillgång|Inköpet är allmän förbrukningsinventarie eller förbrukningsmaterial som hör till 5400|Utgiften avser underentreprenör eller köpt arbete; använd 4600|Beloppet är lokal-, rese-, reklam- eller annan extern kostnad|Betalningen är förskott över 5 000 kronor och leverans inte har påbörjats|Inköpet är privat</x:v>
       </x:c>
       <x:c r="F110" s="14" t="str">
-        <x:v>Bokför den sålda varans anskaffningsvärde|Matcha mot försäljning på 3211|Stäm av marginalen och utgående VMB-moms|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Identifiera varutyp, användning och koppling till företagets försäljning eller produktion|Bokför inköpet exklusive avdragsgill ingående moms|Vid kontantmetoden justeras årets utbetalningar för leverantörsskulder och leverantörsförskott i bokslutet|Vid faktureringsmetoden utgår kostnaden från fakturerade inköp och justeras för förskott samt inköp som borde ha fakturerats|Ta inte med varor som ska aktiveras som anläggningstillgång|Inventera och värdera varor som finns kvar på balansdagen på 1400|Bokför lagerförändringen separat på 4900 så att R5 avser årets varukostnad|Bokför erhållna rabatter och bonusar på 4700 enligt kontoplanen|Stäm av 4000 mot leverantörsreskontra, bank, 1700, 2440, 1400 och 4900|Använd för varor och material som säljs vidare eller direkt ingår i kundens leverans|Klassificera efter inköpets användning|Stäm av mot lager och leverantörsskulder vid bokslut|Bokför varu- och materialinköp som ska säljas vidare eller direkt ingå i leveransen på 4000 exklusive avdragsgill moms|Begär faktura och uppgift om användning när inköpet kan vara inventarie, privat kostnad, förskott eller något som finns kvar i lager|Vid bokslut stäms årets inköp av mot leverantörsskulder, leverantörsförskott och inventeringslistan|Godkänn slutlig R5-kostnad först efter att utgående lager på 1400 och lagerförändringen på 4900 har bokförts</x:v>
       </x:c>
       <x:c r="G110" s="14" t="str">
-        <x:v>1465|1467|3211|2616|2626|2636</x:v>
+        <x:v>2440|1930|2641|1700|1400|4700|4900</x:v>
       </x:c>
       <x:c r="H110" s="14" t="str">
-        <x:v>En VMB-vara som köpts för 1 000 kronor säljs med positiv marginal och 1 000 kronor förs från lager till 4211</x:v>
+        <x:v>Inköpta handelsvaror bokförs på 4000 exklusive avdragsgill moms|Varor som finns kvar vid årets slut tas upp som lager på 1400 och lagerförändringen bokförs på 4900</x:v>
       </x:c>
       <x:c r="I110" s="14" t="str">
-        <x:v>Kontot ska innehålla inköpspris, inte hela kundbetalningen|Ingen ingående moms får lyftas på VMB-inköpet</x:v>
+        <x:v>Varuinköp och varukostnad är inte alltid samma belopp på grund av lagerförändring|Förskott och obetalda leverantörsfakturor måste justeras vid bokslutet|Ej avdragsgill moms ingår i kostnaden eller lagervärdet|Köp av anläggningstillgång får inte kostnadsföras som varor|Använd inte för externa tjänster, förbrukningsinventarier, anläggningstillgångar eller privata inköp</x:v>
       </x:c>
       <x:c r="J110" s="14" t="str">
-        <x:v>varukostnad positiv VMB|inköpspris|såld begagnad vara|positiv marginal</x:v>
+        <x:v>varuinköp|handelsvaror|material|råvara|R5|lager|leverantörsskuld</x:v>
       </x:c>
       <x:c r="K110" s="14" t="str">
-        <x:v>4200|4212|1465|1467|3211|2616|2626|2636</x:v>
+        <x:v>1400|1700|2440|4600|4700|4900|5400|2641</x:v>
       </x:c>
       <x:c r="L110" s="14" t="str">
-        <x:v>BAS_FULL_2022, konto 4211|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 4000, rad R5|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 7.5–7.7 och exemplen 7-3a och 7-3b|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.45–6.55</x:v>
       </x:c>
       <x:c r="M110" s="14" t="str">
-        <x:v>Inköpspriset saknas eller kan inte knytas till varan|Förenklad VMB används och periodens beräkning är oklar</x:v>
+        <x:v>Varans användning eller klassificering är oklar|Leverantörsförskott eller obetald faktura finns|Lagerinventering saknas|Inköpet kan vara anläggningstillgång eller privat|Momsavdraget är begränsat|Användningen är oklar eller bokslutssekvensen mot lager är inte verifierad</x:v>
       </x:c>
       <x:c r="N110" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O110" s="14" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="P110" s="14" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P110" s="14" t="str">
+        <x:v>supplier_advance_over_5000</x:v>
+      </x:c>
       <x:c r="Q110" s="12" t="str"/>
     </x:row>
     <x:row r="111" ht="430" customHeight="1">
       <x:c r="A111" s="14" t="str">
-        <x:v>4212</x:v>
+        <x:v>4200</x:v>
       </x:c>
       <x:c r="B111" s="14" t="str">
-        <x:v>Sålda varor, negativ VMB</x:v>
+        <x:v>Sålda varor VMB</x:v>
       </x:c>
       <x:c r="C111" s="14" t="str">
-        <x:v>Kostnadskonto för inköpspriset på sålda VMB-varor som har negativ vinstmarginal.</x:v>
+        <x:v>Samlat kostnadskonto för anskaffningsvärdet på sålda VMB-varor när materialet inte redan är uppdelat mellan positiv och negativ marginal.</x:v>
       </x:c>
       <x:c r="D111" s="14" t="str">
-        <x:v>En VMB-vara eller tillåten VMB-period har negativ marginal|Inköpspriset ska matchas mot försäljningen på 3212</x:v>
+        <x:v>Importerad bokföring använder BAS 4200 för VMB-varukostnad|VMB-varukostnaden är korrekt men saknar uppdelning på 4211 och 4212</x:v>
       </x:c>
       <x:c r="E111" s="14" t="str">
-        <x:v>Marginalen är positiv; använd 4211|Varan finns kvar i lager|Posten avser lagernedskrivning</x:v>
+        <x:v>Positiv eller negativ marginal kan identifieras; använd 4211 respektive 4212|Varorna omfattas av vanlig moms|Posten avser inköp som fortfarande finns i lager</x:v>
       </x:c>
       <x:c r="F111" s="14" t="str">
-        <x:v>Bokför den sålda varans anskaffningsvärde|Matcha mot försäljning på 3212|Bokför ingen negativ utgående moms|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Stäm av kostnaden mot sålda VMB-varors inköpspris|Försök vid granskning dela upp 4200 mellan 4211 och 4212|Håll VMB-varukostnad skild från vanliga varuinköp|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G111" s="14" t="str">
-        <x:v>1465|1467|3212</x:v>
+        <x:v>1465|1467|3211|3212</x:v>
       </x:c>
       <x:c r="H111" s="14" t="str">
-        <x:v>En VMB-vara säljs för mindre än inköpspriset och anskaffningsvärdet förs från lager till 4212</x:v>
+        <x:v>En importerad SIE-fil har anskaffningsvärdet för sålda VMB-varor bokfört på BAS 4200 och förs över utan att blandas med 4000</x:v>
       </x:c>
       <x:c r="I111" s="14" t="str">
-        <x:v>Negativ marginal är inte samma sak som lagernedskrivning|Kvittning mot positiva marginaler får bara ske när VMB-reglerna uttryckligen medger det</x:v>
+        <x:v>4200 är ett samlingskonto och ger inte ensam tillräckligt underlag för momsberäkningen|Ny löpande bokföring bör använda 4211 eller 4212 när marginalens tecken är känt</x:v>
       </x:c>
       <x:c r="J111" s="14" t="str">
-        <x:v>varukostnad negativ VMB|inköpspris|förlustmarginal|såld begagnad vara</x:v>
+        <x:v>sålda VMB-varor|varukostnad|inköpspris|begagnade varor|BAS 4200</x:v>
       </x:c>
       <x:c r="K111" s="14" t="str">
-        <x:v>4200|4211|1465|1467|3212|2616|2626|2636</x:v>
+        <x:v>4211|4212|1465|1467|3211|3212</x:v>
       </x:c>
       <x:c r="L111" s="14" t="str">
-        <x:v>BAS_FULL_2022, konto 4212|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
+        <x:v>BAS_FULL_2022, konto 4200|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
       </x:c>
       <x:c r="M111" s="14" t="str">
-        <x:v>All negativ periodmarginal vid förenklad VMB|Inköpspriset saknas|Kvittning eller framåtföring av negativ marginal övervägs</x:v>
+        <x:v>4200 används i ny löpande bokföring|Varukostnaden kan inte stämmas av mot lager eller försäljning|Momsberäkningen saknar uppdelning</x:v>
       </x:c>
       <x:c r="N111" s="14" t="str">
         <x:v>active</x:v>
@@ -6311,143 +6315,141 @@
     </x:row>
     <x:row r="112" ht="430" customHeight="1">
       <x:c r="A112" s="14" t="str">
-        <x:v>4600</x:v>
+        <x:v>4211</x:v>
       </x:c>
       <x:c r="B112" s="14" t="str">
-        <x:v>Legoarbeten och underentreprenader</x:v>
+        <x:v>Sålda varor, positiv VMB</x:v>
       </x:c>
       <x:c r="C112" s="14" t="str">
-        <x:v>Kostnadskonto på R5 för köpta arbeten och underentreprenader som är direkt kopplade till företagets egen produktion, entreprenad eller leverans till kund.</x:v>
+        <x:v>Kostnadskonto för inköpspriset på sålda VMB-varor som har positiv vinstmarginal.</x:v>
       </x:c>
       <x:c r="D112" s="14" t="str">
-        <x:v>En extern utförare producerar en del av den vara eller tjänst som företaget säljer|En underentreprenör utför direkt kund- eller projektarbete|Kostnaden är direkt hänförlig till företagets leverans och ska redovisas på R5</x:v>
+        <x:v>En VMB-vara eller tillåten VMB-period har positiv marginal|Inköpspriset ska matchas mot försäljningen på 3211</x:v>
       </x:c>
       <x:c r="E112" s="14" t="str">
-        <x:v>Tjänsten är redovisning, juridik, IT, marknadsföring eller annan allmän extern tjänst; pröva 6500|Utföraren är anställd eller ska behandlas som personal|Inköpet avser varor eller material utan köpt arbete; använd 4000|Arbetet skapar en anläggningstillgång och ska ingå i anskaffningsvärdet|Betalningen är förskott över 5 000 kronor och arbetet inte har påbörjats|Arbetet hör till privatpersonen</x:v>
+        <x:v>Marginalen är negativ; använd 4212|Varan finns kvar i lager|Inköpet omfattas av vanlig moms</x:v>
       </x:c>
       <x:c r="F112" s="14" t="str">
-        <x:v>Identifiera leverantör, avtal, projekt, prestation och direkt koppling till företagets leverans|Bedöm om utföraren är självständig näringsidkare eller om förhållandet kan vara anställning|Kontrollera om svensk omvänd betalningsskyldighet, utlandsförvärv eller vanlig leverantörsmoms gäller|Bokför kostnaden exklusive avdragsgill moms|Justera för leverantörsskulder och förskott i bokslutet enligt vald bokföringsmetod|Aktivera direkt hänförliga utgifter när arbetet avser tillverkning eller förvärv av en anläggningstillgång enligt tillämplig regel|Koppla kostnaden till projekt, kunduppdrag och leverantörsfaktura|Stäm av mot 1700, 2440, momsunderlag och projektkalkyl|Använd när extern företagare utför arbete som direkt ingår i kunduppdraget|Kontrollera F-skatt, avtalsförhållande och momsflöde|Aktivera arbete som skapar företagets egen tillgång|Vid granskningsflagga begär in faktura, avtal, uppdragsbeskrivning och vid behov uppgift om F-skatt och momsbehandling|Sätt ärendet till väntar på underlag tills leverantörens ställning, verksamhetskopplingen och momsbehandlingen är klarlagda|Godkänn 4600 när en självständig leverantör utför arbete som direkt ingår i företagets leverans|Föreslå omklassificering till rätt kostnads- eller tillgångskonto, eller eskalering om förhållandet kan vara anställning eller ligger utanför standardtjänsten</x:v>
+        <x:v>Bokför den sålda varans anskaffningsvärde|Matcha mot försäljning på 3211|Stäm av marginalen och utgående VMB-moms|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G112" s="14" t="str">
-        <x:v>2440|1930|2641|2645|1700|3000|1220|1110</x:v>
+        <x:v>1465|1467|3211|2616|2626|2636</x:v>
       </x:c>
       <x:c r="H112" s="14" t="str">
-        <x:v>En underentreprenör utför en avtalad del av ett kundprojekt; kostnaden bokförs på 4600 med rätt momsbehandling|En konsult som sköter företagets administration bokförs normalt som extern tjänst och inte på 4600</x:v>
+        <x:v>En VMB-vara som köpts för 1 000 kronor säljs med positiv marginal och 1 000 kronor förs från lager till 4211</x:v>
       </x:c>
       <x:c r="I112" s="14" t="str">
-        <x:v>Underentreprenad och inhyrd personal är inte samma sak|Byggtjänster kan omfattas av omvänd betalningsskyldighet|Direkt koppling till kundens leverans måste dokumenteras|Arbete som skapar en anläggningstillgång kan behöva aktiveras|Administration, juridik, kontorsstädning och IT-support hör normalt inte hit</x:v>
+        <x:v>Kontot ska innehålla inköpspris, inte hela kundbetalningen|Ingen ingående moms får lyftas på VMB-inköpet</x:v>
       </x:c>
       <x:c r="J112" s="14" t="str">
-        <x:v>legoarbete|underentreprenör|köpt arbete|direkt kostnad|projekt|R5</x:v>
+        <x:v>varukostnad positiv VMB|inköpspris|såld begagnad vara|positiv marginal</x:v>
       </x:c>
       <x:c r="K112" s="14" t="str">
-        <x:v>4000|1700|2440|6500|6800|2641|2645|3000</x:v>
+        <x:v>4200|4212|1465|1467|3211|2616|2626|2636</x:v>
       </x:c>
       <x:c r="L112" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 4600, rad R5|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7 samt exemplen 7-3a och 7-3b|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sidoordnad bokföring</x:v>
+        <x:v>BAS_FULL_2022, konto 4211|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
       </x:c>
       <x:c r="M112" s="14" t="str">
-        <x:v>Direkt koppling till kunduppdrag saknas|Utföraren kan vara anställd eller inhyrd personal|Omvänd moms, utland eller felaktigt debiterad moms förekommer|Arbetet kan ingå i en anläggningstillgång|Förskott eller ofakturerad kostnad finns|Anställningsrisk, byggmoms, utlandsköp eller projektaktivering förekommer</x:v>
+        <x:v>Inköpspriset saknas eller kan inte knytas till varan|Förenklad VMB används och periodens beräkning är oklar</x:v>
       </x:c>
       <x:c r="N112" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O112" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P112" s="14" t="str">
-        <x:v>supplier_advance_over_5000</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P112" s="14" t="str"/>
       <x:c r="Q112" s="12" t="str"/>
     </x:row>
     <x:row r="113" ht="430" customHeight="1">
       <x:c r="A113" s="14" t="str">
-        <x:v>4700</x:v>
+        <x:v>4212</x:v>
       </x:c>
       <x:c r="B113" s="14" t="str">
-        <x:v>Erhållna rabatter, bonus etc.</x:v>
+        <x:v>Sålda varor, negativ VMB</x:v>
       </x:c>
       <x:c r="C113" s="14" t="str">
-        <x:v>Kostnadsreducerande konto på R6 för rabatter, bonusar, återbäringar och liknande prisnedsättningar som företaget får från leverantörer och som inte redan har dragits av direkt från inköpspriset.</x:v>
+        <x:v>Kostnadskonto för inköpspriset på sålda VMB-varor som har negativ vinstmarginal.</x:v>
       </x:c>
       <x:c r="D113" s="14" t="str">
-        <x:v>Leverantören lämnar en efterhandsrabatt, årsbonus eller återbäring|Prisnedsättningen kan kopplas till ett eller flera företagsinköp|Beloppet ska minska företagets inköps- eller externa kostnader</x:v>
+        <x:v>En VMB-vara eller tillåten VMB-period har negativ marginal|Inköpspriset ska matchas mot försäljningen på 3212</x:v>
       </x:c>
       <x:c r="E113" s="14" t="str">
-        <x:v>Rabatten har redan minskat kostnaden på leverantörsfakturan|Beloppet är rabatt som företaget lämnar till kund; använd 3700|Beloppet avser en anläggningstillgång och ska minska tillgångens anskaffningsvärde eller bokförda värde|Beloppet är ett offentligt bidrag eller försäkringsersättning|Kreditnotan avser retur, feldebitering eller annan händelse som ska rätta ett specifikt kostnads- eller tillgångskonto direkt</x:v>
+        <x:v>Marginalen är positiv; använd 4211|Varan finns kvar i lager|Posten avser lagernedskrivning</x:v>
       </x:c>
       <x:c r="F113" s="14" t="str">
-        <x:v>Identifiera leverantör, bonusavtal, kreditnota och vilka inköp beloppet avser|Bokför rabatten som minskning av kostnad, normalt i kredit på 4700, endast när separat redovisning är motiverad|Justera ingående moms när kreditnotan eller momsregeln kräver det|Om rabatten avser lager ska effekten beaktas i lagrets anskaffningsvärde|Om rabatten avser en anläggningstillgång ska tillgångens anskaffningsvärde eller bokförda värde justeras i stället för att hela beloppet lämnas på 4700|Fördela bonusar som avser flera kostnadsslag enligt dokumenterat underlag|Stäm av mot leverantörsreskontra, betalning och ursprungsfakturor|Kräv manuell granskning vid större årsbonus, flera momssatser eller tillgångsanknutet belopp|Koppla rabatt, bonus eller kreditnota till ursprungligt inköp|Minska rätt kostnad, lager eller anskaffningsvärde|Rätta ingående moms mot ursprungsunderlag|Vid granskningsflagga begär in kreditnota, bonusavtal och underlag som visar vilka ursprungliga inköp rabatten avser|Sätt ärendet till väntar på underlag tills kostnad, period och moms kan kopplas till ursprungstransaktionen|Godkänn 4700 när rabatten är en separat prisnedsättning av vanliga kostnader och rätt momsjustering är dokumenterad|Föreslå omklassificering till ursprungligt kostnads-, lager- eller tillgångskonto när rabatten avser en särskild post</x:v>
+        <x:v>Bokför den sålda varans anskaffningsvärde|Matcha mot försäljning på 3212|Bokför ingen negativ utgående moms|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G113" s="14" t="str">
-        <x:v>2440|1930|2641|4000|4600|5000|5400</x:v>
+        <x:v>1465|1467|3212</x:v>
       </x:c>
       <x:c r="H113" s="14" t="str">
-        <x:v>En leverantörsbonus som avser årets varuinköp krediteras på 4700 och eventuell ingående moms rättas enligt kreditnotan|En rabatt på en ny maskin minskar maskinens anskaffningsvärde och ska inte automatiskt ligga kvar på 4700</x:v>
+        <x:v>En VMB-vara säljs för mindre än inköpspriset och anskaffningsvärdet förs från lager till 4212</x:v>
       </x:c>
       <x:c r="I113" s="14" t="str">
-        <x:v>4700 ska inte bli ett allmänt konto för alla kreditnotor|Rabatten måste kunna kopplas till ursprungliga inköp|Momsjusteringen ska följa kreditnotan och ursprungstransaktionen|Rabatter på lager och anläggningstillgångar kan kräva värdejustering|Generell bokning är inte tillåten när rabatten avser en särskild post</x:v>
+        <x:v>Negativ marginal är inte samma sak som lagernedskrivning|Kvittning mot positiva marginaler får bara ske när VMB-reglerna uttryckligen medger det</x:v>
       </x:c>
       <x:c r="J113" s="14" t="str">
-        <x:v>erhållen rabatt|leverantörsbonus|återbäring|kreditnota|inköpspris|R6</x:v>
+        <x:v>varukostnad negativ VMB|inköpspris|förlustmarginal|såld begagnad vara</x:v>
       </x:c>
       <x:c r="K113" s="14" t="str">
-        <x:v>3700|4000|4600|4900|1220|1230|1240|2440|2641</x:v>
+        <x:v>4200|4211|1465|1467|3212|2616|2626|2636</x:v>
       </x:c>
       <x:c r="L113" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 4700, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 3.18 och kapitel 7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om rättelser och verifikationer</x:v>
+        <x:v>BAS_FULL_2022, konto 4212|SKV_VMB_2026, beskattningsunderlag och vinstmarginal|BFN_K1_WEB_2025, K1-vägledningen</x:v>
       </x:c>
       <x:c r="M113" s="14" t="str">
-        <x:v>Ursprungsinköp eller bonusavtal saknas|Rabatten avser lager eller anläggningstillgång|Flera kostnadsslag, perioder eller momssatser berörs|Kreditnotan kan vara retur eller felrättning i stället för bonus|Årsbonus kräver fördelning eller ursprungsfakturor saknas</x:v>
+        <x:v>All negativ periodmarginal vid förenklad VMB|Inköpspriset saknas|Kvittning eller framåtföring av negativ marginal övervägs</x:v>
       </x:c>
       <x:c r="N113" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O113" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P113" s="14"/>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P113" s="14" t="str"/>
       <x:c r="Q113" s="12" t="str"/>
     </x:row>
     <x:row r="114" ht="430" customHeight="1">
       <x:c r="A114" s="14" t="str">
-        <x:v>4900</x:v>
+        <x:v>4600</x:v>
       </x:c>
       <x:c r="B114" s="14" t="str">
-        <x:v>Förändring av lager</x:v>
+        <x:v>Legoarbeten och underentreprenader</x:v>
       </x:c>
       <x:c r="C114" s="14" t="str">
-        <x:v>Bokslutskonto på R5 för årets förändring av varulager. Kontot kopplar kostnaden för varuinköp till lagervärdet på 1400 så att resultatet endast belastas med årets förbrukade eller sålda varor.</x:v>
+        <x:v>Kostnadskonto på R5 för köpta arbeten och underentreprenader som är direkt kopplade till företagets egen produktion, entreprenad eller leverans till kund.</x:v>
       </x:c>
       <x:c r="D114" s="14" t="str">
-        <x:v>Ett inventerat och värderat lager ska tas upp på 1400 vid årets slut|Utgående lagervärde skiljer sig från ingående lagervärde|Bokslutet ska justera R5 för lagerökning eller lagerminskning</x:v>
+        <x:v>En extern utförare producerar en del av den vara eller tjänst som företaget säljer|En underentreprenör utför direkt kund- eller projektarbete|Kostnaden är direkt hänförlig till företagets leverans och ska redovisas på R5</x:v>
       </x:c>
       <x:c r="E114" s="14" t="str">
-        <x:v>Företaget saknar varulager|Lagrets sammanlagda värde omfattas av K1-regeln som medger att lagret inte tas upp och företaget väljer den förenklingen|Beloppet avser inköp under året; använd 4000|Beloppet är lager av fastigheter eller andra tillgångar som kräver särskild hantering|Inventerings- eller värderingsunderlag saknas</x:v>
+        <x:v>Tjänsten är redovisning, juridik, IT, marknadsföring eller annan allmän extern tjänst; pröva 6500|Utföraren är anställd eller ska behandlas som personal|Inköpet avser varor eller material utan köpt arbete; använd 4000|Arbetet skapar en anläggningstillgång och ska ingå i anskaffningsvärdet|Betalningen är förskott över 5 000 kronor och arbetet inte har påbörjats|Arbetet hör till privatpersonen</x:v>
       </x:c>
       <x:c r="F114" s="14" t="str">
-        <x:v>Fastställ ingående lagervärde från föregående bokslut|Inventera lagret på balansdagen och dokumentera antal, artikel, skick och äganderätt|Värdera lagret enligt K1:s regler om anskaffningsvärde, schablonmässig värdenedgång och större faktisk värdenedgång|Kontrollera om den fysiska personens sammanlagda lager i samtliga verksamheter får kostnadsföras enligt halvt-prisbasbeloppsregeln|Boka utgående lagervärde på 1400|En lagerökning krediterar normalt 4900 och minskar årets R5-kostnad|En lagerminskning debiterar normalt 4900 och ökar årets R5-kostnad|Stäm av 1400 och 4900 mot inventeringslista, 4000 och föregående års saldo|Spara värderingsmetod och regelversion|Använd endast i verifierad bokslutsrutin för lagerförändring|Koppla till inventerat utgående lager och ingående lager|Fastställ ingående lager från föregående bokslut och utgående lager från en verifierad inventeringslista|Om utgående lager är högre än ingående lager bokförs ökningen i debet på 1400 och kredit på 4900|Om utgående lager är lägre än ingående lager bokförs minskningen i debet på 4900 och kredit på 1400|Sätt ärendet till väntar på underlag om inventeringslista, ägande, värdering eller ingående lagervärde saknas; egentillverkat eller svårvärderat lager eskaleras</x:v>
+        <x:v>Identifiera leverantör, avtal, projekt, prestation och direkt koppling till företagets leverans|Bedöm om utföraren är självständig näringsidkare eller om förhållandet kan vara anställning|Kontrollera om svensk omvänd betalningsskyldighet, utlandsförvärv eller vanlig leverantörsmoms gäller|Bokför kostnaden exklusive avdragsgill moms|Justera för leverantörsskulder och förskott i bokslutet enligt vald bokföringsmetod|Aktivera direkt hänförliga utgifter när arbetet avser tillverkning eller förvärv av en anläggningstillgång enligt tillämplig regel|Koppla kostnaden till projekt, kunduppdrag och leverantörsfaktura|Stäm av mot 1700, 2440, momsunderlag och projektkalkyl|Använd när extern företagare utför arbete som direkt ingår i kunduppdraget|Kontrollera F-skatt, avtalsförhållande och momsflöde|Aktivera arbete som skapar företagets egen tillgång|Vid granskningsflagga begär in faktura, avtal, uppdragsbeskrivning och vid behov uppgift om F-skatt och momsbehandling|Sätt ärendet till väntar på underlag tills leverantörens ställning, verksamhetskopplingen och momsbehandlingen är klarlagda|Godkänn 4600 när en självständig leverantör utför arbete som direkt ingår i företagets leverans|Föreslå omklassificering till rätt kostnads- eller tillgångskonto, eller eskalering om förhållandet kan vara anställning eller ligger utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="G114" s="14" t="str">
-        <x:v>1400|4000</x:v>
+        <x:v>2440|1930|2641|2645|1700|3000|1220|1110</x:v>
       </x:c>
       <x:c r="H114" s="14" t="str">
-        <x:v>Lagret ökar från 20 000 till 35 000 kronor: 1400 ökar med 15 000 och 4900 krediteras med 15 000|Lagret minskar från 35 000 till 10 000 kronor: 1400 minskar med 25 000 och 4900 debiteras med 25 000</x:v>
+        <x:v>En underentreprenör utför en avtalad del av ett kundprojekt; kostnaden bokförs på 4600 med rätt momsbehandling|En konsult som sköter företagets administration bokförs normalt som extern tjänst och inte på 4600</x:v>
       </x:c>
       <x:c r="I114" s="14" t="str">
-        <x:v>4900 ska motsvara förändringen mellan ingående och utgående lagervärde|Ett felaktigt tecken vänder resultatpåverkan|Inventering och värdering måste göras innan bokningen|Förenklingsregeln bedöms över den fysiska personens samtliga verksamheter|Fel tecken eller dubbel bokning ger motsatt resultat</x:v>
+        <x:v>Underentreprenad och inhyrd personal är inte samma sak|Byggtjänster kan omfattas av omvänd betalningsskyldighet|Direkt koppling till kundens leverans måste dokumenteras|Arbete som skapar en anläggningstillgång kan behöva aktiveras|Administration, juridik, kontorsstädning och IT-support hör normalt inte hit</x:v>
       </x:c>
       <x:c r="J114" s="14" t="str">
-        <x:v>lagerförändring|varulager|inventering|lagervärde|R5|bokslut</x:v>
+        <x:v>legoarbete|underentreprenör|köpt arbete|direkt kostnad|projekt|R5</x:v>
       </x:c>
       <x:c r="K114" s="14" t="str">
-        <x:v>1400|4000|4700</x:v>
+        <x:v>4000|1700|2440|6500|6800|2641|2645|3000</x:v>
       </x:c>
       <x:c r="L114" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 4900, rad R5|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.45–6.55 och 7.5–7.7 samt exemplen 6-9a, 6-9b och 6-10</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 4600, rad R5|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7 samt exemplen 7-3a och 7-3b|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sidoordnad bokföring</x:v>
       </x:c>
       <x:c r="M114" s="14" t="str">
-        <x:v>Inventeringslista eller ingående lager saknas|Lagret ligger nära halvt prisbasbelopp|Flera verksamheter måste summeras|Lagret innehåller skadade, inkuranta, egentillverkade eller fastighetsrelaterade poster|Bokningens tecken eller föregående års omföring är oklar|Exakt konterings- och återföringsrutin är inte verifierad</x:v>
+        <x:v>Direkt koppling till kunduppdrag saknas|Utföraren kan vara anställd eller inhyrd personal|Omvänd moms, utland eller felaktigt debiterad moms förekommer|Arbetet kan ingå i en anläggningstillgång|Förskott eller ofakturerad kostnad finns|Anställningsrisk, byggmoms, utlandsköp eller projektaktivering förekommer</x:v>
       </x:c>
       <x:c r="N114" s="14" t="str">
         <x:v>active</x:v>
@@ -6456,49 +6458,49 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="P114" s="14" t="str">
-        <x:v>inventory_optional_expensing_half_pbb|inventory_standard_reduction_3_percent</x:v>
+        <x:v>supplier_advance_over_5000</x:v>
       </x:c>
       <x:c r="Q114" s="12" t="str"/>
     </x:row>
     <x:row r="115" ht="430" customHeight="1">
       <x:c r="A115" s="14" t="str">
-        <x:v>5000</x:v>
+        <x:v>4700</x:v>
       </x:c>
       <x:c r="B115" s="14" t="str">
-        <x:v>Lokalkostnader</x:v>
+        <x:v>Erhållna rabatter, bonus etc.</x:v>
       </x:c>
       <x:c r="C115" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för hyrda verksamhetslokaler och kostnader som direkt hör till användningen av sådana lokaler, exempelvis hyra, drift och lokalservice.</x:v>
+        <x:v>Kostnadsreducerande konto på R6 för rabatter, bonusar, återbäringar och liknande prisnedsättningar som företaget får från leverantörer och som inte redan har dragits av direkt från inköpspriset.</x:v>
       </x:c>
       <x:c r="D115" s="14" t="str">
-        <x:v>Företaget hyr en lokal som används i näringsverksamheten|Kostnaden avser lokalens löpande användning, drift, städning eller liknande|Utgiften kan kopplas till lokalavtal, period och verksamhetsanvändning</x:v>
+        <x:v>Leverantören lämnar en efterhandsrabatt, årsbonus eller återbäring|Prisnedsättningen kan kopplas till ett eller flera företagsinköp|Beloppet ska minska företagets inköps- eller externa kostnader</x:v>
       </x:c>
       <x:c r="E115" s="14" t="str">
-        <x:v>Fastigheten ägs av företaget eller ingår som näringsfastighet; pröva 5100|Beloppet är säkerhetsdeposition eller annan återbetalningsbar fordran|Utgiften skapar en bestående förbättring eller anläggningstillgång|Kostnaden avser privat bostad eller ett arbetsrum i bostaden utan verifierad avdragsrätt|Beloppet är hyra av maskin, inventarie eller fordon; använd 5200 eller relevant transportkonto</x:v>
+        <x:v>Rabatten har redan minskat kostnaden på leverantörsfakturan|Beloppet är rabatt som företaget lämnar till kund; använd 3700|Beloppet avser en anläggningstillgång och ska minska tillgångens anskaffningsvärde eller bokförda värde|Beloppet är ett offentligt bidrag eller försäkringsersättning|Kreditnotan avser retur, feldebitering eller annan händelse som ska rätta ett specifikt kostnads- eller tillgångskonto direkt</x:v>
       </x:c>
       <x:c r="F115" s="14" t="str">
-        <x:v>Verifiera hyresvärd, lokal, avtal, period och verksamhetsanvändning|Bokför kostnaden exklusive avdragsgill ingående moms|Skilj löpande hyra och drift från deposition, förskott, inventariehyra och investering i lokalen|BAS 5070 Reparation och underhåll av lokaler får inte mappas automatiskt; kontrollera om arbetet helt eller delvis är en aktiverbar förbättring i hyrd lokal|BAS 5099 Ej avdragsgilla lokalkostnader kräver manuell granskning och dokumenterad skattemässig hantering|Fördela kostnaden vid blandad privat och företagsmässig användning endast enligt dokumenterad regel|Koppla kostnaden till lokal eller kostnadsställe när flera lokaler finns|Kontrollera om lokalen omfattas av frivillig beskattning och om avdragsrätten för moms är begränsad|Stäm av mot avtal, leverantörsfakturor, förskott, leverantörsskuld och betalningar|Kräv manuell granskning för arbetsrum i privatbostad, närståendehyra, större arbeten eller oklar momsbehandling</x:v>
+        <x:v>Identifiera leverantör, bonusavtal, kreditnota och vilka inköp beloppet avser|Bokför rabatten som minskning av kostnad, normalt i kredit på 4700, endast när separat redovisning är motiverad|Justera ingående moms när kreditnotan eller momsregeln kräver det|Om rabatten avser lager ska effekten beaktas i lagrets anskaffningsvärde|Om rabatten avser en anläggningstillgång ska tillgångens anskaffningsvärde eller bokförda värde justeras i stället för att hela beloppet lämnas på 4700|Fördela bonusar som avser flera kostnadsslag enligt dokumenterat underlag|Stäm av mot leverantörsreskontra, betalning och ursprungsfakturor|Kräv manuell granskning vid större årsbonus, flera momssatser eller tillgångsanknutet belopp|Koppla rabatt, bonus eller kreditnota till ursprungligt inköp|Minska rätt kostnad, lager eller anskaffningsvärde|Rätta ingående moms mot ursprungsunderlag|Vid granskningsflagga begär in kreditnota, bonusavtal och underlag som visar vilka ursprungliga inköp rabatten avser|Sätt ärendet till väntar på underlag tills kostnad, period och moms kan kopplas till ursprungstransaktionen|Godkänn 4700 när rabatten är en separat prisnedsättning av vanliga kostnader och rätt momsjustering är dokumenterad|Föreslå omklassificering till ursprungligt kostnads-, lager- eller tillgångskonto när rabatten avser en särskild post</x:v>
       </x:c>
       <x:c r="G115" s="14" t="str">
-        <x:v>2440|1930|2641|2642|1700|1600</x:v>
+        <x:v>2440|1930|2641|4000|4600|5000|5400</x:v>
       </x:c>
       <x:c r="H115" s="14" t="str">
-        <x:v>Månadshyra för en separat verksamhetslokal bokförs på 5000 med avdragsgill moms separat|En återbetalningsbar hyresdeposition bokförs som fordran och inte som lokalkostnad|En reparationsfaktura på BAS 5070 granskas för att skilja löpande återställande arbete från en aktiverbar förbättring i hyrd lokal|En kostnad märkt ej avdragsgill på BAS 5099 granskas och får inte automatiskt behandlas som en vanlig avdragsgill lokalkostnad</x:v>
+        <x:v>En leverantörsbonus som avser årets varuinköp krediteras på 4700 och eventuell ingående moms rättas enligt kreditnotan|En rabatt på en ny maskin minskar maskinens anskaffningsvärde och ska inte automatiskt ligga kvar på 4700</x:v>
       </x:c>
       <x:c r="I115" s="14" t="str">
-        <x:v>Lokalkostnad och kostnad för ägd näringsfastighet måste skiljas åt|Kostnader för privatbostad och arbetsrum i bostaden har särskilda skatteregler|Förbättringar i hyrd lokal kan behöva aktiveras; kontonamnet 5070 bevisar inte att hela utgiften får kostnadsföras direkt|Moms på lokalhyra förutsätter korrekt momsbehandling och kan påverkas av frivillig beskattning|Ej avdragsgilla lokalkostnader måste bevaras för den skattemässiga justeringen</x:v>
+        <x:v>4700 ska inte bli ett allmänt konto för alla kreditnotor|Rabatten måste kunna kopplas till ursprungliga inköp|Momsjusteringen ska följa kreditnotan och ursprungstransaktionen|Rabatter på lager och anläggningstillgångar kan kräva värdejustering|Generell bokning är inte tillåten när rabatten avser en särskild post</x:v>
       </x:c>
       <x:c r="J115" s="14" t="str">
-        <x:v>lokalkostnad|lokalhyra|verksamhetslokal|städning|drift|R6</x:v>
+        <x:v>erhållen rabatt|leverantörsbonus|återbäring|kreditnota|inköpspris|R6</x:v>
       </x:c>
       <x:c r="K115" s="14" t="str">
-        <x:v>5100|5200|5500|1700|1600|2440|2641|2642</x:v>
+        <x:v>3700|4000|4600|4900|1220|1230|1240|2440|2641</x:v>
       </x:c>
       <x:c r="L115" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 5000, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.5–6.27 och 7.5–7.7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och periodavstämning</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 4700, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 3.18 och kapitel 7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om rättelser och verifikationer</x:v>
       </x:c>
       <x:c r="M115" s="14" t="str">
-        <x:v>Lokalen används helt eller delvis privat eller verksamhetsandelen är oklar|Arbetsrum i bostad eller närståendehyra förekommer|Deposition, förskott eller större arbete ingår|Bokningen kommer från BAS 5070 och arbetets karaktär inte har verifierats|Bokningen kommer från BAS 5099 eller är på annat sätt markerad som ej avdragsgill|Moms på hyran, frivillig beskattning eller avdragsrätt är oklar|Kostnaden kan höra till ägd fastighet eller en annan tillgång</x:v>
+        <x:v>Ursprungsinköp eller bonusavtal saknas|Rabatten avser lager eller anläggningstillgång|Flera kostnadsslag, perioder eller momssatser berörs|Kreditnotan kan vara retur eller felrättning i stället för bonus|Årsbonus kräver fördelning eller ursprungsfakturor saknas</x:v>
       </x:c>
       <x:c r="N115" s="14" t="str">
         <x:v>active</x:v>
@@ -6511,92 +6513,94 @@
     </x:row>
     <x:row r="116" ht="430" customHeight="1">
       <x:c r="A116" s="14" t="str">
-        <x:v>5100</x:v>
+        <x:v>4900</x:v>
       </x:c>
       <x:c r="B116" s="14" t="str">
-        <x:v>Fastighetskostnader</x:v>
+        <x:v>Förändring av lager</x:v>
       </x:c>
       <x:c r="C116" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för löpande drift, förvaltning och andra kostnader som hör till en fastighet i näringsverksamheten. Förbättringar och ny-, till- eller ombyggnad ska inte kostnadsföras här.</x:v>
+        <x:v>Bokslutskonto på R5 för årets förändring av varulager. Kontot kopplar kostnaden för varuinköp till lagervärdet på 1400 så att resultatet endast belastas med årets förbrukade eller sålda varor.</x:v>
       </x:c>
       <x:c r="D116" s="14" t="str">
-        <x:v>Företaget eller näringsverksamheten äger eller redovisar fastigheten|Utgiften avser löpande drift, tillsyn, service, förvaltning eller annan fastighetskostnad|Kostnaden hör till årets användning av fastigheten|En byggnad med mycket kort användningstid har efter manuell granskning godkänts för direkt kostnadsföring enligt K1 punkt 6.6</x:v>
+        <x:v>Ett inventerat och värderat lager ska tas upp på 1400 vid årets slut|Utgående lagervärde skiljer sig från ingående lagervärde|Bokslutet ska justera R5 för lagerökning eller lagerminskning</x:v>
       </x:c>
       <x:c r="E116" s="14" t="str">
-        <x:v>Företaget hyr lokalen; använd normalt 5000|Utgiften avser ny-, till- eller ombyggnad eller annan värdehöjande förbättring|Beloppet ska ingå i anskaffningsvärdet för byggnad, markanläggning eller byggnadsinventarie|Utgiften avser ränta, amortering eller privat bostadsdel|Utgiften är reparation av fordon, maskin eller annan tillgång|Objektet är egentligen inventarie, hyrd bod, container eller lokal</x:v>
+        <x:v>Företaget saknar varulager|Lagrets sammanlagda värde omfattas av K1-regeln som medger att lagret inte tas upp och företaget väljer den förenklingen|Beloppet avser inköp under året; använd 4000|Beloppet är lager av fastigheter eller andra tillgångar som kräver särskild hantering|Inventerings- eller värderingsunderlag saknas</x:v>
       </x:c>
       <x:c r="F116" s="14" t="str">
-        <x:v>Verifiera fastighet, ägande eller nyttjanderätt, verksamhetsanknytning och kostnadstyp|Fördela kostnaden mellan näringsdel och privat del när fastigheten används blandat och bokför endast verksamhetsandelen|Skilj löpande drift och återställande reparation från förbättring, nybyggnad, tillbyggnad, ombyggnad och annan anläggningstillgång|BAS 5170 Reparation och underhåll får inte mappas automatiskt; kontrollera alltid om arbetet helt eller delvis ska aktiveras|BAS 5199 Ej avdragsgilla fastighetskostnader kräver manuell granskning och dokumenterad skattemässig hantering|Bokför avdragsgill moms separat och kontrollera fastighetsrelaterade begränsningar, jämkning och ändrad användning|Koppla fakturor och betalningar till fastighetsobjekt och period och stäm av mot relevanta tillgångs- och skuldkonton|Kräv manuell granskning vid näringsfastighet med privat användning, större arbeten, ändrad användning eller oklar fördelningsgrund|Direkt kostnadsförd tillfällig byggnad får endast bokföras här efter manuell granskning enligt K1 punkt 6.6 och ska märkas som sådan|Ta inte upp en godkänd direkt kostnadsförd tillfällig byggnad på 1110 och skriv inte av den via 1119 eller 7820|Pröva först om flyttbar bod, container eller liknande i stället är inventarie, hyra eller lokal</x:v>
+        <x:v>Fastställ ingående lagervärde från föregående bokslut|Inventera lagret på balansdagen och dokumentera antal, artikel, skick och äganderätt|Värdera lagret enligt K1:s regler om anskaffningsvärde, schablonmässig värdenedgång och större faktisk värdenedgång|Kontrollera om den fysiska personens sammanlagda lager i samtliga verksamheter får kostnadsföras enligt halvt-prisbasbeloppsregeln|Boka utgående lagervärde på 1400|En lagerökning krediterar normalt 4900 och minskar årets R5-kostnad|En lagerminskning debiterar normalt 4900 och ökar årets R5-kostnad|Stäm av 1400 och 4900 mot inventeringslista, 4000 och föregående års saldo|Spara värderingsmetod och regelversion|Använd endast i verifierad bokslutsrutin för lagerförändring|Koppla till inventerat utgående lager och ingående lager|Fastställ ingående lager från föregående bokslut och utgående lager från en verifierad inventeringslista|Om utgående lager är högre än ingående lager bokförs ökningen i debet på 1400 och kredit på 4900|Om utgående lager är lägre än ingående lager bokförs minskningen i debet på 4900 och kredit på 1400|Sätt ärendet till väntar på underlag om inventeringslista, ägande, värdering eller ingående lagervärde saknas; egentillverkat eller svårvärderat lager eskaleras</x:v>
       </x:c>
       <x:c r="G116" s="14" t="str">
-        <x:v>2440|1930|2641|2642|1110|1130|1150|1230</x:v>
+        <x:v>1400|4000</x:v>
       </x:c>
       <x:c r="H116" s="14" t="str">
-        <x:v>Löpande el, värme, vatten, sophämtning eller fastighetsskötsel för en verksamhetsfastighet bokförs normalt på 5100|En reparationsfaktura på BAS 5170 granskas för att skilja återställande reparation från aktiverbar förbättring|En tillbyggnad som ger bestående värde aktiveras på relevant tillgångskonto och bokförs inte som fastighetskostnad|En kostnad märkt ej avdragsgill på BAS 5199 granskas och får inte automatiskt behandlas som en vanlig avdragsgill kostnad|En enkel tillfällig byggnad med verifierad kort användningstid bokförs efter manuell granskning på 5100</x:v>
+        <x:v>Lagret ökar från 20 000 till 35 000 kronor: 1400 ökar med 15 000 och 4900 krediteras med 15 000|Lagret minskar från 35 000 till 10 000 kronor: 1400 minskar med 25 000 och 4900 debiteras med 25 000</x:v>
       </x:c>
       <x:c r="I116" s="14" t="str">
-        <x:v>Ägd fastighet och hyrd lokal ska hållas isär|Reparation och förbättring är olika redovisningshändelser; kontonamnet 5170 bevisar inte att hela utgiften får kostnadsföras direkt|Privat del får inte belasta verksamheten|Fastighetsmoms, jämkning och ändrad användning kan kräva särskild bedömning|Direkt kostnadsföring enligt K1 punkt 6.6 är ett undantag och får aldrig väljas automatiskt|Ej avdragsgilla fastighetskostnader måste bevaras för den skattemässiga justeringen</x:v>
+        <x:v>4900 ska motsvara förändringen mellan ingående och utgående lagervärde|Ett felaktigt tecken vänder resultatpåverkan|Inventering och värdering måste göras innan bokningen|Förenklingsregeln bedöms över den fysiska personens samtliga verksamheter|Fel tecken eller dubbel bokning ger motsatt resultat</x:v>
       </x:c>
       <x:c r="J116" s="14" t="str">
-        <x:v>fastighetskostnad|näringsfastighet|drift|förvaltning|reparation|R6</x:v>
+        <x:v>lagerförändring|varulager|inventering|lagervärde|R5|bokslut</x:v>
       </x:c>
       <x:c r="K116" s="14" t="str">
-        <x:v>5000|5500|1110|1130|1150|1230|2642</x:v>
+        <x:v>1400|4000|4700</x:v>
       </x:c>
       <x:c r="L116" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 5100, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.5–6.27 och 7.5–7.7|Skatteverket – Näringsfastigheter, avsnittet Reparation och underhåll, kontrollerat 2026-09-20</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 4900, rad R5|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.45–6.55 och 7.5–7.7 samt exemplen 6-9a, 6-9b och 6-10</x:v>
       </x:c>
       <x:c r="M116" s="14" t="str">
-        <x:v>Fastigheten används helt eller delvis privat eller verksamhetsandelen är oklar|Utgiften kan vara förbättring, ny-, till- eller ombyggnad eller annan anläggningstillgång|Bokningen kommer från BAS 5170 Reparation och underhåll och arbetets karaktär har inte verifierats|Bokningen kommer från BAS 5199 eller är på annat sätt markerad som ej avdragsgill|Moms, jämkning eller ändrad användning är oklar|Fastighetsobjekt, ägandeförhållande, fördelningsgrund eller projektkaraktär saknas eller är oklar|Posten avser tillfällig byggnad, bod eller container och klassificeringen är inte manuellt fastställd</x:v>
+        <x:v>Inventeringslista eller ingående lager saknas|Lagret ligger nära halvt prisbasbelopp|Flera verksamheter måste summeras|Lagret innehåller skadade, inkuranta, egentillverkade eller fastighetsrelaterade poster|Bokningens tecken eller föregående års omföring är oklar|Exakt konterings- och återföringsrutin är inte verifierad</x:v>
       </x:c>
       <x:c r="N116" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O116" s="14" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P116" s="14"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P116" s="14" t="str">
+        <x:v>inventory_optional_expensing_half_pbb|inventory_standard_reduction_3_percent</x:v>
+      </x:c>
       <x:c r="Q116" s="12" t="str"/>
     </x:row>
     <x:row r="117" ht="430" customHeight="1">
       <x:c r="A117" s="14" t="str">
-        <x:v>5200</x:v>
+        <x:v>5000</x:v>
       </x:c>
       <x:c r="B117" s="14" t="str">
-        <x:v>Hyra av anläggningstillgångar</x:v>
+        <x:v>Lokalkostnader</x:v>
       </x:c>
       <x:c r="C117" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för hyra eller leasing av maskiner, inventarier och andra anläggningstillgångar som inte är lokaler eller transportmedel.</x:v>
+        <x:v>Kostnadskonto på R6 för hyrda verksamhetslokaler och kostnader som direkt hör till användningen av sådana lokaler, exempelvis hyra, drift och lokalservice.</x:v>
       </x:c>
       <x:c r="D117" s="14" t="str">
-        <x:v>Företaget hyr eller leasar en maskin, inventarie, dator eller annan utrustning|Äganderätten ligger kvar hos uthyraren och avgiften avser nyttjandet|Kostnaden hör till verksamheten och kan kopplas till avtal och period</x:v>
+        <x:v>Företaget hyr en lokal som används i näringsverksamheten|Kostnaden avser lokalens löpande användning, drift, städning eller liknande|Utgiften kan kopplas till lokalavtal, period och verksamhetsanvändning</x:v>
       </x:c>
       <x:c r="E117" s="14" t="str">
-        <x:v>Avtalet avser lokal; använd 5000|Avtalet avser personbil eller annat transportmedel; använd 5600-serien|Transaktionen är ett köp, avbetalningsköp eller finansierad anskaffning som ska redovisas som tillgång|Beloppet är en återbetalningsbar deposition|Första förhöjda leasingavgiften ska tas upp som förskott enligt K1|Tillgången används privat utan dokumenterad fördelning</x:v>
+        <x:v>Fastigheten ägs av företaget eller ingår som näringsfastighet; pröva 5100|Beloppet är säkerhetsdeposition eller annan återbetalningsbar fordran|Utgiften skapar en bestående förbättring eller anläggningstillgång|Kostnaden avser privat bostad eller ett arbetsrum i bostaden utan verifierad avdragsrätt|Beloppet är hyra av maskin, inventarie eller fordon; använd 5200 eller relevant transportkonto</x:v>
       </x:c>
       <x:c r="F117" s="14" t="str">
-        <x:v>Verifiera avtal, uthyrd tillgång, nyttjandeperiod, avgiftsstruktur och äganderätt|Skilj löpande hyra från deposition, service, försäkring, köpoption och andra avtalsdelar|Bokför löpande avgift exklusive avdragsgill moms på 5200|Ta upp första förhöjd leasinghyra som förskott på B8 när K1:s beloppsvillkor är uppfyllt|Fördela kostnaden vid blandad privat användning enligt dokumenterat underlag|Stäm av mot 1700, 2440, 1930 och avtalsplan|Kräv manuell granskning om avtalet i praktiken kan vara köp eller innehåller större slutbetalning|Använd för vanlig hyra eller operationell leasing av utrustning|Klassificera avtal efter ekonomiskt innehåll|Förhöjd första avgift behandlas preliminärt som förskott|Begär hyres- eller leasingavtal när avgiften innehåller första förhöjd avgift, deposition, köpoption, slutbetalning eller privat användning|Bokför vanlig löpande hyra av utrustning på 5200 exklusive avdragsgill moms|Pröva första förhöjd leasingavgift mot den beslutade K1-rutinen och använd 1700 när belopps- och periodiseringsvillkoren är uppfyllda|Sätt ärendet till väntar på underlag när avtalet kan vara köp eller avbetalning eller när fordon, lokal, moms eller privat användning kräver annan behandling</x:v>
+        <x:v>Verifiera hyresvärd, lokal, avtal, period och verksamhetsanvändning|Bokför kostnaden exklusive avdragsgill ingående moms|Skilj löpande hyra och drift från deposition, förskott, inventariehyra och investering i lokalen|BAS 5070 Reparation och underhåll av lokaler får inte mappas automatiskt; kontrollera om arbetet helt eller delvis är en aktiverbar förbättring i hyrd lokal|BAS 5099 Ej avdragsgilla lokalkostnader kräver manuell granskning och dokumenterad skattemässig hantering|Fördela kostnaden vid blandad privat och företagsmässig användning endast enligt dokumenterad regel|Koppla kostnaden till lokal eller kostnadsställe när flera lokaler finns|Kontrollera om lokalen omfattas av frivillig beskattning och om avdragsrätten för moms är begränsad|Stäm av mot avtal, leverantörsfakturor, förskott, leverantörsskuld och betalningar|Kräv manuell granskning för arbetsrum i privatbostad, närståendehyra, större arbeten eller oklar momsbehandling</x:v>
       </x:c>
       <x:c r="G117" s="14" t="str">
-        <x:v>2440|1930|2641|1700|1600</x:v>
+        <x:v>2440|1930|2641|2642|1700|1600</x:v>
       </x:c>
       <x:c r="H117" s="14" t="str">
-        <x:v>Månadshyra för en kopiator bokförs på 5200|En första förhöjd leasingavgift över K1-gränsen tas upp som förskott och fördelas enligt den fastställda bokslutsrutinen</x:v>
+        <x:v>Månadshyra för en separat verksamhetslokal bokförs på 5000 med avdragsgill moms separat|En återbetalningsbar hyresdeposition bokförs som fordran och inte som lokalkostnad|En reparationsfaktura på BAS 5070 granskas för att skilja löpande återställande arbete från en aktiverbar förbättring i hyrd lokal|En kostnad märkt ej avdragsgill på BAS 5099 granskas och får inte automatiskt behandlas som en vanlig avdragsgill lokalkostnad</x:v>
       </x:c>
       <x:c r="I117" s="14" t="str">
-        <x:v>Avtalets rubrik avgör inte om transaktionen är hyra eller köp|Första förhöjd leasingavgift kan vara en balanspost|Lokaler och transportmedel har egna kontogrupper|Privat användning och begränsad momsavdragsrätt måste bedömas|Köp, avbetalningsköp eller finansiering med ägarövergång ska inte kostnadsföras här</x:v>
+        <x:v>Lokalkostnad och kostnad för ägd näringsfastighet måste skiljas åt|Kostnader för privatbostad och arbetsrum i bostaden har särskilda skatteregler|Förbättringar i hyrd lokal kan behöva aktiveras; kontonamnet 5070 bevisar inte att hela utgiften får kostnadsföras direkt|Moms på lokalhyra förutsätter korrekt momsbehandling och kan påverkas av frivillig beskattning|Ej avdragsgilla lokalkostnader måste bevaras för den skattemässiga justeringen</x:v>
       </x:c>
       <x:c r="J117" s="14" t="str">
-        <x:v>hyra anläggningstillgång|leasing|maskinhyra|inventariehyra|första förhöjd leasingavgift|R6</x:v>
+        <x:v>lokalkostnad|lokalhyra|verksamhetslokal|städning|drift|R6</x:v>
       </x:c>
       <x:c r="K117" s="14" t="str">
-        <x:v>5000|5600|1700|1220|1240|2440|2641</x:v>
+        <x:v>5100|5200|5500|1700|1600|2440|2641|2642</x:v>
       </x:c>
       <x:c r="L117" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 5200, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 6.59 och punkterna 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 5000, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.5–6.27 och 7.5–7.7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och periodavstämning</x:v>
       </x:c>
       <x:c r="M117" s="14" t="str">
-        <x:v>Avtalet kan vara köp eller avbetalning|Första förhöjd avgift, deposition eller köpoption förekommer|Tillgången används privat|Momsavdraget är begränsat|Avtalet avser fordon eller lokal|Köpoption, stor slutbetalning eller periodiseringsrutin är oklar</x:v>
+        <x:v>Lokalen används helt eller delvis privat eller verksamhetsandelen är oklar|Arbetsrum i bostad eller närståendehyra förekommer|Deposition, förskott eller större arbete ingår|Bokningen kommer från BAS 5070 och arbetets karaktär inte har verifierats|Bokningen kommer från BAS 5099 eller är på annat sätt markerad som ej avdragsgill|Moms på hyran, frivillig beskattning eller avdragsrätt är oklar|Kostnaden kan höra till ägd fastighet eller en annan tillgång</x:v>
       </x:c>
       <x:c r="N117" s="14" t="str">
         <x:v>active</x:v>
@@ -6604,50 +6608,48 @@
       <x:c r="O117" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P117" s="14" t="str">
-        <x:v>first_increased_lease_fee_over_5000</x:v>
-      </x:c>
+      <x:c r="P117" s="14"/>
       <x:c r="Q117" s="12" t="str"/>
     </x:row>
     <x:row r="118" ht="430" customHeight="1">
       <x:c r="A118" s="14" t="str">
-        <x:v>5400</x:v>
+        <x:v>5100</x:v>
       </x:c>
       <x:c r="B118" s="14" t="str">
-        <x:v>Förbrukningsinventarier och förbrukningsmaterial</x:v>
+        <x:v>Fastighetskostnader</x:v>
       </x:c>
       <x:c r="C118" s="14" t="str">
-        <x:v>K1-konto på R6 för förbrukningsmaterial samt inventarier som får kostnadsföras direkt därför att anskaffningsvärdet understiger ett halvt prisbasbelopp eller den ekonomiska livslängden är högst tre år.</x:v>
+        <x:v>Kostnadskonto på R6 för löpande drift, förvaltning och andra kostnader som hör till en fastighet i näringsverksamheten. Förbättringar och ny-, till- eller ombyggnad ska inte kostnadsföras här.</x:v>
       </x:c>
       <x:c r="D118" s="14" t="str">
-        <x:v>Inköpet är vanligt förbrukningsmaterial som används i verksamheten och inte ska säljas vidare|Inventariens anskaffningsvärde understiger ett halvt prisbasbelopp efter bedömning av föremål som hör naturligt samman|Inventariens ekonomiska livslängd kan visas vara högst tre år|Kortlivad utrustning, emballage eller skyddsmaterial har tydlig koppling till verksamheten</x:v>
+        <x:v>Företaget eller näringsverksamheten äger eller redovisar fastigheten|Utgiften avser löpande drift, tillsyn, service, förvaltning eller annan fastighetskostnad|Kostnaden hör till årets användning av fastigheten|En byggnad med mycket kort användningstid har efter manuell granskning godkänts för direkt kostnadsföring enligt K1 punkt 6.6</x:v>
       </x:c>
       <x:c r="E118" s="14" t="str">
-        <x:v>Inköpet är en handelsvara, råvara eller material som direkt ingår i kundens leverans; använd 4000|Inventarien överstiger gränsen och har en ekonomisk livslängd längre än tre år; använd normalt 1220|Flera föremål hör naturligt samman eller ingår i en större investering och överstiger gränsen tillsammans|Utgiften avser reparation eller underhåll; använd 5500|Programvaran är ett abonnemang eller en tjänst och ska redovisas som IT-tjänst|Arbetskläderna är vanliga privata kläder utan tydlig skydds- eller yrkesfunktion|Inköpet är privat</x:v>
+        <x:v>Företaget hyr lokalen; använd normalt 5000|Utgiften avser ny-, till- eller ombyggnad eller annan värdehöjande förbättring|Beloppet ska ingå i anskaffningsvärdet för byggnad, markanläggning eller byggnadsinventarie|Utgiften avser ränta, amortering eller privat bostadsdel|Utgiften är reparation av fordon, maskin eller annan tillgång|Objektet är egentligen inventarie, hyrd bod, container eller lokal</x:v>
       </x:c>
       <x:c r="F118" s="14" t="str">
-        <x:v>Identifiera vad som köpts, hur det används, anskaffningsvärde och förväntad ekonomisk livslängd|Vanligt förbrukningsmaterial som inte är lager kan kostnadsföras på 5400|En inventarie får kostnadsföras direkt om anskaffningsvärdet understiger ett halvt prisbasbelopp eller den ekonomiska livslängden är högst tre år|Bedöm föremål med naturligt samband eller som ingår i en större investering tillsammans|Beräkna anskaffningsvärdet exklusive avdragsgill moms men inklusive moms som inte får dras av|Inventarier som både överstiger beloppsgränsen och har längre ekonomisk livslängd än tre år ska normalt föras till 1220|BAS 5412, 5440, 5460, 5492 och 5493 får sammanföras automatiskt till 5400|BAS 5400, 5410, 5411, 5490 och 5491 kräver kontroll av belopp, livslängd och eventuellt naturligt samband|BAS 5420 kräver kontroll av om programvaran är en tillgång, ett mindre direktavdragsgillt inköp eller en löpande tjänst|BAS 5430 kräver kontroll av vad transportinventarien består av och om den ska aktiveras|BAS 5480 kräver kontroll av att kläderna eller skyddsmaterialet är avdragsgilla och tydligt hör till verksamheten</x:v>
+        <x:v>Verifiera fastighet, ägande eller nyttjanderätt, verksamhetsanknytning och kostnadstyp|Fördela kostnaden mellan näringsdel och privat del när fastigheten används blandat och bokför endast verksamhetsandelen|Skilj löpande drift och återställande reparation från förbättring, nybyggnad, tillbyggnad, ombyggnad och annan anläggningstillgång|BAS 5170 Reparation och underhåll får inte mappas automatiskt; kontrollera alltid om arbetet helt eller delvis ska aktiveras|BAS 5199 Ej avdragsgilla fastighetskostnader kräver manuell granskning och dokumenterad skattemässig hantering|Bokför avdragsgill moms separat och kontrollera fastighetsrelaterade begränsningar, jämkning och ändrad användning|Koppla fakturor och betalningar till fastighetsobjekt och period och stäm av mot relevanta tillgångs- och skuldkonton|Kräv manuell granskning vid näringsfastighet med privat användning, större arbeten, ändrad användning eller oklar fördelningsgrund|Direkt kostnadsförd tillfällig byggnad får endast bokföras här efter manuell granskning enligt K1 punkt 6.6 och ska märkas som sådan|Ta inte upp en godkänd direkt kostnadsförd tillfällig byggnad på 1110 och skriv inte av den via 1119 eller 7820|Pröva först om flyttbar bod, container eller liknande i stället är inventarie, hyra eller lokal</x:v>
       </x:c>
       <x:c r="G118" s="14" t="str">
-        <x:v>2440|1930|2641|1220|4000</x:v>
+        <x:v>2440|1930|2641|2642|1110|1130|1150|1230</x:v>
       </x:c>
       <x:c r="H118" s="14" t="str">
-        <x:v>Pennor, rengöringsmaterial och enklare emballage som används i verksamheten bokförs på 5400|Ett fristående verktyg under den aktuella gränsen kan kostnadsföras på 5400|Dator, skärm och tillbehör som köps tillsammans bedöms som en helhet innan direkt kostnadsföring|En dyrare maskin med längre livslängd än tre år bokförs normalt på 1220 och skrivs av|Skyddsglasögon och annan tydlig skyddsutrustning kan bokföras på 5400, medan vanliga privata kläder inte ska göra det</x:v>
+        <x:v>Löpande el, värme, vatten, sophämtning eller fastighetsskötsel för en verksamhetsfastighet bokförs normalt på 5100|En reparationsfaktura på BAS 5170 granskas för att skilja återställande reparation från aktiverbar förbättring|En tillbyggnad som ger bestående värde aktiveras på relevant tillgångskonto och bokförs inte som fastighetskostnad|En kostnad märkt ej avdragsgill på BAS 5199 granskas och får inte automatiskt behandlas som en vanlig avdragsgill kostnad|En enkel tillfällig byggnad med verifierad kort användningstid bokförs efter manuell granskning på 5100</x:v>
       </x:c>
       <x:c r="I118" s="14" t="str">
-        <x:v>Dela inte upp ett sammanhängande inköp för att komma under beloppsgränsen|Beloppsgränsen och högst tre års ekonomisk livslängd är två alternativa grunder för direkt kostnadsföring|Tre år är en bedömning av ekonomisk livslängd och inte en avskrivningstid|Programvara kan behöva redovisas på annat konto beroende på vad som faktiskt köpts|Vanliga kläder är normalt privata även om de används i arbetet</x:v>
+        <x:v>Ägd fastighet och hyrd lokal ska hållas isär|Reparation och förbättring är olika redovisningshändelser; kontonamnet 5170 bevisar inte att hela utgiften får kostnadsföras direkt|Privat del får inte belasta verksamheten|Fastighetsmoms, jämkning och ändrad användning kan kräva särskild bedömning|Direkt kostnadsföring enligt K1 punkt 6.6 är ett undantag och får aldrig väljas automatiskt|Ej avdragsgilla fastighetskostnader måste bevaras för den skattemässiga justeringen</x:v>
       </x:c>
       <x:c r="J118" s="14" t="str">
-        <x:v>förbrukningsinventarie|förbrukningsmaterial|mindre värde|tre år|R6|direkt kostnadsföring</x:v>
+        <x:v>fastighetskostnad|näringsfastighet|drift|förvaltning|reparation|R6</x:v>
       </x:c>
       <x:c r="K118" s="14" t="str">
-        <x:v>1220|4000|5500|6100|6500|2440|2641</x:v>
+        <x:v>5000|5500|1110|1130|1150|1230|2642</x:v>
       </x:c>
       <x:c r="L118" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – konto 5400, rad R6|BFNAR 2006:1, punkterna 6.29–6.36|Skatteverket, Avdrag för värdeminskning, regler för 2026</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 5100, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.5–6.27 och 7.5–7.7|Skatteverket – Näringsfastigheter, avsnittet Reparation och underhåll, kontrollerat 2026-09-20</x:v>
       </x:c>
       <x:c r="M118" s="14" t="str">
-        <x:v>Inventarien ligger nära eller över ett halvt prisbasbelopp|Flera föremål kan höra naturligt samman eller ingå i en större investering|Ekonomisk livslängd är längre än eller osäkert omkring tre år|Posten kommer från BAS 5400, 5410, 5411, 5420, 5430, 5480, 5490 eller 5491|Programvarans form eller arbetsklädernas avdragsrätt är oklar|Inköpet kan vara lager, anläggningstillgång, IT-tjänst eller privat</x:v>
+        <x:v>Fastigheten används helt eller delvis privat eller verksamhetsandelen är oklar|Utgiften kan vara förbättring, ny-, till- eller ombyggnad eller annan anläggningstillgång|Bokningen kommer från BAS 5170 Reparation och underhåll och arbetets karaktär har inte verifierats|Bokningen kommer från BAS 5199 eller är på annat sätt markerad som ej avdragsgill|Moms, jämkning eller ändrad användning är oklar|Fastighetsobjekt, ägandeförhållande, fördelningsgrund eller projektkaraktär saknas eller är oklar|Posten avser tillfällig byggnad, bod eller container och klassificeringen är inte manuellt fastställd</x:v>
       </x:c>
       <x:c r="N118" s="14" t="str">
         <x:v>active</x:v>
@@ -6655,50 +6657,48 @@
       <x:c r="O118" s="14" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="P118" s="14" t="str">
-        <x:v>low_value_inventory_half_pbb|economic_life_max_3_years</x:v>
-      </x:c>
+      <x:c r="P118" s="14"/>
       <x:c r="Q118" s="12" t="str"/>
     </x:row>
     <x:row r="119" ht="430" customHeight="1">
       <x:c r="A119" s="14" t="str">
-        <x:v>5500</x:v>
+        <x:v>5200</x:v>
       </x:c>
       <x:c r="B119" s="14" t="str">
-        <x:v>Reparation och underhåll</x:v>
+        <x:v>Hyra av anläggningstillgångar</x:v>
       </x:c>
       <x:c r="C119" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för åtgärder som återställer eller bibehåller en befintlig tillgångs funktion och skick utan att skapa en ny tillgång eller en väsentlig bestående förbättring.</x:v>
+        <x:v>Kostnadskonto på R6 för hyra eller leasing av maskiner, inventarier och andra anläggningstillgångar som inte är lokaler eller transportmedel.</x:v>
       </x:c>
       <x:c r="D119" s="14" t="str">
-        <x:v>En befintlig maskin, inventarie, lokal eller annan tillgång repareras eller underhålls|Åtgärden återställer normal funktion eller förebygger slitage|Utgiften ska kostnadsföras och kan kopplas till en identifierad tillgång</x:v>
+        <x:v>Företaget hyr eller leasar en maskin, inventarie, dator eller annan utrustning|Äganderätten ligger kvar hos uthyraren och avgiften avser nyttjandet|Kostnaden hör till verksamheten och kan kopplas till avtal och period</x:v>
       </x:c>
       <x:c r="E119" s="14" t="str">
-        <x:v>Åtgärden är nyanskaffning, utbyte som skapar en separat tillgång eller en väsentlig förbättring|Arbetet avser personbil eller annat transportmedel; använd relevant 56-konto|Arbetet hör till ägd fastighets löpande kostnader där 5100 används enligt kontoplanen|Beloppet är garantiåtgärd som leverantören står för utan företagets kostnad|Tillgången är privat</x:v>
+        <x:v>Avtalet avser lokal; använd 5000|Avtalet avser personbil eller annat transportmedel; använd 5600-serien|Transaktionen är ett köp, avbetalningsköp eller finansierad anskaffning som ska redovisas som tillgång|Beloppet är en återbetalningsbar deposition|Första förhöjda leasingavgiften ska tas upp som förskott enligt K1|Tillgången används privat utan dokumenterad fördelning</x:v>
       </x:c>
       <x:c r="F119" s="14" t="str">
-        <x:v>Identifiera den befintliga tillgången och dess funktion före åtgärden|Dokumentera fel, åtgärd, utbytta delar och om kapacitet eller livslängd ökar väsentligt|Kostnadsför åtgärden på 5500 när den endast återställer eller bibehåller funktion|Aktivera utgiften på relevant tillgångskonto när den skapar eller förbättrar en tillgång enligt K1|Dela fakturan när den innehåller både reparation och nyinvestering|Bokför avdragsgill moms separat|Koppla till tillgångs-ID, serviceorder och faktura|Kräv manuell granskning vid större belopp, ombyggnad, komponentbyte eller försäkringsersättning|Kostnadsför arbete som återställer tidigare funktion|Pröva aktivering vid ny komponent eller väsentligt höjd standard, kapacitet eller livslängd|Dela blandad faktura radvis|Vid granskningsflagga begär in fakturaspecifikation, arbetsbeskrivning och uppgift om vilken befintlig tillgång som åtgärdats|Sätt ärendet till väntar på underlag tills reparation kan skiljas från nyanskaffning eller förbättring|Godkänn 5500 när åtgärden endast återställer eller bibehåller tillgångens tidigare funktion|Föreslå uppdelning eller omklassificering till relevant tillgångskonto när åtgärden skapar en ny eller väsentligt förbättrad tillgång</x:v>
+        <x:v>Verifiera avtal, uthyrd tillgång, nyttjandeperiod, avgiftsstruktur och äganderätt|Skilj löpande hyra från deposition, service, försäkring, köpoption och andra avtalsdelar|Bokför löpande avgift exklusive avdragsgill moms på 5200|Ta upp första förhöjd leasinghyra som förskott på B8 när K1:s beloppsvillkor är uppfyllt|Fördela kostnaden vid blandad privat användning enligt dokumenterat underlag|Stäm av mot 1700, 2440, 1930 och avtalsplan|Kräv manuell granskning om avtalet i praktiken kan vara köp eller innehåller större slutbetalning|Använd för vanlig hyra eller operationell leasing av utrustning|Klassificera avtal efter ekonomiskt innehåll|Förhöjd första avgift behandlas preliminärt som förskott|Begär hyres- eller leasingavtal när avgiften innehåller första förhöjd avgift, deposition, köpoption, slutbetalning eller privat användning|Bokför vanlig löpande hyra av utrustning på 5200 exklusive avdragsgill moms|Pröva första förhöjd leasingavgift mot den beslutade K1-rutinen och använd 1700 när belopps- och periodiseringsvillkoren är uppfyllda|Sätt ärendet till väntar på underlag när avtalet kan vara köp eller avbetalning eller när fordon, lokal, moms eller privat användning kräver annan behandling</x:v>
       </x:c>
       <x:c r="G119" s="14" t="str">
-        <x:v>2440|1930|2641|1220|1110|1150|1230</x:v>
+        <x:v>2440|1930|2641|1700|1600</x:v>
       </x:c>
       <x:c r="H119" s="14" t="str">
-        <x:v>Byte av en sliten mindre del för att återställa en maskins funktion bokförs på 5500|En ombyggnad som väsentligt ökar kapacitet eller livslängd aktiveras i stället</x:v>
+        <x:v>Månadshyra för en kopiator bokförs på 5200|En första förhöjd leasingavgift över K1-gränsen tas upp som förskott och fördelas enligt den fastställda bokslutsrutinen</x:v>
       </x:c>
       <x:c r="I119" s="14" t="str">
-        <x:v>Reparation och förbättring måste skiljas åt utifrån åtgärdens ekonomiska innebörd|Fakturans rubrik avgör inte klassificeringen|Större komponentbyten kan behöva delas eller aktiveras|Fordon och vissa fastighetskostnader har mer specifika konton|Saknad specifikation ska kompletteras innan bokning</x:v>
+        <x:v>Avtalets rubrik avgör inte om transaktionen är hyra eller köp|Första förhöjd leasingavgift kan vara en balanspost|Lokaler och transportmedel har egna kontogrupper|Privat användning och begränsad momsavdragsrätt måste bedömas|Köp, avbetalningsköp eller finansiering med ägarövergång ska inte kostnadsföras här</x:v>
       </x:c>
       <x:c r="J119" s="14" t="str">
-        <x:v>reparation|underhåll|service|förbättring|komponentbyte|R6</x:v>
+        <x:v>hyra anläggningstillgång|leasing|maskinhyra|inventariehyra|första förhöjd leasingavgift|R6</x:v>
       </x:c>
       <x:c r="K119" s="14" t="str">
-        <x:v>5100|5400|5613|1220|1110|1150|1230|2440</x:v>
+        <x:v>5000|5600|1700|1220|1240|2440|2641</x:v>
       </x:c>
       <x:c r="L119" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5500, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, reglerna om anskaffningsvärde och kostnadsföring i kapitel 6 samt punkterna 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 5, konto 5200, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 6.59 och punkterna 7.5–7.7</x:v>
       </x:c>
       <x:c r="M119" s="14" t="str">
-        <x:v>Åtgärden kan öka kapacitet, standard eller livslängd|Fakturan innehåller både reparation och investering|Fastighet, fordon eller större komponent berörs|Tillgångs-ID eller arbetsbeskrivning saknas|Försäkringsersättning eller garanti förekommer|Reparation och investering kan inte skiljas åt</x:v>
+        <x:v>Avtalet kan vara köp eller avbetalning|Första förhöjd avgift, deposition eller köpoption förekommer|Tillgången används privat|Momsavdraget är begränsat|Avtalet avser fordon eller lokal|Köpoption, stor slutbetalning eller periodiseringsrutin är oklar</x:v>
       </x:c>
       <x:c r="N119" s="14" t="str">
         <x:v>active</x:v>
@@ -6706,97 +6706,101 @@
       <x:c r="O119" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P119" s="14"/>
+      <x:c r="P119" s="14" t="str">
+        <x:v>first_increased_lease_fee_over_5000</x:v>
+      </x:c>
       <x:c r="Q119" s="12" t="str"/>
     </x:row>
     <x:row r="120" ht="430" customHeight="1">
       <x:c r="A120" s="14" t="str">
-        <x:v>5600</x:v>
+        <x:v>5400</x:v>
       </x:c>
       <x:c r="B120" s="14" t="str">
-        <x:v>Kostnader för transportmedel</x:v>
+        <x:v>Förbrukningsinventarier och förbrukningsmaterial</x:v>
       </x:c>
       <x:c r="C120" s="14" t="str">
-        <x:v>Huvud- eller samlingskonto på R6 för kostnader för företagets transportmedel. Mer specifika underkonton bör användas när fordonstyp och kostnadstyp är kända.</x:v>
+        <x:v>K1-konto på R6 för förbrukningsmaterial samt inventarier som får kostnadsföras direkt därför att anskaffningsvärdet understiger ett halvt prisbasbelopp eller den ekonomiska livslängden är högst tre år.</x:v>
       </x:c>
       <x:c r="D120" s="14" t="str">
-        <x:v>Kostnaden hör till ett transportmedel som används i verksamheten|Fordonstypen eller kostnadstypen är ännu inte särredovisad men systemets kontoplan tillåter 5600|Beloppet ska ingå i R6</x:v>
+        <x:v>Inköpet är vanligt förbrukningsmaterial som används i verksamheten och inte ska säljas vidare|Inventariens anskaffningsvärde understiger ett halvt prisbasbelopp efter bedömning av föremål som hör naturligt samman|Inventariens ekonomiska livslängd kan visas vara högst tre år|Kortlivad utrustning, emballage eller skyddsmaterial har tydlig koppling till verksamheten</x:v>
       </x:c>
       <x:c r="E120" s="14" t="str">
-        <x:v>Kostnaden avser frakt eller transporttjänst köpt från extern transportör; använd 5700|Beloppet är anskaffning av ett fordon; använd 1240/1241|Kostnaden avser privat bil som ersätts enligt schablon; använd 5618|Ett mer specifikt underkonto som 5610–5620 ska användas enligt kontoplanen|Privat användning eller fordonstillhörighet är oklar</x:v>
+        <x:v>Inköpet är en handelsvara, råvara eller material som direkt ingår i kundens leverans; använd 4000|Inventarien överstiger gränsen och har en ekonomisk livslängd längre än tre år; använd normalt 1220|Flera föremål hör naturligt samman eller ingår i en större investering och överstiger gränsen tillsammans|Utgiften avser reparation eller underhåll; använd 5500|Programvaran är ett abonnemang eller en tjänst och ska redovisas som IT-tjänst|Arbetskläderna är vanliga privata kläder utan tydlig skydds- eller yrkesfunktion|Inköpet är privat</x:v>
       </x:c>
       <x:c r="F120" s="14" t="str">
-        <x:v>Identifiera fordon, registreringsnummer, ägande eller leasing och användning|Klassificera kostnaden som drivmedel, försäkring och skatt, reparation, leasing eller övrigt|Använd specifikt underkonto när uppgifterna finns|Bokför endast företagets andel av kostnaden|Bedöm momsavdragsrätten separat per fordonstyp och användning|Koppla kvitto eller faktura till fordonsregister och period|Stäm av mot 1240, leasingavtal, körjournal och eget uttag|Blockera 5600 som ospecificerat restkonto vid bokslut|Använd inte som ospecificerat restkonto|Koppla varje kostnad till fordon och kostnadstyp genom fordonsreskontra|Vid granskningsflagga begär in kvitto eller faktura samt registreringsnummer, ägandeform och kostnadstyp|Sätt ärendet till väntar på underlag tills fordon, verksamhetsandel och momsbehandling är klarlagda|Godkänn 5600 när kostnaden hör till verksamhetens transportmedel men mer specifikt underkonto inte kan fastställas|Föreslå specifikt 56-konto, 5700 eller privat kostnad när underlaget visar en tydligare klassificering</x:v>
+        <x:v>Identifiera vad som köpts, hur det används, anskaffningsvärde och förväntad ekonomisk livslängd|Vanligt förbrukningsmaterial som inte är lager kan kostnadsföras på 5400|En inventarie får kostnadsföras direkt om anskaffningsvärdet understiger ett halvt prisbasbelopp eller den ekonomiska livslängden är högst tre år|Bedöm föremål med naturligt samband eller som ingår i en större investering tillsammans|Beräkna anskaffningsvärdet exklusive avdragsgill moms men inklusive moms som inte får dras av|Inventarier som både överstiger beloppsgränsen och har längre ekonomisk livslängd än tre år ska normalt föras till 1220|BAS 5412, 5440, 5460, 5492 och 5493 får sammanföras automatiskt till 5400|BAS 5400, 5410, 5411, 5490 och 5491 kräver kontroll av belopp, livslängd och eventuellt naturligt samband|BAS 5420 kräver kontroll av om programvaran är en tillgång, ett mindre direktavdragsgillt inköp eller en löpande tjänst|BAS 5430 kräver kontroll av vad transportinventarien består av och om den ska aktiveras|BAS 5480 kräver kontroll av att kläderna eller skyddsmaterialet är avdragsgilla och tydligt hör till verksamheten</x:v>
       </x:c>
       <x:c r="G120" s="14" t="str">
-        <x:v>2440|1930|2641|1240|2014|3200</x:v>
+        <x:v>2440|1930|2641|1220|4000</x:v>
       </x:c>
       <x:c r="H120" s="14" t="str">
-        <x:v>En ospecificerad fordonskostnad kan tillfälligt ligga på 5600 endast om den senare klassificeras till rätt fordons- och kostnadstyp</x:v>
+        <x:v>Pennor, rengöringsmaterial och enklare emballage som används i verksamheten bokförs på 5400|Ett fristående verktyg under den aktuella gränsen kan kostnadsföras på 5400|Dator, skärm och tillbehör som köps tillsammans bedöms som en helhet innan direkt kostnadsföring|En dyrare maskin med längre livslängd än tre år bokförs normalt på 1220 och skrivs av|Skyddsglasögon och annan tydlig skyddsutrustning kan bokföras på 5400, medan vanliga privata kläder inte ska göra det</x:v>
       </x:c>
       <x:c r="I120" s="14" t="str">
-        <x:v>5600 bör inte användas när ett mer specifikt konto kan väljas|Företagsägd bil och privat bil har olika kostnadsmodeller|Momsavdrag och privat användning måste bedömas separat|Frakt- och transporttjänster från extern leverantör hör normalt till 5700|Direktbokning utan fordons- och kostnadsspecifikation ska stoppas</x:v>
+        <x:v>Dela inte upp ett sammanhängande inköp för att komma under beloppsgränsen|Beloppsgränsen och högst tre års ekonomisk livslängd är två alternativa grunder för direkt kostnadsföring|Tre år är en bedömning av ekonomisk livslängd och inte en avskrivningstid|Programvara kan behöva redovisas på annat konto beroende på vad som faktiskt köpts|Vanliga kläder är normalt privata även om de används i arbetet</x:v>
       </x:c>
       <x:c r="J120" s="14" t="str">
-        <x:v>transportmedel|fordonskostnad|bilkostnad|lastbil|R6|samlingskonto</x:v>
+        <x:v>förbrukningsinventarie|förbrukningsmaterial|mindre värde|tre år|R6|direkt kostnadsföring</x:v>
       </x:c>
       <x:c r="K120" s="14" t="str">
-        <x:v>1240|5610|5611|5612|5613|5615|5618|5619|5620|5700</x:v>
+        <x:v>1220|4000|5500|6100|6500|2440|2641</x:v>
       </x:c>
       <x:c r="L120" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5600, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – konto 5400, rad R6|BFNAR 2006:1, punkterna 6.29–6.36|Skatteverket, Avdrag för värdeminskning, regler för 2026</x:v>
       </x:c>
       <x:c r="M120" s="14" t="str">
-        <x:v>Fordon eller kostnadstyp är inte identifierad|Privat användning förekommer|Momsavdragsrätten är oklar|Fordonet kan vara privatägt, leasat eller felklassificerat|Kontot har ospecificerat saldo vid bokslut|Fordon eller kostnadstyp saknas</x:v>
+        <x:v>Inventarien ligger nära eller över ett halvt prisbasbelopp|Flera föremål kan höra naturligt samman eller ingå i en större investering|Ekonomisk livslängd är längre än eller osäkert omkring tre år|Posten kommer från BAS 5400, 5410, 5411, 5420, 5430, 5480, 5490 eller 5491|Programvarans form eller arbetsklädernas avdragsrätt är oklar|Inköpet kan vara lager, anläggningstillgång, IT-tjänst eller privat</x:v>
       </x:c>
       <x:c r="N120" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O120" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P120" s="14"/>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P120" s="14" t="str">
+        <x:v>low_value_inventory_half_pbb|economic_life_max_3_years</x:v>
+      </x:c>
       <x:c r="Q120" s="12" t="str"/>
     </x:row>
     <x:row r="121" ht="430" customHeight="1">
       <x:c r="A121" s="14" t="str">
-        <x:v>5610</x:v>
+        <x:v>5500</x:v>
       </x:c>
       <x:c r="B121" s="14" t="str">
-        <x:v>Personbilskostnader</x:v>
+        <x:v>Reparation och underhåll</x:v>
       </x:c>
       <x:c r="C121" s="14" t="str">
-        <x:v>Huvud- eller samlingskonto på R6 för kostnader för en personbil som hör till näringsverksamheten genom ägande eller leasing. Underkonton 5611–5619 bör användas när kostnadstypen är känd.</x:v>
+        <x:v>Kostnadskonto på R6 för åtgärder som återställer eller bibehåller en befintlig tillgångs funktion och skick utan att skapa en ny tillgång eller en väsentlig bestående förbättring.</x:v>
       </x:c>
       <x:c r="D121" s="14" t="str">
-        <x:v>Kostnaden hör till en personbil som är bokförd som tillgång i verksamheten eller leasas av verksamheten|Fordonet och verksamhetsanvändningen är identifierade|Systemets momskontoplan tillåter samlingskonto 5610</x:v>
+        <x:v>En befintlig maskin, inventarie, lokal eller annan tillgång repareras eller underhålls|Åtgärden återställer normal funktion eller förebygger slitage|Utgiften ska kostnadsföras och kan kopplas till en identifierad tillgång</x:v>
       </x:c>
       <x:c r="E121" s="14" t="str">
-        <x:v>Bilen är privatägd och endast används för resor i verksamheten; använd normalt 5618 enligt aktuell schablonregel|Beloppet är inköp av bilen; använd 1240/1241|Kostnaden avser lastbil eller annat transportmedel|Ett specifikt underkonto 5611–5619 kan användas och krävs|Privat användning eller bilens tillhörighet är inte utredd</x:v>
+        <x:v>Åtgärden är nyanskaffning, utbyte som skapar en separat tillgång eller en väsentlig förbättring|Arbetet avser personbil eller annat transportmedel; använd relevant 56-konto|Arbetet hör till ägd fastighets löpande kostnader där 5100 används enligt kontoplanen|Beloppet är garantiåtgärd som leverantören står för utan företagets kostnad|Tillgången är privat</x:v>
       </x:c>
       <x:c r="F121" s="14" t="str">
-        <x:v>Verifiera registreringsnummer, ägare eller leasingtagare och datum då bilen hör till verksamheten|Koppla kostnaden till bilen och kostnadstyp|Använd specifikt underkonto för drivmedel, försäkring och skatt, reparation, leasing, privat bil eller övrigt när möjligt|Bokför endast företagets kostnadsandel|Registrera privat användning och hantera eget uttag och förmånsintäkt enligt separat regel|Bedöm momsavdragsrätten per kostnad och biltyp|Stäm av mot 1240, körjournal, leasingavtal, 2014 och 3200|Kräv manuell granskning när bilen används blandat|Använd endast med sidoordnad specifikation per personbil|Skilj verksamhetsbil, leasingbil och privat bil|Vid granskningsflagga begär in kvitto eller faktura, registreringsnummer, ägar- eller leasinguppgift och uppgift om användningen|Sätt ärendet till väntar på underlag tills bilen och verksamhetsandelen är verifierade|Godkänn 5610 när kostnaden hör till en företagsbokförd eller leasad personbil men kostnadstypen inte kan specificeras ytterligare|Föreslå 5611–5619 eller privatbilsflödet när kostnadstyp eller ägandeform kan fastställas</x:v>
+        <x:v>Identifiera den befintliga tillgången och dess funktion före åtgärden|Dokumentera fel, åtgärd, utbytta delar och om kapacitet eller livslängd ökar väsentligt|Kostnadsför åtgärden på 5500 när den endast återställer eller bibehåller funktion|Aktivera utgiften på relevant tillgångskonto när den skapar eller förbättrar en tillgång enligt K1|Dela fakturan när den innehåller både reparation och nyinvestering|Bokför avdragsgill moms separat|Koppla till tillgångs-ID, serviceorder och faktura|Kräv manuell granskning vid större belopp, ombyggnad, komponentbyte eller försäkringsersättning|Kostnadsför arbete som återställer tidigare funktion|Pröva aktivering vid ny komponent eller väsentligt höjd standard, kapacitet eller livslängd|Dela blandad faktura radvis|Vid granskningsflagga begär in fakturaspecifikation, arbetsbeskrivning och uppgift om vilken befintlig tillgång som åtgärdats|Sätt ärendet till väntar på underlag tills reparation kan skiljas från nyanskaffning eller förbättring|Godkänn 5500 när åtgärden endast återställer eller bibehåller tillgångens tidigare funktion|Föreslå uppdelning eller omklassificering till relevant tillgångskonto när åtgärden skapar en ny eller väsentligt förbättrad tillgång</x:v>
       </x:c>
       <x:c r="G121" s="14" t="str">
-        <x:v>2440|1930|2641|1240|2014|3200</x:v>
+        <x:v>2440|1930|2641|1220|1110|1150|1230</x:v>
       </x:c>
       <x:c r="H121" s="14" t="str">
-        <x:v>Kostnader för en företagsbokförd personbil samlas under 5610-gruppen och fördelas på rätt underkonto|Resor med en privatägd bil bokförs inte som faktiska personbilskostnader på 5610</x:v>
+        <x:v>Byte av en sliten mindre del för att återställa en maskins funktion bokförs på 5500|En ombyggnad som väsentligt ökar kapacitet eller livslängd aktiveras i stället</x:v>
       </x:c>
       <x:c r="I121" s="14" t="str">
-        <x:v>Företagsbil och privat bil måste skiljas åt|Enskild näringsidkare kan behöva redovisa privat nyttjande som uttag och förmånsintäkt|Momsavdrag är inte automatiskt fullt|Samlingskontot bör inte dölja kostnadstyp|Privat bil ska inte behandlas som företagets tillgång eller faktiska bilkostnad</x:v>
+        <x:v>Reparation och förbättring måste skiljas åt utifrån åtgärdens ekonomiska innebörd|Fakturans rubrik avgör inte klassificeringen|Större komponentbyten kan behöva delas eller aktiveras|Fordon och vissa fastighetskostnader har mer specifika konton|Saknad specifikation ska kompletteras innan bokning</x:v>
       </x:c>
       <x:c r="J121" s="14" t="str">
-        <x:v>personbilskostnad|företagsbil|leasad bil|privat användning|R6</x:v>
+        <x:v>reparation|underhåll|service|förbättring|komponentbyte|R6</x:v>
       </x:c>
       <x:c r="K121" s="14" t="str">
-        <x:v>1240|5611|5612|5613|5615|5618|5619|2014|3200</x:v>
+        <x:v>5100|5400|5613|1220|1110|1150|1230|2440</x:v>
       </x:c>
       <x:c r="L121" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5610, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.3–2.4, 3.17–3.18 och 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5500, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, reglerna om anskaffningsvärde och kostnadsföring i kapitel 6 samt punkterna 7.5–7.7</x:v>
       </x:c>
       <x:c r="M121" s="14" t="str">
-        <x:v>Bilens ägande eller leasing är oklar|Privat användning förekommer|Momsavdragsrätten är begränsad|Bilen kan vara privatägd|Kostnadstypen är ospecificerad|Ägande, leasingform eller användning är oklar</x:v>
+        <x:v>Åtgärden kan öka kapacitet, standard eller livslängd|Fakturan innehåller både reparation och investering|Fastighet, fordon eller större komponent berörs|Tillgångs-ID eller arbetsbeskrivning saknas|Försäkringsersättning eller garanti förekommer|Reparation och investering kan inte skiljas åt</x:v>
       </x:c>
       <x:c r="N121" s="14" t="str">
         <x:v>active</x:v>
@@ -6809,43 +6813,43 @@
     </x:row>
     <x:row r="122" ht="430" customHeight="1">
       <x:c r="A122" s="14" t="str">
-        <x:v>5611</x:v>
+        <x:v>5600</x:v>
       </x:c>
       <x:c r="B122" s="14" t="str">
-        <x:v>Drivmedel för personbilar</x:v>
+        <x:v>Kostnader för transportmedel</x:v>
       </x:c>
       <x:c r="C122" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för drivmedel till en personbil som hör till näringsverksamheten genom ägande eller leasing. Kontot används inte för schablonmässig milkostnad för privat bil.</x:v>
+        <x:v>Huvud- eller samlingskonto på R6 för kostnader för företagets transportmedel. Mer specifika underkonton bör användas när fordonstyp och kostnadstyp är kända.</x:v>
       </x:c>
       <x:c r="D122" s="14" t="str">
-        <x:v>Drivmedlet kan kopplas till en identifierad företagsbokförd eller leasad personbil|Kostnaden avser verksamhetsresor eller den företagsandel som systemet har fastställt|Kvitto, laddningsunderlag eller faktura finns</x:v>
+        <x:v>Kostnaden hör till ett transportmedel som används i verksamheten|Fordonstypen eller kostnadstypen är ännu inte särredovisad men systemets kontoplan tillåter 5600|Beloppet ska ingå i R6</x:v>
       </x:c>
       <x:c r="E122" s="14" t="str">
-        <x:v>Bilen är privatägd och används i verksamheten; använd normalt 5618 efter aktuell schablonregel|Beloppet avser privat körning som företagaren ska bära|Kostnaden gäller lastbil, maskin eller annat transportmedel|Underlag saknas eller fordonet kan inte identifieras|Beloppet är inköp av bil, leasingavgift, reparation, skatt eller försäkring</x:v>
+        <x:v>Kostnaden avser frakt eller transporttjänst köpt från extern transportör; använd 5700|Beloppet är anskaffning av ett fordon; använd 1240/1241|Kostnaden avser privat bil som ersätts enligt schablon; använd 5618|Ett mer specifikt underkonto som 5610–5620 ska användas enligt kontoplanen|Privat användning eller fordonstillhörighet är oklar</x:v>
       </x:c>
       <x:c r="F122" s="14" t="str">
-        <x:v>Identifiera registreringsnummer, drivmedelstyp, datum, mängd och betalningsunderlag|Koppla kostnaden till företagsbokförd eller leasad personbil|Bokför avdragsgill ingående moms separat efter kontroll av biltyp, användning och aktuell momsregel|Fördela eller återför privat del med stöd av körjournal och dokumenterad metod|Hantera privat nyttjande genom 2014 och 3200 när tillämpligt|För laddning hemma: kräv dokumenterad mätning, prisberäkning och beslut om kostnadsmodell innan bokning|Stäm av drivmedelskostnad mot körsträcka, körjournal och fordonsregister|Kräv manuell granskning vid saknade kvitton, blandad användning eller ovanlig förbrukning|Koppla drivmedel och laddning till fordon, biltyp, ägandeform, användning och momsprofil|Kräv körjournal vid privat körning|Hemmaladdning kräver separat mätunderlag|Vid granskningsflagga begär in drivmedelskvitto, registreringsnummer och vid blandad användning körjournal eller motsvarande underlag|Sätt ärendet till väntar på underlag tills fordon, verksamhetsandel och momsbehandling är verifierade|Godkänn 5611 när drivmedlet avser en företagsbokförd eller leasad personbil och verksamhetsdelen är dokumenterad|Föreslå privatbilsflödet, uppdelning eller eskalering när bilen är privatägd, användningen är blandad eller momsfrågan förblir oklar</x:v>
+        <x:v>Identifiera fordon, registreringsnummer, ägande eller leasing och användning|Klassificera kostnaden som drivmedel, försäkring och skatt, reparation, leasing eller övrigt|Använd specifikt underkonto när uppgifterna finns|Bokför endast företagets andel av kostnaden|Bedöm momsavdragsrätten separat per fordonstyp och användning|Koppla kvitto eller faktura till fordonsregister och period|Stäm av mot 1240, leasingavtal, körjournal och eget uttag|Blockera 5600 som ospecificerat restkonto vid bokslut|Använd inte som ospecificerat restkonto|Koppla varje kostnad till fordon och kostnadstyp genom fordonsreskontra|Vid granskningsflagga begär in kvitto eller faktura samt registreringsnummer, ägandeform och kostnadstyp|Sätt ärendet till väntar på underlag tills fordon, verksamhetsandel och momsbehandling är klarlagda|Godkänn 5600 när kostnaden hör till verksamhetens transportmedel men mer specifikt underkonto inte kan fastställas|Föreslå specifikt 56-konto, 5700 eller privat kostnad när underlaget visar en tydligare klassificering</x:v>
       </x:c>
       <x:c r="G122" s="14" t="str">
-        <x:v>2440|1930|2641|2014|3200</x:v>
+        <x:v>2440|1930|2641|1240|2014|3200</x:v>
       </x:c>
       <x:c r="H122" s="14" t="str">
-        <x:v>Bensin till en företagsbokförd personbil bokförs på 5611 med avdragsgill moms separat efter momsbedömning|Drivmedel till privat bil ersätts inte som faktisk kostnad på 5611 utan hanteras enligt 5618 och aktuell schablon</x:v>
+        <x:v>En ospecificerad fordonskostnad kan tillfälligt ligga på 5600 endast om den senare klassificeras till rätt fordons- och kostnadstyp</x:v>
       </x:c>
       <x:c r="I122" s="14" t="str">
-        <x:v>Körjournal behövs för att styrka företagets och privat användning|Momsavdragsrätten beror på fordon och användning|Hemmaladdning kräver särskilt underlag och får inte uppskattas utan beslutad metod|Privat drivmedel får inte belasta verksamheten|Momsavdrag och privat andel får inte bestämmas från kvittot ensamt</x:v>
+        <x:v>5600 bör inte användas när ett mer specifikt konto kan väljas|Företagsägd bil och privat bil har olika kostnadsmodeller|Momsavdrag och privat användning måste bedömas separat|Frakt- och transporttjänster från extern leverantör hör normalt till 5700|Direktbokning utan fordons- och kostnadsspecifikation ska stoppas</x:v>
       </x:c>
       <x:c r="J122" s="14" t="str">
-        <x:v>drivmedel|bensin|diesel|laddning|personbil|körjournal|R6</x:v>
+        <x:v>transportmedel|fordonskostnad|bilkostnad|lastbil|R6|samlingskonto</x:v>
       </x:c>
       <x:c r="K122" s="14" t="str">
-        <x:v>5610|5612|5613|5615|5618|5619|1240|2014|3200|2641</x:v>
+        <x:v>1240|5610|5611|5612|5613|5615|5618|5619|5620|5700</x:v>
       </x:c>
       <x:c r="L122" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5611, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.3–2.4, 3.17–3.18 och 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5600, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7</x:v>
       </x:c>
       <x:c r="M122" s="14" t="str">
-        <x:v>Bilen kan vara privatägd|Privat användning eller körjournal saknas|Momsavdragsrätten är oklar|Hemmaladdning eller delad laddare förekommer|Fordon, drivmedelstyp eller underlag saknas|Privat körning, personbilsmoms eller laddunderlag är oklart</x:v>
+        <x:v>Fordon eller kostnadstyp är inte identifierad|Privat användning förekommer|Momsavdragsrätten är oklar|Fordonet kan vara privatägt, leasat eller felklassificerat|Kontot har ospecificerat saldo vid bokslut|Fordon eller kostnadstyp saknas</x:v>
       </x:c>
       <x:c r="N122" s="14" t="str">
         <x:v>active</x:v>
@@ -6858,43 +6862,43 @@
     </x:row>
     <x:row r="123" ht="430" customHeight="1">
       <x:c r="A123" s="14" t="str">
-        <x:v>5612</x:v>
+        <x:v>5610</x:v>
       </x:c>
       <x:c r="B123" s="14" t="str">
-        <x:v>Försäkring och skatt för personbilar</x:v>
+        <x:v>Personbilskostnader</x:v>
       </x:c>
       <x:c r="C123" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för försäkringspremier, fordonsskatt och liknande obligatoriska avgifter för en personbil som hör till näringsverksamheten genom ägande eller leasing.</x:v>
+        <x:v>Huvud- eller samlingskonto på R6 för kostnader för en personbil som hör till näringsverksamheten genom ägande eller leasing. Underkonton 5611–5619 bör användas när kostnadstypen är känd.</x:v>
       </x:c>
       <x:c r="D123" s="14" t="str">
-        <x:v>Kostnaden kan kopplas till en identifierad företagsbokförd eller leasad personbil|Utgiften avser försäkring, fordonsskatt eller annan verifierad fordonsavgift|Kostnaden hör till verksamhetens innehav och användning av bilen</x:v>
+        <x:v>Kostnaden hör till en personbil som är bokförd som tillgång i verksamheten eller leasas av verksamheten|Fordonet och verksamhetsanvändningen är identifierade|Systemets momskontoplan tillåter samlingskonto 5610</x:v>
       </x:c>
       <x:c r="E123" s="14" t="str">
-        <x:v>Bilen är privatägd och endast används för resor i verksamheten; använd normalt 5618|Beloppet avser drivmedel, reparation, leasingavgift eller övrig personbilskostnad|Beloppet är en återbetalningsbar premie eller fordran|Kostnaden avser privat användning|Fordonet är lastbil eller annat transportmedel</x:v>
+        <x:v>Bilen är privatägd och endast används för resor i verksamheten; använd normalt 5618 enligt aktuell schablonregel|Beloppet är inköp av bilen; använd 1240/1241|Kostnaden avser lastbil eller annat transportmedel|Ett specifikt underkonto 5611–5619 kan användas och krävs|Privat användning eller bilens tillhörighet är inte utredd</x:v>
       </x:c>
       <x:c r="F123" s="14" t="str">
-        <x:v>Identifiera registreringsnummer, ägare eller leasingtagare, försäkringsperiod och skatteperiod|Skilj försäkring, skatt och andra avgifter|Bokför kostnaden på rätt period och hantera förutbetald del endast enligt K1:s regler|Kontrollera återbetalning eller försäkringsersättning|Bokför moms endast om sådan faktiskt debiterats och får dras av|Koppla till försäkringsbrev eller skattebeslut|Stäm av mot 1240, leasingavtal, 2440 och betalning|Kräv granskning vid privat användning eller flera fordon|Bokför försäkring och skatt enligt underlag och K1-förenklingsregler|Koppla återbetalning till ursprunglig kostnad|Koppla försäkringsersättning till skada eller tillgång|Vid granskningsflagga begär in försäkringsbrev eller skattebeslut med registreringsnummer och period|Sätt ärendet till väntar på underlag tills fordonstillhörighet, period och eventuell återbetalning är verifierade|Godkänn 5612 när försäkring eller skatt avser verksamhetens personbil och har rätt period|Föreslå privat kostnad, periodiseringsrutin eller separat hantering av ersättning när underlaget kräver det</x:v>
+        <x:v>Verifiera registreringsnummer, ägare eller leasingtagare och datum då bilen hör till verksamheten|Koppla kostnaden till bilen och kostnadstyp|Använd specifikt underkonto för drivmedel, försäkring och skatt, reparation, leasing, privat bil eller övrigt när möjligt|Bokför endast företagets kostnadsandel|Registrera privat användning och hantera eget uttag och förmånsintäkt enligt separat regel|Bedöm momsavdragsrätten per kostnad och biltyp|Stäm av mot 1240, körjournal, leasingavtal, 2014 och 3200|Kräv manuell granskning när bilen används blandat|Använd endast med sidoordnad specifikation per personbil|Skilj verksamhetsbil, leasingbil och privat bil|Vid granskningsflagga begär in kvitto eller faktura, registreringsnummer, ägar- eller leasinguppgift och uppgift om användningen|Sätt ärendet till väntar på underlag tills bilen och verksamhetsandelen är verifierade|Godkänn 5610 när kostnaden hör till en företagsbokförd eller leasad personbil men kostnadstypen inte kan specificeras ytterligare|Föreslå 5611–5619 eller privatbilsflödet när kostnadstyp eller ägandeform kan fastställas</x:v>
       </x:c>
       <x:c r="G123" s="14" t="str">
-        <x:v>2440|1930|1700|1240</x:v>
+        <x:v>2440|1930|2641|1240|2014|3200</x:v>
       </x:c>
       <x:c r="H123" s="14" t="str">
-        <x:v>Årspremie för en företagsbokförd personbil bokförs på 5612|Fordonsskatt för privatägd bil bokförs inte separat när avdraget görs med schablon på 5618</x:v>
+        <x:v>Kostnader för en företagsbokförd personbil samlas under 5610-gruppen och fördelas på rätt underkonto|Resor med en privatägd bil bokförs inte som faktiska personbilskostnader på 5610</x:v>
       </x:c>
       <x:c r="I123" s="14" t="str">
-        <x:v>Privat bil och företagsbil måste hållas isär|Försäkring och skatt har normalt ingen separat avdragsgill moms|Återbetalning måste kopplas till ursprunglig kostnad|Periodisering får inte göras slentrianmässigt|Totalförlust eller oklar ersättning kräver manuell tillgångshantering</x:v>
+        <x:v>Företagsbil och privat bil måste skiljas åt|Enskild näringsidkare kan behöva redovisa privat nyttjande som uttag och förmånsintäkt|Momsavdrag är inte automatiskt fullt|Samlingskontot bör inte dölja kostnadstyp|Privat bil ska inte behandlas som företagets tillgång eller faktiska bilkostnad</x:v>
       </x:c>
       <x:c r="J123" s="14" t="str">
-        <x:v>personbilsförsäkring|fordonsskatt|trafikförsäkring|bilskatt|R6</x:v>
+        <x:v>personbilskostnad|företagsbil|leasad bil|privat användning|R6</x:v>
       </x:c>
       <x:c r="K123" s="14" t="str">
-        <x:v>5610|5611|5613|5615|5618|5619|1240|1700</x:v>
+        <x:v>1240|5611|5612|5613|5615|5618|5619|2014|3200</x:v>
       </x:c>
       <x:c r="L123" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5612, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18, 6.59 och 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5610, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.3–2.4, 3.17–3.18 och 7.5–7.7</x:v>
       </x:c>
       <x:c r="M123" s="14" t="str">
-        <x:v>Bilens tillhörighet eller användning är oklar|Premien avser flera perioder eller fordon|Återbetalning eller ersättning förekommer|Fordonet kan vara privatägt|Moms har bokförts utan verifierad avdragsrätt|Periodisering, återbetalning eller försäkringsfall är oklart</x:v>
+        <x:v>Bilens ägande eller leasing är oklar|Privat användning förekommer|Momsavdragsrätten är begränsad|Bilen kan vara privatägd|Kostnadstypen är ospecificerad|Ägande, leasingform eller användning är oklar</x:v>
       </x:c>
       <x:c r="N123" s="14" t="str">
         <x:v>active</x:v>
@@ -6907,43 +6911,43 @@
     </x:row>
     <x:row r="124" ht="430" customHeight="1">
       <x:c r="A124" s="14" t="str">
-        <x:v>5613</x:v>
+        <x:v>5611</x:v>
       </x:c>
       <x:c r="B124" s="14" t="str">
-        <x:v>Reparation och underhåll av personbilar</x:v>
+        <x:v>Drivmedel för personbilar</x:v>
       </x:c>
       <x:c r="C124" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för service, reparation och underhåll av en personbil som hör till näringsverksamheten genom ägande eller leasing.</x:v>
+        <x:v>Kostnadskonto på R6 för drivmedel till en personbil som hör till näringsverksamheten genom ägande eller leasing. Kontot används inte för schablonmässig milkostnad för privat bil.</x:v>
       </x:c>
       <x:c r="D124" s="14" t="str">
-        <x:v>Arbetet kan kopplas till en identifierad företagsbokförd eller leasad personbil|Åtgärden återställer eller bibehåller bilens funktion|Faktura beskriver arbete, delar och fordon</x:v>
+        <x:v>Drivmedlet kan kopplas till en identifierad företagsbokförd eller leasad personbil|Kostnaden avser verksamhetsresor eller den företagsandel som systemet har fastställt|Kvitto, laddningsunderlag eller faktura finns</x:v>
       </x:c>
       <x:c r="E124" s="14" t="str">
-        <x:v>Bilen är privatägd och avdrag görs med schablon på 5618|Utgiften är inköp av bilen eller en separat större tillgång|Beloppet avser drivmedel, försäkring, skatt eller leasing|Åtgärden avser privat skada|Fordonet är lastbil</x:v>
+        <x:v>Bilen är privatägd och används i verksamheten; använd normalt 5618 efter aktuell schablonregel|Beloppet avser privat körning som företagaren ska bära|Kostnaden gäller lastbil, maskin eller annat transportmedel|Underlag saknas eller fordonet kan inte identifieras|Beloppet är inköp av bil, leasingavgift, reparation, skatt eller försäkring</x:v>
       </x:c>
       <x:c r="F124" s="14" t="str">
-        <x:v>Identifiera registreringsnummer, mätarställning, serviceorder och fakturarader|Skilj normal service från ny utrustning eller större förbättring|Dela fakturan när den innehåller både reparation, tillbehör och privat kostnad|Bokför ingående moms efter kontroll av biltyp, ägande och användning|Hantera garanti, självrisk och försäkringsersättning spårbart|Koppla till fordonsregister och körjournal|Kräv granskning vid motorbyte, större komponent eller ombyggnad|Kostnadsför service och reparation som återställer funktion|Pröva aktivering vid större komponent, ombyggnad eller väsentligt höjd standard eller livslängd|Vid granskningsflagga begär in fakturaspecifikation, serviceorder och registreringsnummer|Sätt ärendet till väntar på underlag tills reparation, privat del, försäkringsfall och eventuell förbättring kan bedömas|Godkänn 5613 när åtgärden återställer eller underhåller verksamhetens personbil|Föreslå uppdelning eller aktivering när fakturan innehåller privat kostnad, ny utrustning eller en väsentlig förbättring</x:v>
+        <x:v>Identifiera registreringsnummer, drivmedelstyp, datum, mängd och betalningsunderlag|Koppla kostnaden till företagsbokförd eller leasad personbil|Bokför avdragsgill ingående moms separat efter kontroll av biltyp, användning och aktuell momsregel|Fördela eller återför privat del med stöd av körjournal och dokumenterad metod|Hantera privat nyttjande genom 2014 och 3200 när tillämpligt|För laddning hemma: kräv dokumenterad mätning, prisberäkning och beslut om kostnadsmodell innan bokning|Stäm av drivmedelskostnad mot körsträcka, körjournal och fordonsregister|Kräv manuell granskning vid saknade kvitton, blandad användning eller ovanlig förbrukning|Koppla drivmedel och laddning till fordon, biltyp, ägandeform, användning och momsprofil|Kräv körjournal vid privat körning|Hemmaladdning kräver separat mätunderlag|Vid granskningsflagga begär in drivmedelskvitto, registreringsnummer och vid blandad användning körjournal eller motsvarande underlag|Sätt ärendet till väntar på underlag tills fordon, verksamhetsandel och momsbehandling är verifierade|Godkänn 5611 när drivmedlet avser en företagsbokförd eller leasad personbil och verksamhetsdelen är dokumenterad|Föreslå privatbilsflödet, uppdelning eller eskalering när bilen är privatägd, användningen är blandad eller momsfrågan förblir oklar</x:v>
       </x:c>
       <x:c r="G124" s="14" t="str">
-        <x:v>2440|1930|2641|1240|3900</x:v>
+        <x:v>2440|1930|2641|2014|3200</x:v>
       </x:c>
       <x:c r="H124" s="14" t="str">
-        <x:v>Normal service på en företagsbokförd personbil bokförs på 5613|En större ombyggnad prövas som tillgång</x:v>
+        <x:v>Bensin till en företagsbokförd personbil bokförs på 5611 med avdragsgill moms separat efter momsbedömning|Drivmedel till privat bil ersätts inte som faktisk kostnad på 5611 utan hanteras enligt 5618 och aktuell schablon</x:v>
       </x:c>
       <x:c r="I124" s="14" t="str">
-        <x:v>Fakturans rubrik avgör inte om utgiften är reparation eller investering|Momsavdraget måste bedömas separat|Försäkringsersättning och självrisk får inte dubbelräknas|Privata skador hör inte automatiskt till företaget|Moms på personbilsreparation får inte dras av automatiskt</x:v>
+        <x:v>Körjournal behövs för att styrka företagets och privat användning|Momsavdragsrätten beror på fordon och användning|Hemmaladdning kräver särskilt underlag och får inte uppskattas utan beslutad metod|Privat drivmedel får inte belasta verksamheten|Momsavdrag och privat andel får inte bestämmas från kvittot ensamt</x:v>
       </x:c>
       <x:c r="J124" s="14" t="str">
-        <x:v>bilreparation|bilservice|underhåll personbil|reservdel|självrisk|R6</x:v>
+        <x:v>drivmedel|bensin|diesel|laddning|personbil|körjournal|R6</x:v>
       </x:c>
       <x:c r="K124" s="14" t="str">
-        <x:v>5500|5610|5611|5612|5615|5618|5619|1240|2641</x:v>
+        <x:v>5610|5612|5613|5615|5618|5619|1240|2014|3200|2641</x:v>
       </x:c>
       <x:c r="L124" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5613, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5611, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.3–2.4, 3.17–3.18 och 7.5–7.7</x:v>
       </x:c>
       <x:c r="M124" s="14" t="str">
-        <x:v>Åtgärden kan vara investering|Privat skada eller blandad användning förekommer|Försäkringsersättning eller garanti förekommer|Momsavdragsrätten är oklar|Fordon eller arbetsbeskrivning saknas|Större motor-, batteri- eller ombyggnadsarbete förekommer</x:v>
+        <x:v>Bilen kan vara privatägd|Privat användning eller körjournal saknas|Momsavdragsrätten är oklar|Hemmaladdning eller delad laddare förekommer|Fordon, drivmedelstyp eller underlag saknas|Privat körning, personbilsmoms eller laddunderlag är oklart</x:v>
       </x:c>
       <x:c r="N124" s="14" t="str">
         <x:v>active</x:v>
@@ -6956,43 +6960,43 @@
     </x:row>
     <x:row r="125" ht="430" customHeight="1">
       <x:c r="A125" s="14" t="str">
-        <x:v>5615</x:v>
+        <x:v>5612</x:v>
       </x:c>
       <x:c r="B125" s="14" t="str">
-        <x:v>Leasing av personbilar</x:v>
+        <x:v>Försäkring och skatt för personbilar</x:v>
       </x:c>
       <x:c r="C125" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för leasing- och hyresavgifter för en personbil som verksamheten leasar. Första förhöjd avgift och moms hanteras enligt separata regler.</x:v>
+        <x:v>Kostnadskonto på R6 för försäkringspremier, fordonsskatt och liknande obligatoriska avgifter för en personbil som hör till näringsverksamheten genom ägande eller leasing.</x:v>
       </x:c>
       <x:c r="D125" s="14" t="str">
-        <x:v>Verksamheten är leasing- eller hyrestagare för en identifierad personbil|Avgiften avser nyttjandet under en verifierad period|Avtalet är bedömt som leasing eller hyra och inte köp</x:v>
+        <x:v>Kostnaden kan kopplas till en identifierad företagsbokförd eller leasad personbil|Utgiften avser försäkring, fordonsskatt eller annan verifierad fordonsavgift|Kostnaden hör till verksamhetens innehav och användning av bilen</x:v>
       </x:c>
       <x:c r="E125" s="14" t="str">
-        <x:v>Bilen leasas privat av företagaren; använd normalt 5618|Transaktionen är köp, avbetalningsköp eller lösen|Beloppet är drivmedel, service, försäkring, skatt eller deposition|Första förhöjda avgiften ska ligga som förskott|Avtalet avser lastbil</x:v>
+        <x:v>Bilen är privatägd och endast används för resor i verksamheten; använd normalt 5618|Beloppet avser drivmedel, reparation, leasingavgift eller övrig personbilskostnad|Beloppet är en återbetalningsbar premie eller fordran|Kostnaden avser privat användning|Fordonet är lastbil eller annat transportmedel</x:v>
       </x:c>
       <x:c r="F125" s="14" t="str">
-        <x:v>Verifiera leasinggivare, registreringsnummer, avtalsperiod, månadskostnad, första förhöjd avgift, restvärde och köpoption|Skilj leasingavgift från service, försäkring, skatt, deposition och lösenbelopp|Bokför löpande avgift på 5615|Ta upp första förhöjd leasinghyra som förskott på B8 när den överstiger 5 000 kronor exklusive avdragsgill moms|Bedöm om avtalet är hyra eller anskaffning|Vid momspliktig verksamhet får 50 procent av momsen på hyran normalt dras av när bilen används mer än ringa omfattning; villkoren ska verifieras|Bokför ej avdragsgill moms som leasingkostnad|Stäm av mot avtal, 1700, 2440 och 2641|Bedöm avtalet efter ekonomiskt innehåll|Vanlig leasing bokförs som kostnad|Avbetalningsköp eller faktisk ägarövergång redovisas som tillgång och skuld|Verifiera villkor före momsavdrag|Vid granskningsflagga begär in leasingavtal, registreringsnummer, faktura och uppgift om verksamhetsanvändning|Sätt ärendet till väntar på underlag tills leasingform, första avgift, privat användning och momsprofil är verifierade|Godkänn 5615 för vanlig leasing- eller hyresavgift för verksamhetens personbil|Föreslå 1700, tillgång och skuld, privat kostnad eller eskalering när avtalet innehåller förhöjd avgift, faktisk ägarövergång eller oklar användning</x:v>
+        <x:v>Identifiera registreringsnummer, ägare eller leasingtagare, försäkringsperiod och skatteperiod|Skilj försäkring, skatt och andra avgifter|Bokför kostnaden på rätt period och hantera förutbetald del endast enligt K1:s regler|Kontrollera återbetalning eller försäkringsersättning|Bokför moms endast om sådan faktiskt debiterats och får dras av|Koppla till försäkringsbrev eller skattebeslut|Stäm av mot 1240, leasingavtal, 2440 och betalning|Kräv granskning vid privat användning eller flera fordon|Bokför försäkring och skatt enligt underlag och K1-förenklingsregler|Koppla återbetalning till ursprunglig kostnad|Koppla försäkringsersättning till skada eller tillgång|Vid granskningsflagga begär in försäkringsbrev eller skattebeslut med registreringsnummer och period|Sätt ärendet till väntar på underlag tills fordonstillhörighet, period och eventuell återbetalning är verifierade|Godkänn 5612 när försäkring eller skatt avser verksamhetens personbil och har rätt period|Föreslå privat kostnad, periodiseringsrutin eller separat hantering av ersättning när underlaget kräver det</x:v>
       </x:c>
       <x:c r="G125" s="14" t="str">
-        <x:v>2440|1930|2641|1700|1240</x:v>
+        <x:v>2440|1930|1700|1240</x:v>
       </x:c>
       <x:c r="H125" s="14" t="str">
-        <x:v>Månadsleasing bokförs på 5615 med verifierad avdragsgill moms separat|Första förhöjd avgift över K1-gränsen tas upp som förskott</x:v>
+        <x:v>Årspremie för en företagsbokförd personbil bokförs på 5612|Fordonsskatt för privatägd bil bokförs inte separat när avdraget görs med schablon på 5618</x:v>
       </x:c>
       <x:c r="I125" s="14" t="str">
-        <x:v>Avtalets rubrik avgör inte ensam om bilen är hyrd eller köpt|Momsavdraget är begränsat och villkorat|Privatleasing ger inte rätt att bokföra faktiska leasingavgifter|Första förhöjd avgift är inte automatiskt engångskostnad|Stor slutbetalning eller köpoption kräver manuell granskning</x:v>
+        <x:v>Privat bil och företagsbil måste hållas isär|Försäkring och skatt har normalt ingen separat avdragsgill moms|Återbetalning måste kopplas till ursprunglig kostnad|Periodisering får inte göras slentrianmässigt|Totalförlust eller oklar ersättning kräver manuell tillgångshantering</x:v>
       </x:c>
       <x:c r="J125" s="14" t="str">
-        <x:v>leasing personbil|bilhyra|leasingavgift|första förhöjd avgift|leasingmoms|R6</x:v>
+        <x:v>personbilsförsäkring|fordonsskatt|trafikförsäkring|bilskatt|R6</x:v>
       </x:c>
       <x:c r="K125" s="14" t="str">
-        <x:v>5200|5610|5611|5612|5613|5618|5619|1240|1700|2641</x:v>
+        <x:v>5610|5611|5613|5615|5618|5619|1240|1700</x:v>
       </x:c>
       <x:c r="L125" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5615, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 6.59 och punkterna 7.5–7.7|Skatteverket – Bilar och moms, kontrollerad 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5612, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18, 6.59 och 7.5–7.7</x:v>
       </x:c>
       <x:c r="M125" s="14" t="str">
-        <x:v>Avtalet kan vara köp eller avbetalning|Första förhöjd avgift, deposition, restvärde eller köpoption förekommer|Momspliktig användning över 100 mil per år är inte styrkt|Blandad eller momsfri verksamhet förekommer|Bilen kan vara privatleasad|Leasingform, användning eller momsprofil är oklar</x:v>
+        <x:v>Bilens tillhörighet eller användning är oklar|Premien avser flera perioder eller fordon|Återbetalning eller ersättning förekommer|Fordonet kan vara privatägt|Moms har bokförts utan verifierad avdragsrätt|Periodisering, återbetalning eller försäkringsfall är oklart</x:v>
       </x:c>
       <x:c r="N125" s="14" t="str">
         <x:v>active</x:v>
@@ -7000,50 +7004,48 @@
       <x:c r="O125" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P125" s="14" t="str">
-        <x:v>first_increased_lease_fee_over_5000|passenger_car_lease_vat_deduction_50</x:v>
-      </x:c>
+      <x:c r="P125" s="14"/>
       <x:c r="Q125" s="12" t="str"/>
     </x:row>
     <x:row r="126" ht="430" customHeight="1">
       <x:c r="A126" s="14" t="str">
-        <x:v>5618</x:v>
+        <x:v>5613</x:v>
       </x:c>
       <x:c r="B126" s="14" t="str">
-        <x:v>Schablonmässig milkostnad privat personbil</x:v>
+        <x:v>Reparation och underhåll av personbilar</x:v>
       </x:c>
       <x:c r="C126" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för schablonavdrag när företagaren använder sin privatägda eller privatleasade bil för resor i näringsverksamheten. För 2026 är schablonen 25 kronor per mil.</x:v>
+        <x:v>Kostnadskonto på R6 för service, reparation och underhåll av en personbil som hör till näringsverksamheten genom ägande eller leasing.</x:v>
       </x:c>
       <x:c r="D126" s="14" t="str">
-        <x:v>Bilen är privatägd eller privatleasad och inte bokförd i verksamheten|Resan har direkt samband med näringsverksamheten|Körsträcka, datum, resmål och ändamål kan styrkas</x:v>
+        <x:v>Arbetet kan kopplas till en identifierad företagsbokförd eller leasad personbil|Åtgärden återställer eller bibehåller bilens funktion|Faktura beskriver arbete, delar och fordon</x:v>
       </x:c>
       <x:c r="E126" s="14" t="str">
-        <x:v>Bilen är bokförd som tillgång eller leasas av verksamheten|Resan är privat eller inte kvalificerad näringsresa|Faktiska drivmedels-, försäkrings-, reparations- eller leasingkostnader bokförs utöver schablonen|Körjournal saknas|Fel års schablon används</x:v>
+        <x:v>Bilen är privatägd och avdrag görs med schablon på 5618|Utgiften är inköp av bilen eller en separat större tillgång|Beloppet avser drivmedel, försäkring, skatt eller leasing|Åtgärden avser privat skada|Fordonet är lastbil</x:v>
       </x:c>
       <x:c r="F126" s="14" t="str">
-        <x:v>Verifiera att bilen är privat och inte ingår i företagets tillgångar eller leasingavtal|Kräv körjournal med datum, start, mål, ärende och kilometer|Beräkna antal mil gånger versionsstyrd schablon|För 2026 används 25 kronor per mil oavsett drivmedel|Bokför kostnaden på 5618 mot 2018 eller annat beslutat ägarkonto|Bokför ingen ingående moms på schablonen|Bokför styrkta trängsel-, väg-, bro- och färjeavgifter separat|Stäm av mil mot uppdrag och kalender|Använd endast för dokumenterade näringsresor med privat bil|Spara datum, sträcka, syfte, kilometer och fordonsuppgift|Kräv körjournal med datum, resmål, affärsändamål, kilometer och uppgift om att bilen är privatägd eller privatleasad|Beräkna avdraget med den versionsstyrda schablonen; för 2026 används 25 kronor per mil|Bokför kostnaden i debet på 5618 och kredit på 2018 utan ingående moms|Sätt ärendet till väntar på underlag vid saknad körjournal, privat resa, fel årsschablon eller om bilen kan vara bokförd eller leasad i verksamheten</x:v>
+        <x:v>Identifiera registreringsnummer, mätarställning, serviceorder och fakturarader|Skilj normal service från ny utrustning eller större förbättring|Dela fakturan när den innehåller både reparation, tillbehör och privat kostnad|Bokför ingående moms efter kontroll av biltyp, ägande och användning|Hantera garanti, självrisk och försäkringsersättning spårbart|Koppla till fordonsregister och körjournal|Kräv granskning vid motorbyte, större komponent eller ombyggnad|Kostnadsför service och reparation som återställer funktion|Pröva aktivering vid större komponent, ombyggnad eller väsentligt höjd standard eller livslängd|Vid granskningsflagga begär in fakturaspecifikation, serviceorder och registreringsnummer|Sätt ärendet till väntar på underlag tills reparation, privat del, försäkringsfall och eventuell förbättring kan bedömas|Godkänn 5613 när åtgärden återställer eller underhåller verksamhetens personbil|Föreslå uppdelning eller aktivering när fakturan innehåller privat kostnad, ny utrustning eller en väsentlig förbättring</x:v>
       </x:c>
       <x:c r="G126" s="14" t="str">
-        <x:v>2018|2017</x:v>
+        <x:v>2440|1930|2641|1240|3900</x:v>
       </x:c>
       <x:c r="H126" s="14" t="str">
-        <x:v>40 mil med privat bil under 2026 ger 40 × 25 kronor på 5618 mot ägarkonto|Bensin och försäkring bokförs inte dessutom som faktiska kostnader</x:v>
+        <x:v>Normal service på en företagsbokförd personbil bokförs på 5613|En större ombyggnad prövas som tillgång</x:v>
       </x:c>
       <x:c r="I126" s="14" t="str">
-        <x:v>Schablonen ersätter bilens normala faktiska kostnader|Ingen ingående moms bokförs|Körjournal krävs|Beloppet måste versionsstyras|Privat bil och företagsbil får inte blandas|Resa till stadigvarande verksamhetsplats är inte automatiskt näringsresa|Exakt ägarkonto är ännu inte verifierat</x:v>
+        <x:v>Fakturans rubrik avgör inte om utgiften är reparation eller investering|Momsavdraget måste bedömas separat|Försäkringsersättning och självrisk får inte dubbelräknas|Privata skador hör inte automatiskt till företaget|Moms på personbilsreparation får inte dras av automatiskt</x:v>
       </x:c>
       <x:c r="J126" s="14" t="str">
-        <x:v>privat bil|milersättning|schablonmässig milkostnad|25 kronor per mil|körjournal|R6</x:v>
+        <x:v>bilreparation|bilservice|underhåll personbil|reservdel|självrisk|R6</x:v>
       </x:c>
       <x:c r="K126" s="14" t="str">
-        <x:v>5610|5611|5612|5613|5615|5619|2018|1240</x:v>
+        <x:v>5500|5610|5611|5612|5615|5618|5619|1240|2641</x:v>
       </x:c>
       <x:c r="L126" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5618, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 4, kommentaren om privat tillgång och milersättning|Skatteverket – Resor i näringsverksamheten, kontrollerad 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5613, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7</x:v>
       </x:c>
       <x:c r="M126" s="14" t="str">
-        <x:v>Bilens ägande eller leasingform är oklar|Körjournal eller affärsändamål saknas|Bilen kan vara bokförd i verksamheten|Schablonens år eller belopp är fel|Resan kan vara privat eller arbetsresa|Reseklassificering eller motkonto är oklart</x:v>
+        <x:v>Åtgärden kan vara investering|Privat skada eller blandad användning förekommer|Försäkringsersättning eller garanti förekommer|Momsavdragsrätten är oklar|Fordon eller arbetsbeskrivning saknas|Större motor-, batteri- eller ombyggnadsarbete förekommer</x:v>
       </x:c>
       <x:c r="N126" s="14" t="str">
         <x:v>active</x:v>
@@ -7051,50 +7053,48 @@
       <x:c r="O126" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P126" s="14" t="str">
-        <x:v>private_car_mileage_rate_2026</x:v>
-      </x:c>
+      <x:c r="P126" s="14"/>
       <x:c r="Q126" s="12" t="str"/>
     </x:row>
     <x:row r="127" ht="430" customHeight="1">
       <x:c r="A127" s="14" t="str">
-        <x:v>5619</x:v>
+        <x:v>5615</x:v>
       </x:c>
       <x:c r="B127" s="14" t="str">
-        <x:v>Övriga personbilskostnader</x:v>
+        <x:v>Leasing av personbilar</x:v>
       </x:c>
       <x:c r="C127" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för andra verifierade kostnader för en företagsbokförd eller verksamhetsleasad personbil som inte hör till 5611, 5612, 5613 eller 5615.</x:v>
+        <x:v>Kostnadskonto på R6 för leasing- och hyresavgifter för en personbil som verksamheten leasar. Första förhöjd avgift och moms hanteras enligt separata regler.</x:v>
       </x:c>
       <x:c r="D127" s="14" t="str">
-        <x:v>Kostnaden kan kopplas till en identifierad företagsbokförd eller leasad personbil|Utgiften saknar mer specifikt konto|Kostnaden hör till verksamhetsanvändningen</x:v>
+        <x:v>Verksamheten är leasing- eller hyrestagare för en identifierad personbil|Avgiften avser nyttjandet under en verifierad period|Avtalet är bedömt som leasing eller hyra och inte köp</x:v>
       </x:c>
       <x:c r="E127" s="14" t="str">
-        <x:v>Bilen är privatägd och kostnaden täcks av schablon på 5618|Beloppet hör till drivmedel, försäkring, skatt, reparation eller leasing|Beloppet är parkeringsbot eller annan sanktionsavgift|Kostnaden är privat|Fordonet är inte identifierat</x:v>
+        <x:v>Bilen leasas privat av företagaren; använd normalt 5618|Transaktionen är köp, avbetalningsköp eller lösen|Beloppet är drivmedel, service, försäkring, skatt eller deposition|Första förhöjda avgiften ska ligga som förskott|Avtalet avser lastbil</x:v>
       </x:c>
       <x:c r="F127" s="14" t="str">
-        <x:v>Identifiera kostnadstyp, registreringsnummer, datum och affärsändamål|Pröva alltid mer specifikt konto först|Bokför endast verksamhetsandel|Bedöm ingående moms separat|Separera avdragsgilla avgifter från böter och privata utgifter|Koppla till körjournal eller fordonsregister|Använd obligatorisk underkategori|Kräv granskning för parkering, trängselskatt, självrisk, tillbehör och privat användning|Specificera parkering, trängselskatt, vägavgift, självrisk, tvätt, besiktning eller övrigt per fordon|Vid granskningsflagga begär in kvitto eller faktura, registreringsnummer och tydlig uppgift om kostnadstyp och affärsändamål|Sätt ärendet till väntar på underlag tills kostnaden och verksamhetsandelen är verifierade|Godkänn 5619 endast för en verklig personbilskostnad som inte passar på ett mer specifikt 561-konto|Föreslå specifikt bilkonto eller privat kostnad och avvisa böter och andra ej avdragsgilla sanktioner från automatflödet</x:v>
+        <x:v>Verifiera leasinggivare, registreringsnummer, avtalsperiod, månadskostnad, första förhöjd avgift, restvärde och köpoption|Skilj leasingavgift från service, försäkring, skatt, deposition och lösenbelopp|Bokför löpande avgift på 5615|Ta upp första förhöjd leasinghyra som förskott på B8 när den överstiger 5 000 kronor exklusive avdragsgill moms|Bedöm om avtalet är hyra eller anskaffning|Vid momspliktig verksamhet får 50 procent av momsen på hyran normalt dras av när bilen används mer än ringa omfattning; villkoren ska verifieras|Bokför ej avdragsgill moms som leasingkostnad|Stäm av mot avtal, 1700, 2440 och 2641|Bedöm avtalet efter ekonomiskt innehåll|Vanlig leasing bokförs som kostnad|Avbetalningsköp eller faktisk ägarövergång redovisas som tillgång och skuld|Verifiera villkor före momsavdrag|Vid granskningsflagga begär in leasingavtal, registreringsnummer, faktura och uppgift om verksamhetsanvändning|Sätt ärendet till väntar på underlag tills leasingform, första avgift, privat användning och momsprofil är verifierade|Godkänn 5615 för vanlig leasing- eller hyresavgift för verksamhetens personbil|Föreslå 1700, tillgång och skuld, privat kostnad eller eskalering när avtalet innehåller förhöjd avgift, faktisk ägarövergång eller oklar användning</x:v>
       </x:c>
       <x:c r="G127" s="14" t="str">
-        <x:v>2440|1930|2641|2014|3200</x:v>
+        <x:v>2440|1930|2641|1700|1240</x:v>
       </x:c>
       <x:c r="H127" s="14" t="str">
-        <x:v>En mindre verifierad fordonsavgift kan bokföras på 5619 när inget mer specifikt konto passar|En parkeringsbot bokförs inte automatiskt som avdragsgill kostnad</x:v>
+        <x:v>Månadsleasing bokförs på 5615 med verifierad avdragsgill moms separat|Första förhöjd avgift över K1-gränsen tas upp som förskott</x:v>
       </x:c>
       <x:c r="I127" s="14" t="str">
-        <x:v>5619 får inte bli restkonto|Böter och sanktionsavgifter kan vara ej avdragsgilla|Privatbilsschablonen täcker normala bilkostnader|Moms och privat användning bedöms per kostnad|Böter och sanktionsavgifter är normalt ej avdragsgilla och får inte blandas med parkering</x:v>
+        <x:v>Avtalets rubrik avgör inte ensam om bilen är hyrd eller köpt|Momsavdraget är begränsat och villkorat|Privatleasing ger inte rätt att bokföra faktiska leasingavgifter|Första förhöjd avgift är inte automatiskt engångskostnad|Stor slutbetalning eller köpoption kräver manuell granskning</x:v>
       </x:c>
       <x:c r="J127" s="14" t="str">
-        <x:v>övrig personbilskostnad|parkering|trängselskatt|självrisk|biltillbehör|R6</x:v>
+        <x:v>leasing personbil|bilhyra|leasingavgift|första förhöjd avgift|leasingmoms|R6</x:v>
       </x:c>
       <x:c r="K127" s="14" t="str">
-        <x:v>5610|5611|5612|5613|5615|5618|1240|2014|3200</x:v>
+        <x:v>5200|5610|5611|5612|5613|5618|5619|1240|1700|2641</x:v>
       </x:c>
       <x:c r="L127" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5619, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5615, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 6.59 och punkterna 7.5–7.7|Skatteverket – Bilar och moms, kontrollerad 2026-07-30</x:v>
       </x:c>
       <x:c r="M127" s="14" t="str">
-        <x:v>Kostnadstypen är oklar|Böter, sanktionsavgift eller privat kostnad kan ingå|Fordon eller verksamhetsandel saknas|Momsavdragsrätten är oklar|Mer specifikt konto kan vara rätt|Kostnadstyp eller avdragsrätt är oklar</x:v>
+        <x:v>Avtalet kan vara köp eller avbetalning|Första förhöjd avgift, deposition, restvärde eller köpoption förekommer|Momspliktig användning över 100 mil per år är inte styrkt|Blandad eller momsfri verksamhet förekommer|Bilen kan vara privatleasad|Leasingform, användning eller momsprofil är oklar</x:v>
       </x:c>
       <x:c r="N127" s="14" t="str">
         <x:v>active</x:v>
@@ -7102,48 +7102,50 @@
       <x:c r="O127" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P127" s="14"/>
+      <x:c r="P127" s="14" t="str">
+        <x:v>first_increased_lease_fee_over_5000|passenger_car_lease_vat_deduction_50</x:v>
+      </x:c>
       <x:c r="Q127" s="12" t="str"/>
     </x:row>
     <x:row r="128" ht="430" customHeight="1">
       <x:c r="A128" s="14" t="str">
-        <x:v>5620</x:v>
+        <x:v>5618</x:v>
       </x:c>
       <x:c r="B128" s="14" t="str">
-        <x:v>Lastbilskostnader</x:v>
+        <x:v>Schablonmässig milkostnad privat personbil</x:v>
       </x:c>
       <x:c r="C128" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för drivmedel, försäkring, skatt, reparation, leasing och andra kostnader för lastbil eller annat fordon som redovisas i lastbilsgruppen.</x:v>
+        <x:v>Kostnadskonto på R6 för schablonavdrag när företagaren använder sin privatägda eller privatleasade bil för resor i näringsverksamheten. För 2026 är schablonen 25 kronor per mil.</x:v>
       </x:c>
       <x:c r="D128" s="14" t="str">
-        <x:v>Kostnaden hör till en identifierad lastbil i verksamheten|Fordonets registrering, ägande eller leasing och verksamhetsanvändning är verifierade|Utgiften är löpande fordonskostnad</x:v>
+        <x:v>Bilen är privatägd eller privatleasad och inte bokförd i verksamheten|Resan har direkt samband med näringsverksamheten|Körsträcka, datum, resmål och ändamål kan styrkas</x:v>
       </x:c>
       <x:c r="E128" s="14" t="str">
-        <x:v>Fordonet är personbil; använd 5610-gruppen|Beloppet är inköp eller aktiverbar förbättring|Kostnaden är extern frakt- eller transporttjänst; använd 5700|Fordonet är privatägt och annan regel gäller|Fordonstyp eller verksamhetsandel är oklar</x:v>
+        <x:v>Bilen är bokförd som tillgång eller leasas av verksamheten|Resan är privat eller inte kvalificerad näringsresa|Faktiska drivmedels-, försäkrings-, reparations- eller leasingkostnader bokförs utöver schablonen|Körjournal saknas|Fel års schablon används</x:v>
       </x:c>
       <x:c r="F128" s="14" t="str">
-        <x:v>Verifiera registreringsuppgifter, fordonsklass, ägare eller leasingtagare|Koppla kostnaden till registreringsnummer och underkategori|Bokför endast verksamhetsandel|Bedöm moms utifrån fordonets momsrättsliga klassificering|Skilj löpande kostnad från anskaffning eller förbättring|Stäm av mot 1240, körjournal, fordonsregister och leasingavtal|Kräv granskning vid privat användning eller oklar fordonsklass|Klassificera fordon från registrerings- och konstruktionsuppgifter|Specificera kostnader per lastbil och kostnadstyp|Vid granskningsflagga begär in registreringsuppgifter, faktura och uppgift om ägande eller leasing samt användning|Sätt ärendet till väntar på underlag tills fordonsklass, verksamhetsandel och momsbehandling är verifierade|Godkänn 5620 när kostnaden avser verksamhetens lastbil eller motsvarande nyttofordon|Föreslå annat fordonskonto, 5700 eller tillgångskonto när posten avser personbil, köpt transporttjänst eller anskaffning</x:v>
+        <x:v>Verifiera att bilen är privat och inte ingår i företagets tillgångar eller leasingavtal|Kräv körjournal med datum, start, mål, ärende och kilometer|Beräkna antal mil gånger versionsstyrd schablon|För 2026 används 25 kronor per mil oavsett drivmedel|Bokför kostnaden på 5618 mot 2018 eller annat beslutat ägarkonto|Bokför ingen ingående moms på schablonen|Bokför styrkta trängsel-, väg-, bro- och färjeavgifter separat|Stäm av mil mot uppdrag och kalender|Använd endast för dokumenterade näringsresor med privat bil|Spara datum, sträcka, syfte, kilometer och fordonsuppgift|Kräv körjournal med datum, resmål, affärsändamål, kilometer och uppgift om att bilen är privatägd eller privatleasad|Beräkna avdraget med den versionsstyrda schablonen; för 2026 används 25 kronor per mil|Bokför kostnaden i debet på 5618 och kredit på 2018 utan ingående moms|Sätt ärendet till väntar på underlag vid saknad körjournal, privat resa, fel årsschablon eller om bilen kan vara bokförd eller leasad i verksamheten</x:v>
       </x:c>
       <x:c r="G128" s="14" t="str">
-        <x:v>2440|1930|2641|1240|2014|3200</x:v>
+        <x:v>2018|2017</x:v>
       </x:c>
       <x:c r="H128" s="14" t="str">
-        <x:v>Diesel och service för en verksamhetslastbil bokförs på 5620|En extern åkerifaktura bokförs på 5700</x:v>
+        <x:v>40 mil med privat bil under 2026 ger 40 × 25 kronor på 5618 mot ägarkonto|Bensin och försäkring bokförs inte dessutom som faktiska kostnader</x:v>
       </x:c>
       <x:c r="I128" s="14" t="str">
-        <x:v>Momsreglerna kan skilja sig från personbil men fordonsklass måste verifieras|5620 behöver underkategorier|Privat användning hanteras separat|Anskaffning är inte löpande kostnad|Vardaglig benämning avgör inte fordons- eller momsklass</x:v>
+        <x:v>Schablonen ersätter bilens normala faktiska kostnader|Ingen ingående moms bokförs|Körjournal krävs|Beloppet måste versionsstyras|Privat bil och företagsbil får inte blandas|Resa till stadigvarande verksamhetsplats är inte automatiskt näringsresa|Exakt ägarkonto är ännu inte verifierat</x:v>
       </x:c>
       <x:c r="J128" s="14" t="str">
-        <x:v>lastbilskostnad|drivmedel lastbil|lastbilsförsäkring|lastbilsreparation|R6</x:v>
+        <x:v>privat bil|milersättning|schablonmässig milkostnad|25 kronor per mil|körjournal|R6</x:v>
       </x:c>
       <x:c r="K128" s="14" t="str">
-        <x:v>5600|5610|5700|1240|2641|2014|3200</x:v>
+        <x:v>5610|5611|5612|5613|5615|5619|2018|1240</x:v>
       </x:c>
       <x:c r="L128" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5620, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5618, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 4, kommentaren om privat tillgång och milersättning|Skatteverket – Resor i näringsverksamheten, kontrollerad 2026-07-30</x:v>
       </x:c>
       <x:c r="M128" s="14" t="str">
-        <x:v>Fordonsklass eller registrering är oklar|Privat användning förekommer|Momsavdragsrätten är oklar|Kostnaden kan vara anskaffning eller förbättring|Extern transporttjänst kan vara rätt klassificering|Lätt lastbil, specialfordon eller momsprofil är oklar</x:v>
+        <x:v>Bilens ägande eller leasingform är oklar|Körjournal eller affärsändamål saknas|Bilen kan vara bokförd i verksamheten|Schablonens år eller belopp är fel|Resan kan vara privat eller arbetsresa|Reseklassificering eller motkonto är oklart</x:v>
       </x:c>
       <x:c r="N128" s="14" t="str">
         <x:v>active</x:v>
@@ -7151,48 +7153,50 @@
       <x:c r="O128" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P128" s="14"/>
+      <x:c r="P128" s="14" t="str">
+        <x:v>private_car_mileage_rate_2026</x:v>
+      </x:c>
       <x:c r="Q128" s="12" t="str"/>
     </x:row>
     <x:row r="129" ht="430" customHeight="1">
       <x:c r="A129" s="14" t="str">
-        <x:v>5700</x:v>
+        <x:v>5619</x:v>
       </x:c>
       <x:c r="B129" s="14" t="str">
-        <x:v>Frakter och transporter</x:v>
+        <x:v>Övriga personbilskostnader</x:v>
       </x:c>
       <x:c r="C129" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för köpta frakt-, distributions- och transporttjänster för företagets varor, material eller leveranser och inte för egna fordon eller personalresor.</x:v>
+        <x:v>Kostnadskonto på R6 för andra verifierade kostnader för en företagsbokförd eller verksamhetsleasad personbil som inte hör till 5611, 5612, 5613 eller 5615.</x:v>
       </x:c>
       <x:c r="D129" s="14" t="str">
-        <x:v>Företaget köper frakt eller transport från extern transportör|Kostnaden avser transport av varor eller material|Frakten ska kostnadsföras och inte ingå i en tillgångs anskaffningsvärde</x:v>
+        <x:v>Kostnaden kan kopplas till en identifierad företagsbokförd eller leasad personbil|Utgiften saknar mer specifikt konto|Kostnaden hör till verksamhetsanvändningen</x:v>
       </x:c>
       <x:c r="E129" s="14" t="str">
-        <x:v>Kostnaden avser eget fordon; använd 5600-serien|Kostnaden avser företagaren eller personals resa; använd 5800|Frakten är direkt hänförlig till lager eller anläggningstillgång och ska ingå i anskaffningsvärdet|Händelsen är äkta utlägg|Transporten är privat</x:v>
+        <x:v>Bilen är privatägd och kostnaden täcks av schablon på 5618|Beloppet hör till drivmedel, försäkring, skatt, reparation eller leasing|Beloppet är parkeringsbot eller annan sanktionsavgift|Kostnaden är privat|Fordonet är inte identifierat</x:v>
       </x:c>
       <x:c r="F129" s="14" t="str">
-        <x:v>Identifiera transportör, gods, avsändare, mottagare och affärshändelse|Avgör om frakten är löpande kostnad eller direkt förvärvsutgift|Bokför kostnaden exklusive avdragsgill moms|Kontrollera svensk moms, omvänd moms eller importbehandling|Koppla till inköp, försäljning, lager eller projekt|Vid vidarefakturering ligger kostnaden kvar på 5700 och kundersättningen på 3500|Stäm av mot transport- och tullhandlingar|Kräv granskning vid import, export eller större tillgångsförvärv|Kostnadsför frakt som avser leverans till kund eller allmän verksamhet|Lägg direkt hänförlig frakt i lager- eller tillgångsvärde|Koppla till ursprungsinköp eller projekt|Vid granskningsflagga begär in transportfaktura och underlag som visar gods, sträcka, ursprungsinköp eller kundleverans|Sätt ärendet till väntar på underlag tills verksamhetskoppling, moms och eventuell koppling till lager eller tillgång är klarlagda|Godkänn 5700 när en extern transportör utfört en löpande frakt- eller transporttjänst|Föreslå att frakten läggs i lager- eller tillgångsvärde, eller eskalering vid oklar import, export eller momsbehandling</x:v>
+        <x:v>Identifiera kostnadstyp, registreringsnummer, datum och affärsändamål|Pröva alltid mer specifikt konto först|Bokför endast verksamhetsandel|Bedöm ingående moms separat|Separera avdragsgilla avgifter från böter och privata utgifter|Koppla till körjournal eller fordonsregister|Använd obligatorisk underkategori|Kräv granskning för parkering, trängselskatt, självrisk, tillbehör och privat användning|Specificera parkering, trängselskatt, vägavgift, självrisk, tvätt, besiktning eller övrigt per fordon|Vid granskningsflagga begär in kvitto eller faktura, registreringsnummer och tydlig uppgift om kostnadstyp och affärsändamål|Sätt ärendet till väntar på underlag tills kostnaden och verksamhetsandelen är verifierade|Godkänn 5619 endast för en verklig personbilskostnad som inte passar på ett mer specifikt 561-konto|Föreslå specifikt bilkonto eller privat kostnad och avvisa böter och andra ej avdragsgilla sanktioner från automatflödet</x:v>
       </x:c>
       <x:c r="G129" s="14" t="str">
-        <x:v>2440|1930|2641|2645|3500|4000|1220</x:v>
+        <x:v>2440|1930|2641|2014|3200</x:v>
       </x:c>
       <x:c r="H129" s="14" t="str">
-        <x:v>Extern frakt för kundleverans bokförs på 5700 och eventuell kundersättning på 3500|Leveransfrakt för ny maskin kan behöva ingå i anskaffningsvärdet</x:v>
+        <x:v>En mindre verifierad fordonsavgift kan bokföras på 5619 när inget mer specifikt konto passar|En parkeringsbot bokförs inte automatiskt som avdragsgill kostnad</x:v>
       </x:c>
       <x:c r="I129" s="14" t="str">
-        <x:v>Frakt kan vara kostnad eller del av anskaffningsvärde|Eget fordon och personalresa hör till andra konton|Import och export kräver dokumentation|Vidarefakturering minskar inte automatiskt kostnaden|Internationell frakt kräver kontroll av Incoterms, tull och moms</x:v>
+        <x:v>5619 får inte bli restkonto|Böter och sanktionsavgifter kan vara ej avdragsgilla|Privatbilsschablonen täcker normala bilkostnader|Moms och privat användning bedöms per kostnad|Böter och sanktionsavgifter är normalt ej avdragsgilla och får inte blandas med parkering</x:v>
       </x:c>
       <x:c r="J129" s="14" t="str">
-        <x:v>frakt|transport|distribution|spedition|gods|leverans|R6</x:v>
+        <x:v>övrig personbilskostnad|parkering|trängselskatt|självrisk|biltillbehör|R6</x:v>
       </x:c>
       <x:c r="K129" s="14" t="str">
-        <x:v>3500|4000|4600|5600|5800|1220|2641|2645</x:v>
+        <x:v>5610|5611|5612|5613|5615|5618|1240|2014|3200</x:v>
       </x:c>
       <x:c r="L129" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5700, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, reglerna om anskaffningsvärde i kapitel 6 och punkterna 7.5–7.7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5619, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7</x:v>
       </x:c>
       <x:c r="M129" s="14" t="str">
-        <x:v>Det är oklart om frakten ska ingå i lager eller tillgång|Import, export, tull eller Incoterms förekommer|Affärsändamål saknas|Momsbehandlingen är oklar|Händelsen kan vara personalresa eller eget fordon|Import-, export- eller projektkoppling är oklar</x:v>
+        <x:v>Kostnadstypen är oklar|Böter, sanktionsavgift eller privat kostnad kan ingå|Fordon eller verksamhetsandel saknas|Momsavdragsrätten är oklar|Mer specifikt konto kan vara rätt|Kostnadstyp eller avdragsrätt är oklar</x:v>
       </x:c>
       <x:c r="N129" s="14" t="str">
         <x:v>active</x:v>
@@ -7205,43 +7209,43 @@
     </x:row>
     <x:row r="130" ht="430" customHeight="1">
       <x:c r="A130" s="14" t="str">
-        <x:v>5800</x:v>
+        <x:v>5620</x:v>
       </x:c>
       <x:c r="B130" s="14" t="str">
-        <x:v>Resekostnader</x:v>
+        <x:v>Lastbilskostnader</x:v>
       </x:c>
       <x:c r="C130" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för biljetter, logi och andra faktiska kostnader vid resor i näringsverksamheten. Privatbilens schablonmässiga milkostnad redovisas på 5618.</x:v>
+        <x:v>Kostnadskonto på R6 för drivmedel, försäkring, skatt, reparation, leasing och andra kostnader för lastbil eller annat fordon som redovisas i lastbilsgruppen.</x:v>
       </x:c>
       <x:c r="D130" s="14" t="str">
-        <x:v>Resan har direkt samband med företagets inköp, försäljning eller uppdrag|Kostnaden avser tåg, flyg, hotell eller lokal transport|Resmål, datum, deltagare och affärsändamål kan styrkas</x:v>
+        <x:v>Kostnaden hör till en identifierad lastbil i verksamheten|Fordonets registrering, ägande eller leasing och verksamhetsanvändning är verifierade|Utgiften är löpande fordonskostnad</x:v>
       </x:c>
       <x:c r="E130" s="14" t="str">
-        <x:v>Resan är privat eller saknar affärsändamål|Beloppet avser privat bils schablon; använd 5618|Beloppet avser företagets egna fordonskostnader|Utgiften är måltid, representation eller privat levnadskostnad utan avdragsrätt|Resan avser anställds skattepliktiga ersättning som ska hanteras i löneflödet</x:v>
+        <x:v>Fordonet är personbil; använd 5610-gruppen|Beloppet är inköp eller aktiverbar förbättring|Kostnaden är extern frakt- eller transporttjänst; använd 5700|Fordonet är privatägt och annan regel gäller|Fordonstyp eller verksamhetsandel är oklar</x:v>
       </x:c>
       <x:c r="F130" s="14" t="str">
-        <x:v>Kräv reseräkning med resenär, datum, ort, syfte och kund eller uppdrag|Bokför faktiska biljett-, hotell- och transportkostnader exklusive avdragsgill moms|Skilj faktisk resekostnad från ökade levnadskostnader, traktamente, representation och privat kostnad|Använd separat versionsstyrd rutin för schablonavdrag|Kontrollera övernattning, avstånd och fria måltider innan schablon används|Koppla resa till kalender och uppdrag|Stäm av förskott och återbetalningar|Kräv granskning vid utland, kombinerad semester eller medföljande privatperson|Använd endast för verifierad näringsresa|Spara datum, destination, syfte, deltagare och verksamhetskoppling|Hantera traktamente separat och versionsstyrt|Vid granskningsflagga begär in biljetter eller hotellunderlag samt resenär, datum, resmål och affärsändamål|Sätt ärendet till väntar på underlag tills näringsresan och eventuell privat del är verifierade|Godkänn 5800 för dokumenterade faktiska resekostnader i verksamheten|Föreslå uppdelning, privat kostnad eller separat rutin för privat bil, måltid, representation eller traktamente</x:v>
+        <x:v>Verifiera registreringsuppgifter, fordonsklass, ägare eller leasingtagare|Koppla kostnaden till registreringsnummer och underkategori|Bokför endast verksamhetsandel|Bedöm moms utifrån fordonets momsrättsliga klassificering|Skilj löpande kostnad från anskaffning eller förbättring|Stäm av mot 1240, körjournal, fordonsregister och leasingavtal|Kräv granskning vid privat användning eller oklar fordonsklass|Klassificera fordon från registrerings- och konstruktionsuppgifter|Specificera kostnader per lastbil och kostnadstyp|Vid granskningsflagga begär in registreringsuppgifter, faktura och uppgift om ägande eller leasing samt användning|Sätt ärendet till väntar på underlag tills fordonsklass, verksamhetsandel och momsbehandling är verifierade|Godkänn 5620 när kostnaden avser verksamhetens lastbil eller motsvarande nyttofordon|Föreslå annat fordonskonto, 5700 eller tillgångskonto när posten avser personbil, köpt transporttjänst eller anskaffning</x:v>
       </x:c>
       <x:c r="G130" s="14" t="str">
-        <x:v>2440|1930|2641|5618|6070|2013|2018</x:v>
+        <x:v>2440|1930|2641|1240|2014|3200</x:v>
       </x:c>
       <x:c r="H130" s="14" t="str">
-        <x:v>Tågbiljett och hotell för dokumenterat kundbesök bokförs på 5800|Privat bil till kundbesöket bokförs med schablon på 5618</x:v>
+        <x:v>Diesel och service för en verksamhetslastbil bokförs på 5620|En extern åkerifaktura bokförs på 5700</x:v>
       </x:c>
       <x:c r="I130" s="14" t="str">
-        <x:v>Affärsändamålet måste dokumenteras|Biljetter, logi, måltider och schablonavdrag har olika regler|Kombinerad privat- och affärsresa kräver fördelning|Utlandsresor och traktamenten är versionsberoende|Schablonavdrag ska inte skapas automatiskt från rese- eller hotellkvitto</x:v>
+        <x:v>Momsreglerna kan skilja sig från personbil men fordonsklass måste verifieras|5620 behöver underkategorier|Privat användning hanteras separat|Anskaffning är inte löpande kostnad|Vardaglig benämning avgör inte fordons- eller momsklass</x:v>
       </x:c>
       <x:c r="J130" s="14" t="str">
-        <x:v>resekostnad|tåg|flyg|hotell|tjänsteresa|övernattning|R6</x:v>
+        <x:v>lastbilskostnad|drivmedel lastbil|lastbilsförsäkring|lastbilsreparation|R6</x:v>
       </x:c>
       <x:c r="K130" s="14" t="str">
-        <x:v>5618|5700|6070|7300|2440|2641</x:v>
+        <x:v>5600|5610|5700|1240|2641|2014|3200</x:v>
       </x:c>
       <x:c r="L130" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5800, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7|Skatteverket – Resor med övernattning, kontrollerad 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5620, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7</x:v>
       </x:c>
       <x:c r="M130" s="14" t="str">
-        <x:v>Affärsändamål, resenär eller resplan saknas|Privat del eller semester förekommer|Måltider, traktamente eller representation ingår|Utlandsresa eller schablonavdrag förekommer|Momsavdragsrätten är oklar|Privat inslag, arbetsresa eller traktamentsvillkor är oklara</x:v>
+        <x:v>Fordonsklass eller registrering är oklar|Privat användning förekommer|Momsavdragsrätten är oklar|Kostnaden kan vara anskaffning eller förbättring|Extern transporttjänst kan vara rätt klassificering|Lätt lastbil, specialfordon eller momsprofil är oklar</x:v>
       </x:c>
       <x:c r="N130" s="14" t="str">
         <x:v>active</x:v>
@@ -7254,92 +7258,92 @@
     </x:row>
     <x:row r="131" ht="430" customHeight="1">
       <x:c r="A131" s="14" t="str">
-        <x:v>5900</x:v>
+        <x:v>5700</x:v>
       </x:c>
       <x:c r="B131" s="14" t="str">
-        <x:v>Reklam och PR</x:v>
+        <x:v>Frakter och transporter</x:v>
       </x:c>
       <x:c r="C131" s="14" t="str">
-        <x:v>K1-konto på R6 för annonsering, reklam, marknadsföring och PR som hör till verksamheten.</x:v>
+        <x:v>Kostnadskonto på R6 för köpta frakt-, distributions- och transporttjänster för företagets varor, material eller leveranser och inte för egna fordon eller personalresor.</x:v>
       </x:c>
       <x:c r="D131" s="14" t="str">
-        <x:v>Utgiften avser annonsering eller annan tydlig reklam för verksamheten|Utgiften avser mässa, reklamtrycksak, butiksreklam eller annan dokumenterad marknadsföring|Det finns faktura, kvitto eller avtal som visar vad företaget har köpt</x:v>
+        <x:v>Företaget köper frakt eller transport från extern transportör|Kostnaden avser transport av varor eller material|Frakten ska kostnadsföras och inte ingå i en tillgångs anskaffningsvärde</x:v>
       </x:c>
       <x:c r="E131" s="14" t="str">
-        <x:v>Utgiften är privat|Utgiften är representation eller en vanlig gåva|Sponsringen saknar tydlig motprestation eller reklamvärde|Kostnaden hör tydligare hemma på ett annat konto</x:v>
+        <x:v>Kostnaden avser eget fordon; använd 5600-serien|Kostnaden avser företagaren eller personals resa; använd 5800|Frakten är direkt hänförlig till lager eller anläggningstillgång och ska ingå i anskaffningsvärdet|Händelsen är äkta utlägg|Transporten är privat</x:v>
       </x:c>
       <x:c r="F131" s="14" t="str">
-        <x:v>Tydligt angivna reklamkanaler och marknadsföringsåtgärder får sammanföras automatiskt till 5900|Gruppkontot 5900 och övrigt-kontot 5990 kräver kontroll av vad kostnaden faktiskt avser|Varuprover, reklamgåvor, presentreklam och tävlingar kräver kontroll av avdragsrätt och faktisk karaktär|PR och sponsring kräver kontroll av avtal, affärssyfte och motprestation|Vid sponsring får bara den del som motsvaras av en verklig motprestation behandlas som reklam enligt nuvarande regler|Utländsk annonsleverantör kan kräva separat kontroll av omvänd moms men reklamkontot är fortfarande 5900|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Identifiera transportör, gods, avsändare, mottagare och affärshändelse|Avgör om frakten är löpande kostnad eller direkt förvärvsutgift|Bokför kostnaden exklusive avdragsgill moms|Kontrollera svensk moms, omvänd moms eller importbehandling|Koppla till inköp, försäljning, lager eller projekt|Vid vidarefakturering ligger kostnaden kvar på 5700 och kundersättningen på 3500|Stäm av mot transport- och tullhandlingar|Kräv granskning vid import, export eller större tillgångsförvärv|Kostnadsför frakt som avser leverans till kund eller allmän verksamhet|Lägg direkt hänförlig frakt i lager- eller tillgångsvärde|Koppla till ursprungsinköp eller projekt|Vid granskningsflagga begär in transportfaktura och underlag som visar gods, sträcka, ursprungsinköp eller kundleverans|Sätt ärendet till väntar på underlag tills verksamhetskoppling, moms och eventuell koppling till lager eller tillgång är klarlagda|Godkänn 5700 när en extern transportör utfört en löpande frakt- eller transporttjänst|Föreslå att frakten läggs i lager- eller tillgångsvärde, eller eskalering vid oklar import, export eller momsbehandling</x:v>
       </x:c>
       <x:c r="G131" s="14" t="str">
-        <x:v>2440|1930|2641|2645|1700</x:v>
+        <x:v>2440|1930|2641|2645|3500|4000|1220</x:v>
       </x:c>
       <x:c r="H131" s="14" t="str">
-        <x:v>En faktura för annonsering i en svensk tidning bokförs på 5900|Digital annonsering hos Google eller Meta bokförs på 5900; eventuell omvänd moms hanteras separat|Sponsring granskas innan den bokförs eftersom avtalet och motprestationen måste bedömas</x:v>
+        <x:v>Extern frakt för kundleverans bokförs på 5700 och eventuell kundersättning på 3500|Leveransfrakt för ny maskin kan behöva ingå i anskaffningsvärdet</x:v>
       </x:c>
       <x:c r="I131" s="14" t="str">
-        <x:v>Sponsring är inte automatiskt avdragsgill bara för att företagsnamnet syns|Reklamgåvor, tävlingspriser och representation kan ha andra skatte- och momsregler|Utländska annonsplattformar kan medföra omvänd moms</x:v>
+        <x:v>Frakt kan vara kostnad eller del av anskaffningsvärde|Eget fordon och personalresa hör till andra konton|Import och export kräver dokumentation|Vidarefakturering minskar inte automatiskt kostnaden|Internationell frakt kräver kontroll av Incoterms, tull och moms</x:v>
       </x:c>
       <x:c r="J131" s="14" t="str">
-        <x:v>reklam|annonsering|marknadsföring|PR|mässa|sponsring|reklamgåva|R6</x:v>
+        <x:v>frakt|transport|distribution|spedition|gods|leverans|R6</x:v>
       </x:c>
       <x:c r="K131" s="14" t="str">
-        <x:v>6070|6900|6992|6993|2440|2641|2645</x:v>
+        <x:v>3500|4000|4600|5600|5800|1220|2641|2645</x:v>
       </x:c>
       <x:c r="L131" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – konto 5900, rad R6|BFNAR 2006:1 senast ändrat genom BFNAR 2025:1|Skatteverkets rättsliga vägledning om sponsring, 2026</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5700, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, reglerna om anskaffningsvärde i kapitel 6 och punkterna 7.5–7.7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer</x:v>
       </x:c>
       <x:c r="M131" s="14" t="str">
-        <x:v>Posten kommer från BAS 5900, 5960, 5980 eller 5990|Kostnaden kan vara gåva, representation eller tävlingspris|Sponsringsavtal, motprestation eller reklamvärde är oklart|Kostnadens affärsmässiga samband med verksamheten är oklart</x:v>
+        <x:v>Det är oklart om frakten ska ingå i lager eller tillgång|Import, export, tull eller Incoterms förekommer|Affärsändamål saknas|Momsbehandlingen är oklar|Händelsen kan vara personalresa eller eget fordon|Import-, export- eller projektkoppling är oklar</x:v>
       </x:c>
       <x:c r="N131" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O131" s="14" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="P131" s="14"/>
       <x:c r="Q131" s="12" t="str"/>
     </x:row>
     <x:row r="132" ht="430" customHeight="1">
       <x:c r="A132" s="14" t="str">
-        <x:v>6000</x:v>
+        <x:v>5800</x:v>
       </x:c>
       <x:c r="B132" s="14" t="str">
-        <x:v>Övriga försäljningskostnader</x:v>
+        <x:v>Resekostnader</x:v>
       </x:c>
       <x:c r="C132" s="14" t="str">
-        <x:v>Samlingskonto på R6 för försäljningskostnader som inte passar bättre som reklam och PR, representation, frakt, resa eller annan mer specifik extern kostnad.</x:v>
+        <x:v>Kostnadskonto på R6 för biljetter, logi och andra faktiska kostnader vid resor i näringsverksamheten. Privatbilens schablonmässiga milkostnad redovisas på 5618.</x:v>
       </x:c>
       <x:c r="D132" s="14" t="str">
-        <x:v>Utgiften har direkt samband med försäljning eller kundanskaffning|Ingen mer specifik tillåten kontogrupp beskriver kostnaden bättre|Kostnadstyp, motpart, affärsändamål och underlag är dokumenterade|Avgiften avser verifierad kortinlösen eller betalningsförmedling för företagets försäljning</x:v>
+        <x:v>Resan har direkt samband med företagets inköp, försäljning eller uppdrag|Kostnaden avser tåg, flyg, hotell eller lokal transport|Resmål, datum, deltagare och affärsändamål kan styrkas</x:v>
       </x:c>
       <x:c r="E132" s="14" t="str">
-        <x:v>Utgiften är reklam; använd 5900|Utgiften är representation; använd 6070-gruppen|Utgiften är frakt, resa, extern konsulttjänst eller annan kostnad med mer specifikt konto|Beloppet är kundrabatt på 3700|Kostnaden är privat, ej avdragsgill gåva eller okänd banktransaktion</x:v>
+        <x:v>Resan är privat eller saknar affärsändamål|Beloppet avser privat bils schablon; använd 5618|Beloppet avser företagets egna fordonskostnader|Utgiften är måltid, representation eller privat levnadskostnad utan avdragsrätt|Resan avser anställds skattepliktiga ersättning som ska hanteras i löneflödet</x:v>
       </x:c>
       <x:c r="F132" s="14" t="str">
-        <x:v>Identifiera obligatorisk underkategori, exempelvis försäljningsmaterial, orderkostnad, kortavgift, kreditkostnad eller provision|Pröva alltid 3500, 3700, 5700, 5800, 5900, 6070 och 6500 först|Verifiera direkt samband med försäljning|Bokför avdragsgill moms separat|BAS 6040 Kontokortsavgifter får sammanföras automatiskt när kortinlösarens avräkning och utbetalning kan stämmas av|BAS 6000 och 6090 får inte sammanföras automatiskt utan dokumenterad underkategori|BAS 6050 Försäljningsprovisioner kräver kontroll av mottagare, avtal, F-skatt och eventuell löne- eller avgiftshantering|BAS 6055 Franchisekostnader kräver kontroll av om avgiften är löpande, förutbetald eller avser en förvärvad rättighet|BAS 6062 kräver att normala inkassokostnader skiljs från böter, sanktioner och andra ej avdragsgilla avgifter|BAS 6064 Factoringavgifter ska delas upp om underlaget innehåller ränta, kreditkostnad eller annan finansieringsdel|BAS 6069 kräver specifikation av kostnadstyp före sammanföring|BAS 6080 Bankgarantier kräver klassificering och eventuell periodisering|Koppla kostnaden till kampanj, kund, kanal eller aktivitet och dela blandad faktura radvis</x:v>
+        <x:v>Kräv reseräkning med resenär, datum, ort, syfte och kund eller uppdrag|Bokför faktiska biljett-, hotell- och transportkostnader exklusive avdragsgill moms|Skilj faktisk resekostnad från ökade levnadskostnader, traktamente, representation och privat kostnad|Använd separat versionsstyrd rutin för schablonavdrag|Kontrollera övernattning, avstånd och fria måltider innan schablon används|Koppla resa till kalender och uppdrag|Stäm av förskott och återbetalningar|Kräv granskning vid utland, kombinerad semester eller medföljande privatperson|Använd endast för verifierad näringsresa|Spara datum, destination, syfte, deltagare och verksamhetskoppling|Hantera traktamente separat och versionsstyrt|Vid granskningsflagga begär in biljetter eller hotellunderlag samt resenär, datum, resmål och affärsändamål|Sätt ärendet till väntar på underlag tills näringsresan och eventuell privat del är verifierade|Godkänn 5800 för dokumenterade faktiska resekostnader i verksamheten|Föreslå uppdelning, privat kostnad eller separat rutin för privat bil, måltid, representation eller traktamente</x:v>
       </x:c>
       <x:c r="G132" s="14" t="str">
-        <x:v>2440|1930|2641|2645|5900|6070|6500</x:v>
+        <x:v>2440|1930|2641|5618|6070|2013|2018</x:v>
       </x:c>
       <x:c r="H132" s="14" t="str">
-        <x:v>En verifierad kortinlösenavgift från Zettle eller annan kortinlösare bokförs på 6000|En factoringfaktura delas mellan tjänsteavgift på 6000 och eventuell ränta på 8410|En löpande franchiseavgift kan efter granskning bokföras på 6000 medan en startavgift kan kräva annan hantering|En okänd kortbetalning eller ospecificerad post på 6000 eller 6090 får inte godkännas utan underlag</x:v>
+        <x:v>Tågbiljett och hotell för dokumenterat kundbesök bokförs på 5800|Privat bil till kundbesöket bokförs med schablon på 5618</x:v>
       </x:c>
       <x:c r="I132" s="14" t="str">
-        <x:v>6000 får inte bli restkonto|Varje bokning behöver underkategori och affärskoppling|Reklam, representation, resa, frakt och konsulttjänst särredovisas när möjligt|Provision till privatperson kan medföra skyldighet att hantera skatt och avgifter|Factoringavgift kan innehålla ränta som ska hållas isär|Franchise och bankgaranti kan behöva periodiseras eller omklassificeras|Ej avdragsgilla och privata kostnader får inte döljas</x:v>
+        <x:v>Affärsändamålet måste dokumenteras|Biljetter, logi, måltider och schablonavdrag har olika regler|Kombinerad privat- och affärsresa kräver fördelning|Utlandsresor och traktamenten är versionsberoende|Schablonavdrag ska inte skapas automatiskt från rese- eller hotellkvitto</x:v>
       </x:c>
       <x:c r="J132" s="14" t="str">
-        <x:v>övrig försäljningskostnad|marknadsplatsavgift|mässa|event|kundanskaffning|R6</x:v>
+        <x:v>resekostnad|tåg|flyg|hotell|tjänsteresa|övernattning|R6</x:v>
       </x:c>
       <x:c r="K132" s="14" t="str">
-        <x:v>3500|3700|5700|5800|5900|6070|6500|2440|2641</x:v>
+        <x:v>5618|5700|6070|7300|2440|2641</x:v>
       </x:c>
       <x:c r="L132" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 6000, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sidoordnad specifikation</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 5800, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7|Skatteverket – Resor med övernattning, kontrollerad 2026-07-30</x:v>
       </x:c>
       <x:c r="M132" s="14" t="str">
-        <x:v>Mer specifikt konto kan vara rätt|Kostnadstyp eller affärssamband saknas|Gåva, representation eller privat utgift kan ingå|Utland eller omvänd moms förekommer|Posten kommer från BAS 6000, 6050, 6055, 6062, 6064, 6069, 6080 eller 6090|Provisionens mottagare eller F-skatt är oklar|Factoringavgiften kan innehålla ränta eller finansieringsdel|Franchiseavgiftens period eller rättighetens karaktär är oklar|Bankgaranti eller annan avgift kan behöva periodiseras</x:v>
+        <x:v>Affärsändamål, resenär eller resplan saknas|Privat del eller semester förekommer|Måltider, traktamente eller representation ingår|Utlandsresa eller schablonavdrag förekommer|Momsavdragsrätten är oklar|Privat inslag, arbetsresa eller traktamentsvillkor är oklara</x:v>
       </x:c>
       <x:c r="N132" s="14" t="str">
         <x:v>active</x:v>
@@ -7352,94 +7356,92 @@
     </x:row>
     <x:row r="133" ht="430" customHeight="1">
       <x:c r="A133" s="14" t="str">
-        <x:v>6070</x:v>
+        <x:v>5900</x:v>
       </x:c>
       <x:c r="B133" s="14" t="str">
-        <x:v>Representation</x:v>
+        <x:v>Reklam och PR</x:v>
       </x:c>
       <x:c r="C133" s="14" t="str">
-        <x:v>Huvud- eller samlingskonto på R6 för extern representation. Kostnaden ska delas mellan avdragsgill del på 6071 och ej avdragsgill del på 6072 när skattereglerna kräver det.</x:v>
+        <x:v>K1-konto på R6 för annonsering, reklam, marknadsföring och PR som hör till verksamheten.</x:v>
       </x:c>
       <x:c r="D133" s="14" t="str">
-        <x:v>Utgiften har ett omedelbart och dokumenterat samband med näringsverksamheten|Representationen riktar sig till kund, leverantör eller annan extern affärskontakt|Deltagare, syfte, datum, plats och kostnad per person är kända|Systemets kontoplan tillåter samlingskonto 6070</x:v>
+        <x:v>Utgiften avser annonsering eller annan tydlig reklam för verksamheten|Utgiften avser mässa, reklamtrycksak, butiksreklam eller annan dokumenterad marknadsföring|Det finns faktura, kvitto eller avtal som visar vad företaget har köpt</x:v>
       </x:c>
       <x:c r="E133" s="14" t="str">
-        <x:v>Utgiften är privat eller social utan affärssamband|Aktiviteten är reklam eller sponsring med motprestation; pröva 5900|Aktiviteten gäller företagets anställda; pröva personalrepresentation på 7631 eller 7632|Det finns tillräckliga uppgifter för att använda 6071 och 6072|Deltagarförteckning, affärssyfte eller underlag saknas</x:v>
+        <x:v>Utgiften är privat|Utgiften är representation eller en vanlig gåva|Sponsringen saknar tydlig motprestation eller reklamvärde|Kostnaden hör tydligare hemma på ett annat konto</x:v>
       </x:c>
       <x:c r="F133" s="14" t="str">
-        <x:v>Kräv representationstyp, extern eller intern, affärssyfte, deltagare och deras relation till företaget|Kräv datum, plats, antal personer, utgiftsslag och belopp per person|Kontrollera omedelbart samband med verksamheten och skälighet|Dela kostnaden i avdragsgill och ej avdragsgill del enligt aktuell inkomstskatteregel|Beräkna avdragsgill ingående moms separat; inkomstskattemässigt avdrag och momsavdrag är olika bedömningar|Bokför avdragsgill kostnadsdel på 6071 och ej avdragsgill kostnadsdel inklusive ej avdragsgill moms på 6072|Koppla varje post till kvitto, faktura och deltagarlista|Blockera direktbokning på 6070 när fördelningen kan göras|Kräv manuell granskning vid alkohol, gåva, familjemedlem, utlandsrepresentation eller återkommande representation|Kräv datum, plats, affärssyfte, deltagare, relation, antal personer, kostnader och moms|Skilj extern från intern representation|Flagga bokning på 6070 när den kan fördelas mellan avdragsgill och ej avdragsgill representation|Begär kvitto eller faktura, datum, plats, deltagare, relation och affärssyfte och sätt ärendet till väntar på underlag|Godkänn representationen först när verksamhetssamband, kostnadsslag, personbelopp och moms är verifierade|Föreslå uppdelning på 6071 och 6072, privat kostnad eller eskalering när representationstypen förblir oklar</x:v>
+        <x:v>Tydligt angivna reklamkanaler och marknadsföringsåtgärder får sammanföras automatiskt till 5900|Gruppkontot 5900 och övrigt-kontot 5990 kräver kontroll av vad kostnaden faktiskt avser|Varuprover, reklamgåvor, presentreklam och tävlingar kräver kontroll av avdragsrätt och faktisk karaktär|PR och sponsring kräver kontroll av avtal, affärssyfte och motprestation|Vid sponsring får bara den del som motsvaras av en verklig motprestation behandlas som reklam enligt nuvarande regler|Utländsk annonsleverantör kan kräva separat kontroll av omvänd moms men reklamkontot är fortfarande 5900|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G133" s="14" t="str">
-        <x:v>2440|1930|2641|6071|6072</x:v>
+        <x:v>2440|1930|2641|2645|1700</x:v>
       </x:c>
       <x:c r="H133" s="14" t="str">
-        <x:v>En kundmåltid kan vara helt ej avdragsgill vid inkomstbeskattningen men ändå ge ett begränsat momsavdrag; kostnadsdelen bokförs då på 6072 och den avdragsgilla momsen på 2641</x:v>
+        <x:v>En faktura för annonsering i en svensk tidning bokförs på 5900|Digital annonsering hos Google eller Meta bokförs på 5900; eventuell omvänd moms hanteras separat|Sponsring granskas innan den bokförs eftersom avtalet och motprestationen måste bedömas</x:v>
       </x:c>
       <x:c r="I133" s="14" t="str">
-        <x:v>Avdragsgill kostnad och avdragsgill moms är två olika beräkningar|6070 bör normalt inte ha ospecificerat saldo vid bokslut|Affärssamband och deltagare måste dokumenteras|Intern representation hör normalt till personalkostnader|Saknad deltagarlista eller intern representation stoppar standardflödet</x:v>
+        <x:v>Sponsring är inte automatiskt avdragsgill bara för att företagsnamnet syns|Reklamgåvor, tävlingspriser och representation kan ha andra skatte- och momsregler|Utländska annonsplattformar kan medföra omvänd moms</x:v>
       </x:c>
       <x:c r="J133" s="14" t="str">
-        <x:v>representation|extern representation|kundmåltid|deltagarförteckning|R6</x:v>
+        <x:v>reklam|annonsering|marknadsföring|PR|mässa|sponsring|reklamgåva|R6</x:v>
       </x:c>
       <x:c r="K133" s="14" t="str">
-        <x:v>6071|6072|5900|7631|7632|2641</x:v>
+        <x:v>6070|6900|6992|6993|2440|2641|2645</x:v>
       </x:c>
       <x:c r="L133" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 6070 och underkonton, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Belopp och procent 2026 samt Representation, kontrollerat 2026-07-30|Skatteverket – Avdrag för moms vid representation, kontrollerat 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – konto 5900, rad R6|BFNAR 2006:1 senast ändrat genom BFNAR 2025:1|Skatteverkets rättsliga vägledning om sponsring, 2026</x:v>
       </x:c>
       <x:c r="M133" s="14" t="str">
-        <x:v>Deltagare, syfte eller affärssamband saknas|Alkohol, gåva, familjemedlem eller privat inslag förekommer|Intern representation kan vara rätt klassificering|Kostnaden ska delas mellan 6071 och 6072|Momsfördelningen är oklar|Affärssamband eller representationstyp är oklar</x:v>
+        <x:v>Posten kommer från BAS 5900, 5960, 5980 eller 5990|Kostnaden kan vara gåva, representation eller tävlingspris|Sponsringsavtal, motprestation eller reklamvärde är oklart|Kostnadens affärsmässiga samband med verksamheten är oklart</x:v>
       </x:c>
       <x:c r="N133" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O133" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P133" s="14" t="str">
-        <x:v>representation_meal_income_deduction_zero_2026|representation_simple_refreshment_limit_2026|representation_other_expense_limit_2026|representation_meal_vat_base_2026|representation_gift_limit_2026</x:v>
-      </x:c>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P133" s="14"/>
       <x:c r="Q133" s="12" t="str"/>
     </x:row>
     <x:row r="134" ht="430" customHeight="1">
       <x:c r="A134" s="14" t="str">
-        <x:v>6071</x:v>
+        <x:v>6000</x:v>
       </x:c>
       <x:c r="B134" s="14" t="str">
-        <x:v>Representation, avdragsgill</x:v>
+        <x:v>Övriga försäljningskostnader</x:v>
       </x:c>
       <x:c r="C134" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för den del av extern representation som är avdragsgill vid inkomstbeskattningen enligt aktuell belopps- och sambandsregel.</x:v>
+        <x:v>Samlingskonto på R6 för försäljningskostnader som inte passar bättre som reklam och PR, representation, frakt, resa eller annan mer specifik extern kostnad.</x:v>
       </x:c>
       <x:c r="D134" s="14" t="str">
-        <x:v>Representationen har omedelbart samband med verksamheten|Utgiften avser enklare förtäring inom 60 kronor exklusive moms per person|Utgiften avser avdragsgill kringaktivitet inom 180 kronor exklusive moms per person|En representationsgåva uppfyller villkoren och ryms inom 300 kronor exklusive moms</x:v>
+        <x:v>Utgiften har direkt samband med försäljning eller kundanskaffning|Ingen mer specifik tillåten kontogrupp beskriver kostnaden bättre|Kostnadstyp, motpart, affärsändamål och underlag är dokumenterade|Avgiften avser verifierad kortinlösen eller betalningsförmedling för företagets försäljning</x:v>
       </x:c>
       <x:c r="E134" s="14" t="str">
-        <x:v>Utgiften avser frukost, lunch, middag eller annan måltid som inte är enklare förtäring; inkomstskattemässigt avdrag är 0 kronor|Beloppet överstiger avdragsramen; överskjutande del bokförs på 6072|Affärssamband, deltagare eller syfte saknas|Aktiviteten är intern representation|Utgiften är privat, gåva utan representationssamband eller reklam</x:v>
+        <x:v>Utgiften är reklam; använd 5900|Utgiften är representation; använd 6070-gruppen|Utgiften är frakt, resa, extern konsulttjänst eller annan kostnad med mer specifikt konto|Beloppet är kundrabatt på 3700|Kostnaden är privat, ej avdragsgill gåva eller okänd banktransaktion</x:v>
       </x:c>
       <x:c r="F134" s="14" t="str">
-        <x:v>Verifiera extern representation och omedelbart samband med verksamheten|Klassificera utgiften som enklare förtäring, måltid, kringkostnad eller representationsgåva|Beräkna avdragsram per person och tillfälle med versionsstyrd parameter|Bokför endast den inkomstskattemässigt avdragsgilla delen på 6071|Bokför överskjutande eller helt ej avdragsgill kostnadsdel på 6072|Beräkna ingående moms separat enligt momsregeln|Kräv kvitto eller faktura, deltagarlista, syfte, ort och datum|Stäm av belopp per deltagare och mot 6072|Kräv manuell granskning vid gåva, alkohol eller blandade utgiftsslag|Använd endast efter klassificering av enklare förtäring, måltid eller representationsgåva|Koppla till deltagarlista och affärssyfte|Vid granskningsflagga begär in kvitto eller faktura, deltagarlista, datum, plats och affärssyfte|Sätt ärendet till väntar på underlag tills representationstyp, aktuell avdragsram och momsberäkning är verifierade|Godkänn 6071 endast för den dokumenterade inkomstskattemässigt avdragsgilla delen|Föreslå 6072, privat kostnad eller eskalering för överskjutande belopp, saknat samband eller oklar gåva och alkohol</x:v>
+        <x:v>Identifiera obligatorisk underkategori, exempelvis försäljningsmaterial, orderkostnad, kortavgift, kreditkostnad eller provision|Pröva alltid 3500, 3700, 5700, 5800, 5900, 6070 och 6500 först|Verifiera direkt samband med försäljning|Bokför avdragsgill moms separat|BAS 6040 Kontokortsavgifter får sammanföras automatiskt när kortinlösarens avräkning och utbetalning kan stämmas av|BAS 6000 och 6090 får inte sammanföras automatiskt utan dokumenterad underkategori|BAS 6050 Försäljningsprovisioner kräver kontroll av mottagare, avtal, F-skatt och eventuell löne- eller avgiftshantering|BAS 6055 Franchisekostnader kräver kontroll av om avgiften är löpande, förutbetald eller avser en förvärvad rättighet|BAS 6062 kräver att normala inkassokostnader skiljs från böter, sanktioner och andra ej avdragsgilla avgifter|BAS 6064 Factoringavgifter ska delas upp om underlaget innehåller ränta, kreditkostnad eller annan finansieringsdel|BAS 6069 kräver specifikation av kostnadstyp före sammanföring|BAS 6080 Bankgarantier kräver klassificering och eventuell periodisering|Koppla kostnaden till kampanj, kund, kanal eller aktivitet och dela blandad faktura radvis</x:v>
       </x:c>
       <x:c r="G134" s="14" t="str">
-        <x:v>2440|1930|2641|6072</x:v>
+        <x:v>2440|1930|2641|2645|5900|6070|6500</x:v>
       </x:c>
       <x:c r="H134" s="14" t="str">
-        <x:v>Kaffe och enklare smörgås för 55 kronor exklusive moms per kund kan bokföras på 6071 när sambands- och dokumentationskraven är uppfyllda|En kundmiddag bokförs inte som avdragsgill måltidskostnad på 6071</x:v>
+        <x:v>En verifierad kortinlösenavgift från Zettle eller annan kortinlösare bokförs på 6000|En factoringfaktura delas mellan tjänsteavgift på 6000 och eventuell ränta på 8410|En löpande franchiseavgift kan efter granskning bokföras på 6000 medan en startavgift kan kräva annan hantering|En okänd kortbetalning eller ospecificerad post på 6000 eller 6090 får inte godkännas utan underlag</x:v>
       </x:c>
       <x:c r="I134" s="14" t="str">
-        <x:v>En måltid är inte enklare förtäring|Om enklare förtäring överstiger 60 kronor kan hela beloppet bli ej avdragsgillt enligt regeln|Momsavdraget beräknas separat|Avdragsramarna gäller per person och tillfälle|Reklamgåva och vanlig gåva ska inte bokföras här</x:v>
+        <x:v>6000 får inte bli restkonto|Varje bokning behöver underkategori och affärskoppling|Reklam, representation, resa, frakt och konsulttjänst särredovisas när möjligt|Provision till privatperson kan medföra skyldighet att hantera skatt och avgifter|Factoringavgift kan innehålla ränta som ska hållas isär|Franchise och bankgaranti kan behöva periodiseras eller omklassificeras|Ej avdragsgilla och privata kostnader får inte döljas</x:v>
       </x:c>
       <x:c r="J134" s="14" t="str">
-        <x:v>avdragsgill representation|enklare förtäring|kringkostnad|representationsgåva|R6</x:v>
+        <x:v>övrig försäljningskostnad|marknadsplatsavgift|mässa|event|kundanskaffning|R6</x:v>
       </x:c>
       <x:c r="K134" s="14" t="str">
-        <x:v>6070|6072|2641|5900|7631</x:v>
+        <x:v>3500|3700|5700|5800|5900|6070|6500|2440|2641</x:v>
       </x:c>
       <x:c r="L134" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 6071, rad R6|Skatteverket – Belopp och procent 2026 samt Representation, kontrollerat 2026-07-30|Skatteverket – Avdrag för moms vid representation, kontrollerat 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 6000, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sidoordnad specifikation</x:v>
       </x:c>
       <x:c r="M134" s="14" t="str">
-        <x:v>Beloppet ligger nära eller över en avdragsram|Måltid, alkohol eller gåva förekommer|Deltagarantal eller affärssamband saknas|Intern representation kan vara rätt|Flera utgiftsslag eller momssatser ingår|Måltidstyp, gåvotyp eller avdragsram är oklar</x:v>
+        <x:v>Mer specifikt konto kan vara rätt|Kostnadstyp eller affärssamband saknas|Gåva, representation eller privat utgift kan ingå|Utland eller omvänd moms förekommer|Posten kommer från BAS 6000, 6050, 6055, 6062, 6064, 6069, 6080 eller 6090|Provisionens mottagare eller F-skatt är oklar|Factoringavgiften kan innehålla ränta eller finansieringsdel|Franchiseavgiftens period eller rättighetens karaktär är oklar|Bankgaranti eller annan avgift kan behöva periodiseras</x:v>
       </x:c>
       <x:c r="N134" s="14" t="str">
         <x:v>active</x:v>
@@ -7447,50 +7449,48 @@
       <x:c r="O134" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P134" s="14" t="str">
-        <x:v>representation_simple_refreshment_limit_2026|representation_other_expense_limit_2026|representation_gift_limit_2026|representation_meal_vat_base_2026</x:v>
-      </x:c>
+      <x:c r="P134" s="14"/>
       <x:c r="Q134" s="12" t="str"/>
     </x:row>
     <x:row r="135" ht="430" customHeight="1">
       <x:c r="A135" s="14" t="str">
-        <x:v>6072</x:v>
+        <x:v>6070</x:v>
       </x:c>
       <x:c r="B135" s="14" t="str">
-        <x:v>Representation, ej avdragsgill</x:v>
+        <x:v>Representation</x:v>
       </x:c>
       <x:c r="C135" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för den del av extern representation som inte är avdragsgill vid inkomstbeskattningen. Kontot är markerat för skattemässig återläggning i NE-bilagan.</x:v>
+        <x:v>Huvud- eller samlingskonto på R6 för extern representation. Kostnaden ska delas mellan avdragsgill del på 6071 och ej avdragsgill del på 6072 när skattereglerna kräver det.</x:v>
       </x:c>
       <x:c r="D135" s="14" t="str">
-        <x:v>Utgiften är en affärsmässigt motiverad representationskostnad men saknar helt eller delvis inkomstskattemässigt avdrag|Utgiften avser frukost, lunch, middag eller annan måltid med 0 kronor i inkomstskattemässigt avdrag|Beloppet överstiger avdragsramen på 6071|Ej avdragsgill moms ska ingå i kostnaden</x:v>
+        <x:v>Utgiften har ett omedelbart och dokumenterat samband med näringsverksamheten|Representationen riktar sig till kund, leverantör eller annan extern affärskontakt|Deltagare, syfte, datum, plats och kostnad per person är kända|Systemets kontoplan tillåter samlingskonto 6070</x:v>
       </x:c>
       <x:c r="E135" s="14" t="str">
-        <x:v>Utgiften är privat och saknar samband med verksamheten; bokför som eget uttag i stället|Utgiften är avdragsgill och ryms inom 6071|Aktiviteten är intern personalrepresentation|Utgiften är reklam eller sponsring med verifierad motprestation|Underlag och affärssyfte saknas helt</x:v>
+        <x:v>Utgiften är privat eller social utan affärssamband|Aktiviteten är reklam eller sponsring med motprestation; pröva 5900|Aktiviteten gäller företagets anställda; pröva personalrepresentation på 7631 eller 7632|Det finns tillräckliga uppgifter för att använda 6071 och 6072|Deltagarförteckning, affärssyfte eller underlag saknas</x:v>
       </x:c>
       <x:c r="F135" s="14" t="str">
-        <x:v>Verifiera att utgiften trots ej avdragsgill status hör till en faktisk affärshändelse i verksamheten|Klassificera representationstyp och beräkna avdragsgill del på 6071|Bokför resterande kostnad och ej avdragsgill moms på 6072|För måltider är inkomstskattemässigt avdrag 0 kronor men momsavdrag kan finnas på ett underlag om högst 300 kronor exklusive moms per person och tillfälle|Beräkna moms efter faktisk fördelning mellan mat och alkohol när sådan uppdelning finns|Märk kontot för skattemässig återläggning i NE-underlaget|Kräv deltagarlista, syfte, datum och plats även för ej avdragsgill representation|Separera privat del som eget uttag|Kräv manuell granskning vid alkohol, familjemedlem, gåva eller oskäligt belopp|Använd för ej avdragsgill del efter dokumenterad representationsbedömning|Beräkna mat, alkohol, momssatser och personbelopp separat|Vid granskningsflagga begär in kvitto eller faktura, deltagarlista, datum, plats, affärssyfte och momsuppdelning|Sätt ärendet till väntar på underlag tills den faktiska representationen och eventuell privat eller avdragsgill del är verifierad|Godkänn 6072 för den dokumenterade ej avdragsgilla representationsdelen och markera skattemässig återläggning|Föreslå 6071, eget uttag eller eskalering när posten innehåller avdragsgill del, privat kostnad eller oklar moms</x:v>
+        <x:v>Kräv representationstyp, extern eller intern, affärssyfte, deltagare och deras relation till företaget|Kräv datum, plats, antal personer, utgiftsslag och belopp per person|Kontrollera omedelbart samband med verksamheten och skälighet|Dela kostnaden i avdragsgill och ej avdragsgill del enligt aktuell inkomstskatteregel|Beräkna avdragsgill ingående moms separat; inkomstskattemässigt avdrag och momsavdrag är olika bedömningar|Bokför avdragsgill kostnadsdel på 6071 och ej avdragsgill kostnadsdel inklusive ej avdragsgill moms på 6072|Koppla varje post till kvitto, faktura och deltagarlista|Blockera direktbokning på 6070 när fördelningen kan göras|Kräv manuell granskning vid alkohol, gåva, familjemedlem, utlandsrepresentation eller återkommande representation|Kräv datum, plats, affärssyfte, deltagare, relation, antal personer, kostnader och moms|Skilj extern från intern representation|Flagga bokning på 6070 när den kan fördelas mellan avdragsgill och ej avdragsgill representation|Begär kvitto eller faktura, datum, plats, deltagare, relation och affärssyfte och sätt ärendet till väntar på underlag|Godkänn representationen först när verksamhetssamband, kostnadsslag, personbelopp och moms är verifierade|Föreslå uppdelning på 6071 och 6072, privat kostnad eller eskalering när representationstypen förblir oklar</x:v>
       </x:c>
       <x:c r="G135" s="14" t="str">
-        <x:v>2440|1930|2641|6071|2013</x:v>
+        <x:v>2440|1930|2641|6071|6072</x:v>
       </x:c>
       <x:c r="H135" s="14" t="str">
-        <x:v>En kundmiddag bokförs på 6072 exklusive den del av ingående moms som får dras av enligt representationsmomsregeln|Privat middag utan affärssamband bokförs inte på 6072 utan som eget uttag</x:v>
+        <x:v>En kundmåltid kan vara helt ej avdragsgill vid inkomstbeskattningen men ändå ge ett begränsat momsavdrag; kostnadsdelen bokförs då på 6072 och den avdragsgilla momsen på 2641</x:v>
       </x:c>
       <x:c r="I135" s="14" t="str">
-        <x:v>Ej avdragsgill betyder inte att dokumentationskraven försvinner|Privat kostnad får inte döljas som ej avdragsgill representation|Begränsat momsavdrag kan finnas trots 0 kronor i inkomstskattemässigt måltidsavdrag|Kontot ska återläggas skattemässigt|Momsavdrag och inkomstskatteavdrag följer inte samma gräns</x:v>
+        <x:v>Avdragsgill kostnad och avdragsgill moms är två olika beräkningar|6070 bör normalt inte ha ospecificerat saldo vid bokslut|Affärssamband och deltagare måste dokumenteras|Intern representation hör normalt till personalkostnader|Saknad deltagarlista eller intern representation stoppar standardflödet</x:v>
       </x:c>
       <x:c r="J135" s="14" t="str">
-        <x:v>ej avdragsgill representation|kundmiddag|måltid|skattemässig återläggning|NE sid 2|R6</x:v>
+        <x:v>representation|extern representation|kundmåltid|deltagarförteckning|R6</x:v>
       </x:c>
       <x:c r="K135" s="14" t="str">
-        <x:v>6070|6071|2641|2013|7632</x:v>
+        <x:v>6071|6072|5900|7631|7632|2641</x:v>
       </x:c>
       <x:c r="L135" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 6072, rad R6 och NE sidan 2|Skatteverket – Belopp och procent 2026 samt Representation, kontrollerat 2026-07-30|Skatteverket – Avdrag för moms vid representation, kontrollerat 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 6070 och underkonton, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Belopp och procent 2026 samt Representation, kontrollerat 2026-07-30|Skatteverket – Avdrag för moms vid representation, kontrollerat 2026-07-30</x:v>
       </x:c>
       <x:c r="M135" s="14" t="str">
-        <x:v>Privat kostnad kan förekomma|Momsfördelning mellan mat och alkohol är oklar|Deltagare eller affärssyfte saknas|Intern representation kan vara rätt|Kostnaden kan innehålla en avdragsgill del|Kvitto, deltagare eller beräkning saknas</x:v>
+        <x:v>Deltagare, syfte eller affärssamband saknas|Alkohol, gåva, familjemedlem eller privat inslag förekommer|Intern representation kan vara rätt klassificering|Kostnaden ska delas mellan 6071 och 6072|Momsfördelningen är oklar|Affärssamband eller representationstyp är oklar</x:v>
       </x:c>
       <x:c r="N135" s="14" t="str">
         <x:v>active</x:v>
@@ -7499,49 +7499,49 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="P135" s="14" t="str">
-        <x:v>representation_meal_income_deduction_zero_2026|representation_meal_vat_base_2026</x:v>
+        <x:v>representation_meal_income_deduction_zero_2026|representation_simple_refreshment_limit_2026|representation_other_expense_limit_2026|representation_meal_vat_base_2026|representation_gift_limit_2026</x:v>
       </x:c>
       <x:c r="Q135" s="12" t="str"/>
     </x:row>
     <x:row r="136" ht="430" customHeight="1">
       <x:c r="A136" s="14" t="str">
-        <x:v>6100</x:v>
+        <x:v>6071</x:v>
       </x:c>
       <x:c r="B136" s="14" t="str">
-        <x:v>Kontorsmateriel och trycksaker</x:v>
+        <x:v>Representation, avdragsgill</x:v>
       </x:c>
       <x:c r="C136" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för kontorsförbrukning och trycksaker, exempelvis papper, toner, kuvert, blanketter och enklare förbrukningsartiklar för administration.</x:v>
+        <x:v>Kostnadskonto på R6 för den del av extern representation som är avdragsgill vid inkomstbeskattningen enligt aktuell belopps- och sambandsregel.</x:v>
       </x:c>
       <x:c r="D136" s="14" t="str">
-        <x:v>Inköpet förbrukas i kontors- eller administrationsarbetet|Föremålet har lågt värde och är inte en självständig inventarie|Trycksaken används internt eller som normalt administrativt material</x:v>
+        <x:v>Representationen har omedelbart samband med verksamheten|Utgiften avser enklare förtäring inom 60 kronor exklusive moms per person|Utgiften avser avdragsgill kringaktivitet inom 180 kronor exklusive moms per person|En representationsgåva uppfyller villkoren och ryms inom 300 kronor exklusive moms</x:v>
       </x:c>
       <x:c r="E136" s="14" t="str">
-        <x:v>Inköpet är dator, skrivare, möbel eller annan inventarie; pröva 5400 eller 1220|Trycksaken är huvudsakligen reklam- eller kampanjmaterial; använd 5900|Materialet säljs vidare eller ingår direkt i kundens leverans; använd 4000|Beloppet avser abonnemang, programvara eller extern tjänst|Inköpet är privat</x:v>
+        <x:v>Utgiften avser frukost, lunch, middag eller annan måltid som inte är enklare förtäring; inkomstskattemässigt avdrag är 0 kronor|Beloppet överstiger avdragsramen; överskjutande del bokförs på 6072|Affärssamband, deltagare eller syfte saknas|Aktiviteten är intern representation|Utgiften är privat, gåva utan representationssamband eller reklam</x:v>
       </x:c>
       <x:c r="F136" s="14" t="str">
-        <x:v>Identifiera artikel, antal, användning och om föremålen har naturligt samband|Skilj förbrukningsmaterial från inventarie och handelsvara|Bokför kostnaden exklusive avdragsgill ingående moms|Pröva 5400 eller 1220 för utrustning med självständig funktion och längre användning|Pröva 5900 för broschyrer och trycksaker med huvudsakligt marknadsföringssyfte|Koppla fakturan till kontor eller verksamhetsdel vid behov|Stäm av större eller återkommande inköp mot inventariereglerna|Kräv manuell granskning för större skrivare, specialutrustning eller paketköp|Använd för mindre administrativt förbrukningsmaterial|Klassificera trycksak efter administrativt eller reklamändamål|Vid granskningsflagga begär in faktura med artikelspecifikation och uppgift om användningsområde|Sätt ärendet till väntar på underlag tills förbrukningsmaterial kan skiljas från inventarie, handelsvara och reklam|Godkänn 6100 för mindre administrativt förbrukningsmaterial och vanliga trycksaker|Föreslå 5400, 1220, 4000 eller 5900 när inköpet i stället är utrustning, tillgång, handelsvara eller reklam</x:v>
+        <x:v>Verifiera extern representation och omedelbart samband med verksamheten|Klassificera utgiften som enklare förtäring, måltid, kringkostnad eller representationsgåva|Beräkna avdragsram per person och tillfälle med versionsstyrd parameter|Bokför endast den inkomstskattemässigt avdragsgilla delen på 6071|Bokför överskjutande eller helt ej avdragsgill kostnadsdel på 6072|Beräkna ingående moms separat enligt momsregeln|Kräv kvitto eller faktura, deltagarlista, syfte, ort och datum|Stäm av belopp per deltagare och mot 6072|Kräv manuell granskning vid gåva, alkohol eller blandade utgiftsslag|Använd endast efter klassificering av enklare förtäring, måltid eller representationsgåva|Koppla till deltagarlista och affärssyfte|Vid granskningsflagga begär in kvitto eller faktura, deltagarlista, datum, plats och affärssyfte|Sätt ärendet till väntar på underlag tills representationstyp, aktuell avdragsram och momsberäkning är verifierade|Godkänn 6071 endast för den dokumenterade inkomstskattemässigt avdragsgilla delen|Föreslå 6072, privat kostnad eller eskalering för överskjutande belopp, saknat samband eller oklar gåva och alkohol</x:v>
       </x:c>
       <x:c r="G136" s="14" t="str">
-        <x:v>2440|1930|2641|5400|1220</x:v>
+        <x:v>2440|1930|2641|6072</x:v>
       </x:c>
       <x:c r="H136" s="14" t="str">
-        <x:v>Kopieringspapper och toner bokförs på 6100|En ny skrivare prövas som förbrukningsinventarie eller anläggningstillgång</x:v>
+        <x:v>Kaffe och enklare smörgås för 55 kronor exklusive moms per kund kan bokföras på 6071 när sambands- och dokumentationskraven är uppfyllda|En kundmiddag bokförs inte som avdragsgill måltidskostnad på 6071</x:v>
       </x:c>
       <x:c r="I136" s="14" t="str">
-        <x:v>Kontorsmaterial och kontorsinventarie är olika kategorier|Marknadsföringstryck hör normalt till 5900|Flera delar med naturligt samband får inte delas för att undvika aktivering|Privata kontorsinköp får inte belasta verksamheten|Dator, telefon, skrivare, möbel och utrustningspaket ska prövas mot 5400 eller 1220</x:v>
+        <x:v>En måltid är inte enklare förtäring|Om enklare förtäring överstiger 60 kronor kan hela beloppet bli ej avdragsgillt enligt regeln|Momsavdraget beräknas separat|Avdragsramarna gäller per person och tillfälle|Reklamgåva och vanlig gåva ska inte bokföras här</x:v>
       </x:c>
       <x:c r="J136" s="14" t="str">
-        <x:v>kontorsmateriel|papper|toner|kuvert|trycksaker|blanketter|R6</x:v>
+        <x:v>avdragsgill representation|enklare förtäring|kringkostnad|representationsgåva|R6</x:v>
       </x:c>
       <x:c r="K136" s="14" t="str">
-        <x:v>5400|1220|4000|5900|2440|2641</x:v>
+        <x:v>6070|6072|2641|5900|7631</x:v>
       </x:c>
       <x:c r="L136" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6100, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.29–6.36 och 7.5–7.7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 6071, rad R6|Skatteverket – Belopp och procent 2026 samt Representation, kontrollerat 2026-07-30|Skatteverket – Avdrag för moms vid representation, kontrollerat 2026-07-30</x:v>
       </x:c>
       <x:c r="M136" s="14" t="str">
-        <x:v>Föremålet kan vara inventarie eller handelsvara|Trycksaken kan vara reklam|Paketköp eller större utrustning förekommer|Användningen är privat eller blandad|Momsavdragsrätten är oklar|Värde, livslängd, naturligt samband eller användningssyfte är oklart</x:v>
+        <x:v>Beloppet ligger nära eller över en avdragsram|Måltid, alkohol eller gåva förekommer|Deltagarantal eller affärssamband saknas|Intern representation kan vara rätt|Flera utgiftsslag eller momssatser ingår|Måltidstyp, gåvotyp eller avdragsram är oklar</x:v>
       </x:c>
       <x:c r="N136" s="14" t="str">
         <x:v>active</x:v>
@@ -7550,49 +7550,49 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="P136" s="14" t="str">
-        <x:v>low_value_inventory_half_pbb|economic_life_max_3_years</x:v>
+        <x:v>representation_simple_refreshment_limit_2026|representation_other_expense_limit_2026|representation_gift_limit_2026|representation_meal_vat_base_2026</x:v>
       </x:c>
       <x:c r="Q136" s="12" t="str"/>
     </x:row>
     <x:row r="137" ht="430" customHeight="1">
       <x:c r="A137" s="14" t="str">
-        <x:v>6200</x:v>
+        <x:v>6072</x:v>
       </x:c>
       <x:c r="B137" s="14" t="str">
-        <x:v>Tele och post</x:v>
+        <x:v>Representation, ej avdragsgill</x:v>
       </x:c>
       <x:c r="C137" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för telefon-, internet-, porto- och kommunikationstjänster som används i näringsverksamheten.</x:v>
+        <x:v>Kostnadskonto på R6 för den del av extern representation som inte är avdragsgill vid inkomstbeskattningen. Kontot är markerat för skattemässig återläggning i NE-bilagan.</x:v>
       </x:c>
       <x:c r="D137" s="14" t="str">
-        <x:v>Kostnaden avser verksamhetens telefon- eller internetabonnemang|Utgiften avser porto, postbox, brev- eller paketadministration som inte är frakttjänst på 5700|Verksamhetsandelen och underlaget kan verifieras</x:v>
+        <x:v>Utgiften är en affärsmässigt motiverad representationskostnad men saknar helt eller delvis inkomstskattemässigt avdrag|Utgiften avser frukost, lunch, middag eller annan måltid med 0 kronor i inkomstskattemässigt avdrag|Beloppet överstiger avdragsramen på 6071|Ej avdragsgill moms ska ingå i kostnaden</x:v>
       </x:c>
       <x:c r="E137" s="14" t="str">
-        <x:v>Inköpet är telefon, dator, router eller annan utrustning; pröva 5400 eller 1220|Kostnaden är frakt eller transport av varor; använd 5700|Abonnemanget eller samtalet är privat utan företagsandel|Tjänsten är programvara, molntjänst eller konsulttjänst; pröva 6500|Utgiften vidarefaktureras eller är äkta utlägg utan utredd behandling</x:v>
+        <x:v>Utgiften är privat och saknar samband med verksamheten; bokför som eget uttag i stället|Utgiften är avdragsgill och ryms inom 6071|Aktiviteten är intern personalrepresentation|Utgiften är reklam eller sponsring med verifierad motprestation|Underlag och affärssyfte saknas helt</x:v>
       </x:c>
       <x:c r="F137" s="14" t="str">
-        <x:v>Identifiera abonnemang, användare, period, leverantör och tjänst|Skilj abonnemang och trafik från inköp eller avbetalning av utrustning|För privat abonnemang som används i verksamheten: beräkna och dokumentera ett skäligt avdrag för verksamhetsdelen|För företagsabonnemang med privat användning: identifiera och hantera privat del enligt tillämplig uttagsregel|Bokför avdragsgill ingående moms endast för verksamhetsdelen|Skilj porto från frakt, kurir och distribution|Stäm av bindningstid, förskottsbetalning och kreditnotor|Kräv manuell granskning vid familjeabonnemang, telefonpaket, utlandstrafik eller privat betalning|Bokför endast verifierad företagsandel av telefon och internet|Spara abonnent, tjänst, total kostnad, andel, grund och period|Dela paketfaktura radvis|Vid granskningsflagga begär in fullständig faktura med abonnent, period, tjänst, utrustningsdel och eventuell privat andel|Sätt ärendet till väntar på underlag tills verksamhetsandel och eventuell utlands- eller momsbehandling är verifierad|Godkänn 6200 för dokumenterad telefon, internet och porto som hör till verksamheten|Föreslå uppdelning, 5400, 1220, 5700, 6500 eller privat kostnad när fakturan innehåller utrustning, frakt, molntjänst eller privat del</x:v>
+        <x:v>Verifiera att utgiften trots ej avdragsgill status hör till en faktisk affärshändelse i verksamheten|Klassificera representationstyp och beräkna avdragsgill del på 6071|Bokför resterande kostnad och ej avdragsgill moms på 6072|För måltider är inkomstskattemässigt avdrag 0 kronor men momsavdrag kan finnas på ett underlag om högst 300 kronor exklusive moms per person och tillfälle|Beräkna moms efter faktisk fördelning mellan mat och alkohol när sådan uppdelning finns|Märk kontot för skattemässig återläggning i NE-underlaget|Kräv deltagarlista, syfte, datum och plats även för ej avdragsgill representation|Separera privat del som eget uttag|Kräv manuell granskning vid alkohol, familjemedlem, gåva eller oskäligt belopp|Använd för ej avdragsgill del efter dokumenterad representationsbedömning|Beräkna mat, alkohol, momssatser och personbelopp separat|Vid granskningsflagga begär in kvitto eller faktura, deltagarlista, datum, plats, affärssyfte och momsuppdelning|Sätt ärendet till väntar på underlag tills den faktiska representationen och eventuell privat eller avdragsgill del är verifierad|Godkänn 6072 för den dokumenterade ej avdragsgilla representationsdelen och markera skattemässig återläggning|Föreslå 6071, eget uttag eller eskalering när posten innehåller avdragsgill del, privat kostnad eller oklar moms</x:v>
       </x:c>
       <x:c r="G137" s="14" t="str">
-        <x:v>2440|1930|2641|2013|2018|5400|1220</x:v>
+        <x:v>2440|1930|2641|6071|2013</x:v>
       </x:c>
       <x:c r="H137" s="14" t="str">
-        <x:v>Ett separat företagsabonnemang bokförs på 6200 med verksamhetsrelaterad moms|Ett privat mobilabonnemang som används delvis i firman ger endast ett dokumenterat skäligt avdrag för företagsdelen</x:v>
+        <x:v>En kundmiddag bokförs på 6072 exklusive den del av ingående moms som får dras av enligt representationsmomsregeln|Privat middag utan affärssamband bokförs inte på 6072 utan som eget uttag</x:v>
       </x:c>
       <x:c r="I137" s="14" t="str">
-        <x:v>Privat och företagsmässig användning måste fördelas|Telefonutrustning och abonnemang ska skiljas åt|Utländska tele- och molntjänster kan medföra omvänd moms|Porto och varufrakt hör inte alltid till samma konto|Privat eller familjeabonnemang är inte automatiskt fullt avdragsgillt</x:v>
+        <x:v>Ej avdragsgill betyder inte att dokumentationskraven försvinner|Privat kostnad får inte döljas som ej avdragsgill representation|Begränsat momsavdrag kan finnas trots 0 kronor i inkomstskattemässigt måltidsavdrag|Kontot ska återläggas skattemässigt|Momsavdrag och inkomstskatteavdrag följer inte samma gräns</x:v>
       </x:c>
       <x:c r="J137" s="14" t="str">
-        <x:v>telefon|mobilabonnemang|internet|bredband|porto|postbox|R6</x:v>
+        <x:v>ej avdragsgill representation|kundmiddag|måltid|skattemässig återläggning|NE sid 2|R6</x:v>
       </x:c>
       <x:c r="K137" s="14" t="str">
-        <x:v>5400|1220|5700|6500|2013|2018|2440|2641</x:v>
+        <x:v>6070|6071|2641|2013|7632</x:v>
       </x:c>
       <x:c r="L137" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6200, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7|Skatteverkets rättsliga vägledning 2026 – Utgifter för dator och telefon i enskild näringsverksamhet</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 6, konto 6072, rad R6 och NE sidan 2|Skatteverket – Belopp och procent 2026 samt Representation, kontrollerat 2026-07-30|Skatteverket – Avdrag för moms vid representation, kontrollerat 2026-07-30</x:v>
       </x:c>
       <x:c r="M137" s="14" t="str">
-        <x:v>Privat abonnemang eller familjeabonnemang används|Utrustning och abonnemang är paketerade|Verksamhetsandelen saknas|Utlandstjänst eller omvänd moms förekommer|Tjänsten kan vara moln- eller programvarutjänst|Fördelningsgrund, utrustningsdel eller utlandstjänst är oklar</x:v>
+        <x:v>Privat kostnad kan förekomma|Momsfördelning mellan mat och alkohol är oklar|Deltagare eller affärssyfte saknas|Intern representation kan vara rätt|Kostnaden kan innehålla en avdragsgill del|Kvitto, deltagare eller beräkning saknas</x:v>
       </x:c>
       <x:c r="N137" s="14" t="str">
         <x:v>active</x:v>
@@ -7600,97 +7600,101 @@
       <x:c r="O137" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P137" s="14"/>
+      <x:c r="P137" s="14" t="str">
+        <x:v>representation_meal_income_deduction_zero_2026|representation_meal_vat_base_2026</x:v>
+      </x:c>
       <x:c r="Q137" s="12" t="str"/>
     </x:row>
     <x:row r="138" ht="430" customHeight="1">
       <x:c r="A138" s="14" t="str">
-        <x:v>6300</x:v>
+        <x:v>6100</x:v>
       </x:c>
       <x:c r="B138" s="14" t="str">
-        <x:v>Företagsförsäkringar och övriga riskkostnader</x:v>
+        <x:v>Kontorsmateriel och trycksaker</x:v>
       </x:c>
       <x:c r="C138" s="14" t="str">
-        <x:v>Huvud- eller samlingskonto på R6 för försäkringspremier och andra verifierade riskkostnader i verksamheten. Företagsförsäkringspremier bör normalt särredovisas på 6310.</x:v>
+        <x:v>Kostnadskonto på R6 för kontorsförbrukning och trycksaker, exempelvis papper, toner, kuvert, blanketter och enklare förbrukningsartiklar för administration.</x:v>
       </x:c>
       <x:c r="D138" s="14" t="str">
-        <x:v>Utgiften avser en verifierad riskkostnad i näringsverksamheten|Kostnaden gäller avdragsgillt skadestånd, faktisk garantikostnad, bevakning eller larm|Risk, händelse, period, motpart och verksamhetsanknytning är dokumenterade|Ingen mer specifik tillåten kontogrupp beskriver kostnaden bättre</x:v>
+        <x:v>Inköpet förbrukas i kontors- eller administrationsarbetet|Föremålet har lågt värde och är inte en självständig inventarie|Trycksaken används internt eller som normalt administrativt material</x:v>
       </x:c>
       <x:c r="E138" s="14" t="str">
-        <x:v>Utgiften är en vanlig företagsförsäkringspremie; använd normalt 6310|Försäkringen eller risken är privat|Beloppet avser bil-, fastighets- eller annan kostnad med mer specifikt konto|Beloppet avser kundförlust, annan fordringsförlust, självrisk, förlust i pågående arbete eller skadestånd utan verifierad klassificering|Beloppet avser förändring av garantiavsättning; BAS 6361 ligger utanför tjänstens scope|Kontot används som ospecificerat restkonto</x:v>
+        <x:v>Inköpet är dator, skrivare, möbel eller annan inventarie; pröva 5400 eller 1220|Trycksaken är huvudsakligen reklam- eller kampanjmaterial; använd 5900|Materialet säljs vidare eller ingår direkt i kundens leverans; använd 4000|Beloppet avser abonnemang, programvara eller extern tjänst|Inköpet är privat</x:v>
       </x:c>
       <x:c r="F138" s="14" t="str">
-        <x:v>Identifiera kostnadstyp, händelse, motpart, period och verksamhetssamband|Pröva 6310 för ordinarie företagsförsäkringspremier|Pröva mer specifikt fordons-, fastighets-, tillgångs- eller fordringskonto när kostnaden hör dit|BAS 6341 får sammanföras automatiskt endast när skadeståndets avdragsrätt framgår av den valda BAS-underkategorin och underlaget stödjer klassificeringen|BAS 6362 får sammanföras automatiskt när kostnaden är en faktisk, verifierad garantikostnad och inte en avsättning|BAS 6370 får sammanföras automatiskt när kostnaden avser bevakning eller larm i verksamheten|BAS 6300 och 6390 kräver specificerad riskkategori före sammanföring|BAS 6320 kräver kontroll av skada, försäkrat objekt, privat inslag och avdragsrätt|BAS 6330 kräver kontroll mot pågående arbete, värdering och periodens resultat|BAS 6340 och 6342 kräver kontroll av händelse och avdragsrätt|BAS 6350, 6351 och 6352 kräver kontroll av kundfordran, värdering och eventuell momshantering|BAS 6360 kräver uppdelning mellan faktisk garantikostnad och garantiavsättning|BAS 6361 förändring av garantiavsättning ligger utanför tjänstens scope|BAS 6380 kräver identifiering och värdering av den underliggande kortfristiga fordran|Skilj premie, självrisk, skadestånd, garanti, fordringsförlust och försäkringsersättning|Bokför eventuell förutbetald del endast enligt K1:s förenklingsregler|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
+        <x:v>Identifiera artikel, antal, användning och om föremålen har naturligt samband|Skilj förbrukningsmaterial från inventarie och handelsvara|Bokför kostnaden exklusive avdragsgill ingående moms|Pröva 5400 eller 1220 för utrustning med självständig funktion och längre användning|Pröva 5900 för broschyrer och trycksaker med huvudsakligt marknadsföringssyfte|Koppla fakturan till kontor eller verksamhetsdel vid behov|Stäm av större eller återkommande inköp mot inventariereglerna|Kräv manuell granskning för större skrivare, specialutrustning eller paketköp|Använd för mindre administrativt förbrukningsmaterial|Klassificera trycksak efter administrativt eller reklamändamål|Vid granskningsflagga begär in faktura med artikelspecifikation och uppgift om användningsområde|Sätt ärendet till väntar på underlag tills förbrukningsmaterial kan skiljas från inventarie, handelsvara och reklam|Godkänn 6100 för mindre administrativt förbrukningsmaterial och vanliga trycksaker|Föreslå 5400, 1220, 4000 eller 5900 när inköpet i stället är utrustning, tillgång, handelsvara eller reklam</x:v>
       </x:c>
       <x:c r="G138" s="14" t="str">
-        <x:v>2440|1930|1700|6310|6900</x:v>
+        <x:v>2440|1930|2641|5400|1220</x:v>
       </x:c>
       <x:c r="H138" s="14" t="str">
-        <x:v>Kostnad för bevakning eller larm i verksamhetens lokaler bokförs på 6300 när underlaget är tydligt|En faktisk reparationskostnad som omfattas av lämnad garanti bokförs på 6300 när den kan verifieras och ingen avsättning används|Ett avdragsgillt skadestånd med dokumenterad affärshändelse kan bokföras på 6300|En vanlig ansvarsförsäkringspremie bokförs normalt på 6310|En kundförlust granskas separat och får inte automatiskt döljas som allmän riskkostnad</x:v>
+        <x:v>Kopieringspapper och toner bokförs på 6100|En ny skrivare prövas som förbrukningsinventarie eller anläggningstillgång</x:v>
       </x:c>
       <x:c r="I138" s="14" t="str">
-        <x:v>6300 får inte bli ett restkonto|Ordinarie företagsförsäkringspremier bör normalt särredovisas på 6310|Privata personförsäkringar är inte automatiskt avdragsgilla i firman|Försäkringsersättning och premie är olika händelser|Självrisk, skadestånd och fordringsförlust kräver dokumenterad klassificering|Ej avdragsgilla skadestånd får inte behandlas som avdragsgill kostnad|Garantiavsättning får inte sammanblandas med faktisk garantikostnad|Mer specifika tillgångs-, fordons- och fordringskonton ska användas när möjligt</x:v>
+        <x:v>Kontorsmaterial och kontorsinventarie är olika kategorier|Marknadsföringstryck hör normalt till 5900|Flera delar med naturligt samband får inte delas för att undvika aktivering|Privata kontorsinköp får inte belasta verksamheten|Dator, telefon, skrivare, möbel och utrustningspaket ska prövas mot 5400 eller 1220</x:v>
       </x:c>
       <x:c r="J138" s="14" t="str">
-        <x:v>riskkostnad|företagsförsäkring|självrisk|försäkringsrisk|R6</x:v>
+        <x:v>kontorsmateriel|papper|toner|kuvert|trycksaker|blanketter|R6</x:v>
       </x:c>
       <x:c r="K138" s="14" t="str">
-        <x:v>6310|5612|5100|6900|3900|1700</x:v>
+        <x:v>5400|1220|4000|5900|2440|2641</x:v>
       </x:c>
       <x:c r="L138" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6300, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.59 och 7.5–7.7|Skatteverket – Avdragslexikon för företag, Försäkringar, kontrollerat 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6100, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.29–6.36 och 7.5–7.7</x:v>
       </x:c>
       <x:c r="M138" s="14" t="str">
-        <x:v>Försäkringens eller riskens art är oklar|Personförsäkring, pension eller privat risk förekommer|Posten kommer från BAS 6300, 6320, 6330, 6340, 6342, 6350, 6351, 6352, 6360, 6380 eller 6390|Självrisk, skadestånd, kundförlust eller annan fordringsförlust kan vara rätt klassificering|Pågående arbete eller värdering av fordran påverkas|Avdragsrätt eller momshantering är oklar|Mer specifikt konto finns|Periodisering kan vara aktuell</x:v>
+        <x:v>Föremålet kan vara inventarie eller handelsvara|Trycksaken kan vara reklam|Paketköp eller större utrustning förekommer|Användningen är privat eller blandad|Momsavdragsrätten är oklar|Värde, livslängd, naturligt samband eller användningssyfte är oklart</x:v>
       </x:c>
       <x:c r="N138" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O138" s="14" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P138" s="14"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P138" s="14" t="str">
+        <x:v>low_value_inventory_half_pbb|economic_life_max_3_years</x:v>
+      </x:c>
       <x:c r="Q138" s="12" t="str"/>
     </x:row>
     <x:row r="139" ht="430" customHeight="1">
       <x:c r="A139" s="14" t="str">
-        <x:v>6310</x:v>
+        <x:v>6200</x:v>
       </x:c>
       <x:c r="B139" s="14" t="str">
-        <x:v>Företagsförsäkringar</x:v>
+        <x:v>Tele och post</x:v>
       </x:c>
       <x:c r="C139" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för premier på försäkringar som har tecknats för näringsverksamheten, exempelvis ansvars-, avbrotts- och sakförsäkring för verksamhetens tillgångar.</x:v>
+        <x:v>Kostnadskonto på R6 för telefon-, internet-, porto- och kommunikationstjänster som används i näringsverksamheten.</x:v>
       </x:c>
       <x:c r="D139" s="14" t="str">
-        <x:v>Försäkringen är tecknad för verksamheten|Premien avser ansvar, avbrott, egendom eller annan företagsrisk|Försäkringsbrev, period och försäkrade objekt är dokumenterade</x:v>
+        <x:v>Kostnaden avser verksamhetens telefon- eller internetabonnemang|Utgiften avser porto, postbox, brev- eller paketadministration som inte är frakttjänst på 5700|Verksamhetsandelen och underlaget kan verifieras</x:v>
       </x:c>
       <x:c r="E139" s="14" t="str">
-        <x:v>Försäkringen avser privat bostad, privat egendom eller privat levnadskostnad|Premien avser personbil och ska följas på 5612|Premien avser sjuk- eller olycksfallsförsäkring som inte är avdragsgill för näringsidkaren enligt aktuell regel|Beloppet är pensionsförsäkring, gruppliv eller annan personförsäkring utan särskild bedömning|Beloppet är självrisk eller försäkringsersättning</x:v>
+        <x:v>Inköpet är telefon, dator, router eller annan utrustning; pröva 5400 eller 1220|Kostnaden är frakt eller transport av varor; använd 5700|Abonnemanget eller samtalet är privat utan företagsandel|Tjänsten är programvara, molntjänst eller konsulttjänst; pröva 6500|Utgiften vidarefaktureras eller är äkta utlägg utan utredd behandling</x:v>
       </x:c>
       <x:c r="F139" s="14" t="str">
-        <x:v>Verifiera försäkringstagare, försäkrad risk, objekt, period och verksamhetssamband|Kontrollera om premien normalt är avdragsgill därför att den avser näringsverksamheten och eventuell ersättning är hänförlig till verksamheten|Skilj företagsförsäkring från privat personförsäkring och pensionskostnad|Bokför premien på 6310 och eventuell avdragsgill moms endast om sådan har debiterats|Hantera förutbetald premie enligt K1 punkt 6.59 när villkoren är uppfyllda|Koppla premien till försäkringsbrev och förfalloperiod|Stäm av återbetalning och uppsägning|Kräv manuell granskning för sjukvård, olycksfall, gruppliv, reseskydd eller försäkring med privat del|Kräv försäkringsbolag, typ, objekt, period, premie och privat andel|Koppla återbetalning till ursprunglig premie|Följ verifierad periodiseringsrutin|Vid granskningsflagga begär in försäkringsbrev med försäkringstagare, försäkringstyp, objekt, period och premie|Sätt ärendet till väntar på underlag tills verksamhetskoppling, privat andel och period är verifierade|Godkänn 6310 när premien avser en vanlig försäkring för verksamhetens risker eller tillgångar|Föreslå 5612, privat kostnad, periodiseringsrutin eller eskalering när försäkringen avser bil, person, pension eller oklar privat del</x:v>
+        <x:v>Identifiera abonnemang, användare, period, leverantör och tjänst|Skilj abonnemang och trafik från inköp eller avbetalning av utrustning|För privat abonnemang som används i verksamheten: beräkna och dokumentera ett skäligt avdrag för verksamhetsdelen|För företagsabonnemang med privat användning: identifiera och hantera privat del enligt tillämplig uttagsregel|Bokför avdragsgill ingående moms endast för verksamhetsdelen|Skilj porto från frakt, kurir och distribution|Stäm av bindningstid, förskottsbetalning och kreditnotor|Kräv manuell granskning vid familjeabonnemang, telefonpaket, utlandstrafik eller privat betalning|Bokför endast verifierad företagsandel av telefon och internet|Spara abonnent, tjänst, total kostnad, andel, grund och period|Dela paketfaktura radvis|Vid granskningsflagga begär in fullständig faktura med abonnent, period, tjänst, utrustningsdel och eventuell privat andel|Sätt ärendet till väntar på underlag tills verksamhetsandel och eventuell utlands- eller momsbehandling är verifierad|Godkänn 6200 för dokumenterad telefon, internet och porto som hör till verksamheten|Föreslå uppdelning, 5400, 1220, 5700, 6500 eller privat kostnad när fakturan innehåller utrustning, frakt, molntjänst eller privat del</x:v>
       </x:c>
       <x:c r="G139" s="14" t="str">
-        <x:v>2440|1930|1700|6300</x:v>
+        <x:v>2440|1930|2641|2013|2018|5400|1220</x:v>
       </x:c>
       <x:c r="H139" s="14" t="str">
-        <x:v>Premie för verksamhetens ansvarsförsäkring bokförs på 6310|Privat sjuk- och olycksfallsförsäkring bokförs inte automatiskt som företagskostnad</x:v>
+        <x:v>Ett separat företagsabonnemang bokförs på 6200 med verksamhetsrelaterad moms|Ett privat mobilabonnemang som används delvis i firman ger endast ett dokumenterat skäligt avdrag för företagsdelen</x:v>
       </x:c>
       <x:c r="I139" s="14" t="str">
-        <x:v>Försäkringens namn avgör inte ensam avdragsrätten|Personförsäkringar har särskilda regler|Fordon och fastighet kan kräva mer specifikt konto|Försäkringsersättningar redovisas separat|Privat sjuk-, olycksfalls-, liv- eller pensionsförsäkring är inte vanlig företagsförsäkring</x:v>
+        <x:v>Privat och företagsmässig användning måste fördelas|Telefonutrustning och abonnemang ska skiljas åt|Utländska tele- och molntjänster kan medföra omvänd moms|Porto och varufrakt hör inte alltid till samma konto|Privat eller familjeabonnemang är inte automatiskt fullt avdragsgillt</x:v>
       </x:c>
       <x:c r="J139" s="14" t="str">
-        <x:v>företagsförsäkring|ansvarsförsäkring|avbrottsförsäkring|sakförsäkring|premie|R6</x:v>
+        <x:v>telefon|mobilabonnemang|internet|bredband|porto|postbox|R6</x:v>
       </x:c>
       <x:c r="K139" s="14" t="str">
-        <x:v>6300|5612|5100|6900|3900|1700</x:v>
+        <x:v>5400|1220|5700|6500|2013|2018|2440|2641</x:v>
       </x:c>
       <x:c r="L139" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6310, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.59 och 7.5–7.7|Skatteverket – Avdragslexikon för företag, Försäkringar, kontrollerat 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6200, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 2.4, 3.18 och 7.5–7.7|Skatteverkets rättsliga vägledning 2026 – Utgifter för dator och telefon i enskild näringsverksamhet</x:v>
       </x:c>
       <x:c r="M139" s="14" t="str">
-        <x:v>Försäkringen kan vara privat eller en personförsäkring|Försäkringsobjekt eller period saknas|Återbetalning, självrisk eller ersättning förekommer|Mer specifikt kostnadskonto kan vara rätt|Avdragsrätten är särskilt reglerad|Försäkringstyp, privat andel eller periodisering är oklar</x:v>
+        <x:v>Privat abonnemang eller familjeabonnemang används|Utrustning och abonnemang är paketerade|Verksamhetsandelen saknas|Utlandstjänst eller omvänd moms förekommer|Tjänsten kan vara moln- eller programvarutjänst|Fördelningsgrund, utrustningsdel eller utlandstjänst är oklar</x:v>
       </x:c>
       <x:c r="N139" s="14" t="str">
         <x:v>active</x:v>
@@ -7703,92 +7707,92 @@
     </x:row>
     <x:row r="140" ht="430" customHeight="1">
       <x:c r="A140" s="14" t="str">
-        <x:v>6500</x:v>
+        <x:v>6300</x:v>
       </x:c>
       <x:c r="B140" s="14" t="str">
-        <x:v>Övriga externa tjänster</x:v>
+        <x:v>Företagsförsäkringar och övriga riskkostnader</x:v>
       </x:c>
       <x:c r="C140" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för köpta konsult-, redovisnings-, juridik-, IT- och andra externa tjänster som inte är underentreprenad, inhyrd personal eller en tjänst med mer specifikt konto.</x:v>
+        <x:v>Huvud- eller samlingskonto på R6 för försäkringspremier och andra verifierade riskkostnader i verksamheten. Företagsförsäkringspremier bör normalt särredovisas på 6310.</x:v>
       </x:c>
       <x:c r="D140" s="14" t="str">
-        <x:v>En extern leverantör utför en avgränsad administrativ, rådgivande eller specialisttjänst|Tjänsten stödjer verksamheten men är inte direkt del av produktionen på 4600|Leverantören ansvarar för tjänstens resultat och är inte inhyrd under företagets arbetsledning</x:v>
+        <x:v>Utgiften avser en verifierad riskkostnad i näringsverksamheten|Kostnaden gäller avdragsgillt skadestånd, faktisk garantikostnad, bevakning eller larm|Risk, händelse, period, motpart och verksamhetsanknytning är dokumenterade|Ingen mer specifik tillåten kontogrupp beskriver kostnaden bättre</x:v>
       </x:c>
       <x:c r="E140" s="14" t="str">
-        <x:v>Tjänsten är underentreprenad direkt i kundens leverans; använd 4600|Personen ställs till företagets förfogande och leds som personal; använd 6800|Utgiften gäller reklam, tele, försäkring, resa eller annan mer specifik tjänst|Köpet ger en separat rättighet, programvara, webbplats eller annan tillgång som ska aktiveras|Avgiften är en ren medlemsavgift eller en blandad medlems- och serviceavgift där tjänstedelen inte framgår; skicka till manuell granskning</x:v>
+        <x:v>Utgiften är en vanlig företagsförsäkringspremie; använd normalt 6310|Försäkringen eller risken är privat|Beloppet avser bil-, fastighets- eller annan kostnad med mer specifikt konto|Beloppet avser kundförlust, annan fordringsförlust, självrisk, förlust i pågående arbete eller skadestånd utan verifierad klassificering|Beloppet avser förändring av garantiavsättning; BAS 6361 ligger utanför tjänstens scope|Kontot används som ospecificerat restkonto</x:v>
       </x:c>
       <x:c r="F140" s="14" t="str">
-        <x:v>Identifiera leverantör, avtal, leverans, ansvar för resultat och period|Skilj specialist- och konsulttjänst för den egna verksamheten från underentreprenad på 4600 och inhyrd personal på 6800|Använd ett mer specifikt kostnadskonto när tjänstens art omfattas av ett sådant konto|Kontrollera F-skatt när ersättningen avser arbete; om F-skatt saknas ska ärendet granskas med avseende på skatteavdrag, arbetsgivaravgifter och eventuell anställningsrelation|För utländsk leverantör: kontrollera beskattningsland, omvänd moms och eventuell skyldighet att göra skatteavdrag för arbete i Sverige|Bokför kostnaden exklusive avdragsgill moms|Pröva om köpet skapar en identifierbar tillgång eller ska ingå i en annan tillgångs anskaffningsvärde|Koppla kostnaden till avtal, projekt och leverans och stäm av förskott, leverantörsskuld och kreditnota|Periodisera tjänsten när betalnings- och leveransperioden inte sammanfaller enligt tillämplig K1-regel|Bankkostnader kan redovisas på 6500 när ett mer specifikt konto saknas|För serviceavgift till branschorganisation: verifiera att avgiften avser en identifierbar tjänst; ren medlemsavgift eller oklar blandad avgift kräver manuell granskning</x:v>
+        <x:v>Identifiera kostnadstyp, händelse, motpart, period och verksamhetssamband|Pröva 6310 för ordinarie företagsförsäkringspremier|Pröva mer specifikt fordons-, fastighets-, tillgångs- eller fordringskonto när kostnaden hör dit|BAS 6341 får sammanföras automatiskt endast när skadeståndets avdragsrätt framgår av den valda BAS-underkategorin och underlaget stödjer klassificeringen|BAS 6362 får sammanföras automatiskt när kostnaden är en faktisk, verifierad garantikostnad och inte en avsättning|BAS 6370 får sammanföras automatiskt när kostnaden avser bevakning eller larm i verksamheten|BAS 6300 och 6390 kräver specificerad riskkategori före sammanföring|BAS 6320 kräver kontroll av skada, försäkrat objekt, privat inslag och avdragsrätt|BAS 6330 kräver kontroll mot pågående arbete, värdering och periodens resultat|BAS 6340 och 6342 kräver kontroll av händelse och avdragsrätt|BAS 6350, 6351 och 6352 kräver kontroll av kundfordran, värdering och eventuell momshantering|BAS 6360 kräver uppdelning mellan faktisk garantikostnad och garantiavsättning|BAS 6361 förändring av garantiavsättning ligger utanför tjänstens scope|BAS 6380 kräver identifiering och värdering av den underliggande kortfristiga fordran|Skilj premie, självrisk, skadestånd, garanti, fordringsförlust och försäkringsersättning|Bokför eventuell förutbetald del endast enligt K1:s förenklingsregler|Flagga för manuell granskning när någon av granskningssituationerna inträffar|Begär det underlag som behövs för att verifiera belopp, motpart, momsbehandling och kontoklassificering|Sätt ärendet till väntar på underlag och bokför inte posten förrän uppgifterna är verifierade|Godkänn kontot endast när användningsvillkoren är uppfyllda; föreslå annars omklassificering, rättelse eller scope-eskalering</x:v>
       </x:c>
       <x:c r="G140" s="14" t="str">
-        <x:v>2440|1930|2641|2645|1700|4600|6800|1000</x:v>
+        <x:v>2440|1930|1700|6310|6900</x:v>
       </x:c>
       <x:c r="H140" s="14" t="str">
-        <x:v>Redovisnings- eller juridisk rådgivning bokförs normalt på 6500|En person som arbetar under företagets dagliga ledning prövas som inhyrd personal på 6800|En vanlig bankavgift kan bokföras på 6500 när den inte är ränta|En faktura från en branschorganisation som blandar medlemsavgift och serviceavgift granskas om delarna inte framgår</x:v>
+        <x:v>Kostnad för bevakning eller larm i verksamhetens lokaler bokförs på 6300 när underlaget är tydligt|En faktisk reparationskostnad som omfattas av lämnad garanti bokförs på 6300 när den kan verifieras och ingen avsättning används|Ett avdragsgillt skadestånd med dokumenterad affärshändelse kan bokföras på 6300|En vanlig ansvarsförsäkringspremie bokförs normalt på 6310|En kundförlust granskas separat och får inte automatiskt döljas som allmän riskkostnad</x:v>
       </x:c>
       <x:c r="I140" s="14" t="str">
-        <x:v>6500 får inte användas för att dölja underentreprenad eller inhyrd personal|Avsaknad av F-skatt ändrar inte automatiskt kostnadskontot men kan medföra skyldighet att göra skatteavdrag och betala arbetsgivaravgifter|Köpt programvara eller rättighet kan vara en tillgång|Utlandstjänster kan medföra omvänd moms och skatteavdrag|Direkt kundproduktion hör normalt till 4600 och faktisk personaluthyrning till 6800|Ränta är inte en bankkostnad på 6500 utan ska redovisas som räntekostnad</x:v>
+        <x:v>6300 får inte bli ett restkonto|Ordinarie företagsförsäkringspremier bör normalt särredovisas på 6310|Privata personförsäkringar är inte automatiskt avdragsgilla i firman|Försäkringsersättning och premie är olika händelser|Självrisk, skadestånd och fordringsförlust kräver dokumenterad klassificering|Ej avdragsgilla skadestånd får inte behandlas som avdragsgill kostnad|Garantiavsättning får inte sammanblandas med faktisk garantikostnad|Mer specifika tillgångs-, fordons- och fordringskonton ska användas när möjligt</x:v>
       </x:c>
       <x:c r="J140" s="14" t="str">
-        <x:v>extern tjänst|konsult|redovisning|juridik|IT-tjänst|F-skatt|R6</x:v>
+        <x:v>riskkostnad|företagsförsäkring|självrisk|försäkringsrisk|R6</x:v>
       </x:c>
       <x:c r="K140" s="14" t="str">
-        <x:v>4600|6800|6100|6200|5900|1000|2440|2641|2645</x:v>
+        <x:v>6310|5612|5100|6900|3900|1700</x:v>
       </x:c>
       <x:c r="L140" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6500, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och avtal|Skatteverket – F-skatt och företagsuppgifter samt rättslig vägledning om betalningsmottagare utan F-skatt, kontrollerat 2026-09-20</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6300, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.59 och 7.5–7.7|Skatteverket – Avdragslexikon för företag, Försäkringar, kontrollerat 2026-07-30</x:v>
       </x:c>
       <x:c r="M140" s="14" t="str">
-        <x:v>Tjänsten kan vara underentreprenad eller inhyrd personal|Leverantören saknar F-skatt eller relationen kan vara anställning|Leverantören är utländsk eller tjänsten avser arbete i Sverige av ett utländskt företag|Tjänsten kan skapa en identifierbar tillgång eller ingå i en annan tillgångs anskaffningsvärde|Avtal, leverans, beloppsfördelning eller period är oklar|Fakturan innehåller medlemsavgift eller en blandad medlems- och serviceavgift som inte är uppdelad</x:v>
+        <x:v>Försäkringens eller riskens art är oklar|Personförsäkring, pension eller privat risk förekommer|Posten kommer från BAS 6300, 6320, 6330, 6340, 6342, 6350, 6351, 6352, 6360, 6380 eller 6390|Självrisk, skadestånd, kundförlust eller annan fordringsförlust kan vara rätt klassificering|Pågående arbete eller värdering av fordran påverkas|Avdragsrätt eller momshantering är oklar|Mer specifikt konto finns|Periodisering kan vara aktuell</x:v>
       </x:c>
       <x:c r="N140" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O140" s="14" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P140" s="14"/>
       <x:c r="Q140" s="12" t="str"/>
     </x:row>
     <x:row r="141" ht="430" customHeight="1">
       <x:c r="A141" s="14" t="str">
-        <x:v>6800</x:v>
+        <x:v>6310</x:v>
       </x:c>
       <x:c r="B141" s="14" t="str">
-        <x:v>Inhyrd personal</x:v>
+        <x:v>Företagsförsäkringar</x:v>
       </x:c>
       <x:c r="C141" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för personal som hyrs in från bemanningsföretag eller annan leverantör och arbetar under företagets arbetsledning utan att vara anställd av företaget.</x:v>
+        <x:v>Kostnadskonto på R6 för premier på försäkringar som har tecknats för näringsverksamheten, exempelvis ansvars-, avbrotts- och sakförsäkring för verksamhetens tillgångar.</x:v>
       </x:c>
       <x:c r="D141" s="14" t="str">
-        <x:v>Leverantören ställer en person till företagets förfogande|Företaget leder och fördelar det dagliga arbetet|Den formella arbetsgivaren är bemannings- eller uthyrningsföretaget|Faktura, period, person och arbetade timmar kan verifieras</x:v>
+        <x:v>Försäkringen är tecknad för verksamheten|Premien avser ansvar, avbrott, egendom eller annan företagsrisk|Försäkringsbrev, period och försäkrade objekt är dokumenterade</x:v>
       </x:c>
       <x:c r="E141" s="14" t="str">
-        <x:v>Leverantören ansvarar självständigt för ett avgränsat resultat; pröva 4600 eller 6500|Personen är i praktiken anställd av företaget|Leverantören saknar F-skatt och skyldighet till skatteavdrag eller arbetsgivaravgifter inte är utredd|Arbetet är privat eller saknar verksamhetssamband|Fakturan avser rekrytering, konsultprojekt eller annan tjänst</x:v>
+        <x:v>Försäkringen avser privat bostad, privat egendom eller privat levnadskostnad|Premien avser personbil och ska följas på 5612|Premien avser sjuk- eller olycksfallsförsäkring som inte är avdragsgill för näringsidkaren enligt aktuell regel|Beloppet är pensionsförsäkring, gruppliv eller annan personförsäkring utan särskild bedömning|Beloppet är självrisk eller försäkringsersättning</x:v>
       </x:c>
       <x:c r="F141" s="14" t="str">
-        <x:v>Identifiera leverantör, formell arbetsgivare, person, period, timmar och arbetsuppgifter|Bedöm vem som leder arbetet, bär resultatansvar och tillhandahåller arbetsredskap|Skilj personaluthyrning från underentreprenad och konsulttjänst|Kontrollera leverantörens F-skatt och arbetsgivaransvar|För utländsk personaluthyrning: krävs särskild kontroll av skatteavdrag, ekonomisk arbetsgivare, socialförsäkring och arbete i Sverige|Bokför kostnaden exklusive avdragsgill moms|Koppla fakturan till tidrapport och uppdrag|Stäm av mot avtal och betalning|Markera återkommande eller omfattande inhyrning för kundkvalificering eftersom målgruppen normalt saknar anställda|Använd endast för verifierad faktisk personaluthyrning|Bedöm arbetsledning, arbetstid, arbetsplats, ekonomisk risk och resultatansvar|Flagga varje ny eller oklar bokning på 6800 för manuell granskning|Begär avtal, faktura, tidrapport, uppgift om person och arbetsledning samt kontroll av F-skatt|Sätt ärendet till väntar på underlag tills personaluthyrning kan skiljas från underentreprenad, konsulttjänst och anställning|Godkänn 6800 för verifierad begränsad personaluthyrning och föreslå omklassificering eller scope-eskalering vid anställningsliknande, utländskt eller omfattande upplägg</x:v>
+        <x:v>Verifiera försäkringstagare, försäkrad risk, objekt, period och verksamhetssamband|Kontrollera om premien normalt är avdragsgill därför att den avser näringsverksamheten och eventuell ersättning är hänförlig till verksamheten|Skilj företagsförsäkring från privat personförsäkring och pensionskostnad|Bokför premien på 6310 och eventuell avdragsgill moms endast om sådan har debiterats|Hantera förutbetald premie enligt K1 punkt 6.59 när villkoren är uppfyllda|Koppla premien till försäkringsbrev och förfalloperiod|Stäm av återbetalning och uppsägning|Kräv manuell granskning för sjukvård, olycksfall, gruppliv, reseskydd eller försäkring med privat del|Kräv försäkringsbolag, typ, objekt, period, premie och privat andel|Koppla återbetalning till ursprunglig premie|Följ verifierad periodiseringsrutin|Vid granskningsflagga begär in försäkringsbrev med försäkringstagare, försäkringstyp, objekt, period och premie|Sätt ärendet till väntar på underlag tills verksamhetskoppling, privat andel och period är verifierade|Godkänn 6310 när premien avser en vanlig försäkring för verksamhetens risker eller tillgångar|Föreslå 5612, privat kostnad, periodiseringsrutin eller eskalering när försäkringen avser bil, person, pension eller oklar privat del</x:v>
       </x:c>
       <x:c r="G141" s="14" t="str">
-        <x:v>2440|1930|2641|2645|2710|2730</x:v>
+        <x:v>2440|1930|1700|6300</x:v>
       </x:c>
       <x:c r="H141" s="14" t="str">
-        <x:v>Bemanningsföretag fakturerar timmar för en person som arbetar under företagarens dagliga ledning; kostnaden bokförs på 6800|En underentreprenör som själv ansvarar för ett byggmoment bokförs normalt på 4600</x:v>
+        <x:v>Premie för verksamhetens ansvarsförsäkring bokförs på 6310|Privat sjuk- och olycksfallsförsäkring bokförs inte automatiskt som företagskostnad</x:v>
       </x:c>
       <x:c r="I141" s="14" t="str">
-        <x:v>Inhyrd personal och underentreprenad är olika relationer|F-skatt undanröjer inte alltid risken för ett faktiskt anställningsförhållande|Utländsk personaluthyrning har särskilda skatte- och rapporteringsregler|Omfattande inhyrning kan ligga utanför Enkla Boksluts standardkund|Faktura eller F-skatt utesluter inte anställningsförhållande|Återkommande inhyrning ligger normalt utanför standardtjänsten</x:v>
+        <x:v>Försäkringens namn avgör inte ensam avdragsrätten|Personförsäkringar har särskilda regler|Fordon och fastighet kan kräva mer specifikt konto|Försäkringsersättningar redovisas separat|Privat sjuk-, olycksfalls-, liv- eller pensionsförsäkring är inte vanlig företagsförsäkring</x:v>
       </x:c>
       <x:c r="J141" s="14" t="str">
-        <x:v>inhyrd personal|bemanningsföretag|personaluthyrning|ekonomisk arbetsgivare|F-skatt|R6</x:v>
+        <x:v>företagsförsäkring|ansvarsförsäkring|avbrottsförsäkring|sakförsäkring|premie|R6</x:v>
       </x:c>
       <x:c r="K141" s="14" t="str">
-        <x:v>4600|6500|7000|2710|2730|2440|2641|2645</x:v>
+        <x:v>6300|5612|5100|6900|3900|1700</x:v>
       </x:c>
       <x:c r="L141" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6800, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – F- och FA-skatt, kontrollerat 2026-07-30|Skatteverket – Skatteavdrag för arbete och utländsk personaluthyrning, kontrollerat 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6310, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18, 6.59 och 7.5–7.7|Skatteverket – Avdragslexikon för företag, Försäkringar, kontrollerat 2026-07-30</x:v>
       </x:c>
       <x:c r="M141" s="14" t="str">
-        <x:v>Leverantören saknar F-skatt|Relationen kan vara anställning eller underentreprenad|Utländsk leverantör eller arbete i Sverige förekommer|Tidrapport, person eller avtal saknas|Omfattande eller återkommande inhyrning förekommer|Anställningsliknande upplägg eller utländsk arbetskraft förekommer</x:v>
+        <x:v>Försäkringen kan vara privat eller en personförsäkring|Försäkringsobjekt eller period saknas|Återbetalning, självrisk eller ersättning förekommer|Mer specifikt kostnadskonto kan vara rätt|Avdragsrätten är särskilt reglerad|Försäkringstyp, privat andel eller periodisering är oklar</x:v>
       </x:c>
       <x:c r="N141" s="14" t="str">
         <x:v>active</x:v>
@@ -7801,43 +7805,43 @@
     </x:row>
     <x:row r="142" ht="430" customHeight="1">
       <x:c r="A142" s="14" t="str">
-        <x:v>6900</x:v>
+        <x:v>6500</x:v>
       </x:c>
       <x:c r="B142" s="14" t="str">
-        <x:v>Övriga kostnader</x:v>
+        <x:v>Övriga externa tjänster</x:v>
       </x:c>
       <x:c r="C142" s="14" t="str">
-        <x:v>K1-konto på R6 för verksamhetskostnader som inte passar på ett mer specifikt konto, till exempel vissa licens-, patent-, varumärkes-, kontroll- och tillsynsavgifter. Kontot får inte användas som ospecificerat restkonto.</x:v>
+        <x:v>Kostnadskonto på R6 för köpta konsult-, redovisnings-, juridik-, IT- och andra externa tjänster som inte är underentreprenad, inhyrd personal eller en tjänst med mer specifikt konto.</x:v>
       </x:c>
       <x:c r="D142" s="14" t="str">
-        <x:v>Utgiften har ett tydligt samband med verksamheten och ska redovisas som extern kostnad på R6|Ingen mer specifik tillåten kontogrupp beskriver kostnaden bättre|Kostnaden avser exempelvis licens eller royalty, eget patent eller varumärke, kontrollavgift eller tillsynsavgift|Underlaget visar vad som köpts, motpart och affärsändamål</x:v>
+        <x:v>En extern leverantör utför en avgränsad administrativ, rådgivande eller specialisttjänst|Tjänsten stödjer verksamheten men är inte direkt del av produktionen på 4600|Leverantören ansvarar för tjänstens resultat och är inte inhyrd under företagets arbetsledning</x:v>
       </x:c>
       <x:c r="E142" s="14" t="str">
-        <x:v>Utgiften är privat eller saknar tydligt samband med verksamheten|Mer specifikt konto finns, exempelvis 5900, 6100, 6200, 6300, 6500, 6800 eller 6980|Utgiften är varuinköp, inventarie, ränta, avskrivning eller annan post som hör till en annan kontogrupp|Posten är en okänd bank- eller korttransaktion|Posten gäller föreningsavgift; använd 6980|Posten gäller utländsk skatt, utländsk moms eller blandad verksamhet och kräver särskild kontroll</x:v>
+        <x:v>Tjänsten är underentreprenad direkt i kundens leverans; använd 4600|Personen ställs till företagets förfogande och leds som personal; använd 6800|Utgiften gäller reklam, tele, försäkring, resa eller annan mer specifik tjänst|Köpet ger en separat rättighet, programvara, webbplats eller annan tillgång som ska aktiveras|Avgiften är en ren medlemsavgift eller en blandad medlems- och serviceavgift där tjänstedelen inte framgår; skicka till manuell granskning</x:v>
       </x:c>
       <x:c r="F142" s="14" t="str">
-        <x:v>Identifiera alltid kostnadstyp, motpart, belopp, underlag och koppling till verksamheten|Pröva först om ett mer specifikt K1-konto ska användas|BAS 6910, 6920, 6930, 6940, 6950 och 6991 får sammanföras automatiskt till 6900|BAS 6900 och 6990 kräver specificering eftersom de är generella konton|BAS 6970 kräver kontroll av att litteraturen är fackmässig och har tydlig koppling till verksamheten|BAS 6992 kräver att ej avdragsgill företagskostnad skiljs från privat kostnad och hanteras i deklarationen|BAS 6993 kräver kontroll av om posten är en vanlig gåva eller en tillåten reklam- eller representationskostnad|BAS 7990 kräver identifiering av den bakomliggande rörelsekostnaden innan den kan föras till 6900|Föreningsavgifter hålls på 6980 och utländsk skatt, utländsk moms samt blandad verksamhet granskas separat</x:v>
+        <x:v>Identifiera leverantör, avtal, leverans, ansvar för resultat och period|Skilj specialist- och konsulttjänst för den egna verksamheten från underentreprenad på 4600 och inhyrd personal på 6800|Använd ett mer specifikt kostnadskonto när tjänstens art omfattas av ett sådant konto|Kontrollera F-skatt när ersättningen avser arbete; om F-skatt saknas ska ärendet granskas med avseende på skatteavdrag, arbetsgivaravgifter och eventuell anställningsrelation|För utländsk leverantör: kontrollera beskattningsland, omvänd moms och eventuell skyldighet att göra skatteavdrag för arbete i Sverige|Bokför kostnaden exklusive avdragsgill moms|Pröva om köpet skapar en identifierbar tillgång eller ska ingå i en annan tillgångs anskaffningsvärde|Koppla kostnaden till avtal, projekt och leverans och stäm av förskott, leverantörsskuld och kreditnota|Periodisera tjänsten när betalnings- och leveransperioden inte sammanfaller enligt tillämplig K1-regel|Bankkostnader kan redovisas på 6500 när ett mer specifikt konto saknas|För serviceavgift till branschorganisation: verifiera att avgiften avser en identifierbar tjänst; ren medlemsavgift eller oklar blandad avgift kräver manuell granskning</x:v>
       </x:c>
       <x:c r="G142" s="14" t="str">
-        <x:v>2440|1930|2641|6980</x:v>
+        <x:v>2440|1930|2641|2645|1700|4600|6800|1000</x:v>
       </x:c>
       <x:c r="H142" s="14" t="str">
-        <x:v>En dokumenterad tillsynsavgift från en myndighet bokförs på 6900|En licens- eller royaltyavgift som hör till verksamheten bokförs på 6900 när inget mer specifikt konto passar|En bok som direkt behandlar företagets yrkesområde kan bokföras efter kontroll, medan en allmän tidning kräver annan bedömning|En gåva till en organisation granskas och får inte behandlas som avdragsgill kostnad utan stöd|En okänd korttransaktion bokförs inte på 6900 utan utreds först</x:v>
+        <x:v>Redovisnings- eller juridisk rådgivning bokförs normalt på 6500|En person som arbetar under företagets dagliga ledning prövas som inhyrd personal på 6800|En vanlig bankavgift kan bokföras på 6500 när den inte är ränta|En faktura från en branschorganisation som blandar medlemsavgift och serviceavgift granskas om delarna inte framgår</x:v>
       </x:c>
       <x:c r="I142" s="14" t="str">
-        <x:v>6900 får inte bli ett restkonto för kostnader som inte har utretts|Privat kostnad och ej avdragsgill företagskostnad är inte samma sak|Ej avdragsgilla kostnader måste kunna identifieras vid deklarationen|Gåvor och allmänna tidningar är normalt inte automatiskt avdragsgilla|Använd ett mer specifikt konto när det finns</x:v>
+        <x:v>6500 får inte användas för att dölja underentreprenad eller inhyrd personal|Avsaknad av F-skatt ändrar inte automatiskt kostnadskontot men kan medföra skyldighet att göra skatteavdrag och betala arbetsgivaravgifter|Köpt programvara eller rättighet kan vara en tillgång|Utlandstjänster kan medföra omvänd moms och skatteavdrag|Direkt kundproduktion hör normalt till 4600 och faktisk personaluthyrning till 6800|Ränta är inte en bankkostnad på 6500 utan ska redovisas som räntekostnad</x:v>
       </x:c>
       <x:c r="J142" s="14" t="str">
-        <x:v>övrig kostnad|skadestånd|avgift|restkonto|ej avdragsgill kostnad|R6</x:v>
+        <x:v>extern tjänst|konsult|redovisning|juridik|IT-tjänst|F-skatt|R6</x:v>
       </x:c>
       <x:c r="K142" s="14" t="str">
-        <x:v>5900|6100|6200|6300|6500|6800|6980</x:v>
+        <x:v>4600|6800|6100|6200|5900|1000|2440|2641|2645</x:v>
       </x:c>
       <x:c r="L142" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – konto 6900, rad R6|BFNAR 2006:1, reglerna om kostnader och privata utgifter|Skatteverket och verksamt.se, avdrag för kostnader i enskild näringsverksamhet, 2026</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6500, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och avtal|Skatteverket – F-skatt och företagsuppgifter samt rättslig vägledning om betalningsmottagare utan F-skatt, kontrollerat 2026-09-20</x:v>
       </x:c>
       <x:c r="M142" s="14" t="str">
-        <x:v>Posten kommer från BAS 6900, 6970, 6990, 6992, 6993 eller 7990|Mer specifikt konto kan vara rätt|Utgiften kan vara privat eller ej avdragsgill|Litteraturens koppling till verksamheten är oklar|Posten är en gåva, reklamgåva eller representationsgåva|Underlag, motpart eller affärsändamål saknas</x:v>
+        <x:v>Tjänsten kan vara underentreprenad eller inhyrd personal|Leverantören saknar F-skatt eller relationen kan vara anställning|Leverantören är utländsk eller tjänsten avser arbete i Sverige av ett utländskt företag|Tjänsten kan skapa en identifierbar tillgång eller ingå i en annan tillgångs anskaffningsvärde|Avtal, leverans, beloppsfördelning eller period är oklar|Fakturan innehåller medlemsavgift eller en blandad medlems- och serviceavgift som inte är uppdelad</x:v>
       </x:c>
       <x:c r="N142" s="14" t="str">
         <x:v>active</x:v>
@@ -7850,43 +7854,43 @@
     </x:row>
     <x:row r="143" ht="430" customHeight="1">
       <x:c r="A143" s="14" t="str">
-        <x:v>6980</x:v>
+        <x:v>6800</x:v>
       </x:c>
       <x:c r="B143" s="14" t="str">
-        <x:v>Föreningsavgifter</x:v>
+        <x:v>Inhyrd personal</x:v>
       </x:c>
       <x:c r="C143" s="14" t="str">
-        <x:v>Kostnadskonto på R6 för medlemsavgifter till föreningar, branschorganisationer och andra sammanslutningar. Medlemsavgiften är normalt inte skattemässigt avdragsgill och ska skiljas från separat fakturerade serviceavgifter.</x:v>
+        <x:v>Kostnadskonto på R6 för personal som hyrs in från bemanningsföretag eller annan leverantör och arbetar under företagets arbetsledning utan att vara anställd av företaget.</x:v>
       </x:c>
       <x:c r="D143" s="14" t="str">
-        <x:v>Fakturan eller beslutet avser medlemskap i en identifierad förening eller sammanslutning|Medlemsavgiften hör till näringsverksamheten men är skattemässigt ej avdragsgill|Medlemsavgift och eventuell serviceavgift är specificerade var för sig</x:v>
+        <x:v>Leverantören ställer en person till företagets förfogande|Företaget leder och fördelar det dagliga arbetet|Den formella arbetsgivaren är bemannings- eller uthyrningsföretaget|Faktura, period, person och arbetade timmar kan verifieras</x:v>
       </x:c>
       <x:c r="E143" s="14" t="str">
-        <x:v>Beloppet är en separat serviceavgift för direkta tjänster som används i verksamheten; pröva 6500 eller 6900|Avgiften är en myndighets-, tillstånds-, auktorisations- eller registreringsavgift|Medlemskapet är privat|Fakturan avser den anställdas personliga medlemskap utan förmånsbedömning|Beloppet är gåva, sponsring eller bidrag</x:v>
+        <x:v>Leverantören ansvarar självständigt för ett avgränsat resultat; pröva 4600 eller 6500|Personen är i praktiken anställd av företaget|Leverantören saknar F-skatt och skyldighet till skatteavdrag eller arbetsgivaravgifter inte är utredd|Arbetet är privat eller saknar verksamhetssamband|Fakturan avser rekrytering, konsultprojekt eller annan tjänst</x:v>
       </x:c>
       <x:c r="F143" s="14" t="str">
-        <x:v>Identifiera förening, medlem, medlemsperiod och avgiftstyp|Kräv faktura eller medlemsbeslut som skiljer medlemsavgift från serviceavgift|Bokför medlemsavgiften på 6980 och märk den för skattemässig återläggning|Bokför separat avdragsgill serviceavgift på lämpligt tjänstekonto när den avser direkta tjänster som företaget använder|Bokför ingående moms endast på en momsbelagd tjänstedel med giltigt underlag|För arbetsgivarorganisation: identifiera särskilt eventuell del för konfliktändamål|För anställds medlemsavgift: bedöm skattepliktig förmån, skatteavdrag och arbetsgivaravgifter|Stäm av mot betalning och skattekod|Kräv manuell granskning vid blandad faktura eller otydlig avgiftsbenämning|Använd för separat identifierad medlemsavgift|Dela faktura från serviceavgift, momsbelagd tjänst och konfliktfondsdel|Vid granskningsflagga begär in faktura eller medlemsbeslut med uppdelning mellan medlemsavgift och serviceavgift|Sätt ärendet till väntar på underlag tills avgiftstyp, moms och medlemskap är verifierade|Godkänn 6980 för separat identifierad medlemsavgift och markera skattemässig återläggning|Föreslå relevant tjänstekonto, sponsring, gåva eller scope-eskalering när fakturan avser service, annan motprestation eller anställds medlemskap</x:v>
+        <x:v>Identifiera leverantör, formell arbetsgivare, person, period, timmar och arbetsuppgifter|Bedöm vem som leder arbetet, bär resultatansvar och tillhandahåller arbetsredskap|Skilj personaluthyrning från underentreprenad och konsulttjänst|Kontrollera leverantörens F-skatt och arbetsgivaransvar|För utländsk personaluthyrning: krävs särskild kontroll av skatteavdrag, ekonomisk arbetsgivare, socialförsäkring och arbete i Sverige|Bokför kostnaden exklusive avdragsgill moms|Koppla fakturan till tidrapport och uppdrag|Stäm av mot avtal och betalning|Markera återkommande eller omfattande inhyrning för kundkvalificering eftersom målgruppen normalt saknar anställda|Använd endast för verifierad faktisk personaluthyrning|Bedöm arbetsledning, arbetstid, arbetsplats, ekonomisk risk och resultatansvar|Flagga varje ny eller oklar bokning på 6800 för manuell granskning|Begär avtal, faktura, tidrapport, uppgift om person och arbetsledning samt kontroll av F-skatt|Sätt ärendet till väntar på underlag tills personaluthyrning kan skiljas från underentreprenad, konsulttjänst och anställning|Godkänn 6800 för verifierad begränsad personaluthyrning och föreslå omklassificering eller scope-eskalering vid anställningsliknande, utländskt eller omfattande upplägg</x:v>
       </x:c>
       <x:c r="G143" s="14" t="str">
-        <x:v>2440|1930|2013|6500|6900|2641</x:v>
+        <x:v>2440|1930|2641|2645|2710|2730</x:v>
       </x:c>
       <x:c r="H143" s="14" t="str">
-        <x:v>En branschförenings medlemsavgift bokförs på 6980 och återläggs skattemässigt|En separat serviceavgift för kurser och rådgivning kan bokföras på 6500 efter kontroll</x:v>
+        <x:v>Bemanningsföretag fakturerar timmar för en person som arbetar under företagarens dagliga ledning; kostnaden bokförs på 6800|En underentreprenör som själv ansvarar för ett byggmoment bokförs normalt på 4600</x:v>
       </x:c>
       <x:c r="I143" s="14" t="str">
-        <x:v>Medlemsavgifter är normalt inte avdragsgilla|Serviceavgift och medlemsavgift ska inte sammanblandas|Moms får inte lyftas på en momsfri medlemsavgift|Betald medlemsavgift för en anställd kan vara skattepliktig förmån|Serviceavgift för konkreta tjänster kan höra till 6500|Personlig medlemsavgift kan vara personalfråga</x:v>
+        <x:v>Inhyrd personal och underentreprenad är olika relationer|F-skatt undanröjer inte alltid risken för ett faktiskt anställningsförhållande|Utländsk personaluthyrning har särskilda skatte- och rapporteringsregler|Omfattande inhyrning kan ligga utanför Enkla Boksluts standardkund|Faktura eller F-skatt utesluter inte anställningsförhållande|Återkommande inhyrning ligger normalt utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="J143" s="14" t="str">
-        <x:v>föreningsavgift|medlemsavgift|serviceavgift|branschorganisation|skattemässig återläggning|R6</x:v>
+        <x:v>inhyrd personal|bemanningsföretag|personaluthyrning|ekonomisk arbetsgivare|F-skatt|R6</x:v>
       </x:c>
       <x:c r="K143" s="14" t="str">
-        <x:v>6500|6900|7300|7500|2641|2013</x:v>
+        <x:v>4600|6500|7000|2710|2730|2440|2641|2645</x:v>
       </x:c>
       <x:c r="L143" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6980, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Avdragslexikon för företag, Föreningsavgifter, kontrollerat 2026-07-30|Skatteverkets rättsliga vägledning 2026 om medlemsavgifter och serviceavgifter</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6800, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – F- och FA-skatt, kontrollerat 2026-07-30|Skatteverket – Skatteavdrag för arbete och utländsk personaluthyrning, kontrollerat 2026-07-30</x:v>
       </x:c>
       <x:c r="M143" s="14" t="str">
-        <x:v>Fakturan blandar medlems- och serviceavgift|Moms har debiterats utan att tjänstedelen är identifierad|Avgiften avser anställds medlemskap|Arbetsgivarorganisation eller konfliktfond förekommer|Det är oklart om beloppet är avgift, sponsring eller gåva|Fakturan saknar uppdelning eller medlemskapet avser anställd</x:v>
+        <x:v>Leverantören saknar F-skatt|Relationen kan vara anställning eller underentreprenad|Utländsk leverantör eller arbete i Sverige förekommer|Tidrapport, person eller avtal saknas|Omfattande eller återkommande inhyrning förekommer|Anställningsliknande upplägg eller utländsk arbetskraft förekommer</x:v>
       </x:c>
       <x:c r="N143" s="14" t="str">
         <x:v>active</x:v>
@@ -7899,43 +7903,43 @@
     </x:row>
     <x:row r="144" ht="430" customHeight="1">
       <x:c r="A144" s="14" t="str">
-        <x:v>7000</x:v>
+        <x:v>6900</x:v>
       </x:c>
       <x:c r="B144" s="14" t="str">
-        <x:v>Löner till anställda</x:v>
+        <x:v>Övriga kostnader</x:v>
       </x:c>
       <x:c r="C144" s="14" t="str">
-        <x:v>Tekniskt importkonto på R7 för löner till anställda. En förekomst ska stoppa standardflödet eftersom Enkla Boksluts kunder ska sakna anställda.</x:v>
+        <x:v>K1-konto på R6 för verksamhetskostnader som inte passar på ett mer specifikt konto, till exempel vissa licens-, patent-, varumärkes-, kontroll- och tillsynsavgifter. Kontot får inte användas som ospecificerat restkonto.</x:v>
       </x:c>
       <x:c r="D144" s="14" t="str">
-        <x:v>En importerad SIE-fil innehåller lönekostnad på 7000 och posten behöver utredas</x:v>
+        <x:v>Utgiften har ett tydligt samband med verksamheten och ska redovisas som extern kostnad på R6|Ingen mer specifik tillåten kontogrupp beskriver kostnaden bättre|Kostnaden avser exempelvis licens eller royalty, eget patent eller varumärke, kontrollavgift eller tillsynsavgift|Underlaget visar vad som köpts, motpart och affärsändamål</x:v>
       </x:c>
       <x:c r="E144" s="14" t="str">
-        <x:v>Företagarens eget uttag|Ersättning till självständig uppdragstagare med F-skatt|Systemet ska skapa en ny lönepost</x:v>
+        <x:v>Utgiften är privat eller saknar tydligt samband med verksamheten|Mer specifikt konto finns, exempelvis 5900, 6100, 6200, 6300, 6500, 6800 eller 6980|Utgiften är varuinköp, inventarie, ränta, avskrivning eller annan post som hör till en annan kontogrupp|Posten är en okänd bank- eller korttransaktion|Posten gäller föreningsavgift; använd 6980|Posten gäller utländsk skatt, utländsk moms eller blandad verksamhet och kräver särskild kontroll</x:v>
       </x:c>
       <x:c r="F144" s="14" t="str">
-        <x:v>Flagga varje bokning på 7000 för manuell kund- och scope-prövning|Begär anställningsavtal, löneunderlag, arbetsgivardeklaration och betalningsunderlag|Sätt ärendet till väntar på underlag|Om posten avser verklig lön till anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten avser företagaren eller en leverantör: flytta den till eget kapital eller rätt kostnadskonto</x:v>
+        <x:v>Identifiera alltid kostnadstyp, motpart, belopp, underlag och koppling till verksamheten|Pröva först om ett mer specifikt K1-konto ska användas|BAS 6910, 6920, 6930, 6940, 6950 och 6991 får sammanföras automatiskt till 6900|BAS 6900 och 6990 kräver specificering eftersom de är generella konton|BAS 6970 kräver kontroll av att litteraturen är fackmässig och har tydlig koppling till verksamheten|BAS 6992 kräver att ej avdragsgill företagskostnad skiljs från privat kostnad och hanteras i deklarationen|BAS 6993 kräver kontroll av om posten är en vanlig gåva eller en tillåten reklam- eller representationskostnad|BAS 7990 kräver identifiering av den bakomliggande rörelsekostnaden innan den kan föras till 6900|Föreningsavgifter hålls på 6980 och utländsk skatt, utländsk moms samt blandad verksamhet granskas separat</x:v>
       </x:c>
       <x:c r="G144" s="14" t="str">
-        <x:v>2710|2730|1930|2900|7300|7500</x:v>
+        <x:v>2440|1930|2641|6980</x:v>
       </x:c>
       <x:c r="H144" s="14" t="str">
-        <x:v>Lön till anställd innebär scope-prövning|Företagarens privata uttag bokförs mot eget kapital och inte på 7000</x:v>
+        <x:v>En dokumenterad tillsynsavgift från en myndighet bokförs på 6900|En licens- eller royaltyavgift som hör till verksamheten bokförs på 6900 när inget mer specifikt konto passar|En bok som direkt behandlar företagets yrkesområde kan bokföras efter kontroll, medan en allmän tidning kräver annan bedömning|En gåva till en organisation granskas och får inte behandlas som avdragsgill kostnad utan stöd|En okänd korttransaktion bokförs inte på 6900 utan utreds först</x:v>
       </x:c>
       <x:c r="I144" s="14" t="str">
-        <x:v>Företagaren kan inte vara anställd i sin egen enskilda firma|Verklig lönehantering ligger utanför standardtjänsten</x:v>
+        <x:v>6900 får inte bli ett restkonto för kostnader som inte har utretts|Privat kostnad och ej avdragsgill företagskostnad är inte samma sak|Ej avdragsgilla kostnader måste kunna identifieras vid deklarationen|Gåvor och allmänna tidningar är normalt inte automatiskt avdragsgilla|Använd ett mer specifikt konto när det finns</x:v>
       </x:c>
       <x:c r="J144" s="14" t="str">
-        <x:v>lön|bruttolön|anställd|löneutbetalning|arbetsgivardeklaration|AGI|R7</x:v>
+        <x:v>övrig kostnad|skadestånd|avgift|restkonto|ej avdragsgill kostnad|R6</x:v>
       </x:c>
       <x:c r="K144" s="14" t="str">
-        <x:v>2710|2730|7300|7400|7500|7600|1930|2900</x:v>
+        <x:v>5900|6100|6200|6300|6500|6800|6980</x:v>
       </x:c>
       <x:c r="L144" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 7000, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 3.9 om företagarens egna uttag och punkterna 3.18 och 7.5–7.7|Skatteverket – Lön och egna uttag, kontrollerat 2026-07-30|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sidoordnad lönebokföring</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – konto 6900, rad R6|BFNAR 2006:1, reglerna om kostnader och privata utgifter|Skatteverket och verksamt.se, avdrag för kostnader i enskild näringsverksamhet, 2026</x:v>
       </x:c>
       <x:c r="M144" s="14" t="str">
-        <x:v>Varje bokning på 7000|Mottagare, anställningsförhållande, löneunderlag eller AGI saknas</x:v>
+        <x:v>Posten kommer från BAS 6900, 6970, 6990, 6992, 6993 eller 7990|Mer specifikt konto kan vara rätt|Utgiften kan vara privat eller ej avdragsgill|Litteraturens koppling till verksamheten är oklar|Posten är en gåva, reklamgåva eller representationsgåva|Underlag, motpart eller affärsändamål saknas</x:v>
       </x:c>
       <x:c r="N144" s="14" t="str">
         <x:v>active</x:v>
@@ -7943,48 +7947,48 @@
       <x:c r="O144" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P144" s="14" t="str"/>
+      <x:c r="P144" s="14"/>
       <x:c r="Q144" s="12" t="str"/>
     </x:row>
     <x:row r="145" ht="430" customHeight="1">
       <x:c r="A145" s="14" t="str">
-        <x:v>7300</x:v>
+        <x:v>6980</x:v>
       </x:c>
       <x:c r="B145" s="14" t="str">
-        <x:v>Kostnadsersättningar och förmåner</x:v>
+        <x:v>Föreningsavgifter</x:v>
       </x:c>
       <x:c r="C145" s="14" t="str">
-        <x:v>Tekniskt importkonto på R7 för kostnadsersättningar och förmåner till anställda. En förekomst ska stoppa standardflödet och utredas.</x:v>
+        <x:v>Kostnadskonto på R6 för medlemsavgifter till föreningar, branschorganisationer och andra sammanslutningar. Medlemsavgiften är normalt inte skattemässigt avdragsgill och ska skiljas från separat fakturerade serviceavgifter.</x:v>
       </x:c>
       <x:c r="D145" s="14" t="str">
-        <x:v>En importerad SIE-fil innehåller bokning på 7300 och mottagare samt ersättningstyp behöver fastställas</x:v>
+        <x:v>Fakturan eller beslutet avser medlemskap i en identifierad förening eller sammanslutning|Medlemsavgiften hör till näringsverksamheten men är skattemässigt ej avdragsgill|Medlemsavgift och eventuell serviceavgift är specificerade var för sig</x:v>
       </x:c>
       <x:c r="E145" s="14" t="str">
-        <x:v>Företagarens egen resa eller privatbilsschablon|En vanlig företagskostnad som betalats direkt av firman|Systemet ska skapa kostnadsersättning till anställd</x:v>
+        <x:v>Beloppet är en separat serviceavgift för direkta tjänster som används i verksamheten; pröva 6500 eller 6900|Avgiften är en myndighets-, tillstånds-, auktorisations- eller registreringsavgift|Medlemskapet är privat|Fakturan avser den anställdas personliga medlemskap utan förmånsbedömning|Beloppet är gåva, sponsring eller bidrag</x:v>
       </x:c>
       <x:c r="F145" s="14" t="str">
-        <x:v>Flagga varje bokning på 7300 för manuell granskning|Begär uppgift om mottagare, reseräkning eller förmånsunderlag och eventuell arbetsgivardeklaration|Sätt ärendet till väntar på underlag|Om posten avser anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten avser företagaren eller en vanlig företagskostnad: flytta den till rätt rese-, bil-, kostnads- eller egetkapitalkonto</x:v>
+        <x:v>Identifiera förening, medlem, medlemsperiod och avgiftstyp|Kräv faktura eller medlemsbeslut som skiljer medlemsavgift från serviceavgift|Bokför medlemsavgiften på 6980 och märk den för skattemässig återläggning|Bokför separat avdragsgill serviceavgift på lämpligt tjänstekonto när den avser direkta tjänster som företaget använder|Bokför ingående moms endast på en momsbelagd tjänstedel med giltigt underlag|För arbetsgivarorganisation: identifiera särskilt eventuell del för konfliktändamål|För anställds medlemsavgift: bedöm skattepliktig förmån, skatteavdrag och arbetsgivaravgifter|Stäm av mot betalning och skattekod|Kräv manuell granskning vid blandad faktura eller otydlig avgiftsbenämning|Använd för separat identifierad medlemsavgift|Dela faktura från serviceavgift, momsbelagd tjänst och konfliktfondsdel|Vid granskningsflagga begär in faktura eller medlemsbeslut med uppdelning mellan medlemsavgift och serviceavgift|Sätt ärendet till väntar på underlag tills avgiftstyp, moms och medlemskap är verifierade|Godkänn 6980 för separat identifierad medlemsavgift och markera skattemässig återläggning|Föreslå relevant tjänstekonto, sponsring, gåva eller scope-eskalering när fakturan avser service, annan motprestation eller anställds medlemskap</x:v>
       </x:c>
       <x:c r="G145" s="14" t="str">
-        <x:v>1930|2710|2730|7000|7500|2013</x:v>
+        <x:v>2440|1930|2013|6500|6900|2641</x:v>
       </x:c>
       <x:c r="H145" s="14" t="str">
-        <x:v>Importerad kostnadsersättning till anställd leder till scope-prövning|Företagarens egen bilersättning hanteras genom företagets särskilda privatbilsflöde och inte på 7300</x:v>
+        <x:v>En branschförenings medlemsavgift bokförs på 6980 och återläggs skattemässigt|En separat serviceavgift för kurser och rådgivning kan bokföras på 6500 efter kontroll</x:v>
       </x:c>
       <x:c r="I145" s="14" t="str">
-        <x:v>Kontot ska inte användas för företagarens egna resor|Verkliga förmåner eller ersättningar till anställda ligger utanför standardtjänsten</x:v>
+        <x:v>Medlemsavgifter är normalt inte avdragsgilla|Serviceavgift och medlemsavgift ska inte sammanblandas|Moms får inte lyftas på en momsfri medlemsavgift|Betald medlemsavgift för en anställd kan vara skattepliktig förmån|Serviceavgift för konkreta tjänster kan höra till 6500|Personlig medlemsavgift kan vara personalfråga</x:v>
       </x:c>
       <x:c r="J145" s="14" t="str">
-        <x:v>kostnadsersättning|förmån|traktamente|milersättning|tjänsteresa|AGI|R7</x:v>
+        <x:v>föreningsavgift|medlemsavgift|serviceavgift|branschorganisation|skattemässig återläggning|R6</x:v>
       </x:c>
       <x:c r="K145" s="14" t="str">
-        <x:v>7000|7500|7600|5618|5800|2710|2730</x:v>
+        <x:v>6500|6900|7300|7500|2641|2013</x:v>
       </x:c>
       <x:c r="L145" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 7300, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Traktamente och bilersättning, inkomstår 2026, kontrollerat 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 6980, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Avdragslexikon för företag, Föreningsavgifter, kontrollerat 2026-07-30|Skatteverkets rättsliga vägledning 2026 om medlemsavgifter och serviceavgifter</x:v>
       </x:c>
       <x:c r="M145" s="14" t="str">
-        <x:v>Varje bokning på 7300|Mottagare, reseräkning, förmånsunderlag eller AGI saknas</x:v>
+        <x:v>Fakturan blandar medlems- och serviceavgift|Moms har debiterats utan att tjänstedelen är identifierad|Avgiften avser anställds medlemskap|Arbetsgivarorganisation eller konfliktfond förekommer|Det är oklart om beloppet är avgift, sponsring eller gåva|Fakturan saknar uppdelning eller medlemskapet avser anställd</x:v>
       </x:c>
       <x:c r="N145" s="14" t="str">
         <x:v>active</x:v>
@@ -7992,48 +7996,48 @@
       <x:c r="O145" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P145" s="14" t="str"/>
+      <x:c r="P145" s="14"/>
       <x:c r="Q145" s="12" t="str"/>
     </x:row>
     <x:row r="146" ht="430" customHeight="1">
       <x:c r="A146" s="14" t="str">
-        <x:v>7400</x:v>
+        <x:v>7000</x:v>
       </x:c>
       <x:c r="B146" s="14" t="str">
-        <x:v>Pensionskostnader</x:v>
+        <x:v>Löner till anställda</x:v>
       </x:c>
       <x:c r="C146" s="14" t="str">
-        <x:v>Tekniskt importkonto på R7 för pensionskostnader avseende anställda. Företagarens egen pension ska hanteras separat och kontot ska alltid granskas.</x:v>
+        <x:v>Tekniskt importkonto på R7 för löner till anställda. En förekomst ska stoppa standardflödet eftersom Enkla Boksluts kunder ska sakna anställda.</x:v>
       </x:c>
       <x:c r="D146" s="14" t="str">
-        <x:v>En importerad SIE-fil innehåller bokning på 7400 och det behöver fastställas vem pensionen avser</x:v>
+        <x:v>En importerad SIE-fil innehåller lönekostnad på 7000 och posten behöver utredas</x:v>
       </x:c>
       <x:c r="E146" s="14" t="str">
-        <x:v>Företagarens eget pensionssparande som vanlig personalkostnad|Privat sparande eller försäkring utan verifierad pensionsbehandling|Systemet ska skapa en ny tjänstepensionspost</x:v>
+        <x:v>Företagarens eget uttag|Ersättning till självständig uppdragstagare med F-skatt|Systemet ska skapa en ny lönepost</x:v>
       </x:c>
       <x:c r="F146" s="14" t="str">
-        <x:v>Flagga varje bokning på 7400 för manuell granskning|Begär pensionsavtal, uppgift om försäkrad person, premieperiod och betalningsunderlag|Sätt ärendet till väntar på underlag|Om pensionen avser anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om pensionen avser företagaren: bokför betalningen enligt egetkapitalflödet och hantera eventuellt avdrag separat i NE</x:v>
+        <x:v>Flagga varje bokning på 7000 för manuell kund- och scope-prövning|Begär anställningsavtal, löneunderlag, arbetsgivardeklaration och betalningsunderlag|Sätt ärendet till väntar på underlag|Om posten avser verklig lön till anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten avser företagaren eller en leverantör: flytta den till eget kapital eller rätt kostnadskonto</x:v>
       </x:c>
       <x:c r="G146" s="14" t="str">
-        <x:v>2440|1930|7500|2730|2013</x:v>
+        <x:v>2710|2730|1930|2900|7300|7500</x:v>
       </x:c>
       <x:c r="H146" s="14" t="str">
-        <x:v>Tjänstepension till anställd leder till scope-prövning|Företagarens egen pensionspremie bokförs inte som vanlig personalkostnad på 7400</x:v>
+        <x:v>Lön till anställd innebär scope-prövning|Företagarens privata uttag bokförs mot eget kapital och inte på 7000</x:v>
       </x:c>
       <x:c r="I146" s="14" t="str">
-        <x:v>Egen pension och tjänstepension till anställd följer olika flöden|Pension till anställd ligger utanför standardtjänsten</x:v>
+        <x:v>Företagaren kan inte vara anställd i sin egen enskilda firma|Verklig lönehantering ligger utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="J146" s="14" t="str">
-        <x:v>pensionskostnad|tjänstepension|egen pension|R38|R39|särskild löneskatt|R7</x:v>
+        <x:v>lön|bruttolön|anställd|löneutbetalning|arbetsgivardeklaration|AGI|R7</x:v>
       </x:c>
       <x:c r="K146" s="14" t="str">
-        <x:v>7500|2730|2013|7000|6310</x:v>
+        <x:v>2710|2730|7300|7400|7500|7600|1930|2900</x:v>
       </x:c>
       <x:c r="L146" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 7400, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.9, 3.18 och 7.5–7.7|Skatteverket – Kostnader i enskild näringsverksamhet, Avdrag för egna pensionskostnader, kontrollerat 2026-07-30|Skatteverket – Skattemässiga justeringar R38 och R39, kontrollerat 2026-07-30</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 7000, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkt 3.9 om företagarens egna uttag och punkterna 3.18 och 7.5–7.7|Skatteverket – Lön och egna uttag, kontrollerat 2026-07-30|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikationer och sidoordnad lönebokföring</x:v>
       </x:c>
       <x:c r="M146" s="14" t="str">
-        <x:v>Varje bokning på 7400|Det är oklart vem pensionen avser eller pensionsavtal saknas</x:v>
+        <x:v>Varje bokning på 7000|Mottagare, anställningsförhållande, löneunderlag eller AGI saknas</x:v>
       </x:c>
       <x:c r="N146" s="14" t="str">
         <x:v>active</x:v>
@@ -8046,43 +8050,43 @@
     </x:row>
     <x:row r="147" ht="430" customHeight="1">
       <x:c r="A147" s="14" t="str">
-        <x:v>7500</x:v>
+        <x:v>7300</x:v>
       </x:c>
       <x:c r="B147" s="14" t="str">
-        <x:v>Sociala och andra avgifter enligt lag och avtal</x:v>
+        <x:v>Kostnadsersättningar och förmåner</x:v>
       </x:c>
       <x:c r="C147" s="14" t="str">
-        <x:v>Tekniskt importkonto på R7 för arbetsgivaravgifter och andra avgifter för anställda. En förekomst ska stoppa standardflödet.</x:v>
+        <x:v>Tekniskt importkonto på R7 för kostnadsersättningar och förmåner till anställda. En förekomst ska stoppa standardflödet och utredas.</x:v>
       </x:c>
       <x:c r="D147" s="14" t="str">
-        <x:v>En importerad SIE-fil innehåller bokning på 7500 och avgiftstyp samt underlag behöver fastställas</x:v>
+        <x:v>En importerad SIE-fil innehåller bokning på 7300 och mottagare samt ersättningstyp behöver fastställas</x:v>
       </x:c>
       <x:c r="E147" s="14" t="str">
-        <x:v>Företagarens egna egenavgifter|Systemet ska beräkna arbetsgivaravgifter eller personalavgifter</x:v>
+        <x:v>Företagarens egen resa eller privatbilsschablon|En vanlig företagskostnad som betalats direkt av firman|Systemet ska skapa kostnadsersättning till anställd</x:v>
       </x:c>
       <x:c r="F147" s="14" t="str">
-        <x:v>Flagga varje bokning på 7500 för manuell granskning|Begär löneunderlag, arbetsgivardeklaration och beräkning av avgiften|Sätt ärendet till väntar på underlag|Om posten avser anställd eller tjänstepension till anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten avser företagarens egna avgifter eller är felbokad: flytta den till korrekt deklarations- eller egetkapitalflöde</x:v>
+        <x:v>Flagga varje bokning på 7300 för manuell granskning|Begär uppgift om mottagare, reseräkning eller förmånsunderlag och eventuell arbetsgivardeklaration|Sätt ärendet till väntar på underlag|Om posten avser anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten avser företagaren eller en vanlig företagskostnad: flytta den till rätt rese-, bil-, kostnads- eller egetkapitalkonto</x:v>
       </x:c>
       <x:c r="G147" s="14" t="str">
-        <x:v>2730|7000|7300|7400|1930|2012</x:v>
+        <x:v>1930|2710|2730|7000|7500|2013</x:v>
       </x:c>
       <x:c r="H147" s="14" t="str">
-        <x:v>Importerad arbetsgivaravgift leder till scope-prövning|Företagarens egna egenavgifter bokförs inte som arbetsgivaravgift på 7500</x:v>
+        <x:v>Importerad kostnadsersättning till anställd leder till scope-prövning|Företagarens egen bilersättning hanteras genom företagets särskilda privatbilsflöde och inte på 7300</x:v>
       </x:c>
       <x:c r="I147" s="14" t="str">
-        <x:v>Kontot ska inte användas för företagarens egenavgifter|Verkliga personalavgifter ligger utanför standardtjänsten</x:v>
+        <x:v>Kontot ska inte användas för företagarens egna resor|Verkliga förmåner eller ersättningar till anställda ligger utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="J147" s="14" t="str">
-        <x:v>arbetsgivaravgift|sociala avgifter|särskild löneskatt|AGI|2730|R7</x:v>
+        <x:v>kostnadsersättning|förmån|traktamente|milersättning|tjänsteresa|AGI|R7</x:v>
       </x:c>
       <x:c r="K147" s="14" t="str">
-        <x:v>7000|7300|7400|2730|2710|2012</x:v>
+        <x:v>7000|7500|7600|5618|5800|2710|2730</x:v>
       </x:c>
       <x:c r="L147" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7500, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Arbetsgivaravgifter 2026, kontrollerat 2026-07-30|Skatteverket – Särskild löneskatt på pensionskostnader 2026</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 7300, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Traktamente och bilersättning, inkomstår 2026, kontrollerat 2026-07-30</x:v>
       </x:c>
       <x:c r="M147" s="14" t="str">
-        <x:v>Varje bokning på 7500|Avgiftstyp, löneunderlag, AGI eller beräkning saknas</x:v>
+        <x:v>Varje bokning på 7300|Mottagare, reseräkning, förmånsunderlag eller AGI saknas</x:v>
       </x:c>
       <x:c r="N147" s="14" t="str">
         <x:v>active</x:v>
@@ -8095,43 +8099,43 @@
     </x:row>
     <x:row r="148" ht="430" customHeight="1">
       <x:c r="A148" s="14" t="str">
-        <x:v>7600</x:v>
+        <x:v>7400</x:v>
       </x:c>
       <x:c r="B148" s="14" t="str">
-        <x:v>Övriga personalkostnader</x:v>
+        <x:v>Pensionskostnader</x:v>
       </x:c>
       <x:c r="C148" s="14" t="str">
-        <x:v>Tekniskt importkonto på R7 för övriga kostnader som faktiskt avser anställda. En förekomst ska granskas eftersom standardkunden saknar anställda.</x:v>
+        <x:v>Tekniskt importkonto på R7 för pensionskostnader avseende anställda. Företagarens egen pension ska hanteras separat och kontot ska alltid granskas.</x:v>
       </x:c>
       <x:c r="D148" s="14" t="str">
-        <x:v>En importerad SIE-fil innehåller bokning på 7600 och mottagare samt kostnadstyp behöver fastställas</x:v>
+        <x:v>En importerad SIE-fil innehåller bokning på 7400 och det behöver fastställas vem pensionen avser</x:v>
       </x:c>
       <x:c r="E148" s="14" t="str">
-        <x:v>Företagarens egen friskvård eller privata kostnad|En vanlig företagskostnad som hör hemma på ett annat kostnadskonto|Systemet ska skapa en ny personalkostnad</x:v>
+        <x:v>Företagarens eget pensionssparande som vanlig personalkostnad|Privat sparande eller försäkring utan verifierad pensionsbehandling|Systemet ska skapa en ny tjänstepensionspost</x:v>
       </x:c>
       <x:c r="F148" s="14" t="str">
-        <x:v>Flagga varje bokning på 7600 för manuell granskning|Begär underlag med mottagare, kostnadstyp och affärsmässigt syfte|Sätt ärendet till väntar på underlag|Om kostnaden avser anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om kostnaden avser företagaren, är privat eller hör till annan kostnadstyp: flytta den till rätt konto eller eget kapital</x:v>
+        <x:v>Flagga varje bokning på 7400 för manuell granskning|Begär pensionsavtal, uppgift om försäkrad person, premieperiod och betalningsunderlag|Sätt ärendet till väntar på underlag|Om pensionen avser anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om pensionen avser företagaren: bokför betalningen enligt egetkapitalflödet och hantera eventuellt avdrag separat i NE</x:v>
       </x:c>
       <x:c r="G148" s="14" t="str">
-        <x:v>2440|1930|2641|7300|7500|2730</x:v>
+        <x:v>2440|1930|7500|2730|2013</x:v>
       </x:c>
       <x:c r="H148" s="14" t="str">
-        <x:v>Importerad friskvård för anställd leder till scope-prövning|Företagarens eget gymkort är normalt privat och bokförs inte på 7600</x:v>
+        <x:v>Tjänstepension till anställd leder till scope-prövning|Företagarens egen pensionspremie bokförs inte som vanlig personalkostnad på 7400</x:v>
       </x:c>
       <x:c r="I148" s="14" t="str">
-        <x:v>7600 får inte användas som restkonto|Företagarens privata kostnader är inte personalkostnader|Verkliga kostnader för anställda ligger utanför standardtjänsten</x:v>
+        <x:v>Egen pension och tjänstepension till anställd följer olika flöden|Pension till anställd ligger utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="J148" s="14" t="str">
-        <x:v>övrig personalkostnad|friskvård|personalvård|utbildning|rekrytering|personalgåva|R7</x:v>
+        <x:v>pensionskostnad|tjänstepension|egen pension|R38|R39|särskild löneskatt|R7</x:v>
       </x:c>
       <x:c r="K148" s="14" t="str">
-        <x:v>7000|7300|7400|7500|7631|7632|2730|2641</x:v>
+        <x:v>7500|2730|2013|7000|6310</x:v>
       </x:c>
       <x:c r="L148" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7600, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Personalvårdsförmån, motion och friskvård, kontrollerat 2026-07-30|Skatteverket – Gåvor till anställda 2026|Skatteverket – Avdragslexikon för företag, egen friskvård i enskild firma</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 7, konto 7400, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.9, 3.18 och 7.5–7.7|Skatteverket – Kostnader i enskild näringsverksamhet, Avdrag för egna pensionskostnader, kontrollerat 2026-07-30|Skatteverket – Skattemässiga justeringar R38 och R39, kontrollerat 2026-07-30</x:v>
       </x:c>
       <x:c r="M148" s="14" t="str">
-        <x:v>Varje bokning på 7600|Mottagare, kostnadstyp eller affärsmässigt syfte saknas</x:v>
+        <x:v>Varje bokning på 7400|Det är oklart vem pensionen avser eller pensionsavtal saknas</x:v>
       </x:c>
       <x:c r="N148" s="14" t="str">
         <x:v>active</x:v>
@@ -8144,43 +8148,43 @@
     </x:row>
     <x:row r="149" ht="430" customHeight="1">
       <x:c r="A149" s="14" t="str">
-        <x:v>7631</x:v>
+        <x:v>7500</x:v>
       </x:c>
       <x:c r="B149" s="14" t="str">
-        <x:v>Personalrepresentation, avdragsgill</x:v>
+        <x:v>Sociala och andra avgifter enligt lag och avtal</x:v>
       </x:c>
       <x:c r="C149" s="14" t="str">
-        <x:v>Tekniskt importkonto på R7 för avdragsgill del av personalrepresentation. Varje förekomst ska stoppa standardflödet eftersom Enkla Boksluts kunder ska sakna anställda.</x:v>
+        <x:v>Tekniskt importkonto på R7 för arbetsgivaravgifter och andra avgifter för anställda. En förekomst ska stoppa standardflödet.</x:v>
       </x:c>
       <x:c r="D149" s="14" t="str">
-        <x:v>En importerad SIE-fil innehåller bokning på 7631 och posten behöver utredas</x:v>
+        <x:v>En importerad SIE-fil innehåller bokning på 7500 och avgiftstyp samt underlag behöver fastställas</x:v>
       </x:c>
       <x:c r="E149" s="14" t="str">
-        <x:v>Systemet ska skapa intern representation eller personalfest automatiskt|Representationen avser företagaren själv eller externa affärskontakter|Kunden saknar anställda och posten är felklassificerad</x:v>
+        <x:v>Företagarens egna egenavgifter|Systemet ska beräkna arbetsgivaravgifter eller personalavgifter</x:v>
       </x:c>
       <x:c r="F149" s="14" t="str">
-        <x:v>Flagga varje bokning på 7631 för manuell kund- och scope-prövning|Begär deltagarlista, program, syfte, datum, plats och beräkning av avdragsgill del och moms|Sätt ärendet till väntar på underlag|Om posten avser anställda: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten är felklassificerad: flytta den till rätt representations-, privat- eller kostnadskonto innan godkännande</x:v>
+        <x:v>Flagga varje bokning på 7500 för manuell granskning|Begär löneunderlag, arbetsgivardeklaration och beräkning av avgiften|Sätt ärendet till väntar på underlag|Om posten avser anställd eller tjänstepension till anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten avser företagarens egna avgifter eller är felbokad: flytta den till korrekt deklarations- eller egetkapitalflöde</x:v>
       </x:c>
       <x:c r="G149" s="14" t="str">
-        <x:v>2440|1930|2641|7632</x:v>
+        <x:v>2730|7000|7300|7400|1930|2012</x:v>
       </x:c>
       <x:c r="H149" s="14" t="str">
-        <x:v>Importerad personalrepresentation leder till scope-prövning|Extern representation prövas mot 6070–6072 och inte 7631</x:v>
+        <x:v>Importerad arbetsgivaravgift leder till scope-prövning|Företagarens egna egenavgifter bokförs inte som arbetsgivaravgift på 7500</x:v>
       </x:c>
       <x:c r="I149" s="14" t="str">
-        <x:v>Kontot ska aldrig aktivera automatisk personalrepresentation|Verklig intern representation förutsätter normalt anställda och ligger utanför standardtjänsten</x:v>
+        <x:v>Kontot ska inte användas för företagarens egenavgifter|Verkliga personalavgifter ligger utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="J149" s="14" t="str">
-        <x:v>personalrepresentation|intern representation|personalfest|enklare förtäring|kringkostnad|R7</x:v>
+        <x:v>arbetsgivaravgift|sociala avgifter|särskild löneskatt|AGI|2730|R7</x:v>
       </x:c>
       <x:c r="K149" s="14" t="str">
-        <x:v>7632|6071|6072|7600|2641</x:v>
+        <x:v>7000|7300|7400|2730|2710|2012</x:v>
       </x:c>
       <x:c r="L149" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7631, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverkets rättsliga vägledning 2026 om intern representation och personalfest|Skatteverket – Avdrag för moms vid representation</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7500, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Arbetsgivaravgifter 2026, kontrollerat 2026-07-30|Skatteverket – Särskild löneskatt på pensionskostnader 2026</x:v>
       </x:c>
       <x:c r="M149" s="14" t="str">
-        <x:v>Varje bokning på 7631|Deltagare, anställningsrelation, program eller beräkning saknas</x:v>
+        <x:v>Varje bokning på 7500|Avgiftstyp, löneunderlag, AGI eller beräkning saknas</x:v>
       </x:c>
       <x:c r="N149" s="14" t="str">
         <x:v>active</x:v>
@@ -8193,43 +8197,43 @@
     </x:row>
     <x:row r="150" ht="430" customHeight="1">
       <x:c r="A150" s="14" t="str">
-        <x:v>7632</x:v>
+        <x:v>7600</x:v>
       </x:c>
       <x:c r="B150" s="14" t="str">
-        <x:v>Personalrepresentation, ej avdragsgill</x:v>
+        <x:v>Övriga personalkostnader</x:v>
       </x:c>
       <x:c r="C150" s="14" t="str">
-        <x:v>Tekniskt importkonto på R7 för ej avdragsgill del av personalrepresentation. Varje förekomst ska stoppa standardflödet eftersom Enkla Boksluts kunder ska sakna anställda.</x:v>
+        <x:v>Tekniskt importkonto på R7 för övriga kostnader som faktiskt avser anställda. En förekomst ska granskas eftersom standardkunden saknar anställda.</x:v>
       </x:c>
       <x:c r="D150" s="14" t="str">
-        <x:v>En importerad SIE-fil innehåller bokning på 7632 och posten behöver utredas</x:v>
+        <x:v>En importerad SIE-fil innehåller bokning på 7600 och mottagare samt kostnadstyp behöver fastställas</x:v>
       </x:c>
       <x:c r="E150" s="14" t="str">
-        <x:v>Systemet ska skapa intern representation eller personalfest automatiskt|Kostnaden är privat utan koppling till anställda|Representationen avser externa affärskontakter</x:v>
+        <x:v>Företagarens egen friskvård eller privata kostnad|En vanlig företagskostnad som hör hemma på ett annat kostnadskonto|Systemet ska skapa en ny personalkostnad</x:v>
       </x:c>
       <x:c r="F150" s="14" t="str">
-        <x:v>Flagga varje bokning på 7632 för manuell kund- och scope-prövning|Begär deltagarlista, program, syfte, datum, plats och underlag för kostnad och moms|Sätt ärendet till väntar på underlag|Om posten avser anställda: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten är privat eller felklassificerad: flytta den till eget uttag eller rätt konto innan godkännande</x:v>
+        <x:v>Flagga varje bokning på 7600 för manuell granskning|Begär underlag med mottagare, kostnadstyp och affärsmässigt syfte|Sätt ärendet till väntar på underlag|Om kostnaden avser anställd: markera kunden som utanför standardtjänsten och föreslå eskalering|Om kostnaden avser företagaren, är privat eller hör till annan kostnadstyp: flytta den till rätt konto eller eget kapital</x:v>
       </x:c>
       <x:c r="G150" s="14" t="str">
-        <x:v>2440|1930|2641|7631|2013|7300</x:v>
+        <x:v>2440|1930|2641|7300|7500|2730</x:v>
       </x:c>
       <x:c r="H150" s="14" t="str">
-        <x:v>Importerad ej avdragsgill personalrepresentation leder till scope-prövning|Privat måltid bokförs som eget uttag och inte på 7632</x:v>
+        <x:v>Importerad friskvård för anställd leder till scope-prövning|Företagarens eget gymkort är normalt privat och bokförs inte på 7600</x:v>
       </x:c>
       <x:c r="I150" s="14" t="str">
-        <x:v>Kontot ska aldrig aktivera automatisk personalrepresentation|Ej avdragsgill betyder inte att en privat kostnad får bokföras som verksamhetskostnad|Verklig intern representation ligger utanför standardtjänsten</x:v>
+        <x:v>7600 får inte användas som restkonto|Företagarens privata kostnader är inte personalkostnader|Verkliga kostnader för anställda ligger utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="J150" s="14" t="str">
-        <x:v>ej avdragsgill personalrepresentation|personalmiddag|personalfest|skattemässig återläggning|NE sid 2|R7</x:v>
+        <x:v>övrig personalkostnad|friskvård|personalvård|utbildning|rekrytering|personalgåva|R7</x:v>
       </x:c>
       <x:c r="K150" s="14" t="str">
-        <x:v>7631|6072|7300|7500|2641|2013</x:v>
+        <x:v>7000|7300|7400|7500|7631|7632|2730|2641</x:v>
       </x:c>
       <x:c r="L150" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7632, rad R7 och NE sidan 2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverkets rättsliga vägledning 2026 om intern representation och personalfest|Skatteverket – Avdrag för moms vid representation</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7600, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverket – Personalvårdsförmån, motion och friskvård, kontrollerat 2026-07-30|Skatteverket – Gåvor till anställda 2026|Skatteverket – Avdragslexikon för företag, egen friskvård i enskild firma</x:v>
       </x:c>
       <x:c r="M150" s="14" t="str">
-        <x:v>Varje bokning på 7632|Deltagare, anställningsrelation, program, affärssamband eller momsunderlag saknas</x:v>
+        <x:v>Varje bokning på 7600|Mottagare, kostnadstyp eller affärsmässigt syfte saknas</x:v>
       </x:c>
       <x:c r="N150" s="14" t="str">
         <x:v>active</x:v>
@@ -8242,199 +8246,197 @@
     </x:row>
     <x:row r="151" ht="430" customHeight="1">
       <x:c r="A151" s="14" t="str">
-        <x:v>7700</x:v>
+        <x:v>7631</x:v>
       </x:c>
       <x:c r="B151" s="14" t="str">
-        <x:v>Nedskrivningar</x:v>
+        <x:v>Personalrepresentation, avdragsgill</x:v>
       </x:c>
       <x:c r="C151" s="14" t="str">
-        <x:v>Kostnadskonto för nedskrivning av anläggningstillgångar när deras redovisade värde måste sänkas på grund av en tydlig och betydande värdenedgång. Kostnaden redovisas på R9 eller R10 beroende på tillgångsslag.</x:v>
+        <x:v>Tekniskt importkonto på R7 för avdragsgill del av personalrepresentation. Varje förekomst ska stoppa standardflödet eftersom Enkla Boksluts kunder ska sakna anställda.</x:v>
       </x:c>
       <x:c r="D151" s="14" t="str">
-        <x:v>Det finns en dokumenterad värdenedgång som omfattas av K1:s nedskrivningsregler|Byggnad, markanläggning eller mark ska prövas enligt punkt 6.17 eller 6.28|Maskiner, inventarier och förvärvade immateriella tillgångar har inte skrivits av med högsta tillåtna belopp och gruppens ekonomiska värde är betydligt lägre än bokfört värde</x:v>
+        <x:v>En importerad SIE-fil innehåller bokning på 7631 och posten behöver utredas</x:v>
       </x:c>
       <x:c r="E151" s="14" t="str">
-        <x:v>Värdeminskningen är ordinarie avskrivning; använd 7810, 7820 eller 7830|Tillgången har sålts eller utrangerats; pröva 7970 och tillgångskontot|Mindre eller tillfällig marknadssvängning utan stöd för nedskrivning|Maskiner och inventarier har skrivits av med högsta tillåtna belopp varje år och ingen annan K1-regel kräver nedskrivning|Värderingsunderlag eller tillgångsgrupp saknas</x:v>
+        <x:v>Systemet ska skapa intern representation eller personalfest automatiskt|Representationen avser företagaren själv eller externa affärskontakter|Kunden saknar anställda och posten är felklassificerad</x:v>
       </x:c>
       <x:c r="F151" s="14" t="str">
-        <x:v>Identifiera tillgångsslag, bokfört värde, tidigare avskrivningar och värderingstidpunkt|Skilj ordinarie avskrivning, utrangering och nedskrivning|För maskiner, inventarier och förvärvade immateriella tillgångar: gör bedömningen kollektivt enligt K1 punkt 6.40|En värdeminskning på mindre än 10 procent behöver enligt kommentaren till punkt 6.40 inte beaktas|Beräkna gruppens återstående ekonomiska värde och nedskrivningsbelopp|För byggnad, markanläggning och mark: dokumentera tillämplig bedömning enligt punkt 6.17 och koppla till respektive tillgång|Bokför kostnaden på 7700 mot fastställt balanskonto eller ackumulerat värdeminskningskonto|Redovisa kostnaden på R9 för byggnader och markanläggningar och på R10 för maskiner, inventarier och immateriella tillgångar|Uppdatera förteckningen över anläggningstillgångar och dokumentera eventuell senare återföring|Kräv alltid manuell granskning|Kontrollera först om högsta tillåtna skattemässiga avskrivning har gjorts varje år|Om den har gjorts ska ingen nedskrivningsgranskning enligt punkt 6.40 utlösas för denna grupp|Om den inte har gjorts: jämför gruppens dokumenterade ekonomiska värde med bokfört värde|Utlös manuell granskning först vid möjlig värdenedgång på minst 10 procent; bokför aldrig nedskrivning automatiskt|Använd aldrig automatiskt|Kräv dokumenterad skade-, marknads- eller värderingshändelse|Skilj särskild värdenedgång från ordinarie avskrivning|Flagga varje föreslagen eller importerad bokning på 7700 och begär tillgångsförteckning, skade- eller värderingsunderlag, bokfört värde och tidigare avskrivningar|Sätt ärendet till väntar på underlag tills ordinarie avskrivning, utrangering och verklig nedskrivning har skilts åt och tillgångsgruppen är verifierad|Godkänn aldrig en nedskrivning automatiskt; belopp, motkonto, presentationsrad och eventuell återföring kräver manuell bedömning|Föreslå ordinarie avskrivning, utrangering, rättelse eller scope-eskalering när värdenedgången inte är tydlig, betydande och dokumenterad</x:v>
+        <x:v>Flagga varje bokning på 7631 för manuell kund- och scope-prövning|Begär deltagarlista, program, syfte, datum, plats och beräkning av avdragsgill del och moms|Sätt ärendet till väntar på underlag|Om posten avser anställda: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten är felklassificerad: flytta den till rätt representations-, privat- eller kostnadskonto innan godkännande</x:v>
       </x:c>
       <x:c r="G151" s="14" t="str">
-        <x:v>1009|1119|1130|1159|1229|1239|1249</x:v>
+        <x:v>2440|1930|2641|7632</x:v>
       </x:c>
       <x:c r="H151" s="14" t="str">
-        <x:v>En kollektiv nedskrivning av maskiner och förvärvade immateriella tillgångar bokförs på 7700 när gruppens dokumenterade ekonomiska värde betydligt understiger bokfört värde och övriga villkor är uppfyllda</x:v>
+        <x:v>Importerad personalrepresentation leder till scope-prövning|Extern representation prövas mot 6070–6072 och inte 7631</x:v>
       </x:c>
       <x:c r="I151" s="14" t="str">
-        <x:v>Nedskrivning är inte samma sak som ordinarie avskrivning|K1:s inventariebedömning sker kollektivt|Mindre än 10 procents värdenedgång behöver inte beaktas enligt kommentaren till 6.40|Byggnader, mark och inventarier följer olika nedskrivningsregler|10 procent är endast en granskningsgräns; nedskrivning kräver alltid dokumenterad bedömning|Kollektiv gruppindelning och återföringskonto är ännu inte fullt verifierade</x:v>
+        <x:v>Kontot ska aldrig aktivera automatisk personalrepresentation|Verklig intern representation förutsätter normalt anställda och ligger utanför standardtjänsten</x:v>
       </x:c>
       <x:c r="J151" s="14" t="str">
-        <x:v>nedskrivning|värdenedgång|återstående ekonomiskt värde|kollektiv bedömning|R9|R10</x:v>
+        <x:v>personalrepresentation|intern representation|personalfest|enklare förtäring|kringkostnad|R7</x:v>
       </x:c>
       <x:c r="K151" s="14" t="str">
-        <x:v>1009|1110|1119|1130|1150|1159|1220|1229|1230|1239|1240|1249|7810|7820|7830|7970</x:v>
+        <x:v>7632|6071|6072|7600|2641</x:v>
       </x:c>
       <x:c r="L151" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7700, rad R9 alternativt R10|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.17, 6.28, 6.39–6.40 och 7.12|K1-vägledningens kommentar till punkt 6.40 om kollektiv bedömning och värdenedgång under 10 procent</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7631, rad R7|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverkets rättsliga vägledning 2026 om intern representation och personalfest|Skatteverket – Avdrag för moms vid representation</x:v>
       </x:c>
       <x:c r="M151" s="14" t="str">
-        <x:v>Tillgångsslag eller motkonto är inte fastställt|Värderingsunderlag saknas|Det är oklart om händelsen är avskrivning, nedskrivning eller utrangering|Kollektiv värdering eller tidigare avskrivningar är inte verifierade|Återföring kan vara aktuell|Nedskrivning, återföring eller kollektiv värdering aktualiseras</x:v>
+        <x:v>Varje bokning på 7631|Deltagare, anställningsrelation, program eller beräkning saknas</x:v>
       </x:c>
       <x:c r="N151" s="14" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O151" s="14" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P151" s="14" t="str">
-        <x:v>impairment_review_threshold_10_percent</x:v>
-      </x:c>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P151" s="14" t="str"/>
       <x:c r="Q151" s="12" t="str"/>
     </x:row>
     <x:row r="152" ht="430" customHeight="1">
       <x:c r="A152" s="14" t="str">
+        <x:v>7632</x:v>
+      </x:c>
+      <x:c r="B152" s="14" t="str">
+        <x:v>Personalrepresentation, ej avdragsgill</x:v>
+      </x:c>
+      <x:c r="C152" s="14" t="str">
+        <x:v>Tekniskt importkonto på R7 för ej avdragsgill del av personalrepresentation. Varje förekomst ska stoppa standardflödet eftersom Enkla Boksluts kunder ska sakna anställda.</x:v>
+      </x:c>
+      <x:c r="D152" s="14" t="str">
+        <x:v>En importerad SIE-fil innehåller bokning på 7632 och posten behöver utredas</x:v>
+      </x:c>
+      <x:c r="E152" s="14" t="str">
+        <x:v>Systemet ska skapa intern representation eller personalfest automatiskt|Kostnaden är privat utan koppling till anställda|Representationen avser externa affärskontakter</x:v>
+      </x:c>
+      <x:c r="F152" s="14" t="str">
+        <x:v>Flagga varje bokning på 7632 för manuell kund- och scope-prövning|Begär deltagarlista, program, syfte, datum, plats och underlag för kostnad och moms|Sätt ärendet till väntar på underlag|Om posten avser anställda: markera kunden som utanför standardtjänsten och föreslå eskalering|Om posten är privat eller felklassificerad: flytta den till eget uttag eller rätt konto innan godkännande</x:v>
+      </x:c>
+      <x:c r="G152" s="14" t="str">
+        <x:v>2440|1930|2641|7631|2013|7300</x:v>
+      </x:c>
+      <x:c r="H152" s="14" t="str">
+        <x:v>Importerad ej avdragsgill personalrepresentation leder till scope-prövning|Privat måltid bokförs som eget uttag och inte på 7632</x:v>
+      </x:c>
+      <x:c r="I152" s="14" t="str">
+        <x:v>Kontot ska aldrig aktivera automatisk personalrepresentation|Ej avdragsgill betyder inte att en privat kostnad får bokföras som verksamhetskostnad|Verklig intern representation ligger utanför standardtjänsten</x:v>
+      </x:c>
+      <x:c r="J152" s="14" t="str">
+        <x:v>ej avdragsgill personalrepresentation|personalmiddag|personalfest|skattemässig återläggning|NE sid 2|R7</x:v>
+      </x:c>
+      <x:c r="K152" s="14" t="str">
+        <x:v>7631|6072|7300|7500|2641|2013</x:v>
+      </x:c>
+      <x:c r="L152" s="14" t="str">
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7632, rad R7 och NE sidan 2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.18 och 7.5–7.7|Skatteverkets rättsliga vägledning 2026 om intern representation och personalfest|Skatteverket – Avdrag för moms vid representation</x:v>
+      </x:c>
+      <x:c r="M152" s="14" t="str">
+        <x:v>Varje bokning på 7632|Deltagare, anställningsrelation, program, affärssamband eller momsunderlag saknas</x:v>
+      </x:c>
+      <x:c r="N152" s="14" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="O152" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P152" s="14" t="str"/>
+      <x:c r="Q152" s="12" t="str"/>
+    </x:row>
+    <x:row r="153" ht="430" customHeight="1">
+      <x:c r="A153" s="14" t="str">
+        <x:v>7700</x:v>
+      </x:c>
+      <x:c r="B153" s="14" t="str">
+        <x:v>Nedskrivningar</x:v>
+      </x:c>
+      <x:c r="C153" s="14" t="str">
+        <x:v>Kostnadskonto för nedskrivning av anläggningstillgångar när deras redovisade värde måste sänkas på grund av en tydlig och betydande värdenedgång. Kostnaden redovisas på R9 eller R10 beroende på tillgångsslag.</x:v>
+      </x:c>
+      <x:c r="D153" s="14" t="str">
+        <x:v>Det finns en dokumenterad värdenedgång som omfattas av K1:s nedskrivningsregler|Byggnad, markanläggning eller mark ska prövas enligt punkt 6.17 eller 6.28|Maskiner, inventarier och förvärvade immateriella tillgångar har inte skrivits av med högsta tillåtna belopp och gruppens ekonomiska värde är betydligt lägre än bokfört värde</x:v>
+      </x:c>
+      <x:c r="E153" s="14" t="str">
+        <x:v>Värdeminskningen är ordinarie avskrivning; använd 7810, 7820 eller 7830|Tillgången har sålts eller utrangerats; pröva 7970 och tillgångskontot|Mindre eller tillfällig marknadssvängning utan stöd för nedskrivning|Maskiner och inventarier har skrivits av med högsta tillåtna belopp varje år och ingen annan K1-regel kräver nedskrivning|Värderingsunderlag eller tillgångsgrupp saknas</x:v>
+      </x:c>
+      <x:c r="F153" s="14" t="str">
+        <x:v>Identifiera tillgångsslag, bokfört värde, tidigare avskrivningar och värderingstidpunkt|Skilj ordinarie avskrivning, utrangering och nedskrivning|För maskiner, inventarier och förvärvade immateriella tillgångar: gör bedömningen kollektivt enligt K1 punkt 6.40|En värdeminskning på mindre än 10 procent behöver enligt kommentaren till punkt 6.40 inte beaktas|Beräkna gruppens återstående ekonomiska värde och nedskrivningsbelopp|För byggnad, markanläggning och mark: dokumentera tillämplig bedömning enligt punkt 6.17 och koppla till respektive tillgång|Bokför kostnaden på 7700 mot fastställt balanskonto eller ackumulerat värdeminskningskonto|Redovisa kostnaden på R9 för byggnader och markanläggningar och på R10 för maskiner, inventarier och immateriella tillgångar|Uppdatera förteckningen över anläggningstillgångar och dokumentera eventuell senare återföring|Kräv alltid manuell granskning|Kontrollera först om högsta tillåtna skattemässiga avskrivning har gjorts varje år|Om den har gjorts ska ingen nedskrivningsgranskning enligt punkt 6.40 utlösas för denna grupp|Om den inte har gjorts: jämför gruppens dokumenterade ekonomiska värde med bokfört värde|Utlös manuell granskning först vid möjlig värdenedgång på minst 10 procent; bokför aldrig nedskrivning automatiskt|Använd aldrig automatiskt|Kräv dokumenterad skade-, marknads- eller värderingshändelse|Skilj särskild värdenedgång från ordinarie avskrivning|Flagga varje föreslagen eller importerad bokning på 7700 och begär tillgångsförteckning, skade- eller värderingsunderlag, bokfört värde och tidigare avskrivningar|Sätt ärendet till väntar på underlag tills ordinarie avskrivning, utrangering och verklig nedskrivning har skilts åt och tillgångsgruppen är verifierad|Godkänn aldrig en nedskrivning automatiskt; belopp, motkonto, presentationsrad och eventuell återföring kräver manuell bedömning|Föreslå ordinarie avskrivning, utrangering, rättelse eller scope-eskalering när värdenedgången inte är tydlig, betydande och dokumenterad</x:v>
+      </x:c>
+      <x:c r="G153" s="14" t="str">
+        <x:v>1009|1119|1130|1159|1229|1239|1249</x:v>
+      </x:c>
+      <x:c r="H153" s="14" t="str">
+        <x:v>En kollektiv nedskrivning av maskiner och förvärvade immateriella tillgångar bokförs på 7700 när gruppens dokumenterade ekonomiska värde betydligt understiger bokfört värde och övriga villkor är uppfyllda</x:v>
+      </x:c>
+      <x:c r="I153" s="14" t="str">
+        <x:v>Nedskrivning är inte samma sak som ordinarie avskrivning|K1:s inventariebedömning sker kollektivt|Mindre än 10 procents värdenedgång behöver inte beaktas enligt kommentaren till 6.40|Byggnader, mark och inventarier följer olika nedskrivningsregler|10 procent är endast en granskningsgräns; nedskrivning kräver alltid dokumenterad bedömning|Kollektiv gruppindelning och återföringskonto är ännu inte fullt verifierade</x:v>
+      </x:c>
+      <x:c r="J153" s="14" t="str">
+        <x:v>nedskrivning|värdenedgång|återstående ekonomiskt värde|kollektiv bedömning|R9|R10</x:v>
+      </x:c>
+      <x:c r="K153" s="14" t="str">
+        <x:v>1009|1110|1119|1130|1150|1159|1220|1229|1230|1239|1240|1249|7810|7820|7830|7970</x:v>
+      </x:c>
+      <x:c r="L153" s="14" t="str">
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7700, rad R9 alternativt R10|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.17, 6.28, 6.39–6.40 och 7.12|K1-vägledningens kommentar till punkt 6.40 om kollektiv bedömning och värdenedgång under 10 procent</x:v>
+      </x:c>
+      <x:c r="M153" s="14" t="str">
+        <x:v>Tillgångsslag eller motkonto är inte fastställt|Värderingsunderlag saknas|Det är oklart om händelsen är avskrivning, nedskrivning eller utrangering|Kollektiv värdering eller tidigare avskrivningar är inte verifierade|Återföring kan vara aktuell|Nedskrivning, återföring eller kollektiv värdering aktualiseras</x:v>
+      </x:c>
+      <x:c r="N153" s="14" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="O153" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P153" s="14" t="str">
+        <x:v>impairment_review_threshold_10_percent</x:v>
+      </x:c>
+      <x:c r="Q153" s="12" t="str"/>
+    </x:row>
+    <x:row r="154" ht="430" customHeight="1">
+      <x:c r="A154" s="14" t="str">
         <x:v>7810</x:v>
       </x:c>
-      <x:c r="B152" s="14" t="str">
+      <x:c r="B154" s="14" t="str">
         <x:v>Avskrivningar på immateriella anläggningstillgångar</x:v>
       </x:c>
-      <x:c r="C152" s="14" t="str">
+      <x:c r="C154" s="14" t="str">
         <x:v>Kostnadskonto på R10 för årets avskrivning på förvärvade immateriella anläggningstillgångar som redovisas på 1000. Motkontot är normalt 1009.</x:v>
       </x:c>
-      <x:c r="D152" s="14" t="str">
+      <x:c r="D154" s="14" t="str">
         <x:v>En förvärvad immateriell anläggningstillgång finns bokförd på 1000|Årets avskrivning har beräknats enligt K1:s hänvisning till reglerna för maskiner och inventarier|Bokslutsunderlaget fastställer skillnaden mellan bokfört värde före avskrivning och värdet vid beskattningen</x:v>
       </x:c>
-      <x:c r="E152" s="14" t="str">
+      <x:c r="E154" s="14" t="str">
         <x:v>Utgiften avser anskaffning eller utveckling av en immateriell tillgång|Tillgången är internt upparbetad och får inte tas upp enligt K1|Händelsen är nedskrivning; använd 7700|Avskrivningen avser byggnad, markanläggning eller materiella inventarier|Tillgången har sålts, tagits ut eller utrangerats utan att avyttringen först har hanterats</x:v>
       </x:c>
-      <x:c r="F152" s="14" t="str">
+      <x:c r="F154" s="14" t="str">
         <x:v>Stäm av tillgångsförteckning, 1000 och 1009 vid årets ingång|Fastställ årets skattemässiga värde enligt tillämpliga regler för den förvärvade immateriella tillgången|Reglerna om direktavdrag för inventarie av mindre värde och högst tre års ekonomisk livslängd gäller inte för förvärvade immateriella tillgångar|Beräkna avskrivningen som skillnaden mellan bokfört värde före årets avskrivning och värdet som ska redovisas vid beskattningen|Om avskrivningsunderlaget före årets avskrivning är högst ett halvt prisbasbelopp får hela underlaget skrivas av när villkoren i punkt 6.38 är uppfyllda|Bokför avskrivningen i debet på 7810 och kredit på 1009|Hantera försäljning, uttag och utrangering före slutlig avskrivningsberäkning|Pröva separat nedskrivningsbehov enligt 6.40 när högsta tillåtna avskrivning inte görs|Kontrollera att nettot 1000 minus 1009 motsvarar B1 och dokumentera årsomföringen|Om högsta tillåtna avskrivning inte görs och möjlig värdenedgång uppgår till minst 10 procent ska nedskrivning granskas manuellt|Använd endast en skattemässig avskrivningsmetod som har fastställts och dokumenterats manuellt för företagets underlag|Spara anskaffningsvärde, anskaffningsår, ingångsvärde, vald metod och tidigare avskrivningar|Byt aldrig metod automatiskt och skapa inte standardprocentsatser per typ av immateriell rättighet|Använd endast med verifierad skattemässig metod för immateriell tillgång|Spara anskaffningsvärde, år, ingångsvärde, metod och tidigare avskrivningar|Vid granskningsflagga begär in tillgångsförteckning, anskaffningshandling, ingående skattemässigt värde, vald metod och tidigare avskrivningar|Sätt ärendet till väntar på underlag tills tillgången är manuellt godkänd på 1000 och avskrivningen kan stämmas av mot 1009|Godkänn 7810 endast för beräknad avskrivning enligt en dokumenterad och oförändrad skattemässig metod|Föreslå rättelse eller scope-eskalering vid egenutvecklad tillgång, metodbyte, avyttring, uttag, utrangering, nedskrivning eller okänd historik</x:v>
       </x:c>
-      <x:c r="G152" s="14" t="str">
+      <x:c r="G154" s="14" t="str">
         <x:v>1009</x:v>
       </x:c>
-      <x:c r="H152" s="14" t="str">
+      <x:c r="H154" s="14" t="str">
         <x:v>Årets avskrivning på en köpt hemsida med bestående värde bokförs i debet på 7810 och kredit på 1009</x:v>
       </x:c>
-      <x:c r="I152" s="14" t="str">
+      <x:c r="I154" s="14" t="str">
         <x:v>Endast förvärvade immateriella tillgångar får ligga till grund för avskrivning|Låg-värde- och treårsreglerna gäller inte för immateriella tillgångar|Ordinarie avskrivning och nedskrivning ska hållas isär|Skattemässig metod måste fastställas per tillgångstyp|Avskrivningsprocenten följer den verifierade skattemässiga metoden och inte kontonamnet eller typen av rättighet|Ingen automatisk procentsats per tillgångstyp|Årsomföringen mot 1000 och 1009 är ännu inte verifierad</x:v>
       </x:c>
-      <x:c r="J152" s="14" t="str">
+      <x:c r="J154" s="14" t="str">
         <x:v>avskrivning immateriell tillgång|köpt hemsida|licens|1009|skattemässigt värde|R10</x:v>
       </x:c>
-      <x:c r="K152" s="14" t="str">
+      <x:c r="K154" s="14" t="str">
         <x:v>1000|1009|7700|7970</x:v>
       </x:c>
-      <x:c r="L152" s="14" t="str">
+      <x:c r="L154" s="14" t="str">
         <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7810, rad R10|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.2–6.3, 6.37–6.40 och 7.12|K1-vägledningens exempel 6-5, 6-6 och 6-8 i tillämpliga delar</x:v>
       </x:c>
-      <x:c r="M152" s="14" t="str">
+      <x:c r="M154" s="14" t="str">
         <x:v>Tillgången kan vara internt upparbetad|Skattemässig avskrivningsmetod är inte fastställd|Tillgången har avyttrats eller tagits ut|Nedskrivning kan vara rätt åtgärd|1000 och 1009 stämmer inte med tillgångsförteckningen|Vald metod eller tidigare skattemässiga värden är inte verifierade|Historiken visar metodbyte, avvikande räkenskapsår eller ofullständig tillgångsförteckning|Ny, oklar eller metodändrad immateriell tillgång förekommer</x:v>
       </x:c>
-      <x:c r="N152" s="14" t="str">
-        <x:v>active</x:v>
-      </x:c>
-      <x:c r="O152" s="14" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P152" s="14" t="str">
-        <x:v>full_writeoff_remaining_basis_half_pbb|impairment_review_threshold_10_percent</x:v>
-      </x:c>
-      <x:c r="Q152" s="12" t="str"/>
-    </x:row>
-    <x:row r="153">
-      <x:c r="A153" t="str">
-        <x:v>7820</x:v>
-      </x:c>
-      <x:c r="B153" t="str">
-        <x:v>Avskrivningar på byggnader och markanläggningar</x:v>
-      </x:c>
-      <x:c r="C153" t="str">
-        <x:v>Kostnadskonto på R9 för årets planenliga och skattemässigt grundade avskrivning på byggnader och markanläggningar. Motkontot är normalt 1119 respektive 1159.</x:v>
-      </x:c>
-      <x:c r="D153" t="str">
-        <x:v>En byggnad som hör till företaget är bokförd på 1110|En färdigställd markanläggning är bokförd på 1150|Årets avskrivningsbelopp kan härledas till fastighets- och skatteunderlag|Tillgången har varit färdigställd och tagits i bruk</x:v>
-      </x:c>
-      <x:c r="E153" t="str">
-        <x:v>Beloppet avser mark; mark ska inte skrivas av|Utgiften är reparation eller underhåll|Tillgången är byggnads- eller markinventarie; använd 7830|Tillgången är pågående och inte färdigställd; använd 1180|Händelsen är nedskrivning eller avyttring|Avskrivningsunderlag eller tillgångsfördelning saknas</x:v>
-      </x:c>
-      <x:c r="F153" t="str">
-        <x:v>Identifiera fastighet, byggnad, markanläggning, anskaffningsvärde, färdigställandedatum och tidigare avskrivningar|Separera mark från byggnad samt byggnads- och markinventarier från byggnaden|Fastställ skattemässigt avskrivningsunderlag och tillämplig procentsats utifrån verifierad fastighetsklassificering|Beräkna årets avskrivning per byggnad och markanläggning|Bokför kostnaden i debet på 7820 och kredit på 1119 eller 1159|Stäm av nettot 1110 minus 1119 och 1150 minus 1159 mot B2 och tillgångsförteckningen|Hantera försäljning, utrangering, tillbyggnad och omklassificering före slutlig avskrivning|Kräv manuell granskning vid blandad fastighet, delavyttring, privat användning eller osäker skattemässig klass|För befintlig enkel näringsfastighet: beräkna avskrivningen med den procentsats som verifierats från föregående deklaration eller fastighetsunderlag|Vid ny byggnad eller saknad historik krävs manuell startgranskning|Komplexa byggnader, primäravdrag och flera byggnadstyper ligger utanför standardflödet|Fastställ avskrivningsunderlag och procentsats per fastighet från dokumenterad skattemässig klassificering|Koppla delavyttring till specificerad såld del|Vid granskningsflagga begär in fastighets- och objektsförteckning, anskaffningsvärde, färdigställandedatum, tidigare avskrivningar och verifierad skattemässig procentsats|Sätt ärendet till väntar på underlag tills 1110, 1119, 1150 och 1159 kan stämmas av per byggnad eller markanläggning|Godkänn 7820 för en enkel befintlig näringsbyggnad eller markanläggning med dokumenterad och oförändrad avskrivningsprocent|Föreslå scope-eskalering vid ny eller blandad fastighet, primäravdrag, flera byggnadstyper, delavyttring, ombyggnad eller saknad historik</x:v>
-      </x:c>
-      <x:c r="G153" t="str">
-        <x:v>1119|1159</x:v>
-      </x:c>
-      <x:c r="H153" t="str">
-        <x:v>Årets avskrivning på en färdigställd verksamhetsbyggnad debiterar 7820 och krediterar 1119|Markvärdet skrivs inte av</x:v>
-      </x:c>
-      <x:c r="I153" t="str">
-        <x:v>Mark ska alltid hållas skild från avskrivningsbar byggnad|Byggnadsinventarier och markinventarier följer inventariereglerna|Avskrivningsprocenten får inte antas från kontonamnet|Reparation och värdehöjande förbättring måste skiljas åt|En fullständig tabell över alla byggnadstyper ska inte användas automatiskt i Enkla Bokslut|Konto eller vardaglig benämning får inte ensamt styra procentsatsen</x:v>
-      </x:c>
-      <x:c r="J153" t="str">
-        <x:v>avskrivning byggnad|markanläggning|1119|1159|fastighet|R9</x:v>
-      </x:c>
-      <x:c r="K153" t="str">
-        <x:v>1110|1119|1130|1150|1159|1180|1230|1239|5100|5500|7700|7970</x:v>
-      </x:c>
-      <x:c r="L153" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7820, rad R9|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.10–6.18 och 7.12 samt exempel 6-7</x:v>
-      </x:c>
-      <x:c r="M153" t="str">
-        <x:v>Mark och byggnad är inte fördelade|Byggnadsinventarie eller markinventarie kan förekomma|Skattemässig procentsats eller underlag saknas|Tillgången har byggts om, delavyttrats eller används privat|Avskrivningen stämmer inte med tillgångsförteckningen|Historisk procentsats saknas eller byggnaden är ny|Komplex byggnadstyp eller primäravdrag förekommer|Ny fastighet, oklar historik, blandad klassificering eller delavyttring förekommer</x:v>
-      </x:c>
-      <x:c r="N153" t="str">
-        <x:v>active</x:v>
-      </x:c>
-      <x:c r="O153" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="P153" s="14"/>
-      <x:c r="Q153" s="12" t="str"/>
-    </x:row>
-    <x:row r="154">
-      <x:c r="A154" t="str">
-        <x:v>7830</x:v>
-      </x:c>
-      <x:c r="B154" t="str">
-        <x:v>Avskrivningar på maskiner och inventarier</x:v>
-      </x:c>
-      <x:c r="C154" t="str">
-        <x:v>Kostnadskonto på R10 för årets avskrivning på maskiner och inventarier, byggnads- och markinventarier samt bilar och andra transportmedel som redovisas på B4.</x:v>
-      </x:c>
-      <x:c r="D154" t="str">
-        <x:v>Ett kollektivt avskrivningsunderlag för B4 har fastställts|Årets värde vid beskattningen är verifierat|Försäljningsinkomster och årets anskaffningar har först bokförts på respektive B4-underkonto|Årets avskrivning ska bokföras mot 1229, 1239 eller 1249</x:v>
-      </x:c>
-      <x:c r="E154" t="str">
-        <x:v>Beloppet avser immateriell tillgång; använd 7810|Beloppet avser byggnad eller markanläggning; använd 7820|Utgiften får kostnadsföras direkt som inventarie av mindre värde eller med högst tre års livslängd|Händelsen är särskild nedskrivning; använd 7700|Avskrivningen beräknas fritt per enskild inventarie utan avstämning mot den kollektiva skatteregeln</x:v>
-      </x:c>
-      <x:c r="F154" t="str">
-        <x:v>Stäm av ingående B4-värden och årets nyanskaffningar på 1221, 1231 och 1241|Minska underlaget med årets försäljningsinkomster på 1222, 1232 och 1242|Fastställ värdet vid beskattningen och vald tillåten avskrivningsmetod|Beräkna avskrivningen som skillnaden mellan bokfört värde före årets avskrivning och värdet vid beskattningen|Om avskrivningsunderlaget före årets avskrivning är högst ett halvt prisbasbelopp får hela underlaget skrivas av när villkoren är uppfyllda|Fördela den bokförda avskrivningen mot 1229, 1239 och 1249 enligt fastställd systemrutin utan att ändra totalbeloppet|Stäm av B4 och R10 mot tillgångsförteckning och deklarationsunderlag|Pröva separat nedskrivning enligt 6.40 om högsta tillåtna avskrivning inte görs|Kräv manuell granskning vid metodbyte, negativt underlag, delvis privat tillgång eller avyttring|Om högsta tillåtna avskrivning inte görs och möjlig kollektiv värdenedgång uppgår till minst 10 procent ska nedskrivning granskas manuellt|Använd verifierad historisk avskrivningsmetod|Metodbyte får inte göras automatiskt|Total kollektiv avskrivning ska bevaras vid fördelning mellan underkonton|Beräkna årets avskrivning som skillnaden mellan gruppens värde före avskrivning och det verifierade kollektiva B4-värdet vid beskattningen|Bokför hela kostnaden i debet på 7830 och kreditera som standard 1229 när en tillförlitlig kategoriuppdelning saknas|Dela krediten mellan 1229, 1239 och 1249 endast när en verifierad tillgångsförteckning ger en spårbar fördelning; kostnaden på 7830 ska vara oförändrad|Sätt ärendet till väntar på underlag vid okänd metod, negativt underlag, metodbyte, avyttring, privat användning eller bristande avstämning mot B4</x:v>
-      </x:c>
-      <x:c r="G154" t="str">
-        <x:v>1229|1239|1249</x:v>
-      </x:c>
-      <x:c r="H154" t="str">
-        <x:v>Årets kollektivt beräknade inventarieavskrivning bokförs på 7830 mot B4:s avskrivningsunderkonton|En avyttring minskar först avskrivningsunderlaget genom försäljningsinkomsten</x:v>
-      </x:c>
-      <x:c r="I154" t="str">
-        <x:v>K1 kräver kollektiv värdering och avskrivning|Hela underlaget får skrivas av först när halvt-prisbasbeloppsregeln är uppfylld|Direktavdrag vid anskaffningen är en annan regel|Försäljning och utrangering ska hanteras före avskrivningen|Exakt fördelning mellan 1229, 1239 och 1249 är ännu inte verifierad</x:v>
-      </x:c>
-      <x:c r="J154" t="str">
-        <x:v>avskrivning maskiner|inventarier|byggnadsinventarier|bilar|kollektiv avskrivning|R10</x:v>
-      </x:c>
-      <x:c r="K154" t="str">
-        <x:v>1220|1221|1222|1229|1230|1231|1232|1239|1240|1241|1242|1249|5400|7700|7810|7820|7970</x:v>
-      </x:c>
-      <x:c r="L154" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7830, rad R10|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.37–6.40 och 7.12 samt exempel 6-5, 6-6 och 6-8</x:v>
-      </x:c>
-      <x:c r="M154" t="str">
-        <x:v>Avskrivningsmetod eller skattevärde är inte verifierat|Underlaget kan vara negativt eller påverkat av avyttring|Fördelningen mellan 1229, 1239 och 1249 är oklar|Privat användning eller tillskjuten tillgång förekommer|Nedskrivning kan krävas|Historik saknas, metod skiljer sig eller fördelningsrutin är oklar</x:v>
-      </x:c>
-      <x:c r="N154" t="str">
-        <x:v>active</x:v>
-      </x:c>
-      <x:c r="O154" t="n">
+      <x:c r="N154" s="14" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="O154" s="14" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P154" s="14" t="str">
@@ -8444,141 +8446,143 @@
     </x:row>
     <x:row r="155">
       <x:c r="A155" t="str">
-        <x:v>7970</x:v>
+        <x:v>7820</x:v>
       </x:c>
       <x:c r="B155" t="str">
-        <x:v>Förlust vid avyttring av immateriella och materiella anläggningstillgångar</x:v>
+        <x:v>Avskrivningar på byggnader och markanläggningar</x:v>
       </x:c>
       <x:c r="C155" t="str">
-        <x:v>Kostnadskonto på R6 för verifierad förlust vid avyttring av en individuellt värderad immateriell eller materiell anläggningstillgång när försäljningsinkomsten understiger bokfört värde.</x:v>
+        <x:v>Kostnadskonto på R9 för årets planenliga och skattemässigt grundade avskrivning på byggnader och markanläggningar. Motkontot är normalt 1119 respektive 1159.</x:v>
       </x:c>
       <x:c r="D155" t="str">
-        <x:v>En byggnad, mark, markanläggning eller förvärvad immateriell tillgång har avyttrats|Tillgångens bokförda värde och försäljningsinkomst kan fastställas|Tillämplig K1-regel innebär att skillnaden ska redovisas som kostnad|Tillgången har tagits bort ur tillgångsförteckningen</x:v>
+        <x:v>En byggnad som hör till företaget är bokförd på 1110|En färdigställd markanläggning är bokförd på 1150|Årets avskrivningsbelopp kan härledas till fastighets- och skatteunderlag|Tillgången har varit färdigställd och tagits i bruk</x:v>
       </x:c>
       <x:c r="E155" t="str">
-        <x:v>Försäljningsinkomsten överstiger bokfört värde; använd 3970|Avyttringen gäller maskiner och inventarier som först ska hanteras kollektivt genom B4-underkontona|Beloppet är försäljningskostnad, moms eller kundfordran|Tillgången är privat eller har aldrig hört till företaget|Förlusten bygger endast på marknadsvärde utan genomförd avyttring</x:v>
+        <x:v>Beloppet avser mark; mark ska inte skrivas av|Utgiften är reparation eller underhåll|Tillgången är byggnads- eller markinventarie; använd 7830|Tillgången är pågående och inte färdigställd; använd 1180|Händelsen är nedskrivning eller avyttring|Avskrivningsunderlag eller tillgångsfördelning saknas</x:v>
       </x:c>
       <x:c r="F155" t="str">
-        <x:v>Identifiera tillgång, avyttringsdatum, köpare, ersättning exklusive moms, försäljningskostnader och bokfört värde|Bokför försäljningsinkomst och moms separat|Ta bort tillgångens anskaffningsvärde och avskrivningar enligt tillgångsslag|Beräkna resultatet efter att alla tillgångsposter har återförts|Använd 7970 endast när den fastställda nettoskillnaden är en förlust enligt tillämplig K1-regel|För maskiner och inventarier: använd först den kollektiva avyttrings- och avskrivningsmodellen och blockera automatisk 7970|Stäm av mot avtal, betalning, tillgångsförteckning och deklarationsunderlag|Kräv manuell granskning vid delavyttring, byte, försäkringsersättning, uttag eller näringsfastighet|Använd endast vid individuell avyttring och verifierad förlustberäkning|Kräv försäljningspris, bokfört värde, årets avskrivning, kostnader, ersättningar och tillgångsslag|Vid granskningsflagga begär in försäljningsavtal, faktura, betalning och uppdaterad tillgångsförteckning|Sätt ärendet till väntar på underlag tills försäljningspris, bokfört värde, årets avskrivning och moms är avstämda|Godkänn 7970 endast när en individuell avyttring ger en verifierad förlust|Föreslå kollektiv inventariemodell, 3970 eller eskalering vid inbyte, uttag, försäkringsfall eller oklar beräkning</x:v>
+        <x:v>Identifiera fastighet, byggnad, markanläggning, anskaffningsvärde, färdigställandedatum och tidigare avskrivningar|Separera mark från byggnad samt byggnads- och markinventarier från byggnaden|Fastställ skattemässigt avskrivningsunderlag och tillämplig procentsats utifrån verifierad fastighetsklassificering|Beräkna årets avskrivning per byggnad och markanläggning|Bokför kostnaden i debet på 7820 och kredit på 1119 eller 1159|Stäm av nettot 1110 minus 1119 och 1150 minus 1159 mot B2 och tillgångsförteckningen|Hantera försäljning, utrangering, tillbyggnad och omklassificering före slutlig avskrivning|Kräv manuell granskning vid blandad fastighet, delavyttring, privat användning eller osäker skattemässig klass|För befintlig enkel näringsfastighet: beräkna avskrivningen med den procentsats som verifierats från föregående deklaration eller fastighetsunderlag|Vid ny byggnad eller saknad historik krävs manuell startgranskning|Komplexa byggnader, primäravdrag och flera byggnadstyper ligger utanför standardflödet|Fastställ avskrivningsunderlag och procentsats per fastighet från dokumenterad skattemässig klassificering|Koppla delavyttring till specificerad såld del|Vid granskningsflagga begär in fastighets- och objektsförteckning, anskaffningsvärde, färdigställandedatum, tidigare avskrivningar och verifierad skattemässig procentsats|Sätt ärendet till väntar på underlag tills 1110, 1119, 1150 och 1159 kan stämmas av per byggnad eller markanläggning|Godkänn 7820 för en enkel befintlig näringsbyggnad eller markanläggning med dokumenterad och oförändrad avskrivningsprocent|Föreslå scope-eskalering vid ny eller blandad fastighet, primäravdrag, flera byggnadstyper, delavyttring, ombyggnad eller saknad historik</x:v>
       </x:c>
       <x:c r="G155" t="str">
-        <x:v>1000|1009|1110|1119|1130|1150|1159|1930|1500|2610</x:v>
+        <x:v>1119|1159</x:v>
       </x:c>
       <x:c r="H155" t="str">
-        <x:v>En byggnad säljs för mindre än sitt bokförda värde och den verifierade skillnaden redovisas på 7970|Försäljning med vinst redovisas i stället på 3970</x:v>
+        <x:v>Årets avskrivning på en färdigställd verksamhetsbyggnad debiterar 7820 och krediterar 1119|Markvärdet skrivs inte av</x:v>
       </x:c>
       <x:c r="I155" t="str">
-        <x:v>Förlust får inte bokföras innan tillgångens bokförda värde är avstämt|Maskiner och inventarier följer normalt en kollektiv modell|Moms och försäljningskostnader ska hållas isär från reavinsten eller reaförlusten|Privat del får inte belasta företaget|Kollektivt hanterade inventarier ska inte ge separat förlust här</x:v>
+        <x:v>Mark ska alltid hållas skild från avskrivningsbar byggnad|Byggnadsinventarier och markinventarier följer inventariereglerna|Avskrivningsprocenten får inte antas från kontonamnet|Reparation och värdehöjande förbättring måste skiljas åt|En fullständig tabell över alla byggnadstyper ska inte användas automatiskt i Enkla Bokslut|Konto eller vardaglig benämning får inte ensamt styra procentsatsen</x:v>
       </x:c>
       <x:c r="J155" t="str">
-        <x:v>förlust avyttring|anläggningstillgång|reaförlust|bokfört värde|försäljningsinkomst|R6</x:v>
+        <x:v>avskrivning byggnad|markanläggning|1119|1159|fastighet|R9</x:v>
       </x:c>
       <x:c r="K155" t="str">
-        <x:v>3970|1000|1009|1110|1119|1130|1150|1159|1220|1222|1230|1232|1240|1242|7700|7810|7820|7830</x:v>
+        <x:v>1110|1119|1130|1150|1159|1180|1230|1239|5100|5500|7700|7970</x:v>
       </x:c>
       <x:c r="L155" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7970, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.18, 6.27 och 6.37–6.38 samt exempel 6-7 och 6-8</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7820, rad R9|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.10–6.18 och 7.12 samt exempel 6-7</x:v>
       </x:c>
       <x:c r="M155" t="str">
-        <x:v>Tillgången är maskin eller inventarie i kollektiv grupp|Bokfört värde eller försäljningsinkomst är inte avstämt|Avyttringen är byte, delavyttring, uttag eller försäkringsfall|Privat användning eller momsbehandling är oklar|Resultatet kan i stället vara vinst|Tillgångsslag, inbyte, försäkringsersättning eller beräkning är oklar</x:v>
+        <x:v>Mark och byggnad är inte fördelade|Byggnadsinventarie eller markinventarie kan förekomma|Skattemässig procentsats eller underlag saknas|Tillgången har byggts om, delavyttrats eller används privat|Avskrivningen stämmer inte med tillgångsförteckningen|Historisk procentsats saknas eller byggnaden är ny|Komplex byggnadstyp eller primäravdrag förekommer|Ny fastighet, oklar historik, blandad klassificering eller delavyttring förekommer</x:v>
       </x:c>
       <x:c r="N155" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O155" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="P155" s="14"/>
       <x:c r="Q155" s="12" t="str"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" t="str">
-        <x:v>7980</x:v>
+        <x:v>7830</x:v>
       </x:c>
       <x:c r="B156" t="str">
-        <x:v>Ersättningsfonder</x:v>
+        <x:v>Avskrivningar på maskiner och inventarier</x:v>
       </x:c>
       <x:c r="C156" t="str">
-        <x:v>Tekniskt specialistkonto för en godkänd resultateffekt från ersättningsfond. Systemet får inte skapa bokningar på 7980 automatiskt och varje förekomst ska stämmas av mot U3-metadata på 2060.</x:v>
+        <x:v>Kostnadskonto på R10 för årets avskrivning på maskiner och inventarier, byggnads- och markinventarier samt bilar och andra transportmedel som redovisas på B4.</x:v>
       </x:c>
       <x:c r="D156" t="str">
-        <x:v>En specialist har beslutat en dokumenterad resultateffekt vid avsättning, ianspråktagande eller återföring av ersättningsfond</x:v>
+        <x:v>Ett kollektivt avskrivningsunderlag för B4 har fastställts|Årets värde vid beskattningen är verifierat|Försäljningsinkomster och årets anskaffningar har först bokförts på respektive B4-underkonto|Årets avskrivning ska bokföras mot 1229, 1239 eller 1249</x:v>
       </x:c>
       <x:c r="E156" t="str">
-        <x:v>Systemet ska beräkna eller bokföra ersättningsfond automatiskt|Fondtyp, beskattningsår, resultatrad eller motkonto saknas</x:v>
+        <x:v>Beloppet avser immateriell tillgång; använd 7810|Beloppet avser byggnad eller markanläggning; använd 7820|Utgiften får kostnadsföras direkt som inventarie av mindre värde eller med högst tre års livslängd|Händelsen är särskild nedskrivning; använd 7700|Avskrivningen beräknas fritt per enskild inventarie utan avstämning mot den kollektiva skatteregeln</x:v>
       </x:c>
       <x:c r="F156" t="str">
-        <x:v>Flagga varje föreslagen eller importerad bokning på 7980 för specialistgranskning|Begär beslut eller skatteberäkning, fondtyp, beskattningsår, belopp, händelse, presentationsrad och motkonto|Sätt ärendet till väntar på underlag|Godkänn endast en uttryckligen specialistbeslutad bokning och stäm av den mot U3-metadata på 2060|Kontrollera att R9 eller R10, tecken och återföringsfrist är dokumenterade|Markera ny avsättning, ianspråktagande eller återföring som utanför standardflödet</x:v>
+        <x:v>Stäm av ingående B4-värden och årets nyanskaffningar på 1221, 1231 och 1241|Minska underlaget med årets försäljningsinkomster på 1222, 1232 och 1242|Fastställ värdet vid beskattningen och vald tillåten avskrivningsmetod|Beräkna avskrivningen som skillnaden mellan bokfört värde före årets avskrivning och värdet vid beskattningen|Om avskrivningsunderlaget före årets avskrivning är högst ett halvt prisbasbelopp får hela underlaget skrivas av när villkoren är uppfyllda|Fördela den bokförda avskrivningen mot 1229, 1239 och 1249 enligt fastställd systemrutin utan att ändra totalbeloppet|Stäm av B4 och R10 mot tillgångsförteckning och deklarationsunderlag|Pröva separat nedskrivning enligt 6.40 om högsta tillåtna avskrivning inte görs|Kräv manuell granskning vid metodbyte, negativt underlag, delvis privat tillgång eller avyttring|Om högsta tillåtna avskrivning inte görs och möjlig kollektiv värdenedgång uppgår till minst 10 procent ska nedskrivning granskas manuellt|Använd verifierad historisk avskrivningsmetod|Metodbyte får inte göras automatiskt|Total kollektiv avskrivning ska bevaras vid fördelning mellan underkonton|Beräkna årets avskrivning som skillnaden mellan gruppens värde före avskrivning och det verifierade kollektiva B4-värdet vid beskattningen|Bokför hela kostnaden i debet på 7830 och kreditera som standard 1229 när en tillförlitlig kategoriuppdelning saknas|Dela krediten mellan 1229, 1239 och 1249 endast när en verifierad tillgångsförteckning ger en spårbar fördelning; kostnaden på 7830 ska vara oförändrad|Sätt ärendet till väntar på underlag vid okänd metod, negativt underlag, metodbyte, avyttring, privat användning eller bristande avstämning mot B4</x:v>
       </x:c>
       <x:c r="G156" t="str">
-        <x:v>2060</x:v>
+        <x:v>1229|1239|1249</x:v>
       </x:c>
       <x:c r="H156" t="str">
-        <x:v>Specialistgodkänd återföring bokas och stäms av mot U3</x:v>
+        <x:v>Årets kollektivt beräknade inventarieavskrivning bokförs på 7830 mot B4:s avskrivningsunderkonton|En avyttring minskar först avskrivningsunderlaget genom försäljningsinkomsten</x:v>
       </x:c>
       <x:c r="I156" t="str">
-        <x:v>7980 bokas aldrig automatiskt|Ersättningsfond ligger utanför standardflödet</x:v>
+        <x:v>K1 kräver kollektiv värdering och avskrivning|Hela underlaget får skrivas av först när halvt-prisbasbeloppsregeln är uppfylld|Direktavdrag vid anskaffningen är en annan regel|Försäljning och utrangering ska hanteras före avskrivningen|Exakt fördelning mellan 1229, 1239 och 1249 är ännu inte verifierad</x:v>
       </x:c>
       <x:c r="J156" t="str">
-        <x:v>ersättningsfond|avsättning|återföring|ianspråktagande|U3|R9|R10</x:v>
+        <x:v>avskrivning maskiner|inventarier|byggnadsinventarier|bilar|kollektiv avskrivning|R10</x:v>
       </x:c>
       <x:c r="K156" t="str">
-        <x:v>2060|3970|7970|7700|7820|7830|8990</x:v>
+        <x:v>1220|1221|1222|1229|1230|1231|1232|1239|1240|1241|1242|1249|5400|7700|7810|7820|7970</x:v>
       </x:c>
       <x:c r="L156" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7980, rad R9/R10|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 8 om upplysningar om obeskattade reserver och bilaga 2</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7830, rad R10|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.37–6.40 och 7.12 samt exempel 6-5, 6-6 och 6-8</x:v>
       </x:c>
       <x:c r="M156" t="str">
-        <x:v>Varje bokning eller saldo på 7980|Specialistbeslut, U3-avstämning, resultatrad eller motkonto saknas</x:v>
+        <x:v>Avskrivningsmetod eller skattevärde är inte verifierat|Underlaget kan vara negativt eller påverkat av avyttring|Fördelningen mellan 1229, 1239 och 1249 är oklar|Privat användning eller tillskjuten tillgång förekommer|Nedskrivning kan krävas|Historik saknas, metod skiljer sig eller fördelningsrutin är oklar</x:v>
       </x:c>
       <x:c r="N156" t="str">
         <x:v>active</x:v>
       </x:c>
       <x:c r="O156" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P156" s="14" t="str"/>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P156" s="14" t="str">
+        <x:v>full_writeoff_remaining_basis_half_pbb|impairment_review_threshold_10_percent</x:v>
+      </x:c>
       <x:c r="Q156" s="12" t="str"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" t="str">
-        <x:v>8310</x:v>
+        <x:v>7970</x:v>
       </x:c>
       <x:c r="B157" t="str">
-        <x:v>Ränteintäkter och utdelningar</x:v>
+        <x:v>Förlust vid avyttring av immateriella och materiella anläggningstillgångar</x:v>
       </x:c>
       <x:c r="C157" t="str">
-        <x:v>Intäktskonto på R4 för skattepliktiga ränteintäkter och utdelningar som hör till näringsverksamheten.</x:v>
+        <x:v>Kostnadskonto på R6 för verifierad förlust vid avyttring av en individuellt värderad immateriell eller materiell anläggningstillgång när försäljningsinkomsten understiger bokfört värde.</x:v>
       </x:c>
       <x:c r="D157" t="str">
-        <x:v>Räntan härrör från företagets bankmedel, kundfordran eller annan verifierad företagstillgång|Utdelningen avser en andel som får och ska ingå i verksamheten|Intäkten är skattepliktig i näringsverksamheten|Belopp, period och betalare kan verifieras</x:v>
+        <x:v>En byggnad, mark, markanläggning eller förvärvad immateriell tillgång har avyttrats|Tillgångens bokförda värde och försäljningsinkomst kan fastställas|Tillämplig K1-regel innebär att skillnaden ska redovisas som kostnad|Tillgången har tagits bort ur tillgångsförteckningen</x:v>
       </x:c>
       <x:c r="E157" t="str">
-        <x:v>Räntan eller utdelningen hör till privat kapital|Intäkten är skattefri; pröva 8314|Beloppet är försäljningsintäkt, valutakursdifferens eller dröjsmålsavgift med annan klassificering|Rätten till intäkten eller periodtillhörigheten är oklar|Utdelningen avser privat aktieinnehav</x:v>
+        <x:v>Försäljningsinkomsten överstiger bokfört värde; använd 3970|Avyttringen gäller maskiner och inventarier som först ska hanteras kollektivt genom B4-underkontona|Beloppet är försäljningskostnad, moms eller kundfordran|Tillgången är privat eller har aldrig hört till företaget|Förlusten bygger endast på marknadsvärde utan genomförd avyttring</x:v>
       </x:c>
       <x:c r="F157" t="str">
-        <x:v>Identifiera intäktstyp, betalare, underliggande fordran eller andel, skatteplikt och period|Bokför betald ränta mot bank eller fordran|Ta upp upplupen ränteinkomst på 1600 när K1:s sammanlagda 5 000-kronorsgräns överskrids|Ta upp förutbetald ränteinkomst på 2900 när beloppet hör till nästa år och gränsen överskrids|Kräv särskild prövning innan utdelning hänförs till näringsverksamheten|Stäm av mot årsbesked, kontoutdrag, låneavtal och deklarationsunderlag|Separera valutakursdifferens på 8330|Kräv manuell granskning vid närstående lån, privat placering eller skattefri intäkt|Använd endast för ränta eller utdelning som hör till tillgång eller fordran i näringsverksamheten|Spara konto eller depå, avtal, verksamhetskoppling, period och skatteklassificering|Vid granskningsflagga begär in årsbesked, kontoutdrag eller avtal samt uppgift om den underliggande fordran eller andelen|Sätt ärendet till väntar på underlag tills verksamhetskoppling, skatteklassificering och period är verifierade|Godkänn 8310 för skattepliktig ränta eller utdelning som hör till näringsverksamheten|Föreslå privat kapitalinkomst, 8314, periodiseringsrutin eller eskalering när inkomsten inte tydligt hör till verksamheten</x:v>
+        <x:v>Identifiera tillgång, avyttringsdatum, köpare, ersättning exklusive moms, försäljningskostnader och bokfört värde|Bokför försäljningsinkomst och moms separat|Ta bort tillgångens anskaffningsvärde och avskrivningar enligt tillgångsslag|Beräkna resultatet efter att alla tillgångsposter har återförts|Använd 7970 endast när den fastställda nettoskillnaden är en förlust enligt tillämplig K1-regel|För maskiner och inventarier: använd först den kollektiva avyttrings- och avskrivningsmodellen och blockera automatisk 7970|Stäm av mot avtal, betalning, tillgångsförteckning och deklarationsunderlag|Kräv manuell granskning vid delavyttring, byte, försäkringsersättning, uttag eller näringsfastighet|Använd endast vid individuell avyttring och verifierad förlustberäkning|Kräv försäljningspris, bokfört värde, årets avskrivning, kostnader, ersättningar och tillgångsslag|Vid granskningsflagga begär in försäljningsavtal, faktura, betalning och uppdaterad tillgångsförteckning|Sätt ärendet till väntar på underlag tills försäljningspris, bokfört värde, årets avskrivning och moms är avstämda|Godkänn 7970 endast när en individuell avyttring ger en verifierad förlust|Föreslå kollektiv inventariemodell, 3970 eller eskalering vid inbyte, uttag, försäkringsfall eller oklar beräkning</x:v>
       </x:c>
       <x:c r="G157" t="str">
-        <x:v>1930|1940|1970|1600|2900|1300</x:v>
+        <x:v>1000|1009|1110|1119|1130|1150|1159|1930|1500|2610</x:v>
       </x:c>
       <x:c r="H157" t="str">
-        <x:v>Ränta på ett verifierat företagskonto bokförs på 8310|Upplupen företagsränta över K1-gränsen tas upp mot 1600 vid bokslutet</x:v>
+        <x:v>En byggnad säljs för mindre än sitt bokförda värde och den verifierade skillnaden redovisas på 7970|Försäljning med vinst redovisas i stället på 3970</x:v>
       </x:c>
       <x:c r="I157" t="str">
-        <x:v>Finansiell intäkt måste höra till företaget och inte privatpersonen|Utdelning kräver att innehavet får ingå i verksamheten|Periodiseringströskeln gäller den fysiska personens samtliga verksamheter totalt|Skattefri ränta ska hållas isär|Privat sparande och privata värdepapper ska inte tas in i bokföringen</x:v>
+        <x:v>Förlust får inte bokföras innan tillgångens bokförda värde är avstämt|Maskiner och inventarier följer normalt en kollektiv modell|Moms och försäljningskostnader ska hållas isär från reavinsten eller reaförlusten|Privat del får inte belasta företaget|Kollektivt hanterade inventarier ska inte ge separat förlust här</x:v>
       </x:c>
       <x:c r="J157" t="str">
-        <x:v>ränteintäkt|utdelning|företagskonto|upplupen ränta|R4</x:v>
+        <x:v>förlust avyttring|anläggningstillgång|reaförlust|bokfört värde|försäljningsinkomst|R6</x:v>
       </x:c>
       <x:c r="K157" t="str">
-        <x:v>8314|8330|1300|1600|1930|1940|1970|2900</x:v>
+        <x:v>3970|1000|1009|1110|1119|1130|1150|1159|1220|1222|1230|1232|1240|1242|7700|7810|7820|7830</x:v>
       </x:c>
       <x:c r="L157" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8310, rad R4|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.60–6.61 och kapitel 7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikation och periodisering</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7970, rad R6|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.18, 6.27 och 6.37–6.38 samt exempel 6-7 och 6-8</x:v>
       </x:c>
       <x:c r="M157" t="str">
-        <x:v>Intäkten kan vara privat kapitalinkomst|Utdelningens tillgångstillhörighet är oklar|Skatteplikten är inte verifierad|Upplupen eller förutbetald ränta kan behöva periodiseras|Närstående part eller utländsk betalare förekommer|Verksamhetskoppling eller periodisering är oklar</x:v>
+        <x:v>Tillgången är maskin eller inventarie i kollektiv grupp|Bokfört värde eller försäljningsinkomst är inte avstämt|Avyttringen är byte, delavyttring, uttag eller försäkringsfall|Privat användning eller momsbehandling är oklar|Resultatet kan i stället vara vinst|Tillgångsslag, inbyte, försäkringsersättning eller beräkning är oklar</x:v>
       </x:c>
       <x:c r="N157" t="str">
         <x:v>active</x:v>
@@ -8586,50 +8590,48 @@
       <x:c r="O157" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P157" s="14" t="str">
-        <x:v>accrued_interest_income_over_5000|prepaid_interest_income_over_5000</x:v>
-      </x:c>
+      <x:c r="P157" s="14"/>
       <x:c r="Q157" s="12" t="str"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" t="str">
-        <x:v>8314</x:v>
+        <x:v>7980</x:v>
       </x:c>
       <x:c r="B158" t="str">
-        <x:v>Skattefria ränteintäkter</x:v>
+        <x:v>Ersättningsfonder</x:v>
       </x:c>
       <x:c r="C158" t="str">
-        <x:v>Underkonto på R4 för ränteintäkter som hör till verksamhetens redovisning men är skattefria och därför ska hanteras som skattemässig justering på NE-bilagans sida 2.</x:v>
+        <x:v>Tekniskt specialistkonto för en godkänd resultateffekt från ersättningsfond. Systemet får inte skapa bokningar på 7980 automatiskt och varje förekomst ska stämmas av mot U3-metadata på 2060.</x:v>
       </x:c>
       <x:c r="D158" t="str">
-        <x:v>Ränteintäkten är verifierad som skattefri enligt aktuell regel|Intäkten hör till en post som redovisas i företagets bokföring|Beloppet ska ingå i bokfört resultat men undantas vid beskattningen</x:v>
+        <x:v>En specialist har beslutat en dokumenterad resultateffekt vid avsättning, ianspråktagande eller återföring av ersättningsfond</x:v>
       </x:c>
       <x:c r="E158" t="str">
-        <x:v>Räntan är skattepliktig; använd 8310|Beloppet hör till privatpersonen och ska inte bokföras i företaget|Skattefriheten antas enbart utifrån betalaren eller kontots namn|Beloppet är återbetalning, kapitalinsättning eller valutakursdifferens</x:v>
+        <x:v>Systemet ska beräkna eller bokföra ersättningsfond automatiskt|Fondtyp, beskattningsår, resultatrad eller motkonto saknas</x:v>
       </x:c>
       <x:c r="F158" t="str">
-        <x:v>Identifiera betalare, underliggande fordran eller konto, regelstöd, period och belopp|Dokumentera varför intäkten är skattefri|Bokför intäkten på 8314 endast om den samtidigt hör till företagets bokföring|Märk beloppet för skattemässig justering på NE-bilagans sida 2|Pröva K1:s periodiseringsregler för upplupen eller förutbetald ränta när de är tillämpliga|Stäm av mot årsbesked och deklarationsunderlag|Blockera automatisk användning baserad endast på transaktionstext|Kräv manuell granskning av ränta på skattekonto och andra gränsfall mellan privat och företag|Använd endast när skattefriheten har tydlig rättslig grund och skattekod|Koppla ränta på skattekontot till verifierad skattekontorutin|Flagga varje föreslagen eller importerad bokning på 8314 och begär årsbesked, betalare, kontotyp, regelstöd och förklaring till varför räntan hör till företagets bokföring|Sätt ärendet till väntar på underlag tills både verksamhetsanknytningen och skattefriheten är verifierade och NE-justeringen är definierad|Godkänn 8314 endast för dokumenterad skattefri ränteintäkt som ska ingå i bokföringen och samtidigt justeras skattemässigt|Ränta på företagarens privata skattekonto ska inte automatiskt bokas som företagsintäkt; föreslå 2012, privat hantering eller manuell eskalering efter underlaget</x:v>
+        <x:v>Flagga varje föreslagen eller importerad bokning på 7980 för specialistgranskning|Begär beslut eller skatteberäkning, fondtyp, beskattningsår, belopp, händelse, presentationsrad och motkonto|Sätt ärendet till väntar på underlag|Godkänn endast en uttryckligen specialistbeslutad bokning och stäm av den mot U3-metadata på 2060|Kontrollera att R9 eller R10, tecken och återföringsfrist är dokumenterade|Markera ny avsättning, ianspråktagande eller återföring som utanför standardflödet</x:v>
       </x:c>
       <x:c r="G158" t="str">
-        <x:v>1930|1940|1970|1600|2900|2012</x:v>
+        <x:v>2060</x:v>
       </x:c>
       <x:c r="H158" t="str">
-        <x:v>En dokumenterat skattefri ränteintäkt bokförs på 8314 och märks för skattemässig justering|Ränta som hör till privatpersonen bokförs inte som företagsintäkt</x:v>
+        <x:v>Specialistgodkänd återföring bokas och stäms av mot U3</x:v>
       </x:c>
       <x:c r="I158" t="str">
-        <x:v>Skattefrihet och tillhörighet till företaget är två separata prövningar|Kontot ska kopplas till NE-justering|Ränta på skattekonto kräver fastställd ägarkontering|Beloppet får inte lämnas utan regelreferens|Kontot får inte användas utifrån kundens antagande|Exakt bokning mot 2012 är ännu inte verifierad</x:v>
+        <x:v>7980 bokas aldrig automatiskt|Ersättningsfond ligger utanför standardflödet</x:v>
       </x:c>
       <x:c r="J158" t="str">
-        <x:v>skattefri ränta|ränteintäkt|skattemässig justering|NE sidan 2|R4</x:v>
+        <x:v>ersättningsfond|avsättning|återföring|ianspråktagande|U3|R9|R10</x:v>
       </x:c>
       <x:c r="K158" t="str">
-        <x:v>8310|8330|1600|2012|2900</x:v>
+        <x:v>2060|3970|7970|7700|7820|7830|8990</x:v>
       </x:c>
       <x:c r="L158" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8314, rad R4 och NE sidan 2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.13–3.14, 6.60–6.61 och kapitel 7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 8, konto 7980, rad R9/R10|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 8 om upplysningar om obeskattade reserver och bilaga 2</x:v>
       </x:c>
       <x:c r="M158" t="str">
-        <x:v>Regelstödet för skattefrihet saknas|Räntan kan vara privat|Skattekontoränta förekommer|Periodisering kan krävas|NE-justeringen är inte kopplad|Rättslig grund eller skattekontorutin saknas</x:v>
+        <x:v>Varje bokning eller saldo på 7980|Specialistbeslut, U3-avstämning, resultatrad eller motkonto saknas</x:v>
       </x:c>
       <x:c r="N158" t="str">
         <x:v>active</x:v>
@@ -8637,99 +8639,99 @@
       <x:c r="O158" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P158" s="14" t="str">
+      <x:c r="P158" s="14" t="str"/>
+      <x:c r="Q158" s="12" t="str"/>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>8310</x:v>
+      </x:c>
+      <x:c r="B159" t="str">
+        <x:v>Ränteintäkter och utdelningar</x:v>
+      </x:c>
+      <x:c r="C159" t="str">
+        <x:v>Intäktskonto på R4 för skattepliktiga ränteintäkter och utdelningar som hör till näringsverksamheten.</x:v>
+      </x:c>
+      <x:c r="D159" t="str">
+        <x:v>Räntan härrör från företagets bankmedel, kundfordran eller annan verifierad företagstillgång|Utdelningen avser en andel som får och ska ingå i verksamheten|Intäkten är skattepliktig i näringsverksamheten|Belopp, period och betalare kan verifieras</x:v>
+      </x:c>
+      <x:c r="E159" t="str">
+        <x:v>Räntan eller utdelningen hör till privat kapital|Intäkten är skattefri; pröva 8314|Beloppet är försäljningsintäkt, valutakursdifferens eller dröjsmålsavgift med annan klassificering|Rätten till intäkten eller periodtillhörigheten är oklar|Utdelningen avser privat aktieinnehav</x:v>
+      </x:c>
+      <x:c r="F159" t="str">
+        <x:v>Identifiera intäktstyp, betalare, underliggande fordran eller andel, skatteplikt och period|Bokför betald ränta mot bank eller fordran|Ta upp upplupen ränteinkomst på 1600 när K1:s sammanlagda 5 000-kronorsgräns överskrids|Ta upp förutbetald ränteinkomst på 2900 när beloppet hör till nästa år och gränsen överskrids|Kräv särskild prövning innan utdelning hänförs till näringsverksamheten|Stäm av mot årsbesked, kontoutdrag, låneavtal och deklarationsunderlag|Separera valutakursdifferens på 8330|Kräv manuell granskning vid närstående lån, privat placering eller skattefri intäkt|Använd endast för ränta eller utdelning som hör till tillgång eller fordran i näringsverksamheten|Spara konto eller depå, avtal, verksamhetskoppling, period och skatteklassificering|Vid granskningsflagga begär in årsbesked, kontoutdrag eller avtal samt uppgift om den underliggande fordran eller andelen|Sätt ärendet till väntar på underlag tills verksamhetskoppling, skatteklassificering och period är verifierade|Godkänn 8310 för skattepliktig ränta eller utdelning som hör till näringsverksamheten|Föreslå privat kapitalinkomst, 8314, periodiseringsrutin eller eskalering när inkomsten inte tydligt hör till verksamheten</x:v>
+      </x:c>
+      <x:c r="G159" t="str">
+        <x:v>1930|1940|1970|1600|2900|1300</x:v>
+      </x:c>
+      <x:c r="H159" t="str">
+        <x:v>Ränta på ett verifierat företagskonto bokförs på 8310|Upplupen företagsränta över K1-gränsen tas upp mot 1600 vid bokslutet</x:v>
+      </x:c>
+      <x:c r="I159" t="str">
+        <x:v>Finansiell intäkt måste höra till företaget och inte privatpersonen|Utdelning kräver att innehavet får ingå i verksamheten|Periodiseringströskeln gäller den fysiska personens samtliga verksamheter totalt|Skattefri ränta ska hållas isär|Privat sparande och privata värdepapper ska inte tas in i bokföringen</x:v>
+      </x:c>
+      <x:c r="J159" t="str">
+        <x:v>ränteintäkt|utdelning|företagskonto|upplupen ränta|R4</x:v>
+      </x:c>
+      <x:c r="K159" t="str">
+        <x:v>8314|8330|1300|1600|1930|1940|1970|2900</x:v>
+      </x:c>
+      <x:c r="L159" t="str">
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8310, rad R4|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 6.60–6.61 och kapitel 7|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om verifikation och periodisering</x:v>
+      </x:c>
+      <x:c r="M159" t="str">
+        <x:v>Intäkten kan vara privat kapitalinkomst|Utdelningens tillgångstillhörighet är oklar|Skatteplikten är inte verifierad|Upplupen eller förutbetald ränta kan behöva periodiseras|Närstående part eller utländsk betalare förekommer|Verksamhetskoppling eller periodisering är oklar</x:v>
+      </x:c>
+      <x:c r="N159" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="O159" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P159" s="14" t="str">
         <x:v>accrued_interest_income_over_5000|prepaid_interest_income_over_5000</x:v>
       </x:c>
-      <x:c r="Q158" s="12" t="str"/>
-    </x:row>
-    <x:row r="159" ht="430" customHeight="1">
-      <x:c r="A159" s="14" t="str">
-        <x:v>8330</x:v>
-      </x:c>
-      <x:c r="B159" s="14" t="str">
-        <x:v>Valutakursdifferenser på fordringar och placeringar</x:v>
-      </x:c>
-      <x:c r="C159" s="14" t="str">
-        <x:v>Intäktskonto på R4 för positiva valutakursdifferenser på företagets fordringar, bankmedel och tillåtna placeringar. Negativa differenser prövas mot 8430.</x:v>
-      </x:c>
-      <x:c r="D159" s="14" t="str">
-        <x:v>En företagstillgång eller fordran är uttryckt i annan valuta än svenska kronor|Ursprungsbelopp, använd kurs och betalnings- eller balansdagskurs kan verifieras|Omräkningen ger en positiv differens som hör till verksamheten</x:v>
-      </x:c>
-      <x:c r="E159" s="14" t="str">
-        <x:v>Beloppet är ursprunglig försäljningsintäkt, ränta eller bankavgift|Differensen avser leverantörsskuld eller lån; pröva 8430|Tillgången eller placeringen är privat|Kursen eller värderingstidpunkten saknas|Beloppet uppkommer genom spekulation eller säkring utan särskild bedömning</x:v>
-      </x:c>
-      <x:c r="F159" s="14" t="str">
-        <x:v>Identifiera valuta, ursprungstransaktion, transaktionsdatum, ursprungskurs, regleringsdatum eller balansdag och använd kurskälla|Räkna om den ursprungliga affärshändelsen enligt avistakurs eller tillåten approximation|Beräkna realiserad differens vid betalning och dokumentera återföring av fordran|Pröva separat om oreglerade fordringar och bankmedel ska räknas om vid bokslutet enligt tillämplig K1- och skatteregel|Bokför endast positiv nettodifferens på 8330 enligt fastställd kontomodell|Bokför negativ differens på 8430 när den hör till skuldkostnad eller enligt beslutad symmetrisk modell|Håll ränta och bankavgift separata|Stäm av per valuta och mot reskontra, bank och kurskälla|Kräv manuell granskning vid valutasäkring, kryptotillgång, utländsk placering eller större kursrörelse|Använd för verifierad positiv realiserad eller orealiserad valutakursdifferens|Spara ursprungskurs, betalnings- eller bokslutskurs, källa och transaktionskoppling|Vid granskningsflagga begär in ursprungsfaktura eller fordran, betalningsunderlag, valuta, datum och dokumenterad kurskälla|Sätt ärendet till väntar på underlag tills ursprungskurs, betalnings- eller bokslutskurs och positiv differens är verifierade|Godkänn 8330 för en enkel dokumenterad positiv valutakursdifferens som hör till verksamheten|Föreslå 8430, privat post, rätt period eller scope-eskalering vid negativ differens, säkring, kryptotillgång eller komplicerad flervalutahantering</x:v>
-      </x:c>
-      <x:c r="G159" s="14" t="str">
-        <x:v>1500|1600|1920|1930|1940|1970|1300</x:v>
-      </x:c>
-      <x:c r="H159" s="14" t="str">
-        <x:v>En kundfordran i euro betalas när kronkursen är högre än vid faktureringen; den positiva differensen bokförs på 8330</x:v>
-      </x:c>
-      <x:c r="I159" s="14" t="str">
-        <x:v>Ursprunglig intäkt ska inte bokföras om som kursdifferens|Kurskälla och datum måste sparas|Privata placeringar ska inte ingå|Positiv och negativ differens måste hanteras konsekvent|Nettning över olika transaktioner är inte tillåten|Växlingspåslag är inte kursdifferens</x:v>
-      </x:c>
-      <x:c r="J159" s="14" t="str">
-        <x:v>valutakursvinst|kursdifferens|fordran|bankkonto|utländsk valuta|R4</x:v>
-      </x:c>
-      <x:c r="K159" s="14" t="str">
-        <x:v>8430|1500|1600|1920|1930|1940|1970|8310</x:v>
-      </x:c>
-      <x:c r="L159" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8330, rad R4|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, punkterna 2.4–2.7 om omräkning till redovisningsvaluta|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 6 och 7</x:v>
-      </x:c>
-      <x:c r="M159" s="14" t="str">
-        <x:v>Kurskälla eller värderingstidpunkt saknas|Tillgången kan vara privat eller otillåten placering|Orealiserad bokslutsdifferens förekommer|Valutasäkring eller flera valutor förekommer|Det är oklart om negativ differens ska nettas eller bokföras på 8430|Kurskälla, realisationsstatus eller säkringsinstrument är oklart</x:v>
-      </x:c>
-      <x:c r="N159" s="14" t="str">
-        <x:v>active</x:v>
-      </x:c>
-      <x:c r="O159" s="14" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P159" s="14"/>
-      <x:c r="Q159" s="14" t="str"/>
+      <x:c r="Q159" s="12" t="str"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" t="str">
-        <x:v>8410</x:v>
+        <x:v>8314</x:v>
       </x:c>
       <x:c r="B160" t="str">
-        <x:v>Räntekostnader för skulder</x:v>
+        <x:v>Skattefria ränteintäkter</x:v>
       </x:c>
       <x:c r="C160" t="str">
-        <x:v>Kostnadskonto på R8 för ränta på lån och andra skulder som hör till näringsverksamheten.</x:v>
+        <x:v>Underkonto på R4 för ränteintäkter som hör till verksamhetens redovisning men är skattefria och därför ska hanteras som skattemässig justering på NE-bilagans sida 2.</x:v>
       </x:c>
       <x:c r="D160" t="str">
-        <x:v>Skulden är bokförd eller på annat sätt verifierad som företagsskuld|Räntan kan skiljas från amortering och avgifter|Kostnaden hör till verksamheten och rätt period|Långivare, kapitalbelopp, räntesats och betalning kan verifieras</x:v>
+        <x:v>Ränteintäkten är verifierad som skattefri enligt aktuell regel|Intäkten hör till en post som redovisas i företagets bokföring|Beloppet ska ingå i bokfört resultat men undantas vid beskattningen</x:v>
       </x:c>
       <x:c r="E160" t="str">
-        <x:v>Beloppet är amortering; minska skuldkontot|Beloppet är bank- eller serviceavgift som inte är ränta eller annan utgift för kredit|Skulden eller räntan är privat|Beloppet är företagarens skatt eller ränta på privat skattekonto|Posten är en valutakursdifferens eller annan orealiserad värdeförändring som ska klassificeras separat|Räntebelopp eller period kan inte skiljas från övrig betalning</x:v>
+        <x:v>Räntan är skattepliktig; använd 8310|Beloppet hör till privatpersonen och ska inte bokföras i företaget|Skattefriheten antas enbart utifrån betalaren eller kontots namn|Beloppet är återbetalning, kapitalinsättning eller valutakursdifferens</x:v>
       </x:c>
       <x:c r="F160" t="str">
-        <x:v>Identifiera skuld, långivare, kapitaldel, räntedel, avgifter, period och betalningsdatum|Fördela lån som används både privat och i företaget enligt dokumenterad användning|Bokför betald företagsränta på 8410 och amortering mot 2330, 2350 eller 2390|Ta upp upplupen ränteutgift på 2900 när den sammanlagt överstiger 5 000 kronor enligt K1|Ta upp förutbetald ränteutgift på 1600 när den hör till nästa år och gränsen överskrids|Stäm av mot lånebesked, amorteringsplan, bank och B13/B16|Separera valutakursdifferens på 8430|BAS 8417, 8423, 8424, 8480 och 8490 får inte mappas automatiskt utan kräver manuell klassificering|BAS 8450 och 8451 ska granskas mot 8430 eller annan relevant hantering och får inte automatiskt behandlas som ränta|BAS 8411 hör inte till en vanlig K1-enskild firma och BAS 8412 ligger utanför tjänstens scope|Märk ej avdragsgill eller privat ränta för skattemässig justering eller eget uttag i stället för vanlig avdragsgill räntekostnad|Kräv manuell granskning vid närstående lån, blandad användning, utländsk skuld, byggnadskreditiv eller kapitaliserad ränta</x:v>
+        <x:v>Identifiera betalare, underliggande fordran eller konto, regelstöd, period och belopp|Dokumentera varför intäkten är skattefri|Bokför intäkten på 8314 endast om den samtidigt hör till företagets bokföring|Märk beloppet för skattemässig justering på NE-bilagans sida 2|Pröva K1:s periodiseringsregler för upplupen eller förutbetald ränta när de är tillämpliga|Stäm av mot årsbesked och deklarationsunderlag|Blockera automatisk användning baserad endast på transaktionstext|Kräv manuell granskning av ränta på skattekonto och andra gränsfall mellan privat och företag|Använd endast när skattefriheten har tydlig rättslig grund och skattekod|Koppla ränta på skattekontot till verifierad skattekontorutin|Flagga varje föreslagen eller importerad bokning på 8314 och begär årsbesked, betalare, kontotyp, regelstöd och förklaring till varför räntan hör till företagets bokföring|Sätt ärendet till väntar på underlag tills både verksamhetsanknytningen och skattefriheten är verifierade och NE-justeringen är definierad|Godkänn 8314 endast för dokumenterad skattefri ränteintäkt som ska ingå i bokföringen och samtidigt justeras skattemässigt|Ränta på företagarens privata skattekonto ska inte automatiskt bokas som företagsintäkt; föreslå 2012, privat hantering eller manuell eskalering efter underlaget</x:v>
       </x:c>
       <x:c r="G160" t="str">
-        <x:v>2330|2350|2390|2900|1600|1930</x:v>
+        <x:v>1930|1940|1970|1600|2900|2012</x:v>
       </x:c>
       <x:c r="H160" t="str">
-        <x:v>En lånebetalning delas mellan amortering mot 2350 och ränta på 8410|Upplupen företagsränta över K1-gränsen bokförs mot 2900 vid bokslutet|Ränta från BAS 8423 granskas för att skilja avdragsgill företagsränta från ej avdragsgill eller privat skatteränta|En post på BAS 8450 eller 8451 granskas och förs vid valutakursdifferens till 8430 i stället för 8410</x:v>
+        <x:v>En dokumenterat skattefri ränteintäkt bokförs på 8314 och märks för skattemässig justering|Ränta som hör till privatpersonen bokförs inte som företagsintäkt</x:v>
       </x:c>
       <x:c r="I160" t="str">
-        <x:v>Amortering är inte kostnad|Endast företagets räntedel får belasta R8|Utgiftsränta på skattekontot är inte skattemässigt avdragsgill|Periodiseringströskeln gäller den fysiska personens samtliga verksamheter totalt|Avgifter, valutakursdifferenser och orealiserade värdeförändringar ska hållas isär från ränta|Hela bankdragningen får inte bokföras som ränta</x:v>
+        <x:v>Skattefrihet och tillhörighet till företaget är två separata prövningar|Kontot ska kopplas till NE-justering|Ränta på skattekonto kräver fastställd ägarkontering|Beloppet får inte lämnas utan regelreferens|Kontot får inte användas utifrån kundens antagande|Exakt bokning mot 2012 är ännu inte verifierad</x:v>
       </x:c>
       <x:c r="J160" t="str">
-        <x:v>räntekostnad|lån|amortering|upplupen ränta|förutbetald ränta|R8</x:v>
+        <x:v>skattefri ränta|ränteintäkt|skattemässig justering|NE sidan 2|R4</x:v>
       </x:c>
       <x:c r="K160" t="str">
-        <x:v>2330|2350|2390|2900|1600|8430|2013</x:v>
+        <x:v>8310|8330|1600|2012|2900</x:v>
       </x:c>
       <x:c r="L160" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8410, rad R8|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.17, 6.59, 6.73 och 7.11 samt exempel 3-4 och 7-4|Skatteverket – Ränteutgifter, kontrollerat 2026-09-20</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8314, rad R4 och NE sidan 2|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.13–3.14, 6.60–6.61 och kapitel 7</x:v>
       </x:c>
       <x:c r="M160" t="str">
-        <x:v>Skulden kan vara privat eller blandad|Amortering och ränta är inte separerade|Upplupen eller förutbetald ränta kan behöva periodiseras|Närstående eller utländsk långivare förekommer|Posten kommer från BAS 8417, 8423, 8424, 8480 eller 8490|Posten kommer från BAS 8450 eller 8451 och klassificeringen mot 8430 är inte verifierad|Avgiften kan vara annat än ränta eller den skattemässiga avdragsrätten är oklar</x:v>
+        <x:v>Regelstödet för skattefrihet saknas|Räntan kan vara privat|Skattekontoränta förekommer|Periodisering kan krävas|NE-justeringen är inte kopplad|Rättslig grund eller skattekontorutin saknas</x:v>
       </x:c>
       <x:c r="N160" t="str">
         <x:v>active</x:v>
@@ -8738,49 +8740,49 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="P160" s="14" t="str">
-        <x:v>accrued_interest_expense_over_5000|prepaid_interest_expense_over_5000</x:v>
+        <x:v>accrued_interest_income_over_5000|prepaid_interest_income_over_5000</x:v>
       </x:c>
       <x:c r="Q160" s="12" t="str"/>
     </x:row>
     <x:row r="161" ht="430" customHeight="1">
       <x:c r="A161" s="14" t="str">
-        <x:v>8430</x:v>
+        <x:v>8330</x:v>
       </x:c>
       <x:c r="B161" s="14" t="str">
-        <x:v>Valutakursdifferenser på skulder</x:v>
+        <x:v>Valutakursdifferenser på fordringar och placeringar</x:v>
       </x:c>
       <x:c r="C161" s="14" t="str">
-        <x:v>Kostnadskonto på R8 för negativa valutakursdifferenser på företagets leverantörsskulder, lån och andra skulder i utländsk valuta.</x:v>
+        <x:v>Intäktskonto på R4 för positiva valutakursdifferenser på företagets fordringar, bankmedel och tillåtna placeringar. Negativa differenser prövas mot 8430.</x:v>
       </x:c>
       <x:c r="D161" s="14" t="str">
-        <x:v>En verifierad företagsskuld är uttryckt i annan valuta än svenska kronor|Ursprungskurs och betalnings- eller balansdagskurs kan verifieras|Omräkningen ger en negativ differens som hör till skulden</x:v>
+        <x:v>En företagstillgång eller fordran är uttryckt i annan valuta än svenska kronor|Ursprungsbelopp, använd kurs och betalnings- eller balansdagskurs kan verifieras|Omräkningen ger en positiv differens som hör till verksamheten</x:v>
       </x:c>
       <x:c r="E161" s="14" t="str">
-        <x:v>Beloppet är inköp, ränta, amortering, bankavgift eller leverantörsskuldens kapitalbelopp|Differensen avser fordran, bankmedel eller placering; pröva 8330|Skulden är privat|Kurskälla eller värderingstidpunkt saknas|Valutasäkring förekommer utan särskild bedömning</x:v>
+        <x:v>Beloppet är ursprunglig försäljningsintäkt, ränta eller bankavgift|Differensen avser leverantörsskuld eller lån; pröva 8430|Tillgången eller placeringen är privat|Kursen eller värderingstidpunkten saknas|Beloppet uppkommer genom spekulation eller säkring utan särskild bedömning</x:v>
       </x:c>
       <x:c r="F161" s="14" t="str">
-        <x:v>Identifiera valuta, ursprungstransaktion, skuld, transaktionsdatum, ursprungskurs, regleringsdatum eller balansdag och kurskälla|Räkna om ursprungshändelsen enligt avistakurs eller tillåten approximation|Beräkna realiserad differens när skulden betalas och stäng leverantörs- eller låneposten|Pröva separat om oreglerad skuld ska räknas om vid bokslutet enligt tillämplig K1- och skatteregel|Bokför negativ differens på 8430 enligt fastställd kontomodell|Bokför positiv differens på 8330 eller enligt beslutad symmetrisk modell|Separera ränta, amortering och bankavgift|Stäm av per valuta mot reskontra, låneunderlag och kurskälla|Kräv manuell granskning vid säkring, närstående, flera valutor eller större kursrörelse|Använd för verifierad negativ realiserad eller orealiserad valutakursdifferens|Spara samma valutadata som för 8330|Vid granskningsflagga begär in ursprungsfaktura eller skuld, betalningsunderlag, valuta, datum och dokumenterad kurskälla|Sätt ärendet till väntar på underlag tills ursprungskurs, betalnings- eller bokslutskurs och negativ differens är verifierade|Godkänn 8430 för en enkel dokumenterad negativ valutakursdifferens som hör till verksamheten|Föreslå 8330, privat post, rätt period eller scope-eskalering vid positiv differens, säkring eller komplicerad flervalutahantering</x:v>
+        <x:v>Identifiera valuta, ursprungstransaktion, transaktionsdatum, ursprungskurs, regleringsdatum eller balansdag och använd kurskälla|Räkna om den ursprungliga affärshändelsen enligt avistakurs eller tillåten approximation|Beräkna realiserad differens vid betalning och dokumentera återföring av fordran|Pröva separat om oreglerade fordringar och bankmedel ska räknas om vid bokslutet enligt tillämplig K1- och skatteregel|Bokför endast positiv nettodifferens på 8330 enligt fastställd kontomodell|Bokför negativ differens på 8430 när den hör till skuldkostnad eller enligt beslutad symmetrisk modell|Håll ränta och bankavgift separata|Stäm av per valuta och mot reskontra, bank och kurskälla|Kräv manuell granskning vid valutasäkring, kryptotillgång, utländsk placering eller större kursrörelse|Använd för verifierad positiv realiserad eller orealiserad valutakursdifferens|Spara ursprungskurs, betalnings- eller bokslutskurs, källa och transaktionskoppling|Vid granskningsflagga begär in ursprungsfaktura eller fordran, betalningsunderlag, valuta, datum och dokumenterad kurskälla|Sätt ärendet till väntar på underlag tills ursprungskurs, betalnings- eller bokslutskurs och positiv differens är verifierade|Godkänn 8330 för en enkel dokumenterad positiv valutakursdifferens som hör till verksamheten|Föreslå 8430, privat post, rätt period eller scope-eskalering vid negativ differens, säkring, kryptotillgång eller komplicerad flervalutahantering</x:v>
       </x:c>
       <x:c r="G161" s="14" t="str">
-        <x:v>2440|2330|2350|2390|2900|1930</x:v>
+        <x:v>1500|1600|1920|1930|1940|1970|1300</x:v>
       </x:c>
       <x:c r="H161" s="14" t="str">
-        <x:v>En leverantörsskuld i euro betalas när euron blivit dyrare; den negativa differensen bokförs på 8430</x:v>
+        <x:v>En kundfordran i euro betalas när kronkursen är högre än vid faktureringen; den positiva differensen bokförs på 8330</x:v>
       </x:c>
       <x:c r="I161" s="14" t="str">
-        <x:v>Ursprunglig kostnad får inte dubbelbokföras som kursdifferens|Kurskälla och datum måste sparas|Privata skulder ska inte ingå|Positiva och negativa differenser måste behandlas konsekvent|Bankavgift, växlingspåslag och valutasäkring ska behandlas separat</x:v>
+        <x:v>Ursprunglig intäkt ska inte bokföras om som kursdifferens|Kurskälla och datum måste sparas|Privata placeringar ska inte ingå|Positiv och negativ differens måste hanteras konsekvent|Nettning över olika transaktioner är inte tillåten|Växlingspåslag är inte kursdifferens</x:v>
       </x:c>
       <x:c r="J161" s="14" t="str">
-        <x:v>valutakursförlust|kursdifferens|leverantörsskuld|lån|utländsk valuta|R8</x:v>
+        <x:v>valutakursvinst|kursdifferens|fordran|bankkonto|utländsk valuta|R4</x:v>
       </x:c>
       <x:c r="K161" s="14" t="str">
-        <x:v>8330|2440|2330|2350|2390|2900|8410</x:v>
+        <x:v>8430|1500|1600|1920|1930|1940|1970|8310</x:v>
       </x:c>
       <x:c r="L161" s="14" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8430, rad R8|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, punkterna 2.4–2.7 om omräkning till redovisningsvaluta|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 6 och 7</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8330, rad R4|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, punkterna 2.4–2.7 om omräkning till redovisningsvaluta|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 6 och 7</x:v>
       </x:c>
       <x:c r="M161" s="14" t="str">
-        <x:v>Kurskälla eller värderingstidpunkt saknas|Skulden kan vara privat|Orealiserad bokslutsdifferens förekommer|Valutasäkring eller flera valutor förekommer|Det är oklart om positiv differens ska nettas eller bokföras på 8330|Kurskälla, realisationsstatus eller säkringsinstrument är oklart</x:v>
+        <x:v>Kurskälla eller värderingstidpunkt saknas|Tillgången kan vara privat eller otillåten placering|Orealiserad bokslutsdifferens förekommer|Valutasäkring eller flera valutor förekommer|Det är oklart om negativ differens ska nettas eller bokföras på 8430|Kurskälla, realisationsstatus eller säkringsinstrument är oklart</x:v>
       </x:c>
       <x:c r="N161" s="14" t="str">
         <x:v>active</x:v>
@@ -8793,43 +8795,43 @@
     </x:row>
     <x:row r="162">
       <x:c r="A162" t="str">
-        <x:v>8990</x:v>
+        <x:v>8410</x:v>
       </x:c>
       <x:c r="B162" t="str">
-        <x:v>Resultat</x:v>
+        <x:v>Räntekostnader för skulder</x:v>
       </x:c>
       <x:c r="C162" t="str">
-        <x:v>Tekniskt importkonto för resultatposter från källsystem som använder 8990. Enkla Bokslut skapar inte nya bokningar på kontot utan använder 8999 som enda konto för resultatstängningen.</x:v>
+        <x:v>Kostnadskonto på R8 för ränta på lån och andra skulder som hör till näringsverksamheten.</x:v>
       </x:c>
       <x:c r="D162" t="str">
-        <x:v>En importerad SIE-fil innehåller saldo eller bokning på 8990 som måste stämmas av mot resultatrapporten och 8999</x:v>
+        <x:v>Skulden är bokförd eller på annat sätt verifierad som företagsskuld|Räntan kan skiljas från amortering och avgifter|Kostnaden hör till verksamheten och rätt period|Långivare, kapitalbelopp, räntesats och betalning kan verifieras</x:v>
       </x:c>
       <x:c r="E162" t="str">
-        <x:v>Systemet ska avsluta årets resultat|En ny manuell resultatbokning ska skapas|8990 och 8999 används parallellt för samma resultat</x:v>
+        <x:v>Beloppet är amortering; minska skuldkontot|Beloppet är bank- eller serviceavgift som inte är ränta eller annan utgift för kredit|Skulden eller räntan är privat|Beloppet är företagarens skatt eller ränta på privat skattekonto|Posten är en valutakursdifferens eller annan orealiserad värdeförändring som ska klassificeras separat|Räntebelopp eller period kan inte skiljas från övrig betalning</x:v>
       </x:c>
       <x:c r="F162" t="str">
-        <x:v>Flagga varje importerat saldo eller bokning på 8990 för manuell avstämning|Begär resultatrapport, bokslutsverifikation och uppgift om källsystemets avslutningsrutin|Sätt ärendet till väntar på underlag tills relationen mellan 8990, 8999 och 2019 är verifierad|Om 8990 avser samma resultat som 8999: omklassificera eller neutralisera posten utan dubbelräkning|Systemets nya resultatstängning ska alltid använda 8999 och därefter 2019|Godkänn endast när 8990 är noll efter avstämningen</x:v>
+        <x:v>Identifiera skuld, långivare, kapitaldel, räntedel, avgifter, period och betalningsdatum|Fördela lån som används både privat och i företaget enligt dokumenterad användning|Bokför betald företagsränta på 8410 och amortering mot 2330, 2350 eller 2390|Ta upp upplupen ränteutgift på 2900 när den sammanlagt överstiger 5 000 kronor enligt K1|Ta upp förutbetald ränteutgift på 1600 när den hör till nästa år och gränsen överskrids|Stäm av mot lånebesked, amorteringsplan, bank och B13/B16|Separera valutakursdifferens på 8430|BAS 8417, 8423, 8424, 8480 och 8490 får inte mappas automatiskt utan kräver manuell klassificering|BAS 8450 och 8451 ska granskas mot 8430 eller annan relevant hantering och får inte automatiskt behandlas som ränta|BAS 8411 hör inte till en vanlig K1-enskild firma och BAS 8412 ligger utanför tjänstens scope|Märk ej avdragsgill eller privat ränta för skattemässig justering eller eget uttag i stället för vanlig avdragsgill räntekostnad|Kräv manuell granskning vid närstående lån, blandad användning, utländsk skuld, byggnadskreditiv eller kapitaliserad ränta</x:v>
       </x:c>
       <x:c r="G162" t="str">
-        <x:v>8999|2019</x:v>
+        <x:v>2330|2350|2390|2900|1600|1930</x:v>
       </x:c>
       <x:c r="H162" t="str">
-        <x:v>Importerat 8990-saldo stäms av och förs in i den beslutade 8999/2019-kedjan</x:v>
+        <x:v>En lånebetalning delas mellan amortering mot 2350 och ränta på 8410|Upplupen företagsränta över K1-gränsen bokförs mot 2900 vid bokslutet|Ränta från BAS 8423 granskas för att skilja avdragsgill företagsränta från ej avdragsgill eller privat skatteränta|En post på BAS 8450 eller 8451 granskas och förs vid valutakursdifferens till 8430 i stället för 8410</x:v>
       </x:c>
       <x:c r="I162" t="str">
-        <x:v>Systemet får aldrig skapa både 8990 och 8999 för samma årsresultat</x:v>
+        <x:v>Amortering är inte kostnad|Endast företagets räntedel får belasta R8|Utgiftsränta på skattekontot är inte skattemässigt avdragsgill|Periodiseringströskeln gäller den fysiska personens samtliga verksamheter totalt|Avgifter, valutakursdifferenser och orealiserade värdeförändringar ska hållas isär från ränta|Hela bankdragningen får inte bokföras som ränta</x:v>
       </x:c>
       <x:c r="J162" t="str">
-        <x:v>resultat|bokslut|R11|samlingskonto|resultatomföring</x:v>
+        <x:v>räntekostnad|lån|amortering|upplupen ränta|förutbetald ränta|R8</x:v>
       </x:c>
       <x:c r="K162" t="str">
-        <x:v>8999|2019|2010</x:v>
+        <x:v>2330|2350|2390|2900|1600|8430|2013</x:v>
       </x:c>
       <x:c r="L162" t="str">
-        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8990, rad R11|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 5 och bilaga 2|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om bokslutstransaktioner, systemdokumentation och behandlingshistorik</x:v>
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8410, rad R8|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, punkterna 3.17, 6.59, 6.73 och 7.11 samt exempel 3-4 och 7-4|Skatteverket – Ränteutgifter, kontrollerat 2026-09-20</x:v>
       </x:c>
       <x:c r="M162" t="str">
-        <x:v>Varje saldo eller bokning på 8990|Källsystemets avslutningskedja eller relationen till 8999 är oklar</x:v>
+        <x:v>Skulden kan vara privat eller blandad|Amortering och ränta är inte separerade|Upplupen eller förutbetald ränta kan behöva periodiseras|Närstående eller utländsk långivare förekommer|Posten kommer från BAS 8417, 8423, 8424, 8480 eller 8490|Posten kommer från BAS 8450 eller 8451 och klassificeringen mot 8430 är inte verifierad|Avgiften kan vara annat än ränta eller den skattemässiga avdragsrätten är oklar</x:v>
       </x:c>
       <x:c r="N162" t="str">
         <x:v>active</x:v>
@@ -8837,63 +8839,157 @@
       <x:c r="O162" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P162" s="14" t="str"/>
+      <x:c r="P162" s="14" t="str">
+        <x:v>accrued_interest_expense_over_5000|prepaid_interest_expense_over_5000</x:v>
+      </x:c>
       <x:c r="Q162" s="12" t="str"/>
     </x:row>
-    <x:row r="163">
-      <x:c r="A163" t="str">
+    <x:row r="163" ht="430" customHeight="1">
+      <x:c r="A163" s="14" t="str">
+        <x:v>8430</x:v>
+      </x:c>
+      <x:c r="B163" s="14" t="str">
+        <x:v>Valutakursdifferenser på skulder</x:v>
+      </x:c>
+      <x:c r="C163" s="14" t="str">
+        <x:v>Kostnadskonto på R8 för negativa valutakursdifferenser på företagets leverantörsskulder, lån och andra skulder i utländsk valuta.</x:v>
+      </x:c>
+      <x:c r="D163" s="14" t="str">
+        <x:v>En verifierad företagsskuld är uttryckt i annan valuta än svenska kronor|Ursprungskurs och betalnings- eller balansdagskurs kan verifieras|Omräkningen ger en negativ differens som hör till skulden</x:v>
+      </x:c>
+      <x:c r="E163" s="14" t="str">
+        <x:v>Beloppet är inköp, ränta, amortering, bankavgift eller leverantörsskuldens kapitalbelopp|Differensen avser fordran, bankmedel eller placering; pröva 8330|Skulden är privat|Kurskälla eller värderingstidpunkt saknas|Valutasäkring förekommer utan särskild bedömning</x:v>
+      </x:c>
+      <x:c r="F163" s="14" t="str">
+        <x:v>Identifiera valuta, ursprungstransaktion, skuld, transaktionsdatum, ursprungskurs, regleringsdatum eller balansdag och kurskälla|Räkna om ursprungshändelsen enligt avistakurs eller tillåten approximation|Beräkna realiserad differens när skulden betalas och stäng leverantörs- eller låneposten|Pröva separat om oreglerad skuld ska räknas om vid bokslutet enligt tillämplig K1- och skatteregel|Bokför negativ differens på 8430 enligt fastställd kontomodell|Bokför positiv differens på 8330 eller enligt beslutad symmetrisk modell|Separera ränta, amortering och bankavgift|Stäm av per valuta mot reskontra, låneunderlag och kurskälla|Kräv manuell granskning vid säkring, närstående, flera valutor eller större kursrörelse|Använd för verifierad negativ realiserad eller orealiserad valutakursdifferens|Spara samma valutadata som för 8330|Vid granskningsflagga begär in ursprungsfaktura eller skuld, betalningsunderlag, valuta, datum och dokumenterad kurskälla|Sätt ärendet till väntar på underlag tills ursprungskurs, betalnings- eller bokslutskurs och negativ differens är verifierade|Godkänn 8430 för en enkel dokumenterad negativ valutakursdifferens som hör till verksamheten|Föreslå 8330, privat post, rätt period eller scope-eskalering vid positiv differens, säkring eller komplicerad flervalutahantering</x:v>
+      </x:c>
+      <x:c r="G163" s="14" t="str">
+        <x:v>2440|2330|2350|2390|2900|1930</x:v>
+      </x:c>
+      <x:c r="H163" s="14" t="str">
+        <x:v>En leverantörsskuld i euro betalas när euron blivit dyrare; den negativa differensen bokförs på 8430</x:v>
+      </x:c>
+      <x:c r="I163" s="14" t="str">
+        <x:v>Ursprunglig kostnad får inte dubbelbokföras som kursdifferens|Kurskälla och datum måste sparas|Privata skulder ska inte ingå|Positiva och negativa differenser måste behandlas konsekvent|Bankavgift, växlingspåslag och valutasäkring ska behandlas separat</x:v>
+      </x:c>
+      <x:c r="J163" s="14" t="str">
+        <x:v>valutakursförlust|kursdifferens|leverantörsskuld|lån|utländsk valuta|R8</x:v>
+      </x:c>
+      <x:c r="K163" s="14" t="str">
+        <x:v>8330|2440|2330|2350|2390|2900|8410</x:v>
+      </x:c>
+      <x:c r="L163" s="14" t="str">
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8430, rad R8|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, punkterna 2.4–2.7 om omräkning till redovisningsvaluta|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 6 och 7</x:v>
+      </x:c>
+      <x:c r="M163" s="14" t="str">
+        <x:v>Kurskälla eller värderingstidpunkt saknas|Skulden kan vara privat|Orealiserad bokslutsdifferens förekommer|Valutasäkring eller flera valutor förekommer|Det är oklart om positiv differens ska nettas eller bokföras på 8330|Kurskälla, realisationsstatus eller säkringsinstrument är oklart</x:v>
+      </x:c>
+      <x:c r="N163" s="14" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="O163" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P163" s="14"/>
+      <x:c r="Q163" s="14" t="str"/>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>8990</x:v>
+      </x:c>
+      <x:c r="B164" t="str">
+        <x:v>Resultat</x:v>
+      </x:c>
+      <x:c r="C164" t="str">
+        <x:v>Tekniskt importkonto för resultatposter från källsystem som använder 8990. Enkla Bokslut skapar inte nya bokningar på kontot utan använder 8999 som enda konto för resultatstängningen.</x:v>
+      </x:c>
+      <x:c r="D164" t="str">
+        <x:v>En importerad SIE-fil innehåller saldo eller bokning på 8990 som måste stämmas av mot resultatrapporten och 8999</x:v>
+      </x:c>
+      <x:c r="E164" t="str">
+        <x:v>Systemet ska avsluta årets resultat|En ny manuell resultatbokning ska skapas|8990 och 8999 används parallellt för samma resultat</x:v>
+      </x:c>
+      <x:c r="F164" t="str">
+        <x:v>Flagga varje importerat saldo eller bokning på 8990 för manuell avstämning|Begär resultatrapport, bokslutsverifikation och uppgift om källsystemets avslutningsrutin|Sätt ärendet till väntar på underlag tills relationen mellan 8990, 8999 och 2019 är verifierad|Om 8990 avser samma resultat som 8999: omklassificera eller neutralisera posten utan dubbelräkning|Systemets nya resultatstängning ska alltid använda 8999 och därefter 2019|Godkänn endast när 8990 är noll efter avstämningen</x:v>
+      </x:c>
+      <x:c r="G164" t="str">
+        <x:v>8999|2019</x:v>
+      </x:c>
+      <x:c r="H164" t="str">
+        <x:v>Importerat 8990-saldo stäms av och förs in i den beslutade 8999/2019-kedjan</x:v>
+      </x:c>
+      <x:c r="I164" t="str">
+        <x:v>Systemet får aldrig skapa både 8990 och 8999 för samma årsresultat</x:v>
+      </x:c>
+      <x:c r="J164" t="str">
+        <x:v>resultat|bokslut|R11|samlingskonto|resultatomföring</x:v>
+      </x:c>
+      <x:c r="K164" t="str">
+        <x:v>8999|2019|2010</x:v>
+      </x:c>
+      <x:c r="L164" t="str">
+        <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8990, rad R11|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, kapitel 5 och bilaga 2|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, reglerna om bokslutstransaktioner, systemdokumentation och behandlingshistorik</x:v>
+      </x:c>
+      <x:c r="M164" t="str">
+        <x:v>Varje saldo eller bokning på 8990|Källsystemets avslutningskedja eller relationen till 8999 är oklar</x:v>
+      </x:c>
+      <x:c r="N164" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="O164" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P164" s="14" t="str"/>
+      <x:c r="Q164" s="12" t="str"/>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" t="str">
         <x:v>8999</x:v>
       </x:c>
-      <x:c r="B163" t="str">
+      <x:c r="B165" t="str">
         <x:v>Årets resultat</x:v>
       </x:c>
-      <x:c r="C163" t="str">
+      <x:c r="C165" t="str">
         <x:v>Tekniskt bokslutskonto på R11 för räkenskapsårets slutliga bokförda vinst eller förlust. Kontot används när resultatkontona avslutas och resultatet förs till 2019 Årets resultat, delägare 1.</x:v>
       </x:c>
-      <x:c r="D163" t="str">
+      <x:c r="D165" t="str">
         <x:v>Samtliga intäkts- och kostnadskonton är avstämda och bokslutstransaktionerna är färdiga|Räkenskapsårets resultat enligt R11 är fastställt|En spårbar bokslutsverifikation ska avsluta resultatkontona och föra resultatet till eget kapital|Systemets beslutade avslutningsrutin använder 8999 som bokningskonto</x:v>
       </x:c>
-      <x:c r="E163" t="str">
+      <x:c r="E165" t="str">
         <x:v>En vanlig affärshändelse eller rättelse bokförs|Resultatet är preliminärt eller balansräkningen är inte avstämd|Beloppet avser eget uttag, egen insättning, skatt eller fondavsättning|Systemets avslutningsrutin använder 8990 som bokningskonto och 8999 endast som underkonto eller rapportkonto|Resultatet ska fördelas mellan flera deltagare utan dokumenterad fördelningsgrund</x:v>
       </x:c>
-      <x:c r="F163" t="str">
+      <x:c r="F165" t="str">
         <x:v>Beräkna årets bokförda resultat efter att alla poster på R1–R10 har stämts av|Kontrollera att resultatet motsvarar R11 i det förenklade årsbokslutet|Skapa en separat och reproducerbar bokslutsverifikation för avslutningen|Avsluta samtliga intäkts- och kostnadskonton mot 8999 enligt systemets fastställda rutin|I en rutin där 8999 används som bokningskonto får en vinst ett kreditsaldo på 8999 före överföringen och förs därefter med debet 8999 och kredit 2019|En förlust får ett debetsaldo på 8999 före överföringen och förs därefter med kredit 8999 och debet 2019|Kontrollera att 8999 är noll efter överföringen till eget kapital|Kontrollera att 2019 överensstämmer med årets resultat och att tillgångar minus skulder motsvarar eget kapital|För nästa år förs 2019 vidare till 2010 enligt den beslutade årsomföringsrutinen|Bokför inte både 8990 och 8999 för samma resultat om detta skapar dubbelräkning|Använd endast inom verifierad slutlig resultatbokning|Koppla till 2019 och efterföljande årsomföring till 2010|Använd 8999 som systemets enda konto för den slutliga resultatstängningen; systemet ska inte samtidigt skapa en bokning på 8990|Stäng intäkts- och kostnadskontona mot 8999 först när samtliga bokslutsposter och R1–R10 är avstämda|Kontrollera att saldot på 8999 motsvarar R11 och för därefter hela saldot till 2019 med motsatt bokning|Godkänn bokslutet först när 8999 är noll, 2019 motsvarar årets resultat och stängningsverifikationen bara finns en gång</x:v>
       </x:c>
-      <x:c r="G163" t="str">
+      <x:c r="G165" t="str">
         <x:v>8990|2019|2010</x:v>
       </x:c>
-      <x:c r="H163" t="str">
+      <x:c r="H165" t="str">
         <x:v>Vid vinst avslutas resultatkontona så att 8999 får ett kreditsaldo; därefter debiteras 8999 och 2019 krediteras|Vid förlust får 8999 ett debetsaldo; därefter krediteras 8999 och 2019 debiteras</x:v>
       </x:c>
-      <x:c r="I163" t="str">
+      <x:c r="I165" t="str">
         <x:v>8999 är ett tekniskt avslutningskonto och inte en löpande intäkt eller kostnad|Kontot ska normalt vara noll efter resultatöverföringen|8990 och 8999 får inte båda ge resultatpåverkan|Resultatfördelning mellan flera deltagare måste beslutas innan överföringen|Ändringar efter avslutad bokslutsverifikation kräver att hela avslutningskedjan görs om och stäms av|Får inte skapa dubbelbokning med 8990</x:v>
       </x:c>
-      <x:c r="J163" t="str">
+      <x:c r="J165" t="str">
         <x:v>årets resultat|bokslut|resultatöverföring|R11|8999|2019|eget kapital|årsomföring</x:v>
       </x:c>
-      <x:c r="K163" t="str">
+      <x:c r="K165" t="str">
         <x:v>8990|2019|2010|2020|2030|2040</x:v>
       </x:c>
-      <x:c r="L163" t="str">
+      <x:c r="L165" t="str">
         <x:v>BAS Förenklat årsbokslut (K1) – Kontoplan 2018, sida 9, konto 8999, rad R11|BFNAR 2006:1, K1-vägledningen uppdaterad 2025-03-24, bilaga 2 och exempel 5-1 om resultat och eget kapital|BFNAR 2013:2, vägledningen Bokföring uppdaterad 2024-09-16, avsnitten om bokslutstransaktioner, rättelser och systemdokumentation</x:v>
       </x:c>
-      <x:c r="M163" t="str">
+      <x:c r="M165" t="str">
         <x:v>Avslutningsrutinen mellan 8990, 8999, 2019 och 2010 är inte fastställd|R11 stämmer inte med resultaträkningen|8999 är inte noll efter resultatöverföringen|Bokslutsverifikation eller avstämning saknas|Flera deltagare eller resultatandelar förekommer|Bokningskonto, tecken eller nollkontroll är inte verifierad</x:v>
       </x:c>
-      <x:c r="N163" t="str">
-        <x:v>active</x:v>
-      </x:c>
-      <x:c r="O163" t="n">
+      <x:c r="N165" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="O165" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P163" s="14"/>
-      <x:c r="Q163" s="12" t="str"/>
-    </x:row>
-    <x:row r="164">
-      <x:c r="P164" s="14"/>
-    </x:row>
-    <x:row r="165">
       <x:c r="P165" s="14"/>
+      <x:c r="Q165" s="12" t="str"/>
     </x:row>
     <x:row r="166">
       <x:c r="P166" s="14"/>
@@ -11400,9 +11496,15 @@
     <x:row r="1000">
       <x:c r="P1000" s="14"/>
     </x:row>
+    <x:row r="1001">
+      <x:c r="P1001" s="14"/>
+    </x:row>
+    <x:row r="1002">
+      <x:c r="P1002" s="14"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="N2:N1000">
+    <x:dataValidation type="list" sqref="N2:N1002">
       <x:formula1>"draft,reviewed,active"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>